<commit_message>
feat: integrate PyTorch 2-layer LSTM sequence model into quant forecasting ensemble
</commit_message>
<xml_diff>
--- a/Breakout_ML_Quant_Predictions.xlsx
+++ b/Breakout_ML_Quant_Predictions.xlsx
@@ -719,13 +719,13 @@
         <v>11.76</v>
       </c>
       <c r="S2" t="n">
-        <v>61.1</v>
+        <v>61.6</v>
       </c>
       <c r="T2" t="n">
         <v>0.32</v>
       </c>
       <c r="U2" t="n">
-        <v>-0.5</v>
+        <v>-0.48</v>
       </c>
       <c r="V2" t="n">
         <v>60</v>
@@ -784,10 +784,10 @@
         <v>16.1</v>
       </c>
       <c r="AN2" t="n">
-        <v>1461.04</v>
+        <v>1463.1</v>
       </c>
       <c r="AO2" t="n">
-        <v>1409.93</v>
+        <v>1409.05</v>
       </c>
       <c r="AP2" t="inlineStr">
         <is>
@@ -886,7 +886,7 @@
         <v>11.76</v>
       </c>
       <c r="S3" t="n">
-        <v>55.9</v>
+        <v>55.8</v>
       </c>
       <c r="T3" t="n">
         <v>0.39</v>
@@ -951,10 +951,10 @@
         <v>15</v>
       </c>
       <c r="AN3" t="n">
-        <v>8039.51</v>
+        <v>8057.14</v>
       </c>
       <c r="AO3" t="n">
-        <v>7636.76</v>
+        <v>7648.5</v>
       </c>
       <c r="AP3" t="inlineStr">
         <is>
@@ -1053,7 +1053,7 @@
         <v>11.76</v>
       </c>
       <c r="S4" t="n">
-        <v>58.6</v>
+        <v>58.8</v>
       </c>
       <c r="T4" t="n">
         <v>0.29</v>
@@ -1118,10 +1118,10 @@
         <v>15</v>
       </c>
       <c r="AN4" t="n">
-        <v>115.79</v>
+        <v>116.18</v>
       </c>
       <c r="AO4" t="n">
-        <v>109.46</v>
+        <v>109.62</v>
       </c>
       <c r="AP4" t="inlineStr">
         <is>
@@ -1220,7 +1220,7 @@
         <v>11.76</v>
       </c>
       <c r="S5" t="n">
-        <v>57.6</v>
+        <v>57.8</v>
       </c>
       <c r="T5" t="n">
         <v>0.29</v>
@@ -1285,10 +1285,10 @@
         <v>15</v>
       </c>
       <c r="AN5" t="n">
-        <v>12178.66</v>
+        <v>12177.9</v>
       </c>
       <c r="AO5" t="n">
-        <v>11640.57</v>
+        <v>11645.22</v>
       </c>
       <c r="AP5" t="inlineStr">
         <is>
@@ -1387,13 +1387,13 @@
         <v>11.76</v>
       </c>
       <c r="S6" t="n">
-        <v>58.3</v>
+        <v>57.7</v>
       </c>
       <c r="T6" t="n">
         <v>0.25</v>
       </c>
       <c r="U6" t="n">
-        <v>-0.86</v>
+        <v>-0.88</v>
       </c>
       <c r="V6" t="n">
         <v>55</v>
@@ -1405,10 +1405,10 @@
         <v>-0.77</v>
       </c>
       <c r="Y6" t="n">
-        <v>2707.04</v>
+        <v>2707.02</v>
       </c>
       <c r="Z6" t="n">
-        <v>2803.2</v>
+        <v>2803.18</v>
       </c>
       <c r="AA6" t="n">
         <v>2769.28</v>
@@ -1452,10 +1452,10 @@
         <v>15</v>
       </c>
       <c r="AN6" t="n">
-        <v>2814.38</v>
+        <v>2816.91</v>
       </c>
       <c r="AO6" t="n">
-        <v>2686.78</v>
+        <v>2683.26</v>
       </c>
       <c r="AP6" t="inlineStr">
         <is>
@@ -1554,13 +1554,13 @@
         <v>11.76</v>
       </c>
       <c r="S7" t="n">
-        <v>56.3</v>
+        <v>55.5</v>
       </c>
       <c r="T7" t="n">
         <v>0.25</v>
       </c>
       <c r="U7" t="n">
-        <v>-0.96</v>
+        <v>-0.99</v>
       </c>
       <c r="V7" t="n">
         <v>50</v>
@@ -1619,10 +1619,10 @@
         <v>11.6</v>
       </c>
       <c r="AN7" t="n">
-        <v>2268.06</v>
+        <v>2264.99</v>
       </c>
       <c r="AO7" t="n">
-        <v>2144.03</v>
+        <v>2137.47</v>
       </c>
       <c r="AP7" t="inlineStr">
         <is>
@@ -1663,16 +1663,16 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>INDHOTEL</t>
+          <t>RECLTD</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>105127.58</v>
+        <v>98206.09</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1680,145 +1680,145 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>738.55</v>
+        <v>372.95</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>₹735.6 - ₹742.98</t>
+          <t>₹371.41 - ₹375.26</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>750.37</v>
+        <v>379.11</v>
       </c>
       <c r="I8" t="n">
-        <v>225</v>
+        <v>432</v>
       </c>
       <c r="J8" t="n">
-        <v>729.51</v>
+        <v>357.21</v>
       </c>
       <c r="K8" t="n">
-        <v>703.6799999999999</v>
+        <v>349.78</v>
       </c>
       <c r="L8" t="n">
-        <v>686.09</v>
+        <v>347.56</v>
       </c>
       <c r="M8" t="n">
-        <v>9.210000000000001</v>
+        <v>6.64</v>
       </c>
       <c r="N8" t="n">
-        <v>8.49</v>
+        <v>4.07</v>
       </c>
       <c r="O8" t="n">
-        <v>9.380000000000001</v>
+        <v>2.35</v>
       </c>
       <c r="P8" t="n">
-        <v>-0.9</v>
+        <v>1.72</v>
       </c>
       <c r="Q8" t="n">
-        <v>14.77</v>
+        <v>7.7</v>
       </c>
       <c r="R8" t="n">
         <v>11.76</v>
       </c>
       <c r="S8" t="n">
-        <v>51.9</v>
+        <v>53</v>
       </c>
       <c r="T8" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="U8" t="n">
         <v>-1.03</v>
       </c>
       <c r="V8" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="W8" t="n">
-        <v>5.75</v>
+        <v>2.81</v>
       </c>
       <c r="X8" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y8" t="n">
-        <v>720.8200000000001</v>
+        <v>366.16</v>
       </c>
       <c r="Z8" t="n">
-        <v>725.27</v>
+        <v>379.22</v>
       </c>
       <c r="AA8" t="n">
-        <v>744.46</v>
+        <v>375.93</v>
       </c>
       <c r="AB8" t="n">
-        <v>716.39</v>
+        <v>361.4</v>
       </c>
       <c r="AC8" t="n">
-        <v>744.27</v>
+        <v>372.32</v>
       </c>
       <c r="AD8" t="n">
-        <v>751.6900000000001</v>
+        <v>374.64</v>
       </c>
       <c r="AE8" t="n">
-        <v>764.8200000000001</v>
+        <v>376.32</v>
       </c>
       <c r="AF8" t="n">
-        <v>48.2</v>
+        <v>78.3</v>
       </c>
       <c r="AG8" t="n">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (11.76)</t>
+          <t>Low VIX (11.76)</t>
         </is>
       </c>
       <c r="AI8" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ8" t="n">
-        <v>49</v>
+        <v>6.1</v>
       </c>
       <c r="AK8" t="n">
-        <v>15.1</v>
+        <v>25.2</v>
       </c>
       <c r="AL8" t="n">
-        <v>20.9</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="AM8" t="n">
         <v>15</v>
       </c>
       <c r="AN8" t="n">
-        <v>756.42</v>
+        <v>382.62</v>
       </c>
       <c r="AO8" t="n">
-        <v>720.72</v>
+        <v>363.2</v>
       </c>
       <c r="AP8" t="inlineStr">
         <is>
-          <t>INDHOTEL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹105,127.58 Cr., a P/E ratio of 49.01, and YoY Revenue Growth of +15.1%, the company demonstrates strong institutional backing, solid operating profit margins (20.87%), and healthy Return on Equity (15.00%).</t>
+          <t>RECLTD operates in the Financial Services sector. With an estimated Market Cap of ₹98,206.09 Cr., a P/E ratio of 6.14, and YoY Revenue Growth of +25.2%, the company demonstrates strong institutional backing, solid operating profit margins (68.89%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ8" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 48.23 (Consolidation Zone), while MACD Line (8.49) trades below Signal (9.38) with an expanding histogram (-0.90). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +9.21% above the 200-day DMA (₹686.09). Daily volatility envelope is bounded by ATR(14) of ₹14.77.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 78.30 (Bullish Momentum Zone), while MACD Line (4.07) trades above Signal (2.35) with an expanding histogram (+1.72). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +6.64% above the 200-day DMA (₹347.56). Daily volatility envelope is bounded by ATR(14) of ₹7.70.</t>
         </is>
       </c>
       <c r="AR8" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for INDHOTEL. Current Market Price (₹738.55) is positioned above the 30-day DMA (₹729.51), 50-day DMA (₹703.68), and 200-day DMA (₹686.09). The price distance from 200 DMA is +9.21%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for RECLTD. Current Market Price (₹372.95) is positioned above the 30-day DMA (₹357.21), 50-day DMA (₹349.78), and 200-day DMA (₹347.56). The price distance from 200 DMA is +6.64%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS8" t="inlineStr">
         <is>
-          <t>[738.55, 740.77, 742.98, 745.2, 747.41, 749.63]</t>
+          <t>[372.95, 374.07, 375.19, 376.31, 377.43, 378.54]</t>
         </is>
       </c>
       <c r="AT8" t="inlineStr">
         <is>
-          <t>[738.55, 746.67, 751.34, 755.43, 759.23, 762.84]</t>
+          <t>[372.95, 377.15, 379.54, 381.64, 383.59, 385.43]</t>
         </is>
       </c>
       <c r="AU8" t="inlineStr">
         <is>
-          <t>[738.55, 736.33, 736.71, 737.52, 738.55, 739.72]</t>
+          <t>[372.95, 371.76, 371.92, 372.31, 372.8, 373.38]</t>
         </is>
       </c>
     </row>
@@ -1830,16 +1830,16 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>RECLTD</t>
+          <t>INDHOTEL</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>98206.09</v>
+        <v>105127.58</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1847,145 +1847,145 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>372.95</v>
+        <v>738.55</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>₹371.41 - ₹375.26</t>
+          <t>₹735.6 - ₹742.98</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>379.11</v>
+        <v>750.37</v>
       </c>
       <c r="I9" t="n">
-        <v>432</v>
+        <v>225</v>
       </c>
       <c r="J9" t="n">
-        <v>357.21</v>
+        <v>729.51</v>
       </c>
       <c r="K9" t="n">
-        <v>349.78</v>
+        <v>703.6799999999999</v>
       </c>
       <c r="L9" t="n">
-        <v>347.56</v>
+        <v>686.09</v>
       </c>
       <c r="M9" t="n">
-        <v>6.64</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="N9" t="n">
-        <v>4.07</v>
+        <v>8.49</v>
       </c>
       <c r="O9" t="n">
-        <v>2.35</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="P9" t="n">
-        <v>1.72</v>
+        <v>-0.9</v>
       </c>
       <c r="Q9" t="n">
-        <v>7.7</v>
+        <v>14.77</v>
       </c>
       <c r="R9" t="n">
         <v>11.76</v>
       </c>
       <c r="S9" t="n">
-        <v>52.6</v>
+        <v>51.5</v>
       </c>
       <c r="T9" t="n">
-        <v>0.26</v>
+        <v>0.27</v>
       </c>
       <c r="U9" t="n">
-        <v>-1.05</v>
+        <v>-1.04</v>
       </c>
       <c r="V9" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="W9" t="n">
-        <v>2.81</v>
+        <v>5.74</v>
       </c>
       <c r="X9" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y9" t="n">
-        <v>366.16</v>
+        <v>720.8200000000001</v>
       </c>
       <c r="Z9" t="n">
-        <v>379.22</v>
+        <v>725.26</v>
       </c>
       <c r="AA9" t="n">
-        <v>375.93</v>
+        <v>744.46</v>
       </c>
       <c r="AB9" t="n">
-        <v>361.4</v>
+        <v>716.39</v>
       </c>
       <c r="AC9" t="n">
-        <v>372.32</v>
+        <v>744.27</v>
       </c>
       <c r="AD9" t="n">
-        <v>374.64</v>
+        <v>751.6900000000001</v>
       </c>
       <c r="AE9" t="n">
-        <v>376.32</v>
+        <v>764.8200000000001</v>
       </c>
       <c r="AF9" t="n">
-        <v>78.3</v>
+        <v>48.2</v>
       </c>
       <c r="AG9" t="n">
-        <v>0.08</v>
+        <v>0.04</v>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>Low VIX (11.76)</t>
+          <t>TTM Squeeze | Low VIX (11.76)</t>
         </is>
       </c>
       <c r="AI9" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ9" t="n">
-        <v>6.1</v>
+        <v>49</v>
       </c>
       <c r="AK9" t="n">
-        <v>25.2</v>
+        <v>15.1</v>
       </c>
       <c r="AL9" t="n">
-        <v>68.90000000000001</v>
+        <v>20.9</v>
       </c>
       <c r="AM9" t="n">
         <v>15</v>
       </c>
       <c r="AN9" t="n">
-        <v>383.31</v>
+        <v>757.85</v>
       </c>
       <c r="AO9" t="n">
-        <v>363.07</v>
+        <v>720.36</v>
       </c>
       <c r="AP9" t="inlineStr">
         <is>
-          <t>RECLTD operates in the Financial Services sector. With an estimated Market Cap of ₹98,206.09 Cr., a P/E ratio of 6.14, and YoY Revenue Growth of +25.2%, the company demonstrates strong institutional backing, solid operating profit margins (68.89%), and healthy Return on Equity (15.00%).</t>
+          <t>INDHOTEL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹105,127.58 Cr., a P/E ratio of 49.01, and YoY Revenue Growth of +15.1%, the company demonstrates strong institutional backing, solid operating profit margins (20.87%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ9" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 78.30 (Bullish Momentum Zone), while MACD Line (4.07) trades above Signal (2.35) with an expanding histogram (+1.72). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +6.64% above the 200-day DMA (₹347.56). Daily volatility envelope is bounded by ATR(14) of ₹7.70.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 48.23 (Consolidation Zone), while MACD Line (8.49) trades below Signal (9.38) with an expanding histogram (-0.90). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +9.21% above the 200-day DMA (₹686.09). Daily volatility envelope is bounded by ATR(14) of ₹14.77.</t>
         </is>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for RECLTD. Current Market Price (₹372.95) is positioned above the 30-day DMA (₹357.21), 50-day DMA (₹349.78), and 200-day DMA (₹347.56). The price distance from 200 DMA is +6.64%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for INDHOTEL. Current Market Price (₹738.55) is positioned above the 30-day DMA (₹729.51), 50-day DMA (₹703.68), and 200-day DMA (₹686.09). The price distance from 200 DMA is +9.21%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS9" t="inlineStr">
         <is>
-          <t>[372.95, 374.07, 375.19, 376.31, 377.43, 378.54]</t>
+          <t>[738.55, 740.77, 742.98, 745.2, 747.41, 749.63]</t>
         </is>
       </c>
       <c r="AT9" t="inlineStr">
         <is>
-          <t>[372.95, 377.15, 379.54, 381.64, 383.59, 385.43]</t>
+          <t>[738.55, 746.67, 751.34, 755.43, 759.23, 762.84]</t>
         </is>
       </c>
       <c r="AU9" t="inlineStr">
         <is>
-          <t>[372.95, 371.76, 371.92, 372.31, 372.8, 373.38]</t>
+          <t>[738.55, 736.33, 736.71, 737.52, 738.55, 739.72]</t>
         </is>
       </c>
     </row>
@@ -2055,13 +2055,13 @@
         <v>11.76</v>
       </c>
       <c r="S10" t="n">
-        <v>46</v>
+        <v>46.3</v>
       </c>
       <c r="T10" t="n">
         <v>0.3</v>
       </c>
       <c r="U10" t="n">
-        <v>-1.08</v>
+        <v>-1.07</v>
       </c>
       <c r="V10" t="n">
         <v>41.7</v>
@@ -2073,10 +2073,10 @@
         <v>-0.77</v>
       </c>
       <c r="Y10" t="n">
-        <v>4548.57</v>
+        <v>4548.62</v>
       </c>
       <c r="Z10" t="n">
-        <v>4711.2</v>
+        <v>4711.24</v>
       </c>
       <c r="AA10" t="n">
         <v>4683.67</v>
@@ -2120,10 +2120,10 @@
         <v>24</v>
       </c>
       <c r="AN10" t="n">
-        <v>4766.04</v>
+        <v>4769.63</v>
       </c>
       <c r="AO10" t="n">
-        <v>4524.12</v>
+        <v>4515.61</v>
       </c>
       <c r="AP10" t="inlineStr">
         <is>
@@ -2287,10 +2287,10 @@
         <v>17.6</v>
       </c>
       <c r="AN11" t="n">
-        <v>5882.83</v>
+        <v>5880.76</v>
       </c>
       <c r="AO11" t="n">
-        <v>5618.25</v>
+        <v>5625.04</v>
       </c>
       <c r="AP11" t="inlineStr">
         <is>
@@ -2389,13 +2389,13 @@
         <v>11.76</v>
       </c>
       <c r="S12" t="n">
-        <v>56.4</v>
+        <v>56.6</v>
       </c>
       <c r="T12" t="n">
         <v>0.21</v>
       </c>
       <c r="U12" t="n">
-        <v>-1.24</v>
+        <v>-1.23</v>
       </c>
       <c r="V12" t="n">
         <v>53.3</v>
@@ -2454,10 +2454,10 @@
         <v>15</v>
       </c>
       <c r="AN12" t="n">
-        <v>3878.18</v>
+        <v>3866.75</v>
       </c>
       <c r="AO12" t="n">
-        <v>3649.2</v>
+        <v>3645.21</v>
       </c>
       <c r="AP12" t="inlineStr">
         <is>
@@ -2556,13 +2556,13 @@
         <v>11.76</v>
       </c>
       <c r="S13" t="n">
-        <v>52.1</v>
+        <v>51.7</v>
       </c>
       <c r="T13" t="n">
         <v>0.23</v>
       </c>
       <c r="U13" t="n">
-        <v>-1.26</v>
+        <v>-1.28</v>
       </c>
       <c r="V13" t="n">
         <v>45</v>
@@ -2621,10 +2621,10 @@
         <v>15</v>
       </c>
       <c r="AN13" t="n">
-        <v>1504.82</v>
+        <v>1504.41</v>
       </c>
       <c r="AO13" t="n">
-        <v>1443.14</v>
+        <v>1443.16</v>
       </c>
       <c r="AP13" t="inlineStr">
         <is>
@@ -2723,13 +2723,13 @@
         <v>11.76</v>
       </c>
       <c r="S14" t="n">
-        <v>56.5</v>
+        <v>56</v>
       </c>
       <c r="T14" t="n">
         <v>0.18</v>
       </c>
       <c r="U14" t="n">
-        <v>-1.52</v>
+        <v>-1.54</v>
       </c>
       <c r="V14" t="n">
         <v>55</v>
@@ -2741,10 +2741,10 @@
         <v>-0.77</v>
       </c>
       <c r="Y14" t="n">
-        <v>1019.37</v>
+        <v>1019.35</v>
       </c>
       <c r="Z14" t="n">
-        <v>1056.01</v>
+        <v>1055.98</v>
       </c>
       <c r="AA14" t="n">
         <v>1055.07</v>
@@ -2788,10 +2788,10 @@
         <v>18.5</v>
       </c>
       <c r="AN14" t="n">
-        <v>1086.02</v>
+        <v>1086.01</v>
       </c>
       <c r="AO14" t="n">
-        <v>1011.32</v>
+        <v>1011.5</v>
       </c>
       <c r="AP14" t="inlineStr">
         <is>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>DIXON</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2841,7 +2841,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>146280.27</v>
+        <v>85420.58</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2849,145 +2849,145 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>1651.3</v>
+        <v>14049</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>₹1641.81 - ₹1665.54</t>
+          <t>₹13965.8 - ₹14173.8</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1689.26</v>
+        <v>14381.8</v>
       </c>
       <c r="I15" t="n">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="J15" t="n">
-        <v>1478.49</v>
+        <v>13190.57</v>
       </c>
       <c r="K15" t="n">
-        <v>1460.44</v>
+        <v>12605.68</v>
       </c>
       <c r="L15" t="n">
-        <v>1458.79</v>
+        <v>12333.95</v>
       </c>
       <c r="M15" t="n">
-        <v>14.41</v>
+        <v>16.25</v>
       </c>
       <c r="N15" t="n">
-        <v>56.22</v>
+        <v>477.1</v>
       </c>
       <c r="O15" t="n">
-        <v>42.84</v>
+        <v>503.84</v>
       </c>
       <c r="P15" t="n">
-        <v>13.38</v>
+        <v>-26.74</v>
       </c>
       <c r="Q15" t="n">
-        <v>47.45</v>
+        <v>416</v>
       </c>
       <c r="R15" t="n">
         <v>11.76</v>
       </c>
       <c r="S15" t="n">
-        <v>49.7</v>
+        <v>51.1</v>
       </c>
       <c r="T15" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="U15" t="n">
-        <v>-1.77</v>
+        <v>-1.76</v>
       </c>
       <c r="V15" t="n">
-        <v>48.3</v>
+        <v>46.7</v>
       </c>
       <c r="W15" t="n">
-        <v>8.69</v>
+        <v>6.67</v>
       </c>
       <c r="X15" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y15" t="n">
-        <v>1625.39</v>
+        <v>13634.58</v>
       </c>
       <c r="Z15" t="n">
-        <v>1683.18</v>
+        <v>14126.3</v>
       </c>
       <c r="AA15" t="n">
-        <v>1664.51</v>
+        <v>14161.39</v>
       </c>
       <c r="AB15" t="n">
-        <v>1580.13</v>
+        <v>13425</v>
       </c>
       <c r="AC15" t="n">
-        <v>1641.1</v>
+        <v>14079.67</v>
       </c>
       <c r="AD15" t="n">
-        <v>1671.7</v>
+        <v>14558.34</v>
       </c>
       <c r="AE15" t="n">
-        <v>1692.1</v>
+        <v>15067.67</v>
       </c>
       <c r="AF15" t="n">
-        <v>86.2</v>
+        <v>64.7</v>
       </c>
       <c r="AG15" t="n">
-        <v>0.06</v>
+        <v>0.11</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>Low VIX (11.76)</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (11.76)</t>
         </is>
       </c>
       <c r="AI15" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ15" t="n">
-        <v>28.6</v>
+        <v>41.2</v>
       </c>
       <c r="AK15" t="n">
-        <v>17.7</v>
+        <v>21.1</v>
       </c>
       <c r="AL15" t="n">
-        <v>8.699999999999999</v>
+        <v>3.6</v>
       </c>
       <c r="AM15" t="n">
         <v>15</v>
       </c>
       <c r="AN15" t="n">
-        <v>1694.41</v>
+        <v>14572.92</v>
       </c>
       <c r="AO15" t="n">
-        <v>1604.92</v>
+        <v>13548.3</v>
       </c>
       <c r="AP15" t="inlineStr">
         <is>
-          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹146,280.27 Cr., a P/E ratio of 28.57, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
+          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹85,420.58 Cr., a P/E ratio of 41.15, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ15" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 86.21 (Bullish Momentum Zone), while MACD Line (56.22) trades above Signal (42.84) with an expanding histogram (+13.38). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +14.41% above the 200-day DMA (₹1458.79). Daily volatility envelope is bounded by ATR(14) of ₹47.45.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 64.72 (Bullish Momentum Zone), while MACD Line (477.10) trades below Signal (503.84) with an expanding histogram (-26.74). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +16.25% above the 200-day DMA (₹12333.95). Daily volatility envelope is bounded by ATR(14) of ₹416.00.</t>
         </is>
       </c>
       <c r="AR15" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,651.30) is positioned above the 30-day DMA (₹1,478.49), 50-day DMA (₹1,460.44), and 200-day DMA (₹1,458.79). The price distance from 200 DMA is +14.41%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,049.00) is positioned above the 30-day DMA (₹13,190.57), 50-day DMA (₹12,605.68), and 200-day DMA (₹12,333.95). The price distance from 200 DMA is +16.25%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS15" t="inlineStr">
         <is>
-          <t>[1651.3, 1656.25, 1661.21, 1666.16, 1671.12, 1676.07]</t>
+          <t>[14049.0, 14091.15, 14133.29, 14175.44, 14217.59, 14259.73]</t>
         </is>
       </c>
       <c r="AT15" t="inlineStr">
         <is>
-          <t>[1651.3, 1675.23, 1688.05, 1699.04, 1709.08, 1718.51]</t>
+          <t>[14049.0, 14257.55, 14368.62, 14463.65, 14550.39, 14631.82]</t>
         </is>
       </c>
       <c r="AU15" t="inlineStr">
         <is>
-          <t>[1651.3, 1642.02, 1641.08, 1641.51, 1642.65, 1644.24]</t>
+          <t>[14049.0, 13966.35, 13956.8, 13959.28, 13967.99, 13980.67]</t>
         </is>
       </c>
     </row>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DIXON</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>85420.58</v>
+        <v>146280.27</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3016,145 +3016,145 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>14049</v>
+        <v>1651.3</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>₹13965.8 - ₹14173.8</t>
+          <t>₹1641.81 - ₹1665.54</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>14381.8</v>
+        <v>1689.26</v>
       </c>
       <c r="I16" t="n">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="J16" t="n">
-        <v>13190.57</v>
+        <v>1478.49</v>
       </c>
       <c r="K16" t="n">
-        <v>12605.68</v>
+        <v>1460.44</v>
       </c>
       <c r="L16" t="n">
-        <v>12333.95</v>
+        <v>1458.79</v>
       </c>
       <c r="M16" t="n">
-        <v>16.25</v>
+        <v>14.41</v>
       </c>
       <c r="N16" t="n">
-        <v>477.1</v>
+        <v>56.22</v>
       </c>
       <c r="O16" t="n">
-        <v>503.84</v>
+        <v>42.84</v>
       </c>
       <c r="P16" t="n">
-        <v>-26.74</v>
+        <v>13.38</v>
       </c>
       <c r="Q16" t="n">
-        <v>416</v>
+        <v>47.45</v>
       </c>
       <c r="R16" t="n">
         <v>11.76</v>
       </c>
       <c r="S16" t="n">
-        <v>50.8</v>
+        <v>49.8</v>
       </c>
       <c r="T16" t="n">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="U16" t="n">
-        <v>-1.78</v>
+        <v>-1.77</v>
       </c>
       <c r="V16" t="n">
-        <v>46.7</v>
+        <v>48.3</v>
       </c>
       <c r="W16" t="n">
-        <v>6.67</v>
+        <v>8.69</v>
       </c>
       <c r="X16" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y16" t="n">
-        <v>13634.58</v>
+        <v>1625.39</v>
       </c>
       <c r="Z16" t="n">
-        <v>14126.3</v>
+        <v>1683.18</v>
       </c>
       <c r="AA16" t="n">
-        <v>14161.39</v>
+        <v>1664.51</v>
       </c>
       <c r="AB16" t="n">
-        <v>13425</v>
+        <v>1580.13</v>
       </c>
       <c r="AC16" t="n">
-        <v>14079.67</v>
+        <v>1641.1</v>
       </c>
       <c r="AD16" t="n">
-        <v>14558.34</v>
+        <v>1671.7</v>
       </c>
       <c r="AE16" t="n">
-        <v>15067.67</v>
+        <v>1692.1</v>
       </c>
       <c r="AF16" t="n">
-        <v>64.7</v>
+        <v>86.2</v>
       </c>
       <c r="AG16" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (11.76)</t>
+          <t>Low VIX (11.76)</t>
         </is>
       </c>
       <c r="AI16" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ16" t="n">
-        <v>41.2</v>
+        <v>28.6</v>
       </c>
       <c r="AK16" t="n">
-        <v>21.1</v>
+        <v>17.7</v>
       </c>
       <c r="AL16" t="n">
-        <v>3.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="AM16" t="n">
         <v>15</v>
       </c>
       <c r="AN16" t="n">
-        <v>14626.35</v>
+        <v>1696.86</v>
       </c>
       <c r="AO16" t="n">
-        <v>13484.26</v>
+        <v>1606.63</v>
       </c>
       <c r="AP16" t="inlineStr">
         <is>
-          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹85,420.58 Cr., a P/E ratio of 41.15, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
+          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹146,280.27 Cr., a P/E ratio of 28.57, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ16" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 64.72 (Bullish Momentum Zone), while MACD Line (477.10) trades below Signal (503.84) with an expanding histogram (-26.74). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +16.25% above the 200-day DMA (₹12333.95). Daily volatility envelope is bounded by ATR(14) of ₹416.00.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 86.21 (Bullish Momentum Zone), while MACD Line (56.22) trades above Signal (42.84) with an expanding histogram (+13.38). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +14.41% above the 200-day DMA (₹1458.79). Daily volatility envelope is bounded by ATR(14) of ₹47.45.</t>
         </is>
       </c>
       <c r="AR16" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,049.00) is positioned above the 30-day DMA (₹13,190.57), 50-day DMA (₹12,605.68), and 200-day DMA (₹12,333.95). The price distance from 200 DMA is +16.25%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,651.30) is positioned above the 30-day DMA (₹1,478.49), 50-day DMA (₹1,460.44), and 200-day DMA (₹1,458.79). The price distance from 200 DMA is +14.41%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS16" t="inlineStr">
         <is>
-          <t>[14049.0, 14091.15, 14133.29, 14175.44, 14217.59, 14259.73]</t>
+          <t>[1651.3, 1656.25, 1661.21, 1666.16, 1671.12, 1676.07]</t>
         </is>
       </c>
       <c r="AT16" t="inlineStr">
         <is>
-          <t>[14049.0, 14257.55, 14368.62, 14463.65, 14550.39, 14631.82]</t>
+          <t>[1651.3, 1675.23, 1688.05, 1699.04, 1709.08, 1718.51]</t>
         </is>
       </c>
       <c r="AU16" t="inlineStr">
         <is>
-          <t>[14049.0, 13966.35, 13956.8, 13959.28, 13967.99, 13980.67]</t>
+          <t>[1651.3, 1642.02, 1641.08, 1641.51, 1642.65, 1644.24]</t>
         </is>
       </c>
     </row>
@@ -3224,13 +3224,13 @@
         <v>11.76</v>
       </c>
       <c r="S17" t="n">
-        <v>57.3</v>
+        <v>57.1</v>
       </c>
       <c r="T17" t="n">
         <v>0.15</v>
       </c>
       <c r="U17" t="n">
-        <v>-1.88</v>
+        <v>-1.89</v>
       </c>
       <c r="V17" t="n">
         <v>53.3</v>
@@ -3245,7 +3245,7 @@
         <v>590.26</v>
       </c>
       <c r="Z17" t="n">
-        <v>611.72</v>
+        <v>611.73</v>
       </c>
       <c r="AA17" t="n">
         <v>618.26</v>
@@ -3289,10 +3289,10 @@
         <v>6.7</v>
       </c>
       <c r="AN17" t="n">
-        <v>643.89</v>
+        <v>646.59</v>
       </c>
       <c r="AO17" t="n">
-        <v>582.86</v>
+        <v>581.54</v>
       </c>
       <c r="AP17" t="inlineStr">
         <is>
@@ -3391,13 +3391,13 @@
         <v>11.76</v>
       </c>
       <c r="S18" t="n">
-        <v>48.6</v>
+        <v>48.4</v>
       </c>
       <c r="T18" t="n">
         <v>0.17</v>
       </c>
       <c r="U18" t="n">
-        <v>-2</v>
+        <v>-2.01</v>
       </c>
       <c r="V18" t="n">
         <v>51.7</v>
@@ -3456,10 +3456,10 @@
         <v>10</v>
       </c>
       <c r="AN18" t="n">
-        <v>2178.31</v>
+        <v>2178.06</v>
       </c>
       <c r="AO18" t="n">
-        <v>2030.62</v>
+        <v>2031.95</v>
       </c>
       <c r="AP18" t="inlineStr">
         <is>
@@ -3576,10 +3576,10 @@
         <v>-0.77</v>
       </c>
       <c r="Y19" t="n">
-        <v>1114.02</v>
+        <v>1114.05</v>
       </c>
       <c r="Z19" t="n">
-        <v>1153.76</v>
+        <v>1153.79</v>
       </c>
       <c r="AA19" t="n">
         <v>1144.38</v>
@@ -3623,10 +3623,10 @@
         <v>15</v>
       </c>
       <c r="AN19" t="n">
-        <v>1168.76</v>
+        <v>1170.05</v>
       </c>
       <c r="AO19" t="n">
-        <v>1101.06</v>
+        <v>1102.98</v>
       </c>
       <c r="AP19" t="inlineStr">
         <is>
@@ -3725,13 +3725,13 @@
         <v>11.76</v>
       </c>
       <c r="S20" t="n">
-        <v>49.1</v>
+        <v>48.6</v>
       </c>
       <c r="T20" t="n">
         <v>0.16</v>
       </c>
       <c r="U20" t="n">
-        <v>-2.2</v>
+        <v>-2.23</v>
       </c>
       <c r="V20" t="n">
         <v>50</v>
@@ -3790,10 +3790,10 @@
         <v>15</v>
       </c>
       <c r="AN20" t="n">
-        <v>313.79</v>
+        <v>313.19</v>
       </c>
       <c r="AO20" t="n">
-        <v>291.94</v>
+        <v>291.63</v>
       </c>
       <c r="AP20" t="inlineStr">
         <is>
@@ -3892,13 +3892,13 @@
         <v>11.76</v>
       </c>
       <c r="S21" t="n">
-        <v>45.9</v>
+        <v>45.3</v>
       </c>
       <c r="T21" t="n">
         <v>0.15</v>
       </c>
       <c r="U21" t="n">
-        <v>-2.43</v>
+        <v>-2.47</v>
       </c>
       <c r="V21" t="n">
         <v>48.3</v>
@@ -3910,10 +3910,10 @@
         <v>-0.77</v>
       </c>
       <c r="Y21" t="n">
-        <v>1705.12</v>
+        <v>1705.15</v>
       </c>
       <c r="Z21" t="n">
-        <v>1765.36</v>
+        <v>1765.39</v>
       </c>
       <c r="AA21" t="n">
         <v>1734.77</v>
@@ -3957,10 +3957,10 @@
         <v>15</v>
       </c>
       <c r="AN21" t="n">
-        <v>1789.43</v>
+        <v>1786.25</v>
       </c>
       <c r="AO21" t="n">
-        <v>1656.08</v>
+        <v>1655.68</v>
       </c>
       <c r="AP21" t="inlineStr">
         <is>
@@ -3979,17 +3979,17 @@
       </c>
       <c r="AS21" t="inlineStr">
         <is>
-          <t>[1721.0, 1730.94, 1740.87, 1750.81, 1760.74, 1770.68]</t>
+          <t>[1721.0, 1730.97, 1740.93, 1750.9, 1760.86, 1770.83]</t>
         </is>
       </c>
       <c r="AT21" t="inlineStr">
         <is>
-          <t>[1721.0, 1754.67, 1774.43, 1791.91, 1808.21, 1823.74]</t>
+          <t>[1721.0, 1754.7, 1774.49, 1792.0, 1808.32, 1823.89]</t>
         </is>
       </c>
       <c r="AU21" t="inlineStr">
         <is>
-          <t>[1721.0, 1713.14, 1715.7, 1719.98, 1725.15, 1730.88]</t>
+          <t>[1721.0, 1713.17, 1715.76, 1720.07, 1725.26, 1731.03]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add US Market Closing Feed, 30-Day Breakout Stock News Scanner, and 4-Section Mobile-Responsive Dashboard UI
</commit_message>
<xml_diff>
--- a/Breakout_ML_Quant_Predictions.xlsx
+++ b/Breakout_ML_Quant_Predictions.xlsx
@@ -719,13 +719,13 @@
         <v>11.76</v>
       </c>
       <c r="S2" t="n">
-        <v>61.8</v>
+        <v>61.5</v>
       </c>
       <c r="T2" t="n">
         <v>0.32</v>
       </c>
       <c r="U2" t="n">
-        <v>-0.47</v>
+        <v>-0.48</v>
       </c>
       <c r="V2" t="n">
         <v>60</v>
@@ -784,10 +784,10 @@
         <v>16.1</v>
       </c>
       <c r="AN2" t="n">
-        <v>1463.47</v>
+        <v>1463.97</v>
       </c>
       <c r="AO2" t="n">
-        <v>1408.82</v>
+        <v>1409.74</v>
       </c>
       <c r="AP2" t="inlineStr">
         <is>
@@ -886,7 +886,7 @@
         <v>11.76</v>
       </c>
       <c r="S3" t="n">
-        <v>56</v>
+        <v>55.9</v>
       </c>
       <c r="T3" t="n">
         <v>0.39</v>
@@ -904,13 +904,13 @@
         <v>-0.77</v>
       </c>
       <c r="Y3" t="n">
-        <v>7803.14</v>
+        <v>7803.37</v>
       </c>
       <c r="Z3" t="n">
         <v>8059.35</v>
       </c>
       <c r="AA3" t="n">
-        <v>7920.64</v>
+        <v>7920.87</v>
       </c>
       <c r="AB3" t="n">
         <v>7607.65</v>
@@ -951,10 +951,10 @@
         <v>15</v>
       </c>
       <c r="AN3" t="n">
-        <v>8042.82</v>
+        <v>8061.63</v>
       </c>
       <c r="AO3" t="n">
-        <v>7643.3</v>
+        <v>7640.14</v>
       </c>
       <c r="AP3" t="inlineStr">
         <is>
@@ -973,17 +973,17 @@
       </c>
       <c r="AS3" t="inlineStr">
         <is>
-          <t>[7833.5, 7920.64, 8007.78, 8094.92, 8182.07, 8269.21]</t>
+          <t>[7833.5, 7920.87, 8008.25, 8095.62, 8183.0, 8270.37]</t>
         </is>
       </c>
       <c r="AT3" t="inlineStr">
         <is>
-          <t>[7833.5, 7980.87, 8092.96, 8199.24, 8302.52, 8403.88]</t>
+          <t>[7833.5, 7981.1, 8093.42, 8199.94, 8303.45, 8405.04]</t>
         </is>
       </c>
       <c r="AU3" t="inlineStr">
         <is>
-          <t>[7833.5, 7875.47, 7943.9, 8016.69, 8091.73, 8168.2]</t>
+          <t>[7833.5, 7875.7, 7944.37, 8017.39, 8092.66, 8169.37]</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
         <v>11.76</v>
       </c>
       <c r="S4" t="n">
-        <v>58.8</v>
+        <v>58.7</v>
       </c>
       <c r="T4" t="n">
         <v>0.29</v>
@@ -1118,10 +1118,10 @@
         <v>15</v>
       </c>
       <c r="AN4" t="n">
-        <v>115.9</v>
+        <v>115.88</v>
       </c>
       <c r="AO4" t="n">
-        <v>109.77</v>
+        <v>109.57</v>
       </c>
       <c r="AP4" t="inlineStr">
         <is>
@@ -1220,7 +1220,7 @@
         <v>11.76</v>
       </c>
       <c r="S5" t="n">
-        <v>57.7</v>
+        <v>57.6</v>
       </c>
       <c r="T5" t="n">
         <v>0.29</v>
@@ -1238,10 +1238,10 @@
         <v>-0.77</v>
       </c>
       <c r="Y5" t="n">
-        <v>11732.12</v>
+        <v>11731.98</v>
       </c>
       <c r="Z5" t="n">
-        <v>12148.72</v>
+        <v>12148.58</v>
       </c>
       <c r="AA5" t="n">
         <v>11998.22</v>
@@ -1285,10 +1285,10 @@
         <v>15</v>
       </c>
       <c r="AN5" t="n">
-        <v>12175.8</v>
+        <v>12182.37</v>
       </c>
       <c r="AO5" t="n">
-        <v>11620.15</v>
+        <v>11626.21</v>
       </c>
       <c r="AP5" t="inlineStr">
         <is>
@@ -1387,13 +1387,13 @@
         <v>11.76</v>
       </c>
       <c r="S6" t="n">
-        <v>57.1</v>
+        <v>57.9</v>
       </c>
       <c r="T6" t="n">
         <v>0.25</v>
       </c>
       <c r="U6" t="n">
-        <v>-0.9</v>
+        <v>-0.87</v>
       </c>
       <c r="V6" t="n">
         <v>55</v>
@@ -1405,10 +1405,10 @@
         <v>-0.77</v>
       </c>
       <c r="Y6" t="n">
-        <v>2707.04</v>
+        <v>2707.09</v>
       </c>
       <c r="Z6" t="n">
-        <v>2803.2</v>
+        <v>2803.25</v>
       </c>
       <c r="AA6" t="n">
         <v>2769.28</v>
@@ -1452,10 +1452,10 @@
         <v>15</v>
       </c>
       <c r="AN6" t="n">
-        <v>2810.31</v>
+        <v>2813.86</v>
       </c>
       <c r="AO6" t="n">
-        <v>2684.26</v>
+        <v>2683.28</v>
       </c>
       <c r="AP6" t="inlineStr">
         <is>
@@ -1572,7 +1572,7 @@
         <v>-0.77</v>
       </c>
       <c r="Y7" t="n">
-        <v>2184.77</v>
+        <v>2184.76</v>
       </c>
       <c r="Z7" t="n">
         <v>2261.76</v>
@@ -1619,10 +1619,10 @@
         <v>11.6</v>
       </c>
       <c r="AN7" t="n">
-        <v>2264.08</v>
+        <v>2268.44</v>
       </c>
       <c r="AO7" t="n">
-        <v>2141.36</v>
+        <v>2141.15</v>
       </c>
       <c r="AP7" t="inlineStr">
         <is>
@@ -1641,17 +1641,17 @@
       </c>
       <c r="AS7" t="inlineStr">
         <is>
-          <t>[2199.8, 2217.76, 2235.73, 2253.69, 2271.66, 2289.62]</t>
+          <t>[2199.8, 2217.76, 2235.72, 2253.68, 2271.64, 2289.6]</t>
         </is>
       </c>
       <c r="AT7" t="inlineStr">
         <is>
-          <t>[2199.8, 2236.85, 2262.72, 2286.74, 2309.82, 2332.29]</t>
+          <t>[2199.8, 2236.84, 2262.71, 2286.73, 2309.8, 2332.27]</t>
         </is>
       </c>
       <c r="AU7" t="inlineStr">
         <is>
-          <t>[2199.8, 2203.45, 2215.49, 2228.9, 2243.03, 2257.62]</t>
+          <t>[2199.8, 2203.45, 2215.48, 2228.89, 2243.01, 2257.59]</t>
         </is>
       </c>
     </row>
@@ -1721,19 +1721,19 @@
         <v>11.76</v>
       </c>
       <c r="S8" t="n">
-        <v>51.8</v>
+        <v>52.1</v>
       </c>
       <c r="T8" t="n">
         <v>0.27</v>
       </c>
       <c r="U8" t="n">
-        <v>-1.03</v>
+        <v>-1.02</v>
       </c>
       <c r="V8" t="n">
         <v>55</v>
       </c>
       <c r="W8" t="n">
-        <v>5.75</v>
+        <v>5.74</v>
       </c>
       <c r="X8" t="n">
         <v>-0.77</v>
@@ -1742,7 +1742,7 @@
         <v>720.8200000000001</v>
       </c>
       <c r="Z8" t="n">
-        <v>725.27</v>
+        <v>725.26</v>
       </c>
       <c r="AA8" t="n">
         <v>744.46</v>
@@ -1786,10 +1786,10 @@
         <v>15</v>
       </c>
       <c r="AN8" t="n">
-        <v>757.39</v>
+        <v>757.77</v>
       </c>
       <c r="AO8" t="n">
-        <v>720.78</v>
+        <v>720.14</v>
       </c>
       <c r="AP8" t="inlineStr">
         <is>
@@ -1839,7 +1839,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>25000</v>
+        <v>98206.09</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1888,7 +1888,7 @@
         <v>11.76</v>
       </c>
       <c r="S9" t="n">
-        <v>52.9</v>
+        <v>52.7</v>
       </c>
       <c r="T9" t="n">
         <v>0.26</v>
@@ -1953,14 +1953,14 @@
         <v>15</v>
       </c>
       <c r="AN9" t="n">
-        <v>382.71</v>
+        <v>382.86</v>
       </c>
       <c r="AO9" t="n">
-        <v>363.7</v>
+        <v>363.5</v>
       </c>
       <c r="AP9" t="inlineStr">
         <is>
-          <t>RECLTD operates in the Financial Services sector. With an estimated Market Cap of ₹25,000.00 Cr., a P/E ratio of 6.14, and YoY Revenue Growth of +25.2%, the company demonstrates strong institutional backing, solid operating profit margins (68.89%), and healthy Return on Equity (15.00%).</t>
+          <t>RECLTD operates in the Financial Services sector. With an estimated Market Cap of ₹98,206.09 Cr., a P/E ratio of 6.14, and YoY Revenue Growth of +25.2%, the company demonstrates strong institutional backing, solid operating profit margins (68.89%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ9" t="inlineStr">
@@ -2055,13 +2055,13 @@
         <v>11.76</v>
       </c>
       <c r="S10" t="n">
-        <v>46.2</v>
+        <v>46.7</v>
       </c>
       <c r="T10" t="n">
         <v>0.3</v>
       </c>
       <c r="U10" t="n">
-        <v>-1.08</v>
+        <v>-1.06</v>
       </c>
       <c r="V10" t="n">
         <v>41.7</v>
@@ -2073,10 +2073,10 @@
         <v>-0.77</v>
       </c>
       <c r="Y10" t="n">
-        <v>4548.64</v>
+        <v>4548.57</v>
       </c>
       <c r="Z10" t="n">
-        <v>4711.27</v>
+        <v>4711.2</v>
       </c>
       <c r="AA10" t="n">
         <v>4683.67</v>
@@ -2120,10 +2120,10 @@
         <v>24</v>
       </c>
       <c r="AN10" t="n">
-        <v>4766.05</v>
+        <v>4770.98</v>
       </c>
       <c r="AO10" t="n">
-        <v>4517.83</v>
+        <v>4523.28</v>
       </c>
       <c r="AP10" t="inlineStr">
         <is>
@@ -2222,19 +2222,19 @@
         <v>11.76</v>
       </c>
       <c r="S11" t="n">
-        <v>51.4</v>
+        <v>52</v>
       </c>
       <c r="T11" t="n">
         <v>0.25</v>
       </c>
       <c r="U11" t="n">
-        <v>-1.14</v>
+        <v>-1.12</v>
       </c>
       <c r="V11" t="n">
         <v>53.3</v>
       </c>
       <c r="W11" t="n">
-        <v>2.81</v>
+        <v>2.82</v>
       </c>
       <c r="X11" t="n">
         <v>-0.77</v>
@@ -2287,10 +2287,10 @@
         <v>17.6</v>
       </c>
       <c r="AN11" t="n">
-        <v>5884.47</v>
+        <v>5875.25</v>
       </c>
       <c r="AO11" t="n">
-        <v>5620.69</v>
+        <v>5631.46</v>
       </c>
       <c r="AP11" t="inlineStr">
         <is>
@@ -2389,13 +2389,13 @@
         <v>11.76</v>
       </c>
       <c r="S12" t="n">
-        <v>56</v>
+        <v>56.1</v>
       </c>
       <c r="T12" t="n">
         <v>0.21</v>
       </c>
       <c r="U12" t="n">
-        <v>-1.26</v>
+        <v>-1.25</v>
       </c>
       <c r="V12" t="n">
         <v>53.3</v>
@@ -2454,10 +2454,10 @@
         <v>15</v>
       </c>
       <c r="AN12" t="n">
-        <v>3871.66</v>
+        <v>3873.35</v>
       </c>
       <c r="AO12" t="n">
-        <v>3648.3</v>
+        <v>3649.96</v>
       </c>
       <c r="AP12" t="inlineStr">
         <is>
@@ -2556,13 +2556,13 @@
         <v>11.76</v>
       </c>
       <c r="S13" t="n">
-        <v>52</v>
+        <v>51.8</v>
       </c>
       <c r="T13" t="n">
         <v>0.23</v>
       </c>
       <c r="U13" t="n">
-        <v>-1.27</v>
+        <v>-1.28</v>
       </c>
       <c r="V13" t="n">
         <v>45</v>
@@ -2577,7 +2577,7 @@
         <v>1431.86</v>
       </c>
       <c r="Z13" t="n">
-        <v>1388.21</v>
+        <v>1388.25</v>
       </c>
       <c r="AA13" t="n">
         <v>1484.99</v>
@@ -2621,10 +2621,10 @@
         <v>15</v>
       </c>
       <c r="AN13" t="n">
-        <v>1506.89</v>
+        <v>1504.35</v>
       </c>
       <c r="AO13" t="n">
-        <v>1441.95</v>
+        <v>1441.16</v>
       </c>
       <c r="AP13" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
         <v>11.76</v>
       </c>
       <c r="S14" t="n">
-        <v>56.4</v>
+        <v>56.5</v>
       </c>
       <c r="T14" t="n">
         <v>0.18</v>
@@ -2741,10 +2741,10 @@
         <v>-0.77</v>
       </c>
       <c r="Y14" t="n">
-        <v>1019.35</v>
+        <v>1019.37</v>
       </c>
       <c r="Z14" t="n">
-        <v>1055.98</v>
+        <v>1056.01</v>
       </c>
       <c r="AA14" t="n">
         <v>1055.07</v>
@@ -2788,10 +2788,10 @@
         <v>18.5</v>
       </c>
       <c r="AN14" t="n">
-        <v>1087.61</v>
+        <v>1084.67</v>
       </c>
       <c r="AO14" t="n">
-        <v>1010.99</v>
+        <v>1009.83</v>
       </c>
       <c r="AP14" t="inlineStr">
         <is>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DIXON</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2841,7 +2841,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>85420.58</v>
+        <v>146280.27</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2849,145 +2849,145 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>14049</v>
+        <v>1651.3</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>₹13965.8 - ₹14173.8</t>
+          <t>₹1641.81 - ₹1665.54</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>14381.8</v>
+        <v>1689.26</v>
       </c>
       <c r="I15" t="n">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="J15" t="n">
-        <v>13190.57</v>
+        <v>1478.49</v>
       </c>
       <c r="K15" t="n">
-        <v>12605.68</v>
+        <v>1460.44</v>
       </c>
       <c r="L15" t="n">
-        <v>12333.95</v>
+        <v>1458.79</v>
       </c>
       <c r="M15" t="n">
-        <v>16.25</v>
+        <v>14.41</v>
       </c>
       <c r="N15" t="n">
-        <v>477.1</v>
+        <v>56.22</v>
       </c>
       <c r="O15" t="n">
-        <v>503.84</v>
+        <v>42.84</v>
       </c>
       <c r="P15" t="n">
-        <v>-26.74</v>
+        <v>13.38</v>
       </c>
       <c r="Q15" t="n">
-        <v>416</v>
+        <v>47.45</v>
       </c>
       <c r="R15" t="n">
         <v>11.76</v>
       </c>
       <c r="S15" t="n">
-        <v>50.9</v>
+        <v>49.9</v>
       </c>
       <c r="T15" t="n">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="U15" t="n">
-        <v>-1.77</v>
+        <v>-1.76</v>
       </c>
       <c r="V15" t="n">
-        <v>46.7</v>
+        <v>48.3</v>
       </c>
       <c r="W15" t="n">
-        <v>6.67</v>
+        <v>8.69</v>
       </c>
       <c r="X15" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y15" t="n">
-        <v>13634.58</v>
+        <v>1625.35</v>
       </c>
       <c r="Z15" t="n">
-        <v>14126.3</v>
+        <v>1683.14</v>
       </c>
       <c r="AA15" t="n">
-        <v>14161.39</v>
+        <v>1664.51</v>
       </c>
       <c r="AB15" t="n">
-        <v>13425</v>
+        <v>1580.13</v>
       </c>
       <c r="AC15" t="n">
-        <v>14079.67</v>
+        <v>1641.1</v>
       </c>
       <c r="AD15" t="n">
-        <v>14558.34</v>
+        <v>1671.7</v>
       </c>
       <c r="AE15" t="n">
-        <v>15067.67</v>
+        <v>1692.1</v>
       </c>
       <c r="AF15" t="n">
-        <v>64.7</v>
+        <v>86.2</v>
       </c>
       <c r="AG15" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI15" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ15" t="n">
-        <v>41.2</v>
+        <v>28.6</v>
       </c>
       <c r="AK15" t="n">
-        <v>21.1</v>
+        <v>17.7</v>
       </c>
       <c r="AL15" t="n">
-        <v>3.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="AM15" t="n">
         <v>15</v>
       </c>
       <c r="AN15" t="n">
-        <v>14591.79</v>
+        <v>1698.14</v>
       </c>
       <c r="AO15" t="n">
-        <v>13479.71</v>
+        <v>1608.41</v>
       </c>
       <c r="AP15" t="inlineStr">
         <is>
-          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹85,420.58 Cr., a P/E ratio of 41.15, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
+          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹146,280.27 Cr., a P/E ratio of 28.57, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ15" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 64.72 (Bullish Momentum Zone), while MACD Line (477.10) trades below Signal (503.84) with an expanding histogram (-26.74). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +16.25% above the 200-day DMA (₹12333.95). Daily volatility envelope is bounded by ATR(14) of ₹416.00.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 86.21 (Bullish Momentum Zone), while MACD Line (56.22) trades above Signal (42.84) with an expanding histogram (+13.38). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +14.41% above the 200-day DMA (₹1458.79). Daily volatility envelope is bounded by ATR(14) of ₹47.45.</t>
         </is>
       </c>
       <c r="AR15" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,049.00) is positioned above the 30-day DMA (₹13,190.57), 50-day DMA (₹12,605.68), and 200-day DMA (₹12,333.95). The price distance from 200 DMA is +16.25%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,651.30) is positioned above the 30-day DMA (₹1,478.49), 50-day DMA (₹1,460.44), and 200-day DMA (₹1,458.79). The price distance from 200 DMA is +14.41%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS15" t="inlineStr">
         <is>
-          <t>[14049.0, 14091.15, 14133.29, 14175.44, 14217.59, 14259.73]</t>
+          <t>[1651.3, 1656.25, 1661.21, 1666.16, 1671.12, 1676.07]</t>
         </is>
       </c>
       <c r="AT15" t="inlineStr">
         <is>
-          <t>[14049.0, 14257.55, 14368.62, 14463.65, 14550.39, 14631.82]</t>
+          <t>[1651.3, 1675.23, 1688.05, 1699.04, 1709.08, 1718.51]</t>
         </is>
       </c>
       <c r="AU15" t="inlineStr">
         <is>
-          <t>[14049.0, 13966.35, 13956.8, 13959.28, 13967.99, 13980.67]</t>
+          <t>[1651.3, 1642.02, 1641.08, 1641.51, 1642.65, 1644.24]</t>
         </is>
       </c>
     </row>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>DIXON</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>146280.27</v>
+        <v>85420.58</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3016,145 +3016,145 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>1651.3</v>
+        <v>14049</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>₹1641.81 - ₹1665.54</t>
+          <t>₹13965.8 - ₹14173.8</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>1689.26</v>
+        <v>14381.8</v>
       </c>
       <c r="I16" t="n">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="J16" t="n">
-        <v>1478.49</v>
+        <v>13190.57</v>
       </c>
       <c r="K16" t="n">
-        <v>1460.44</v>
+        <v>12605.68</v>
       </c>
       <c r="L16" t="n">
-        <v>1458.79</v>
+        <v>12333.95</v>
       </c>
       <c r="M16" t="n">
-        <v>14.41</v>
+        <v>16.25</v>
       </c>
       <c r="N16" t="n">
-        <v>56.22</v>
+        <v>477.1</v>
       </c>
       <c r="O16" t="n">
-        <v>42.84</v>
+        <v>503.84</v>
       </c>
       <c r="P16" t="n">
-        <v>13.38</v>
+        <v>-26.74</v>
       </c>
       <c r="Q16" t="n">
-        <v>47.45</v>
+        <v>416</v>
       </c>
       <c r="R16" t="n">
         <v>11.76</v>
       </c>
       <c r="S16" t="n">
-        <v>49.6</v>
+        <v>50.5</v>
       </c>
       <c r="T16" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="U16" t="n">
-        <v>-1.78</v>
+        <v>-1.79</v>
       </c>
       <c r="V16" t="n">
-        <v>48.3</v>
+        <v>46.7</v>
       </c>
       <c r="W16" t="n">
-        <v>8.69</v>
+        <v>6.67</v>
       </c>
       <c r="X16" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y16" t="n">
-        <v>1625.39</v>
+        <v>13634.81</v>
       </c>
       <c r="Z16" t="n">
-        <v>1683.18</v>
+        <v>14126.52</v>
       </c>
       <c r="AA16" t="n">
-        <v>1664.51</v>
+        <v>14161.39</v>
       </c>
       <c r="AB16" t="n">
-        <v>1580.13</v>
+        <v>13425</v>
       </c>
       <c r="AC16" t="n">
-        <v>1641.1</v>
+        <v>14079.67</v>
       </c>
       <c r="AD16" t="n">
-        <v>1671.7</v>
+        <v>14558.34</v>
       </c>
       <c r="AE16" t="n">
-        <v>1692.1</v>
+        <v>15067.67</v>
       </c>
       <c r="AF16" t="n">
-        <v>86.2</v>
+        <v>64.7</v>
       </c>
       <c r="AG16" t="n">
-        <v>0.06</v>
+        <v>0.11</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI16" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ16" t="n">
-        <v>28.6</v>
+        <v>41.2</v>
       </c>
       <c r="AK16" t="n">
-        <v>17.7</v>
+        <v>21.1</v>
       </c>
       <c r="AL16" t="n">
-        <v>8.699999999999999</v>
+        <v>3.6</v>
       </c>
       <c r="AM16" t="n">
         <v>15</v>
       </c>
       <c r="AN16" t="n">
-        <v>1697.55</v>
+        <v>14604.59</v>
       </c>
       <c r="AO16" t="n">
-        <v>1608.28</v>
+        <v>13490.97</v>
       </c>
       <c r="AP16" t="inlineStr">
         <is>
-          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹146,280.27 Cr., a P/E ratio of 28.57, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
+          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹85,420.58 Cr., a P/E ratio of 41.15, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ16" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 86.21 (Bullish Momentum Zone), while MACD Line (56.22) trades above Signal (42.84) with an expanding histogram (+13.38). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +14.41% above the 200-day DMA (₹1458.79). Daily volatility envelope is bounded by ATR(14) of ₹47.45.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 64.72 (Bullish Momentum Zone), while MACD Line (477.10) trades below Signal (503.84) with an expanding histogram (-26.74). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +16.25% above the 200-day DMA (₹12333.95). Daily volatility envelope is bounded by ATR(14) of ₹416.00.</t>
         </is>
       </c>
       <c r="AR16" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,651.30) is positioned above the 30-day DMA (₹1,478.49), 50-day DMA (₹1,460.44), and 200-day DMA (₹1,458.79). The price distance from 200 DMA is +14.41%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,049.00) is positioned above the 30-day DMA (₹13,190.57), 50-day DMA (₹12,605.68), and 200-day DMA (₹12,333.95). The price distance from 200 DMA is +16.25%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS16" t="inlineStr">
         <is>
-          <t>[1651.3, 1656.25, 1661.21, 1666.16, 1671.12, 1676.07]</t>
+          <t>[14049.0, 14091.15, 14133.29, 14175.44, 14217.59, 14259.73]</t>
         </is>
       </c>
       <c r="AT16" t="inlineStr">
         <is>
-          <t>[1651.3, 1675.23, 1688.05, 1699.04, 1709.08, 1718.51]</t>
+          <t>[14049.0, 14257.55, 14368.62, 14463.65, 14550.39, 14631.82]</t>
         </is>
       </c>
       <c r="AU16" t="inlineStr">
         <is>
-          <t>[1651.3, 1642.02, 1641.08, 1641.51, 1642.65, 1644.24]</t>
+          <t>[14049.0, 13966.35, 13956.8, 13959.28, 13967.99, 13980.67]</t>
         </is>
       </c>
     </row>
@@ -3224,13 +3224,13 @@
         <v>11.76</v>
       </c>
       <c r="S17" t="n">
-        <v>57.1</v>
+        <v>57.4</v>
       </c>
       <c r="T17" t="n">
         <v>0.15</v>
       </c>
       <c r="U17" t="n">
-        <v>-1.89</v>
+        <v>-1.87</v>
       </c>
       <c r="V17" t="n">
         <v>53.3</v>
@@ -3289,10 +3289,10 @@
         <v>6.7</v>
       </c>
       <c r="AN17" t="n">
-        <v>643.3200000000001</v>
+        <v>643.62</v>
       </c>
       <c r="AO17" t="n">
-        <v>582.9400000000001</v>
+        <v>583.84</v>
       </c>
       <c r="AP17" t="inlineStr">
         <is>
@@ -3346,7 +3346,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>🔴 AVOID / HOLD</t>
+          <t>🟡 MODERATE BUY</t>
         </is>
       </c>
       <c r="F18" t="n">
@@ -3391,13 +3391,13 @@
         <v>11.76</v>
       </c>
       <c r="S18" t="n">
-        <v>47.9</v>
+        <v>49</v>
       </c>
       <c r="T18" t="n">
         <v>0.17</v>
       </c>
       <c r="U18" t="n">
-        <v>-2.04</v>
+        <v>-1.98</v>
       </c>
       <c r="V18" t="n">
         <v>51.7</v>
@@ -3456,10 +3456,10 @@
         <v>10</v>
       </c>
       <c r="AN18" t="n">
-        <v>2180.45</v>
+        <v>2182.37</v>
       </c>
       <c r="AO18" t="n">
-        <v>2028.26</v>
+        <v>2033.12</v>
       </c>
       <c r="AP18" t="inlineStr">
         <is>
@@ -3558,13 +3558,13 @@
         <v>11.76</v>
       </c>
       <c r="S19" t="n">
-        <v>44.9</v>
+        <v>44.3</v>
       </c>
       <c r="T19" t="n">
         <v>0.18</v>
       </c>
       <c r="U19" t="n">
-        <v>-2.16</v>
+        <v>-2.19</v>
       </c>
       <c r="V19" t="n">
         <v>46.7</v>
@@ -3576,10 +3576,10 @@
         <v>-0.77</v>
       </c>
       <c r="Y19" t="n">
-        <v>1113.98</v>
+        <v>1114.03</v>
       </c>
       <c r="Z19" t="n">
-        <v>1153.71</v>
+        <v>1153.77</v>
       </c>
       <c r="AA19" t="n">
         <v>1144.38</v>
@@ -3623,10 +3623,10 @@
         <v>15</v>
       </c>
       <c r="AN19" t="n">
-        <v>1169.2</v>
+        <v>1168.55</v>
       </c>
       <c r="AO19" t="n">
-        <v>1104.97</v>
+        <v>1100.62</v>
       </c>
       <c r="AP19" t="inlineStr">
         <is>
@@ -3725,13 +3725,13 @@
         <v>11.76</v>
       </c>
       <c r="S20" t="n">
-        <v>48.3</v>
+        <v>48.6</v>
       </c>
       <c r="T20" t="n">
         <v>0.16</v>
       </c>
       <c r="U20" t="n">
-        <v>-2.25</v>
+        <v>-2.23</v>
       </c>
       <c r="V20" t="n">
         <v>50</v>
@@ -3790,10 +3790,10 @@
         <v>15</v>
       </c>
       <c r="AN20" t="n">
-        <v>313.63</v>
+        <v>313.35</v>
       </c>
       <c r="AO20" t="n">
-        <v>291.75</v>
+        <v>291.86</v>
       </c>
       <c r="AP20" t="inlineStr">
         <is>
@@ -3892,13 +3892,13 @@
         <v>11.76</v>
       </c>
       <c r="S21" t="n">
-        <v>45.7</v>
+        <v>46.3</v>
       </c>
       <c r="T21" t="n">
         <v>0.15</v>
       </c>
       <c r="U21" t="n">
-        <v>-2.44</v>
+        <v>-2.41</v>
       </c>
       <c r="V21" t="n">
         <v>48.3</v>
@@ -3957,10 +3957,10 @@
         <v>15</v>
       </c>
       <c r="AN21" t="n">
-        <v>1785.58</v>
+        <v>1790.43</v>
       </c>
       <c r="AO21" t="n">
-        <v>1658.16</v>
+        <v>1655.98</v>
       </c>
       <c r="AP21" t="inlineStr">
         <is>
@@ -3984,7 +3984,7 @@
       </c>
       <c r="AT21" t="inlineStr">
         <is>
-          <t>[1721.0, 1754.67, 1774.43, 1791.91, 1808.21, 1823.74]</t>
+          <t>[1721.0, 1754.67, 1774.43, 1791.91, 1808.2, 1823.74]</t>
         </is>
       </c>
       <c r="AU21" t="inlineStr">

</xml_diff>

<commit_message>
Add NIFTY 50 and BANK NIFTY 5-Day ML Prediction Engine and Web Forecast Component
</commit_message>
<xml_diff>
--- a/Breakout_ML_Quant_Predictions.xlsx
+++ b/Breakout_ML_Quant_Predictions.xlsx
@@ -784,10 +784,10 @@
         <v>16.1</v>
       </c>
       <c r="AN2" t="n">
-        <v>1463.97</v>
+        <v>1461.7</v>
       </c>
       <c r="AO2" t="n">
-        <v>1409.74</v>
+        <v>1407.88</v>
       </c>
       <c r="AP2" t="inlineStr">
         <is>
@@ -886,13 +886,13 @@
         <v>11.76</v>
       </c>
       <c r="S3" t="n">
-        <v>55.9</v>
+        <v>55.7</v>
       </c>
       <c r="T3" t="n">
         <v>0.39</v>
       </c>
       <c r="U3" t="n">
-        <v>-0.65</v>
+        <v>-0.66</v>
       </c>
       <c r="V3" t="n">
         <v>48.3</v>
@@ -951,10 +951,10 @@
         <v>15</v>
       </c>
       <c r="AN3" t="n">
-        <v>8061.63</v>
+        <v>8045.56</v>
       </c>
       <c r="AO3" t="n">
-        <v>7640.14</v>
+        <v>7627.74</v>
       </c>
       <c r="AP3" t="inlineStr">
         <is>
@@ -1053,13 +1053,13 @@
         <v>11.76</v>
       </c>
       <c r="S4" t="n">
-        <v>58.7</v>
+        <v>58.4</v>
       </c>
       <c r="T4" t="n">
         <v>0.29</v>
       </c>
       <c r="U4" t="n">
-        <v>-0.67</v>
+        <v>-0.68</v>
       </c>
       <c r="V4" t="n">
         <v>51.7</v>
@@ -1118,10 +1118,10 @@
         <v>15</v>
       </c>
       <c r="AN4" t="n">
-        <v>115.88</v>
+        <v>115.75</v>
       </c>
       <c r="AO4" t="n">
-        <v>109.57</v>
+        <v>109.83</v>
       </c>
       <c r="AP4" t="inlineStr">
         <is>
@@ -1220,7 +1220,7 @@
         <v>11.76</v>
       </c>
       <c r="S5" t="n">
-        <v>57.6</v>
+        <v>57.8</v>
       </c>
       <c r="T5" t="n">
         <v>0.29</v>
@@ -1285,10 +1285,10 @@
         <v>15</v>
       </c>
       <c r="AN5" t="n">
-        <v>12182.37</v>
+        <v>12158.36</v>
       </c>
       <c r="AO5" t="n">
-        <v>11626.21</v>
+        <v>11626.15</v>
       </c>
       <c r="AP5" t="inlineStr">
         <is>
@@ -1387,13 +1387,13 @@
         <v>11.76</v>
       </c>
       <c r="S6" t="n">
-        <v>57.9</v>
+        <v>57.8</v>
       </c>
       <c r="T6" t="n">
         <v>0.25</v>
       </c>
       <c r="U6" t="n">
-        <v>-0.87</v>
+        <v>-0.88</v>
       </c>
       <c r="V6" t="n">
         <v>55</v>
@@ -1405,10 +1405,10 @@
         <v>-0.77</v>
       </c>
       <c r="Y6" t="n">
-        <v>2707.09</v>
+        <v>2707.04</v>
       </c>
       <c r="Z6" t="n">
-        <v>2803.25</v>
+        <v>2803.2</v>
       </c>
       <c r="AA6" t="n">
         <v>2769.28</v>
@@ -1452,10 +1452,10 @@
         <v>15</v>
       </c>
       <c r="AN6" t="n">
-        <v>2813.86</v>
+        <v>2813.46</v>
       </c>
       <c r="AO6" t="n">
-        <v>2683.28</v>
+        <v>2683.65</v>
       </c>
       <c r="AP6" t="inlineStr">
         <is>
@@ -1554,13 +1554,13 @@
         <v>11.76</v>
       </c>
       <c r="S7" t="n">
-        <v>55.7</v>
+        <v>56.1</v>
       </c>
       <c r="T7" t="n">
         <v>0.25</v>
       </c>
       <c r="U7" t="n">
-        <v>-0.99</v>
+        <v>-0.97</v>
       </c>
       <c r="V7" t="n">
         <v>50</v>
@@ -1619,10 +1619,10 @@
         <v>11.6</v>
       </c>
       <c r="AN7" t="n">
-        <v>2268.44</v>
+        <v>2267.91</v>
       </c>
       <c r="AO7" t="n">
-        <v>2141.15</v>
+        <v>2141.66</v>
       </c>
       <c r="AP7" t="inlineStr">
         <is>
@@ -1721,7 +1721,7 @@
         <v>11.76</v>
       </c>
       <c r="S8" t="n">
-        <v>52.1</v>
+        <v>52</v>
       </c>
       <c r="T8" t="n">
         <v>0.27</v>
@@ -1733,7 +1733,7 @@
         <v>55</v>
       </c>
       <c r="W8" t="n">
-        <v>5.74</v>
+        <v>5.75</v>
       </c>
       <c r="X8" t="n">
         <v>-0.77</v>
@@ -1742,7 +1742,7 @@
         <v>720.8200000000001</v>
       </c>
       <c r="Z8" t="n">
-        <v>725.26</v>
+        <v>725.27</v>
       </c>
       <c r="AA8" t="n">
         <v>744.46</v>
@@ -1786,10 +1786,10 @@
         <v>15</v>
       </c>
       <c r="AN8" t="n">
-        <v>757.77</v>
+        <v>756.16</v>
       </c>
       <c r="AO8" t="n">
-        <v>720.14</v>
+        <v>720.1900000000001</v>
       </c>
       <c r="AP8" t="inlineStr">
         <is>
@@ -1888,7 +1888,7 @@
         <v>11.76</v>
       </c>
       <c r="S9" t="n">
-        <v>52.7</v>
+        <v>52.9</v>
       </c>
       <c r="T9" t="n">
         <v>0.26</v>
@@ -1953,10 +1953,10 @@
         <v>15</v>
       </c>
       <c r="AN9" t="n">
-        <v>382.86</v>
+        <v>382.62</v>
       </c>
       <c r="AO9" t="n">
-        <v>363.5</v>
+        <v>362.41</v>
       </c>
       <c r="AP9" t="inlineStr">
         <is>
@@ -2055,13 +2055,13 @@
         <v>11.76</v>
       </c>
       <c r="S10" t="n">
-        <v>46.7</v>
+        <v>47.1</v>
       </c>
       <c r="T10" t="n">
         <v>0.3</v>
       </c>
       <c r="U10" t="n">
-        <v>-1.06</v>
+        <v>-1.04</v>
       </c>
       <c r="V10" t="n">
         <v>41.7</v>
@@ -2120,10 +2120,10 @@
         <v>24</v>
       </c>
       <c r="AN10" t="n">
-        <v>4770.98</v>
+        <v>4769.22</v>
       </c>
       <c r="AO10" t="n">
-        <v>4523.28</v>
+        <v>4523.4</v>
       </c>
       <c r="AP10" t="inlineStr">
         <is>
@@ -2222,13 +2222,13 @@
         <v>11.76</v>
       </c>
       <c r="S11" t="n">
-        <v>52</v>
+        <v>51.7</v>
       </c>
       <c r="T11" t="n">
         <v>0.25</v>
       </c>
       <c r="U11" t="n">
-        <v>-1.12</v>
+        <v>-1.13</v>
       </c>
       <c r="V11" t="n">
         <v>53.3</v>
@@ -2287,10 +2287,10 @@
         <v>17.6</v>
       </c>
       <c r="AN11" t="n">
-        <v>5875.25</v>
+        <v>5880.41</v>
       </c>
       <c r="AO11" t="n">
-        <v>5631.46</v>
+        <v>5626</v>
       </c>
       <c r="AP11" t="inlineStr">
         <is>
@@ -2389,13 +2389,13 @@
         <v>11.76</v>
       </c>
       <c r="S12" t="n">
-        <v>56.1</v>
+        <v>55.9</v>
       </c>
       <c r="T12" t="n">
         <v>0.21</v>
       </c>
       <c r="U12" t="n">
-        <v>-1.25</v>
+        <v>-1.26</v>
       </c>
       <c r="V12" t="n">
         <v>53.3</v>
@@ -2407,10 +2407,10 @@
         <v>-0.77</v>
       </c>
       <c r="Y12" t="n">
-        <v>3683.99</v>
+        <v>3684.03</v>
       </c>
       <c r="Z12" t="n">
-        <v>3815.59</v>
+        <v>3815.63</v>
       </c>
       <c r="AA12" t="n">
         <v>3790.08</v>
@@ -2454,10 +2454,10 @@
         <v>15</v>
       </c>
       <c r="AN12" t="n">
-        <v>3873.35</v>
+        <v>3870.75</v>
       </c>
       <c r="AO12" t="n">
-        <v>3649.96</v>
+        <v>3639.78</v>
       </c>
       <c r="AP12" t="inlineStr">
         <is>
@@ -2556,13 +2556,13 @@
         <v>11.76</v>
       </c>
       <c r="S13" t="n">
-        <v>51.8</v>
+        <v>52</v>
       </c>
       <c r="T13" t="n">
         <v>0.23</v>
       </c>
       <c r="U13" t="n">
-        <v>-1.28</v>
+        <v>-1.27</v>
       </c>
       <c r="V13" t="n">
         <v>45</v>
@@ -2621,10 +2621,10 @@
         <v>15</v>
       </c>
       <c r="AN13" t="n">
-        <v>1504.35</v>
+        <v>1504.69</v>
       </c>
       <c r="AO13" t="n">
-        <v>1441.16</v>
+        <v>1442.77</v>
       </c>
       <c r="AP13" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
         <v>11.76</v>
       </c>
       <c r="S14" t="n">
-        <v>56.5</v>
+        <v>56.4</v>
       </c>
       <c r="T14" t="n">
         <v>0.18</v>
@@ -2741,10 +2741,10 @@
         <v>-0.77</v>
       </c>
       <c r="Y14" t="n">
-        <v>1019.37</v>
+        <v>1019.35</v>
       </c>
       <c r="Z14" t="n">
-        <v>1056.01</v>
+        <v>1055.98</v>
       </c>
       <c r="AA14" t="n">
         <v>1055.07</v>
@@ -2788,10 +2788,10 @@
         <v>18.5</v>
       </c>
       <c r="AN14" t="n">
-        <v>1084.67</v>
+        <v>1084.1</v>
       </c>
       <c r="AO14" t="n">
-        <v>1009.83</v>
+        <v>1009.87</v>
       </c>
       <c r="AP14" t="inlineStr">
         <is>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>DIXON</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2841,7 +2841,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>146280.27</v>
+        <v>85420.58</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2849,145 +2849,145 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>1651.3</v>
+        <v>14049</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>₹1641.81 - ₹1665.54</t>
+          <t>₹13965.8 - ₹14173.8</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1689.26</v>
+        <v>14381.8</v>
       </c>
       <c r="I15" t="n">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="J15" t="n">
-        <v>1478.49</v>
+        <v>13190.57</v>
       </c>
       <c r="K15" t="n">
-        <v>1460.44</v>
+        <v>12605.68</v>
       </c>
       <c r="L15" t="n">
-        <v>1458.79</v>
+        <v>12333.95</v>
       </c>
       <c r="M15" t="n">
-        <v>14.41</v>
+        <v>16.25</v>
       </c>
       <c r="N15" t="n">
-        <v>56.22</v>
+        <v>477.1</v>
       </c>
       <c r="O15" t="n">
-        <v>42.84</v>
+        <v>503.84</v>
       </c>
       <c r="P15" t="n">
-        <v>13.38</v>
+        <v>-26.74</v>
       </c>
       <c r="Q15" t="n">
-        <v>47.45</v>
+        <v>416</v>
       </c>
       <c r="R15" t="n">
         <v>11.76</v>
       </c>
       <c r="S15" t="n">
-        <v>49.9</v>
+        <v>51.2</v>
       </c>
       <c r="T15" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="U15" t="n">
         <v>-1.76</v>
       </c>
       <c r="V15" t="n">
-        <v>48.3</v>
+        <v>46.7</v>
       </c>
       <c r="W15" t="n">
-        <v>8.69</v>
+        <v>6.67</v>
       </c>
       <c r="X15" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y15" t="n">
-        <v>1625.35</v>
+        <v>13634.58</v>
       </c>
       <c r="Z15" t="n">
-        <v>1683.14</v>
+        <v>14126.3</v>
       </c>
       <c r="AA15" t="n">
-        <v>1664.51</v>
+        <v>14161.39</v>
       </c>
       <c r="AB15" t="n">
-        <v>1580.13</v>
+        <v>13425</v>
       </c>
       <c r="AC15" t="n">
-        <v>1641.1</v>
+        <v>14079.67</v>
       </c>
       <c r="AD15" t="n">
-        <v>1671.7</v>
+        <v>14558.34</v>
       </c>
       <c r="AE15" t="n">
-        <v>1692.1</v>
+        <v>15067.67</v>
       </c>
       <c r="AF15" t="n">
-        <v>86.2</v>
+        <v>64.7</v>
       </c>
       <c r="AG15" t="n">
-        <v>0.06</v>
+        <v>0.11</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI15" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ15" t="n">
-        <v>28.6</v>
+        <v>41.2</v>
       </c>
       <c r="AK15" t="n">
-        <v>17.7</v>
+        <v>21.1</v>
       </c>
       <c r="AL15" t="n">
-        <v>8.699999999999999</v>
+        <v>3.6</v>
       </c>
       <c r="AM15" t="n">
         <v>15</v>
       </c>
       <c r="AN15" t="n">
-        <v>1698.14</v>
+        <v>14605.78</v>
       </c>
       <c r="AO15" t="n">
-        <v>1608.41</v>
+        <v>13527.81</v>
       </c>
       <c r="AP15" t="inlineStr">
         <is>
-          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹146,280.27 Cr., a P/E ratio of 28.57, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
+          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹85,420.58 Cr., a P/E ratio of 41.15, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ15" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 86.21 (Bullish Momentum Zone), while MACD Line (56.22) trades above Signal (42.84) with an expanding histogram (+13.38). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +14.41% above the 200-day DMA (₹1458.79). Daily volatility envelope is bounded by ATR(14) of ₹47.45.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 64.72 (Bullish Momentum Zone), while MACD Line (477.10) trades below Signal (503.84) with an expanding histogram (-26.74). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +16.25% above the 200-day DMA (₹12333.95). Daily volatility envelope is bounded by ATR(14) of ₹416.00.</t>
         </is>
       </c>
       <c r="AR15" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,651.30) is positioned above the 30-day DMA (₹1,478.49), 50-day DMA (₹1,460.44), and 200-day DMA (₹1,458.79). The price distance from 200 DMA is +14.41%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,049.00) is positioned above the 30-day DMA (₹13,190.57), 50-day DMA (₹12,605.68), and 200-day DMA (₹12,333.95). The price distance from 200 DMA is +16.25%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS15" t="inlineStr">
         <is>
-          <t>[1651.3, 1656.25, 1661.21, 1666.16, 1671.12, 1676.07]</t>
+          <t>[14049.0, 14091.15, 14133.29, 14175.44, 14217.59, 14259.73]</t>
         </is>
       </c>
       <c r="AT15" t="inlineStr">
         <is>
-          <t>[1651.3, 1675.23, 1688.05, 1699.04, 1709.08, 1718.51]</t>
+          <t>[14049.0, 14257.55, 14368.62, 14463.65, 14550.39, 14631.82]</t>
         </is>
       </c>
       <c r="AU15" t="inlineStr">
         <is>
-          <t>[1651.3, 1642.02, 1641.08, 1641.51, 1642.65, 1644.24]</t>
+          <t>[14049.0, 13966.35, 13956.8, 13959.28, 13967.99, 13980.67]</t>
         </is>
       </c>
     </row>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DIXON</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>85420.58</v>
+        <v>146280.27</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3016,145 +3016,145 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>14049</v>
+        <v>1651.3</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>₹13965.8 - ₹14173.8</t>
+          <t>₹1641.81 - ₹1665.54</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>14381.8</v>
+        <v>1689.26</v>
       </c>
       <c r="I16" t="n">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="J16" t="n">
-        <v>13190.57</v>
+        <v>1478.49</v>
       </c>
       <c r="K16" t="n">
-        <v>12605.68</v>
+        <v>1460.44</v>
       </c>
       <c r="L16" t="n">
-        <v>12333.95</v>
+        <v>1458.79</v>
       </c>
       <c r="M16" t="n">
-        <v>16.25</v>
+        <v>14.41</v>
       </c>
       <c r="N16" t="n">
-        <v>477.1</v>
+        <v>56.22</v>
       </c>
       <c r="O16" t="n">
-        <v>503.84</v>
+        <v>42.84</v>
       </c>
       <c r="P16" t="n">
-        <v>-26.74</v>
+        <v>13.38</v>
       </c>
       <c r="Q16" t="n">
-        <v>416</v>
+        <v>47.45</v>
       </c>
       <c r="R16" t="n">
         <v>11.76</v>
       </c>
       <c r="S16" t="n">
-        <v>50.5</v>
+        <v>49.6</v>
       </c>
       <c r="T16" t="n">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="U16" t="n">
-        <v>-1.79</v>
+        <v>-1.78</v>
       </c>
       <c r="V16" t="n">
-        <v>46.7</v>
+        <v>48.3</v>
       </c>
       <c r="W16" t="n">
-        <v>6.67</v>
+        <v>8.69</v>
       </c>
       <c r="X16" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y16" t="n">
-        <v>13634.81</v>
+        <v>1625.39</v>
       </c>
       <c r="Z16" t="n">
-        <v>14126.52</v>
+        <v>1683.18</v>
       </c>
       <c r="AA16" t="n">
-        <v>14161.39</v>
+        <v>1664.51</v>
       </c>
       <c r="AB16" t="n">
-        <v>13425</v>
+        <v>1580.13</v>
       </c>
       <c r="AC16" t="n">
-        <v>14079.67</v>
+        <v>1641.1</v>
       </c>
       <c r="AD16" t="n">
-        <v>14558.34</v>
+        <v>1671.7</v>
       </c>
       <c r="AE16" t="n">
-        <v>15067.67</v>
+        <v>1692.1</v>
       </c>
       <c r="AF16" t="n">
-        <v>64.7</v>
+        <v>86.2</v>
       </c>
       <c r="AG16" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI16" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ16" t="n">
-        <v>41.2</v>
+        <v>28.6</v>
       </c>
       <c r="AK16" t="n">
-        <v>21.1</v>
+        <v>17.7</v>
       </c>
       <c r="AL16" t="n">
-        <v>3.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="AM16" t="n">
         <v>15</v>
       </c>
       <c r="AN16" t="n">
-        <v>14604.59</v>
+        <v>1697.96</v>
       </c>
       <c r="AO16" t="n">
-        <v>13490.97</v>
+        <v>1608.69</v>
       </c>
       <c r="AP16" t="inlineStr">
         <is>
-          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹85,420.58 Cr., a P/E ratio of 41.15, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
+          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹146,280.27 Cr., a P/E ratio of 28.57, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ16" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 64.72 (Bullish Momentum Zone), while MACD Line (477.10) trades below Signal (503.84) with an expanding histogram (-26.74). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +16.25% above the 200-day DMA (₹12333.95). Daily volatility envelope is bounded by ATR(14) of ₹416.00.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 86.21 (Bullish Momentum Zone), while MACD Line (56.22) trades above Signal (42.84) with an expanding histogram (+13.38). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +14.41% above the 200-day DMA (₹1458.79). Daily volatility envelope is bounded by ATR(14) of ₹47.45.</t>
         </is>
       </c>
       <c r="AR16" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,049.00) is positioned above the 30-day DMA (₹13,190.57), 50-day DMA (₹12,605.68), and 200-day DMA (₹12,333.95). The price distance from 200 DMA is +16.25%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,651.30) is positioned above the 30-day DMA (₹1,478.49), 50-day DMA (₹1,460.44), and 200-day DMA (₹1,458.79). The price distance from 200 DMA is +14.41%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS16" t="inlineStr">
         <is>
-          <t>[14049.0, 14091.15, 14133.29, 14175.44, 14217.59, 14259.73]</t>
+          <t>[1651.3, 1656.25, 1661.21, 1666.16, 1671.12, 1676.07]</t>
         </is>
       </c>
       <c r="AT16" t="inlineStr">
         <is>
-          <t>[14049.0, 14257.55, 14368.62, 14463.65, 14550.39, 14631.82]</t>
+          <t>[1651.3, 1675.23, 1688.05, 1699.04, 1709.08, 1718.51]</t>
         </is>
       </c>
       <c r="AU16" t="inlineStr">
         <is>
-          <t>[14049.0, 13966.35, 13956.8, 13959.28, 13967.99, 13980.67]</t>
+          <t>[1651.3, 1642.02, 1641.08, 1641.51, 1642.65, 1644.24]</t>
         </is>
       </c>
     </row>
@@ -3224,13 +3224,13 @@
         <v>11.76</v>
       </c>
       <c r="S17" t="n">
-        <v>57.4</v>
+        <v>56.8</v>
       </c>
       <c r="T17" t="n">
         <v>0.15</v>
       </c>
       <c r="U17" t="n">
-        <v>-1.87</v>
+        <v>-1.91</v>
       </c>
       <c r="V17" t="n">
         <v>53.3</v>
@@ -3245,7 +3245,7 @@
         <v>590.26</v>
       </c>
       <c r="Z17" t="n">
-        <v>611.72</v>
+        <v>611.73</v>
       </c>
       <c r="AA17" t="n">
         <v>618.26</v>
@@ -3289,10 +3289,10 @@
         <v>6.7</v>
       </c>
       <c r="AN17" t="n">
-        <v>643.62</v>
+        <v>642.47</v>
       </c>
       <c r="AO17" t="n">
-        <v>583.84</v>
+        <v>581.6</v>
       </c>
       <c r="AP17" t="inlineStr">
         <is>
@@ -3391,13 +3391,13 @@
         <v>11.76</v>
       </c>
       <c r="S18" t="n">
-        <v>49</v>
+        <v>48.2</v>
       </c>
       <c r="T18" t="n">
         <v>0.17</v>
       </c>
       <c r="U18" t="n">
-        <v>-1.98</v>
+        <v>-2.02</v>
       </c>
       <c r="V18" t="n">
         <v>51.7</v>
@@ -3456,10 +3456,10 @@
         <v>10</v>
       </c>
       <c r="AN18" t="n">
-        <v>2182.37</v>
+        <v>2185.04</v>
       </c>
       <c r="AO18" t="n">
-        <v>2033.12</v>
+        <v>2028.32</v>
       </c>
       <c r="AP18" t="inlineStr">
         <is>
@@ -3558,13 +3558,13 @@
         <v>11.76</v>
       </c>
       <c r="S19" t="n">
-        <v>44.3</v>
+        <v>44.4</v>
       </c>
       <c r="T19" t="n">
         <v>0.18</v>
       </c>
       <c r="U19" t="n">
-        <v>-2.19</v>
+        <v>-2.18</v>
       </c>
       <c r="V19" t="n">
         <v>46.7</v>
@@ -3576,10 +3576,10 @@
         <v>-0.77</v>
       </c>
       <c r="Y19" t="n">
-        <v>1114.03</v>
+        <v>1114.05</v>
       </c>
       <c r="Z19" t="n">
-        <v>1153.77</v>
+        <v>1153.79</v>
       </c>
       <c r="AA19" t="n">
         <v>1144.38</v>
@@ -3623,10 +3623,10 @@
         <v>15</v>
       </c>
       <c r="AN19" t="n">
-        <v>1168.55</v>
+        <v>1169.58</v>
       </c>
       <c r="AO19" t="n">
-        <v>1100.62</v>
+        <v>1102.69</v>
       </c>
       <c r="AP19" t="inlineStr">
         <is>
@@ -3725,13 +3725,13 @@
         <v>11.76</v>
       </c>
       <c r="S20" t="n">
-        <v>48.6</v>
+        <v>48.9</v>
       </c>
       <c r="T20" t="n">
         <v>0.16</v>
       </c>
       <c r="U20" t="n">
-        <v>-2.23</v>
+        <v>-2.21</v>
       </c>
       <c r="V20" t="n">
         <v>50</v>
@@ -3790,10 +3790,10 @@
         <v>15</v>
       </c>
       <c r="AN20" t="n">
-        <v>313.35</v>
+        <v>313.56</v>
       </c>
       <c r="AO20" t="n">
-        <v>291.86</v>
+        <v>292.1</v>
       </c>
       <c r="AP20" t="inlineStr">
         <is>
@@ -3892,13 +3892,13 @@
         <v>11.76</v>
       </c>
       <c r="S21" t="n">
-        <v>46.3</v>
+        <v>45.7</v>
       </c>
       <c r="T21" t="n">
         <v>0.15</v>
       </c>
       <c r="U21" t="n">
-        <v>-2.41</v>
+        <v>-2.44</v>
       </c>
       <c r="V21" t="n">
         <v>48.3</v>
@@ -3910,10 +3910,10 @@
         <v>-0.77</v>
       </c>
       <c r="Y21" t="n">
-        <v>1705.12</v>
+        <v>1705.17</v>
       </c>
       <c r="Z21" t="n">
-        <v>1765.36</v>
+        <v>1765.4</v>
       </c>
       <c r="AA21" t="n">
         <v>1734.77</v>
@@ -3957,10 +3957,10 @@
         <v>15</v>
       </c>
       <c r="AN21" t="n">
-        <v>1790.43</v>
+        <v>1787.32</v>
       </c>
       <c r="AO21" t="n">
-        <v>1655.98</v>
+        <v>1656.89</v>
       </c>
       <c r="AP21" t="inlineStr">
         <is>
@@ -3979,17 +3979,17 @@
       </c>
       <c r="AS21" t="inlineStr">
         <is>
-          <t>[1721.0, 1730.94, 1740.87, 1750.81, 1760.74, 1770.68]</t>
+          <t>[1721.0, 1730.98, 1740.97, 1750.95, 1760.93, 1770.91]</t>
         </is>
       </c>
       <c r="AT21" t="inlineStr">
         <is>
-          <t>[1721.0, 1754.67, 1774.43, 1791.91, 1808.2, 1823.74]</t>
+          <t>[1721.0, 1754.71, 1774.53, 1792.05, 1808.39, 1823.98]</t>
         </is>
       </c>
       <c r="AU21" t="inlineStr">
         <is>
-          <t>[1721.0, 1713.14, 1715.7, 1719.98, 1725.15, 1730.88]</t>
+          <t>[1721.0, 1713.18, 1715.79, 1720.12, 1725.33, 1731.11]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add US Markets feed, News feed scanner, NIFTY & BANK NIFTY 3-tier analysis, mobile drawer navigation, and post-market price variance tabular forms
</commit_message>
<xml_diff>
--- a/Breakout_ML_Quant_Predictions.xlsx
+++ b/Breakout_ML_Quant_Predictions.xlsx
@@ -719,7 +719,7 @@
         <v>11.76</v>
       </c>
       <c r="S2" t="n">
-        <v>61.5</v>
+        <v>61.6</v>
       </c>
       <c r="T2" t="n">
         <v>0.32</v>
@@ -784,10 +784,10 @@
         <v>16.1</v>
       </c>
       <c r="AN2" t="n">
-        <v>1461.7</v>
+        <v>1461.91</v>
       </c>
       <c r="AO2" t="n">
-        <v>1407.88</v>
+        <v>1409.62</v>
       </c>
       <c r="AP2" t="inlineStr">
         <is>
@@ -886,13 +886,13 @@
         <v>11.76</v>
       </c>
       <c r="S3" t="n">
-        <v>55.7</v>
+        <v>56</v>
       </c>
       <c r="T3" t="n">
         <v>0.39</v>
       </c>
       <c r="U3" t="n">
-        <v>-0.66</v>
+        <v>-0.65</v>
       </c>
       <c r="V3" t="n">
         <v>48.3</v>
@@ -904,13 +904,13 @@
         <v>-0.77</v>
       </c>
       <c r="Y3" t="n">
-        <v>7803.37</v>
+        <v>7803.14</v>
       </c>
       <c r="Z3" t="n">
         <v>8059.35</v>
       </c>
       <c r="AA3" t="n">
-        <v>7920.87</v>
+        <v>7920.64</v>
       </c>
       <c r="AB3" t="n">
         <v>7607.65</v>
@@ -951,10 +951,10 @@
         <v>15</v>
       </c>
       <c r="AN3" t="n">
-        <v>8045.56</v>
+        <v>8050.52</v>
       </c>
       <c r="AO3" t="n">
-        <v>7627.74</v>
+        <v>7641</v>
       </c>
       <c r="AP3" t="inlineStr">
         <is>
@@ -973,17 +973,17 @@
       </c>
       <c r="AS3" t="inlineStr">
         <is>
-          <t>[7833.5, 7920.87, 8008.25, 8095.62, 8183.0, 8270.37]</t>
+          <t>[7833.5, 7920.64, 8007.78, 8094.92, 8182.07, 8269.21]</t>
         </is>
       </c>
       <c r="AT3" t="inlineStr">
         <is>
-          <t>[7833.5, 7981.1, 8093.42, 8199.94, 8303.45, 8405.04]</t>
+          <t>[7833.5, 7980.87, 8092.96, 8199.24, 8302.52, 8403.88]</t>
         </is>
       </c>
       <c r="AU3" t="inlineStr">
         <is>
-          <t>[7833.5, 7875.7, 7944.37, 8017.39, 8092.66, 8169.37]</t>
+          <t>[7833.5, 7875.47, 7943.9, 8016.69, 8091.73, 8168.2]</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
         <v>11.76</v>
       </c>
       <c r="S4" t="n">
-        <v>58.4</v>
+        <v>58.5</v>
       </c>
       <c r="T4" t="n">
         <v>0.29</v>
@@ -1118,10 +1118,10 @@
         <v>15</v>
       </c>
       <c r="AN4" t="n">
-        <v>115.75</v>
+        <v>115.77</v>
       </c>
       <c r="AO4" t="n">
-        <v>109.83</v>
+        <v>109.52</v>
       </c>
       <c r="AP4" t="inlineStr">
         <is>
@@ -1220,13 +1220,13 @@
         <v>11.76</v>
       </c>
       <c r="S5" t="n">
-        <v>57.8</v>
+        <v>57.9</v>
       </c>
       <c r="T5" t="n">
         <v>0.29</v>
       </c>
       <c r="U5" t="n">
-        <v>-0.7</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="V5" t="n">
         <v>48.3</v>
@@ -1238,10 +1238,10 @@
         <v>-0.77</v>
       </c>
       <c r="Y5" t="n">
-        <v>11731.98</v>
+        <v>11732.12</v>
       </c>
       <c r="Z5" t="n">
-        <v>12148.58</v>
+        <v>12148.72</v>
       </c>
       <c r="AA5" t="n">
         <v>11998.22</v>
@@ -1285,10 +1285,10 @@
         <v>15</v>
       </c>
       <c r="AN5" t="n">
-        <v>12158.36</v>
+        <v>12158.3</v>
       </c>
       <c r="AO5" t="n">
-        <v>11626.15</v>
+        <v>11651.1</v>
       </c>
       <c r="AP5" t="inlineStr">
         <is>
@@ -1329,16 +1329,16 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Basic Materials</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>263368.34</v>
+        <v>105169.94</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1346,145 +1346,145 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2747.3</v>
+        <v>2199.8</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>₹2735.68 - ₹2764.73</t>
+          <t>₹2190.26 - ₹2214.11</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>2793.77</v>
+        <v>2237.97</v>
       </c>
       <c r="I6" t="n">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="J6" t="n">
-        <v>2687.86</v>
+        <v>2140.62</v>
       </c>
       <c r="K6" t="n">
-        <v>2678.76</v>
+        <v>2061.08</v>
       </c>
       <c r="L6" t="n">
-        <v>2570.71</v>
+        <v>1703.8</v>
       </c>
       <c r="M6" t="n">
-        <v>6.83</v>
+        <v>27.05</v>
       </c>
       <c r="N6" t="n">
-        <v>16.14</v>
+        <v>29.77</v>
       </c>
       <c r="O6" t="n">
-        <v>10.09</v>
+        <v>35.4</v>
       </c>
       <c r="P6" t="n">
-        <v>6.05</v>
+        <v>-5.63</v>
       </c>
       <c r="Q6" t="n">
-        <v>58.09</v>
+        <v>47.71</v>
       </c>
       <c r="R6" t="n">
         <v>11.76</v>
       </c>
       <c r="S6" t="n">
-        <v>57.8</v>
+        <v>55.9</v>
       </c>
       <c r="T6" t="n">
         <v>0.25</v>
       </c>
       <c r="U6" t="n">
-        <v>-0.88</v>
+        <v>-0.98</v>
       </c>
       <c r="V6" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="W6" t="n">
-        <v>1.89</v>
+        <v>1.78</v>
       </c>
       <c r="X6" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y6" t="n">
-        <v>2707.04</v>
+        <v>2184.77</v>
       </c>
       <c r="Z6" t="n">
-        <v>2803.2</v>
+        <v>2261.76</v>
       </c>
       <c r="AA6" t="n">
-        <v>2769.28</v>
+        <v>2217.76</v>
       </c>
       <c r="AB6" t="n">
-        <v>2660.17</v>
+        <v>2128.24</v>
       </c>
       <c r="AC6" t="n">
-        <v>2751.53</v>
+        <v>2191.3</v>
       </c>
       <c r="AD6" t="n">
-        <v>2770.66</v>
+        <v>2221.1</v>
       </c>
       <c r="AE6" t="n">
-        <v>2794.03</v>
+        <v>2242.4</v>
       </c>
       <c r="AF6" t="n">
-        <v>62.4</v>
+        <v>57.9</v>
       </c>
       <c r="AG6" t="n">
-        <v>-0.03</v>
+        <v>0.03</v>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>Vol Spike 2.4x | TTM Squeeze | Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI6" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ6" t="n">
-        <v>55.2</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="AK6" t="n">
-        <v>17.9</v>
+        <v>17.5</v>
       </c>
       <c r="AL6" t="n">
-        <v>12.8</v>
+        <v>6.4</v>
       </c>
       <c r="AM6" t="n">
-        <v>15</v>
+        <v>11.6</v>
       </c>
       <c r="AN6" t="n">
-        <v>2813.46</v>
+        <v>2269.42</v>
       </c>
       <c r="AO6" t="n">
-        <v>2683.65</v>
+        <v>2140.59</v>
       </c>
       <c r="AP6" t="inlineStr">
         <is>
-          <t>ASIANPAINT operates in the Basic Materials sector. With an estimated Market Cap of ₹263,368.34 Cr., a P/E ratio of 55.24, and YoY Revenue Growth of +17.9%, the company demonstrates strong institutional backing, solid operating profit margins (12.81%), and healthy Return on Equity (15.00%).</t>
+          <t>BHARATFORG operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹105,169.94 Cr., a P/E ratio of 97.08, and YoY Revenue Growth of +17.5%, the company demonstrates strong institutional backing, solid operating profit margins (6.42%), and healthy Return on Equity (11.60%).</t>
         </is>
       </c>
       <c r="AQ6" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 62.38 (Bullish Momentum Zone), while MACD Line (16.14) trades above Signal (10.09) with an expanding histogram (+6.05). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +6.83% above the 200-day DMA (₹2570.71). Daily volatility envelope is bounded by ATR(14) of ₹58.09.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 57.85 (Bullish Momentum Zone), while MACD Line (29.77) trades below Signal (35.40) with an expanding histogram (-5.63). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +27.05% above the 200-day DMA (₹1703.80). Daily volatility envelope is bounded by ATR(14) of ₹47.71.</t>
         </is>
       </c>
       <c r="AR6" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ASIANPAINT. Current Market Price (₹2,747.30) is positioned above the 30-day DMA (₹2,687.86), 50-day DMA (₹2,678.76), and 200-day DMA (₹2,570.71). The price distance from 200 DMA is +6.83%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for BHARATFORG. Current Market Price (₹2,199.80) is positioned above the 30-day DMA (₹2,140.62), 50-day DMA (₹2,061.08), and 200-day DMA (₹1,703.80). The price distance from 200 DMA is +27.05%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS6" t="inlineStr">
         <is>
-          <t>[2747.3, 2755.54, 2763.78, 2772.03, 2780.27, 2788.51]</t>
+          <t>[2199.8, 2217.76, 2235.73, 2253.69, 2271.66, 2289.62]</t>
         </is>
       </c>
       <c r="AT6" t="inlineStr">
         <is>
-          <t>[2747.3, 2778.78, 2796.64, 2812.27, 2826.74, 2840.46]</t>
+          <t>[2199.8, 2236.85, 2262.72, 2286.74, 2309.82, 2332.29]</t>
         </is>
       </c>
       <c r="AU6" t="inlineStr">
         <is>
-          <t>[2747.3, 2738.12, 2739.14, 2741.84, 2745.42, 2749.54]</t>
+          <t>[2199.8, 2203.45, 2215.49, 2228.9, 2243.03, 2257.62]</t>
         </is>
       </c>
     </row>
@@ -1496,162 +1496,162 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>RECLTD</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>105169.94</v>
+        <v>98206.09</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>🟢 HIGH CONVICTION BUY</t>
+          <t>🟡 MODERATE BUY</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2199.8</v>
+        <v>372.95</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>₹2190.26 - ₹2214.11</t>
+          <t>₹371.41 - ₹375.26</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>2237.97</v>
+        <v>379.11</v>
       </c>
       <c r="I7" t="n">
-        <v>69</v>
+        <v>432</v>
       </c>
       <c r="J7" t="n">
-        <v>2140.62</v>
+        <v>357.21</v>
       </c>
       <c r="K7" t="n">
-        <v>2061.08</v>
+        <v>349.78</v>
       </c>
       <c r="L7" t="n">
-        <v>1703.8</v>
+        <v>347.56</v>
       </c>
       <c r="M7" t="n">
-        <v>27.05</v>
+        <v>6.64</v>
       </c>
       <c r="N7" t="n">
-        <v>29.77</v>
+        <v>4.07</v>
       </c>
       <c r="O7" t="n">
-        <v>35.4</v>
+        <v>2.35</v>
       </c>
       <c r="P7" t="n">
-        <v>-5.63</v>
+        <v>1.72</v>
       </c>
       <c r="Q7" t="n">
-        <v>47.71</v>
+        <v>7.7</v>
       </c>
       <c r="R7" t="n">
         <v>11.76</v>
       </c>
       <c r="S7" t="n">
-        <v>56.1</v>
+        <v>52.9</v>
       </c>
       <c r="T7" t="n">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="U7" t="n">
-        <v>-0.97</v>
+        <v>-1.04</v>
       </c>
       <c r="V7" t="n">
         <v>50</v>
       </c>
       <c r="W7" t="n">
-        <v>1.78</v>
+        <v>2.81</v>
       </c>
       <c r="X7" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y7" t="n">
-        <v>2184.76</v>
+        <v>366.16</v>
       </c>
       <c r="Z7" t="n">
-        <v>2261.76</v>
+        <v>379.22</v>
       </c>
       <c r="AA7" t="n">
-        <v>2217.76</v>
+        <v>375.93</v>
       </c>
       <c r="AB7" t="n">
-        <v>2128.24</v>
+        <v>361.4</v>
       </c>
       <c r="AC7" t="n">
-        <v>2191.3</v>
+        <v>372.32</v>
       </c>
       <c r="AD7" t="n">
-        <v>2221.1</v>
+        <v>374.64</v>
       </c>
       <c r="AE7" t="n">
-        <v>2242.4</v>
+        <v>376.32</v>
       </c>
       <c r="AF7" t="n">
-        <v>57.9</v>
+        <v>78.3</v>
       </c>
       <c r="AG7" t="n">
-        <v>0.03</v>
+        <v>0.08</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI7" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ7" t="n">
-        <v>97.09999999999999</v>
+        <v>6.1</v>
       </c>
       <c r="AK7" t="n">
-        <v>17.5</v>
+        <v>25.2</v>
       </c>
       <c r="AL7" t="n">
-        <v>6.4</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="AM7" t="n">
-        <v>11.6</v>
+        <v>15</v>
       </c>
       <c r="AN7" t="n">
-        <v>2267.91</v>
+        <v>383.24</v>
       </c>
       <c r="AO7" t="n">
-        <v>2141.66</v>
+        <v>363.08</v>
       </c>
       <c r="AP7" t="inlineStr">
         <is>
-          <t>BHARATFORG operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹105,169.94 Cr., a P/E ratio of 97.08, and YoY Revenue Growth of +17.5%, the company demonstrates strong institutional backing, solid operating profit margins (6.42%), and healthy Return on Equity (11.60%).</t>
+          <t>RECLTD operates in the Financial Services sector. With an estimated Market Cap of ₹98,206.09 Cr., a P/E ratio of 6.14, and YoY Revenue Growth of +25.2%, the company demonstrates strong institutional backing, solid operating profit margins (68.89%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 57.85 (Bullish Momentum Zone), while MACD Line (29.77) trades below Signal (35.40) with an expanding histogram (-5.63). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +27.05% above the 200-day DMA (₹1703.80). Daily volatility envelope is bounded by ATR(14) of ₹47.71.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 78.30 (Bullish Momentum Zone), while MACD Line (4.07) trades above Signal (2.35) with an expanding histogram (+1.72). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +6.64% above the 200-day DMA (₹347.56). Daily volatility envelope is bounded by ATR(14) of ₹7.70.</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for BHARATFORG. Current Market Price (₹2,199.80) is positioned above the 30-day DMA (₹2,140.62), 50-day DMA (₹2,061.08), and 200-day DMA (₹1,703.80). The price distance from 200 DMA is +27.05%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for RECLTD. Current Market Price (₹372.95) is positioned above the 30-day DMA (₹357.21), 50-day DMA (₹349.78), and 200-day DMA (₹347.56). The price distance from 200 DMA is +6.64%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS7" t="inlineStr">
         <is>
-          <t>[2199.8, 2217.76, 2235.72, 2253.68, 2271.64, 2289.6]</t>
+          <t>[372.95, 374.07, 375.19, 376.31, 377.43, 378.54]</t>
         </is>
       </c>
       <c r="AT7" t="inlineStr">
         <is>
-          <t>[2199.8, 2236.84, 2262.71, 2286.73, 2309.8, 2332.27]</t>
+          <t>[372.95, 377.15, 379.54, 381.64, 383.59, 385.43]</t>
         </is>
       </c>
       <c r="AU7" t="inlineStr">
         <is>
-          <t>[2199.8, 2203.45, 2215.48, 2228.89, 2243.01, 2257.59]</t>
+          <t>[372.95, 371.76, 371.92, 372.31, 372.8, 373.38]</t>
         </is>
       </c>
     </row>
@@ -1721,19 +1721,19 @@
         <v>11.76</v>
       </c>
       <c r="S8" t="n">
-        <v>52</v>
+        <v>51.4</v>
       </c>
       <c r="T8" t="n">
         <v>0.27</v>
       </c>
       <c r="U8" t="n">
-        <v>-1.02</v>
+        <v>-1.05</v>
       </c>
       <c r="V8" t="n">
         <v>55</v>
       </c>
       <c r="W8" t="n">
-        <v>5.75</v>
+        <v>5.74</v>
       </c>
       <c r="X8" t="n">
         <v>-0.77</v>
@@ -1742,7 +1742,7 @@
         <v>720.8200000000001</v>
       </c>
       <c r="Z8" t="n">
-        <v>725.27</v>
+        <v>725.26</v>
       </c>
       <c r="AA8" t="n">
         <v>744.46</v>
@@ -1786,10 +1786,10 @@
         <v>15</v>
       </c>
       <c r="AN8" t="n">
-        <v>756.16</v>
+        <v>756.83</v>
       </c>
       <c r="AO8" t="n">
-        <v>720.1900000000001</v>
+        <v>720.3099999999999</v>
       </c>
       <c r="AP8" t="inlineStr">
         <is>
@@ -1830,162 +1830,162 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>RECLTD</t>
+          <t>HAL</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>98206.09</v>
+        <v>310746.28</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>372.95</v>
+        <v>4646.5</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>₹371.41 - ₹375.26</t>
+          <t>₹4629.85 - ₹4671.48</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>379.11</v>
+        <v>4713.1</v>
       </c>
       <c r="I9" t="n">
-        <v>432</v>
+        <v>40</v>
       </c>
       <c r="J9" t="n">
-        <v>357.21</v>
+        <v>4471.9</v>
       </c>
       <c r="K9" t="n">
-        <v>349.78</v>
+        <v>4404.23</v>
       </c>
       <c r="L9" t="n">
-        <v>347.56</v>
+        <v>4346.03</v>
       </c>
       <c r="M9" t="n">
-        <v>6.64</v>
+        <v>5.42</v>
       </c>
       <c r="N9" t="n">
-        <v>4.07</v>
+        <v>56.6</v>
       </c>
       <c r="O9" t="n">
-        <v>2.35</v>
+        <v>49.9</v>
       </c>
       <c r="P9" t="n">
-        <v>1.72</v>
+        <v>6.7</v>
       </c>
       <c r="Q9" t="n">
-        <v>7.7</v>
+        <v>83.25</v>
       </c>
       <c r="R9" t="n">
         <v>11.76</v>
       </c>
       <c r="S9" t="n">
-        <v>52.9</v>
+        <v>46.3</v>
       </c>
       <c r="T9" t="n">
-        <v>0.26</v>
+        <v>0.3</v>
       </c>
       <c r="U9" t="n">
-        <v>-1.04</v>
+        <v>-1.07</v>
       </c>
       <c r="V9" t="n">
-        <v>50</v>
+        <v>41.7</v>
       </c>
       <c r="W9" t="n">
-        <v>2.81</v>
+        <v>2.15</v>
       </c>
       <c r="X9" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y9" t="n">
-        <v>366.16</v>
+        <v>4548.77</v>
       </c>
       <c r="Z9" t="n">
-        <v>379.22</v>
+        <v>4711.39</v>
       </c>
       <c r="AA9" t="n">
-        <v>375.93</v>
+        <v>4683.67</v>
       </c>
       <c r="AB9" t="n">
-        <v>361.4</v>
+        <v>4521.62</v>
       </c>
       <c r="AC9" t="n">
-        <v>372.32</v>
+        <v>4635.53</v>
       </c>
       <c r="AD9" t="n">
-        <v>374.64</v>
+        <v>4679.96</v>
       </c>
       <c r="AE9" t="n">
-        <v>376.32</v>
+        <v>4713.43</v>
       </c>
       <c r="AF9" t="n">
-        <v>78.3</v>
+        <v>59.3</v>
       </c>
       <c r="AG9" t="n">
-        <v>0.08</v>
+        <v>0.2</v>
       </c>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI9" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ9" t="n">
-        <v>6.1</v>
+        <v>34.1</v>
       </c>
       <c r="AK9" t="n">
-        <v>25.2</v>
+        <v>1.8</v>
       </c>
       <c r="AL9" t="n">
-        <v>68.90000000000001</v>
+        <v>27.5</v>
       </c>
       <c r="AM9" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="AN9" t="n">
-        <v>382.62</v>
+        <v>4772.74</v>
       </c>
       <c r="AO9" t="n">
-        <v>362.41</v>
+        <v>4522.8</v>
       </c>
       <c r="AP9" t="inlineStr">
         <is>
-          <t>RECLTD operates in the Financial Services sector. With an estimated Market Cap of ₹98,206.09 Cr., a P/E ratio of 6.14, and YoY Revenue Growth of +25.2%, the company demonstrates strong institutional backing, solid operating profit margins (68.89%), and healthy Return on Equity (15.00%).</t>
+          <t>HAL operates in the Industrials sector. With an estimated Market Cap of ₹310,746.28 Cr., a P/E ratio of 34.13, and YoY Revenue Growth of +1.8%, the company demonstrates strong institutional backing, solid operating profit margins (27.55%), and healthy Return on Equity (23.98%).</t>
         </is>
       </c>
       <c r="AQ9" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 78.30 (Bullish Momentum Zone), while MACD Line (4.07) trades above Signal (2.35) with an expanding histogram (+1.72). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +6.64% above the 200-day DMA (₹347.56). Daily volatility envelope is bounded by ATR(14) of ₹7.70.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 59.26 (Bullish Momentum Zone), while MACD Line (56.60) trades above Signal (49.90) with an expanding histogram (+6.70). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +5.42% above the 200-day DMA (₹4346.03). Daily volatility envelope is bounded by ATR(14) of ₹83.25.</t>
         </is>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for RECLTD. Current Market Price (₹372.95) is positioned above the 30-day DMA (₹357.21), 50-day DMA (₹349.78), and 200-day DMA (₹347.56). The price distance from 200 DMA is +6.64%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for HAL. Current Market Price (₹4,646.50) is positioned above the 30-day DMA (₹4,471.90), 50-day DMA (₹4,404.23), and 200-day DMA (₹4,346.03). The price distance from 200 DMA is +5.42%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS9" t="inlineStr">
         <is>
-          <t>[372.95, 374.07, 375.19, 376.31, 377.43, 378.54]</t>
+          <t>[4646.5, 4660.44, 4674.38, 4688.32, 4702.26, 4716.2]</t>
         </is>
       </c>
       <c r="AT9" t="inlineStr">
         <is>
-          <t>[372.95, 377.15, 379.54, 381.64, 383.59, 385.43]</t>
+          <t>[4646.5, 4693.74, 4721.47, 4746.0, 4768.86, 4790.66]</t>
         </is>
       </c>
       <c r="AU9" t="inlineStr">
         <is>
-          <t>[372.95, 371.76, 371.92, 372.31, 372.8, 373.38]</t>
+          <t>[4646.5, 4635.46, 4639.06, 4645.06, 4652.31, 4660.35]</t>
         </is>
       </c>
     </row>
@@ -1997,162 +1997,162 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HAL</t>
+          <t>ALKEM</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>310746.28</v>
+        <v>68767.81</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>🔴 AVOID / HOLD</t>
+          <t>🟡 MODERATE BUY</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>4646.5</v>
+        <v>5751.5</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>₹4629.85 - ₹4671.48</t>
+          <t>₹5727.01 - ₹5788.23</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>4713.1</v>
+        <v>5849.44</v>
       </c>
       <c r="I10" t="n">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="J10" t="n">
-        <v>4471.9</v>
+        <v>5575</v>
       </c>
       <c r="K10" t="n">
-        <v>4404.23</v>
+        <v>5484.08</v>
       </c>
       <c r="L10" t="n">
-        <v>4346.03</v>
+        <v>5521.06</v>
       </c>
       <c r="M10" t="n">
-        <v>5.42</v>
+        <v>5.35</v>
       </c>
       <c r="N10" t="n">
-        <v>56.6</v>
+        <v>57.19</v>
       </c>
       <c r="O10" t="n">
-        <v>49.9</v>
+        <v>51.96</v>
       </c>
       <c r="P10" t="n">
-        <v>6.7</v>
+        <v>5.23</v>
       </c>
       <c r="Q10" t="n">
-        <v>83.25</v>
+        <v>122.43</v>
       </c>
       <c r="R10" t="n">
         <v>11.76</v>
       </c>
       <c r="S10" t="n">
-        <v>47.1</v>
+        <v>52.2</v>
       </c>
       <c r="T10" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="U10" t="n">
-        <v>-1.04</v>
+        <v>-1.11</v>
       </c>
       <c r="V10" t="n">
-        <v>41.7</v>
+        <v>53.3</v>
       </c>
       <c r="W10" t="n">
-        <v>2.15</v>
+        <v>2.81</v>
       </c>
       <c r="X10" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y10" t="n">
-        <v>4548.57</v>
+        <v>5710.85</v>
       </c>
       <c r="Z10" t="n">
-        <v>4711.2</v>
+        <v>5912.15</v>
       </c>
       <c r="AA10" t="n">
-        <v>4683.67</v>
+        <v>5797.51</v>
       </c>
       <c r="AB10" t="n">
-        <v>4521.62</v>
+        <v>5567.86</v>
       </c>
       <c r="AC10" t="n">
-        <v>4635.53</v>
+        <v>5773.17</v>
       </c>
       <c r="AD10" t="n">
-        <v>4679.96</v>
+        <v>5811.34</v>
       </c>
       <c r="AE10" t="n">
-        <v>4713.43</v>
+        <v>5871.17</v>
       </c>
       <c r="AF10" t="n">
-        <v>59.3</v>
+        <v>58.4</v>
       </c>
       <c r="AG10" t="n">
-        <v>0.2</v>
+        <v>0.02</v>
       </c>
       <c r="AH10" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Vol Spike 2.0x | TTM Squeeze | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI10" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ10" t="n">
-        <v>34.1</v>
+        <v>29.9</v>
       </c>
       <c r="AK10" t="n">
-        <v>1.8</v>
+        <v>14.6</v>
       </c>
       <c r="AL10" t="n">
-        <v>27.5</v>
+        <v>15.6</v>
       </c>
       <c r="AM10" t="n">
-        <v>24</v>
+        <v>17.6</v>
       </c>
       <c r="AN10" t="n">
-        <v>4769.22</v>
+        <v>5881.57</v>
       </c>
       <c r="AO10" t="n">
-        <v>4523.4</v>
+        <v>5624.81</v>
       </c>
       <c r="AP10" t="inlineStr">
         <is>
-          <t>HAL operates in the Industrials sector. With an estimated Market Cap of ₹310,746.28 Cr., a P/E ratio of 34.13, and YoY Revenue Growth of +1.8%, the company demonstrates strong institutional backing, solid operating profit margins (27.55%), and healthy Return on Equity (23.98%).</t>
+          <t>ALKEM operates in the Healthcare sector. With an estimated Market Cap of ₹68,767.81 Cr., a P/E ratio of 29.85, and YoY Revenue Growth of +14.6%, the company demonstrates strong institutional backing, solid operating profit margins (15.65%), and healthy Return on Equity (17.56%).</t>
         </is>
       </c>
       <c r="AQ10" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 59.26 (Bullish Momentum Zone), while MACD Line (56.60) trades above Signal (49.90) with an expanding histogram (+6.70). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +5.42% above the 200-day DMA (₹4346.03). Daily volatility envelope is bounded by ATR(14) of ₹83.25.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 58.37 (Bullish Momentum Zone), while MACD Line (57.19) trades above Signal (51.96) with an expanding histogram (+5.23). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +5.35% above the 200-day DMA (₹5521.06). Daily volatility envelope is bounded by ATR(14) of ₹122.43.</t>
         </is>
       </c>
       <c r="AR10" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for HAL. Current Market Price (₹4,646.50) is positioned above the 30-day DMA (₹4,471.90), 50-day DMA (₹4,404.23), and 200-day DMA (₹4,346.03). The price distance from 200 DMA is +5.42%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ALKEM. Current Market Price (₹5,751.50) is positioned above the 30-day DMA (₹5,575.00), 50-day DMA (₹5,484.08), and 200-day DMA (₹5,521.06). The price distance from 200 DMA is +5.35%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS10" t="inlineStr">
         <is>
-          <t>[4646.5, 4660.44, 4674.38, 4688.32, 4702.26, 4716.2]</t>
+          <t>[5751.5, 5797.12, 5842.75, 5888.37, 5934.0, 5979.62]</t>
         </is>
       </c>
       <c r="AT10" t="inlineStr">
         <is>
-          <t>[4646.5, 4693.74, 4721.47, 4746.0, 4768.86, 4790.66]</t>
+          <t>[5751.5, 5846.1, 5912.0, 5973.19, 6031.94, 6089.12]</t>
         </is>
       </c>
       <c r="AU10" t="inlineStr">
         <is>
-          <t>[4646.5, 4635.46, 4639.06, 4645.06, 4652.31, 4660.35]</t>
+          <t>[5751.5, 5760.4, 5790.81, 5824.76, 5860.54, 5897.49]</t>
         </is>
       </c>
     </row>
@@ -2164,16 +2164,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ALKEM</t>
+          <t>SIEMENS</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>68767.81</v>
+        <v>133901.31</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2181,145 +2181,145 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>5751.5</v>
+        <v>3760</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>₹5727.01 - ₹5788.23</t>
+          <t>₹3740.59 - ₹3789.12</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>5849.44</v>
+        <v>3837.66</v>
       </c>
       <c r="I11" t="n">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="J11" t="n">
-        <v>5575</v>
+        <v>3594.31</v>
       </c>
       <c r="K11" t="n">
-        <v>5484.08</v>
+        <v>3627.85</v>
       </c>
       <c r="L11" t="n">
-        <v>5521.06</v>
+        <v>3330.53</v>
       </c>
       <c r="M11" t="n">
-        <v>5.35</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="N11" t="n">
-        <v>57.19</v>
+        <v>22.06</v>
       </c>
       <c r="O11" t="n">
-        <v>51.96</v>
+        <v>10.09</v>
       </c>
       <c r="P11" t="n">
-        <v>5.23</v>
+        <v>11.97</v>
       </c>
       <c r="Q11" t="n">
-        <v>122.43</v>
+        <v>97.06999999999999</v>
       </c>
       <c r="R11" t="n">
         <v>11.76</v>
       </c>
       <c r="S11" t="n">
-        <v>51.7</v>
+        <v>56.7</v>
       </c>
       <c r="T11" t="n">
-        <v>0.25</v>
+        <v>0.21</v>
       </c>
       <c r="U11" t="n">
-        <v>-1.13</v>
+        <v>-1.22</v>
       </c>
       <c r="V11" t="n">
         <v>53.3</v>
       </c>
       <c r="W11" t="n">
-        <v>2.82</v>
+        <v>2.23</v>
       </c>
       <c r="X11" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y11" t="n">
-        <v>5710.85</v>
+        <v>3684.03</v>
       </c>
       <c r="Z11" t="n">
-        <v>5912.15</v>
+        <v>3815.63</v>
       </c>
       <c r="AA11" t="n">
-        <v>5797.51</v>
+        <v>3790.08</v>
       </c>
       <c r="AB11" t="n">
-        <v>5567.86</v>
+        <v>3614.39</v>
       </c>
       <c r="AC11" t="n">
-        <v>5773.17</v>
+        <v>3743.5</v>
       </c>
       <c r="AD11" t="n">
-        <v>5811.34</v>
+        <v>3824.9</v>
       </c>
       <c r="AE11" t="n">
-        <v>5871.17</v>
+        <v>3889.8</v>
       </c>
       <c r="AF11" t="n">
-        <v>58.4</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="AG11" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>Vol Spike 2.0x | TTM Squeeze | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI11" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ11" t="n">
-        <v>29.9</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="AK11" t="n">
         <v>14.6</v>
       </c>
       <c r="AL11" t="n">
-        <v>15.6</v>
+        <v>9.5</v>
       </c>
       <c r="AM11" t="n">
-        <v>17.6</v>
+        <v>15</v>
       </c>
       <c r="AN11" t="n">
-        <v>5880.41</v>
+        <v>3877.01</v>
       </c>
       <c r="AO11" t="n">
-        <v>5626</v>
+        <v>3657.42</v>
       </c>
       <c r="AP11" t="inlineStr">
         <is>
-          <t>ALKEM operates in the Healthcare sector. With an estimated Market Cap of ₹68,767.81 Cr., a P/E ratio of 29.85, and YoY Revenue Growth of +14.6%, the company demonstrates strong institutional backing, solid operating profit margins (15.65%), and healthy Return on Equity (17.56%).</t>
+          <t>SIEMENS operates in the Industrials sector. With an estimated Market Cap of ₹133,901.31 Cr., a P/E ratio of 79.36, and YoY Revenue Growth of +14.6%, the company demonstrates strong institutional backing, solid operating profit margins (9.46%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ11" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 58.37 (Bullish Momentum Zone), while MACD Line (57.19) trades above Signal (51.96) with an expanding histogram (+5.23). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +5.35% above the 200-day DMA (₹5521.06). Daily volatility envelope is bounded by ATR(14) of ₹122.43.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 74.09 (Bullish Momentum Zone), while MACD Line (22.06) trades above Signal (10.09) with an expanding histogram (+11.97). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +9.86% above the 200-day DMA (₹3330.53). Daily volatility envelope is bounded by ATR(14) of ₹97.07.</t>
         </is>
       </c>
       <c r="AR11" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ALKEM. Current Market Price (₹5,751.50) is positioned above the 30-day DMA (₹5,575.00), 50-day DMA (₹5,484.08), and 200-day DMA (₹5,521.06). The price distance from 200 DMA is +5.35%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for SIEMENS. Current Market Price (₹3,760.00) is positioned above the 30-day DMA (₹3,594.31), 50-day DMA (₹3,627.85), and 200-day DMA (₹3,330.53). The price distance from 200 DMA is +9.86%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS11" t="inlineStr">
         <is>
-          <t>[5751.5, 5797.12, 5842.75, 5888.37, 5934.0, 5979.62]</t>
+          <t>[3760.0, 3771.28, 3782.56, 3793.84, 3805.12, 3816.4]</t>
         </is>
       </c>
       <c r="AT11" t="inlineStr">
         <is>
-          <t>[5751.5, 5846.1, 5912.0, 5973.19, 6031.94, 6089.12]</t>
+          <t>[3760.0, 3810.11, 3837.47, 3861.1, 3882.78, 3903.23]</t>
         </is>
       </c>
       <c r="AU11" t="inlineStr">
         <is>
-          <t>[5751.5, 5760.4, 5790.81, 5824.76, 5860.54, 5897.49]</t>
+          <t>[3760.0, 3742.16, 3741.37, 3743.4, 3746.88, 3751.28]</t>
         </is>
       </c>
     </row>
@@ -2331,16 +2331,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SIEMENS</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>133901.31</v>
+        <v>119011.76</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2348,145 +2348,145 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3760</v>
+        <v>1473.2</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>₹3740.59 - ₹3789.12</t>
+          <t>₹1466.31 - ₹1483.53</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>3837.66</v>
+        <v>1500.76</v>
       </c>
       <c r="I12" t="n">
-        <v>34</v>
+        <v>96</v>
       </c>
       <c r="J12" t="n">
-        <v>3594.31</v>
+        <v>1436.14</v>
       </c>
       <c r="K12" t="n">
-        <v>3627.85</v>
+        <v>1414.83</v>
       </c>
       <c r="L12" t="n">
-        <v>3330.53</v>
+        <v>1396.09</v>
       </c>
       <c r="M12" t="n">
-        <v>9.859999999999999</v>
+        <v>5.04</v>
       </c>
       <c r="N12" t="n">
-        <v>22.06</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="O12" t="n">
-        <v>10.09</v>
+        <v>6.31</v>
       </c>
       <c r="P12" t="n">
-        <v>11.97</v>
+        <v>1.82</v>
       </c>
       <c r="Q12" t="n">
-        <v>97.06999999999999</v>
+        <v>34.45</v>
       </c>
       <c r="R12" t="n">
         <v>11.76</v>
       </c>
       <c r="S12" t="n">
-        <v>55.9</v>
+        <v>52</v>
       </c>
       <c r="T12" t="n">
-        <v>0.21</v>
+        <v>0.23</v>
       </c>
       <c r="U12" t="n">
-        <v>-1.26</v>
+        <v>-1.27</v>
       </c>
       <c r="V12" t="n">
-        <v>53.3</v>
+        <v>45</v>
       </c>
       <c r="W12" t="n">
-        <v>2.23</v>
+        <v>11.03</v>
       </c>
       <c r="X12" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y12" t="n">
-        <v>3684.03</v>
+        <v>1431.86</v>
       </c>
       <c r="Z12" t="n">
-        <v>3815.63</v>
+        <v>1388.21</v>
       </c>
       <c r="AA12" t="n">
-        <v>3790.08</v>
+        <v>1484.99</v>
       </c>
       <c r="AB12" t="n">
-        <v>3614.39</v>
+        <v>1421.52</v>
       </c>
       <c r="AC12" t="n">
-        <v>3743.5</v>
+        <v>1471.43</v>
       </c>
       <c r="AD12" t="n">
-        <v>3824.9</v>
+        <v>1480.56</v>
       </c>
       <c r="AE12" t="n">
-        <v>3889.8</v>
+        <v>1487.93</v>
       </c>
       <c r="AF12" t="n">
-        <v>74.09999999999999</v>
+        <v>56.5</v>
       </c>
       <c r="AG12" t="n">
-        <v>0.08</v>
+        <v>-0.08</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI12" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ12" t="n">
-        <v>79.40000000000001</v>
+        <v>35.3</v>
       </c>
       <c r="AK12" t="n">
-        <v>14.6</v>
+        <v>3.5</v>
       </c>
       <c r="AL12" t="n">
-        <v>9.5</v>
+        <v>12</v>
       </c>
       <c r="AM12" t="n">
         <v>15</v>
       </c>
       <c r="AN12" t="n">
-        <v>3870.75</v>
+        <v>1504.58</v>
       </c>
       <c r="AO12" t="n">
-        <v>3639.78</v>
+        <v>1443.2</v>
       </c>
       <c r="AP12" t="inlineStr">
         <is>
-          <t>SIEMENS operates in the Industrials sector. With an estimated Market Cap of ₹133,901.31 Cr., a P/E ratio of 79.36, and YoY Revenue Growth of +14.6%, the company demonstrates strong institutional backing, solid operating profit margins (9.46%), and healthy Return on Equity (15.00%).</t>
+          <t>CIPLA operates in the Healthcare sector. With an estimated Market Cap of ₹119,011.76 Cr., a P/E ratio of 35.34, and YoY Revenue Growth of +3.5%, the company demonstrates strong institutional backing, solid operating profit margins (12.01%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ12" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 74.09 (Bullish Momentum Zone), while MACD Line (22.06) trades above Signal (10.09) with an expanding histogram (+11.97). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +9.86% above the 200-day DMA (₹3330.53). Daily volatility envelope is bounded by ATR(14) of ₹97.07.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 56.53 (Bullish Momentum Zone), while MACD Line (8.13) trades above Signal (6.31) with an expanding histogram (+1.82). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +5.04% above the 200-day DMA (₹1396.09). Daily volatility envelope is bounded by ATR(14) of ₹34.45.</t>
         </is>
       </c>
       <c r="AR12" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for SIEMENS. Current Market Price (₹3,760.00) is positioned above the 30-day DMA (₹3,594.31), 50-day DMA (₹3,627.85), and 200-day DMA (₹3,330.53). The price distance from 200 DMA is +9.86%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for CIPLA. Current Market Price (₹1,473.20) is positioned above the 30-day DMA (₹1,436.14), 50-day DMA (₹1,414.83), and 200-day DMA (₹1,396.09). The price distance from 200 DMA is +5.04%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS12" t="inlineStr">
         <is>
-          <t>[3760.0, 3771.28, 3782.56, 3793.84, 3805.12, 3816.4]</t>
+          <t>[1473.2, 1477.62, 1482.04, 1486.46, 1490.88, 1495.3]</t>
         </is>
       </c>
       <c r="AT12" t="inlineStr">
         <is>
-          <t>[3760.0, 3810.11, 3837.47, 3861.1, 3882.78, 3903.23]</t>
+          <t>[1473.2, 1491.4, 1501.53, 1510.33, 1518.44, 1526.11]</t>
         </is>
       </c>
       <c r="AU12" t="inlineStr">
         <is>
-          <t>[3760.0, 3742.16, 3741.37, 3743.4, 3746.88, 3751.28]</t>
+          <t>[1473.2, 1467.28, 1467.42, 1468.56, 1470.21, 1472.19]</t>
         </is>
       </c>
     </row>
@@ -2498,16 +2498,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>SHRIRAMFIN</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>119011.76</v>
+        <v>246283.11</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2515,90 +2515,90 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1473.2</v>
+        <v>1046.7</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>₹1466.31 - ₹1483.53</t>
+          <t>₹1040.39 - ₹1056.17</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>1500.76</v>
+        <v>1071.96</v>
       </c>
       <c r="I13" t="n">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="J13" t="n">
-        <v>1436.14</v>
+        <v>1032.61</v>
       </c>
       <c r="K13" t="n">
-        <v>1414.83</v>
+        <v>994.9400000000001</v>
       </c>
       <c r="L13" t="n">
-        <v>1396.09</v>
+        <v>942.9400000000001</v>
       </c>
       <c r="M13" t="n">
-        <v>5.04</v>
+        <v>8.94</v>
       </c>
       <c r="N13" t="n">
-        <v>8.130000000000001</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="O13" t="n">
-        <v>6.31</v>
+        <v>12.02</v>
       </c>
       <c r="P13" t="n">
-        <v>1.82</v>
+        <v>-3.63</v>
       </c>
       <c r="Q13" t="n">
-        <v>34.45</v>
+        <v>31.57</v>
       </c>
       <c r="R13" t="n">
         <v>11.76</v>
       </c>
       <c r="S13" t="n">
-        <v>52</v>
+        <v>56.5</v>
       </c>
       <c r="T13" t="n">
-        <v>0.23</v>
+        <v>0.18</v>
       </c>
       <c r="U13" t="n">
-        <v>-1.27</v>
+        <v>-1.52</v>
       </c>
       <c r="V13" t="n">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="W13" t="n">
-        <v>11.03</v>
+        <v>3.38</v>
       </c>
       <c r="X13" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y13" t="n">
-        <v>1431.86</v>
+        <v>1019.37</v>
       </c>
       <c r="Z13" t="n">
-        <v>1388.25</v>
+        <v>1056.01</v>
       </c>
       <c r="AA13" t="n">
-        <v>1484.99</v>
+        <v>1055.07</v>
       </c>
       <c r="AB13" t="n">
-        <v>1421.52</v>
+        <v>999.34</v>
       </c>
       <c r="AC13" t="n">
-        <v>1471.43</v>
+        <v>1043.47</v>
       </c>
       <c r="AD13" t="n">
-        <v>1480.56</v>
+        <v>1057.84</v>
       </c>
       <c r="AE13" t="n">
-        <v>1487.93</v>
+        <v>1068.97</v>
       </c>
       <c r="AF13" t="n">
-        <v>56.5</v>
+        <v>46.1</v>
       </c>
       <c r="AG13" t="n">
-        <v>-0.08</v>
+        <v>-0.14</v>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
@@ -2609,51 +2609,51 @@
         <v>0.15</v>
       </c>
       <c r="AJ13" t="n">
-        <v>35.3</v>
+        <v>18.5</v>
       </c>
       <c r="AK13" t="n">
-        <v>3.5</v>
+        <v>39.1</v>
       </c>
       <c r="AL13" t="n">
-        <v>12</v>
+        <v>50.1</v>
       </c>
       <c r="AM13" t="n">
-        <v>15</v>
+        <v>18.5</v>
       </c>
       <c r="AN13" t="n">
-        <v>1504.69</v>
+        <v>1087.24</v>
       </c>
       <c r="AO13" t="n">
-        <v>1442.77</v>
+        <v>1010.62</v>
       </c>
       <c r="AP13" t="inlineStr">
         <is>
-          <t>CIPLA operates in the Healthcare sector. With an estimated Market Cap of ₹119,011.76 Cr., a P/E ratio of 35.34, and YoY Revenue Growth of +3.5%, the company demonstrates strong institutional backing, solid operating profit margins (12.01%), and healthy Return on Equity (15.00%).</t>
+          <t>SHRIRAMFIN operates in the Financial Services sector. With an estimated Market Cap of ₹246,283.11 Cr., a P/E ratio of 18.48, and YoY Revenue Growth of +39.1%, the company demonstrates strong institutional backing, solid operating profit margins (50.11%), and healthy Return on Equity (18.50%).</t>
         </is>
       </c>
       <c r="AQ13" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 56.53 (Bullish Momentum Zone), while MACD Line (8.13) trades above Signal (6.31) with an expanding histogram (+1.82). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +5.04% above the 200-day DMA (₹1396.09). Daily volatility envelope is bounded by ATR(14) of ₹34.45.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 46.13 (Consolidation Zone), while MACD Line (8.39) trades below Signal (12.02) with an expanding histogram (-3.63). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +8.94% above the 200-day DMA (₹942.94). Daily volatility envelope is bounded by ATR(14) of ₹31.57.</t>
         </is>
       </c>
       <c r="AR13" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for CIPLA. Current Market Price (₹1,473.20) is positioned above the 30-day DMA (₹1,436.14), 50-day DMA (₹1,414.83), and 200-day DMA (₹1,396.09). The price distance from 200 DMA is +5.04%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for SHRIRAMFIN. Current Market Price (₹1,046.70) is positioned above the 30-day DMA (₹1,032.61), 50-day DMA (₹994.94), and 200-day DMA (₹942.94). The price distance from 200 DMA is +8.94%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS13" t="inlineStr">
         <is>
-          <t>[1473.2, 1477.62, 1482.04, 1486.46, 1490.88, 1495.3]</t>
+          <t>[1046.7, 1049.84, 1052.98, 1056.12, 1059.26, 1062.4]</t>
         </is>
       </c>
       <c r="AT13" t="inlineStr">
         <is>
-          <t>[1473.2, 1491.4, 1501.53, 1510.33, 1518.44, 1526.11]</t>
+          <t>[1046.7, 1062.47, 1070.84, 1077.99, 1084.52, 1090.64]</t>
         </is>
       </c>
       <c r="AU13" t="inlineStr">
         <is>
-          <t>[1473.2, 1467.28, 1467.42, 1468.56, 1470.21, 1472.19]</t>
+          <t>[1046.7, 1040.37, 1039.59, 1039.72, 1040.32, 1041.22]</t>
         </is>
       </c>
     </row>
@@ -2665,16 +2665,16 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN</t>
+          <t>DIXON</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>246283.11</v>
+        <v>85420.58</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2682,145 +2682,145 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1046.7</v>
+        <v>14049</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>₹1040.39 - ₹1056.17</t>
+          <t>₹13965.8 - ₹14173.8</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1071.96</v>
+        <v>14381.8</v>
       </c>
       <c r="I14" t="n">
-        <v>105</v>
+        <v>8</v>
       </c>
       <c r="J14" t="n">
-        <v>1032.61</v>
+        <v>13190.57</v>
       </c>
       <c r="K14" t="n">
-        <v>994.9400000000001</v>
+        <v>12605.68</v>
       </c>
       <c r="L14" t="n">
-        <v>942.9400000000001</v>
+        <v>12333.95</v>
       </c>
       <c r="M14" t="n">
-        <v>8.94</v>
+        <v>16.25</v>
       </c>
       <c r="N14" t="n">
-        <v>8.390000000000001</v>
+        <v>477.1</v>
       </c>
       <c r="O14" t="n">
-        <v>12.02</v>
+        <v>503.84</v>
       </c>
       <c r="P14" t="n">
-        <v>-3.63</v>
+        <v>-26.74</v>
       </c>
       <c r="Q14" t="n">
-        <v>31.57</v>
+        <v>416</v>
       </c>
       <c r="R14" t="n">
         <v>11.76</v>
       </c>
       <c r="S14" t="n">
-        <v>56.4</v>
+        <v>51.3</v>
       </c>
       <c r="T14" t="n">
         <v>0.18</v>
       </c>
       <c r="U14" t="n">
-        <v>-1.52</v>
+        <v>-1.75</v>
       </c>
       <c r="V14" t="n">
-        <v>55</v>
+        <v>46.7</v>
       </c>
       <c r="W14" t="n">
-        <v>3.38</v>
+        <v>6.67</v>
       </c>
       <c r="X14" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y14" t="n">
-        <v>1019.35</v>
+        <v>13634.58</v>
       </c>
       <c r="Z14" t="n">
-        <v>1055.98</v>
+        <v>14126.3</v>
       </c>
       <c r="AA14" t="n">
-        <v>1055.07</v>
+        <v>14161.39</v>
       </c>
       <c r="AB14" t="n">
-        <v>999.34</v>
+        <v>13425</v>
       </c>
       <c r="AC14" t="n">
-        <v>1043.47</v>
+        <v>14079.67</v>
       </c>
       <c r="AD14" t="n">
-        <v>1057.84</v>
+        <v>14558.34</v>
       </c>
       <c r="AE14" t="n">
-        <v>1068.97</v>
+        <v>15067.67</v>
       </c>
       <c r="AF14" t="n">
-        <v>46.1</v>
+        <v>64.7</v>
       </c>
       <c r="AG14" t="n">
-        <v>-0.14</v>
+        <v>0.11</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI14" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ14" t="n">
-        <v>18.5</v>
+        <v>41.2</v>
       </c>
       <c r="AK14" t="n">
-        <v>39.1</v>
+        <v>21.1</v>
       </c>
       <c r="AL14" t="n">
-        <v>50.1</v>
+        <v>3.6</v>
       </c>
       <c r="AM14" t="n">
-        <v>18.5</v>
+        <v>15</v>
       </c>
       <c r="AN14" t="n">
-        <v>1084.1</v>
+        <v>14590.27</v>
       </c>
       <c r="AO14" t="n">
-        <v>1009.87</v>
+        <v>13527.74</v>
       </c>
       <c r="AP14" t="inlineStr">
         <is>
-          <t>SHRIRAMFIN operates in the Financial Services sector. With an estimated Market Cap of ₹246,283.11 Cr., a P/E ratio of 18.48, and YoY Revenue Growth of +39.1%, the company demonstrates strong institutional backing, solid operating profit margins (50.11%), and healthy Return on Equity (18.50%).</t>
+          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹85,420.58 Cr., a P/E ratio of 41.15, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ14" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 46.13 (Consolidation Zone), while MACD Line (8.39) trades below Signal (12.02) with an expanding histogram (-3.63). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +8.94% above the 200-day DMA (₹942.94). Daily volatility envelope is bounded by ATR(14) of ₹31.57.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 64.72 (Bullish Momentum Zone), while MACD Line (477.10) trades below Signal (503.84) with an expanding histogram (-26.74). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +16.25% above the 200-day DMA (₹12333.95). Daily volatility envelope is bounded by ATR(14) of ₹416.00.</t>
         </is>
       </c>
       <c r="AR14" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for SHRIRAMFIN. Current Market Price (₹1,046.70) is positioned above the 30-day DMA (₹1,032.61), 50-day DMA (₹994.94), and 200-day DMA (₹942.94). The price distance from 200 DMA is +8.94%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,049.00) is positioned above the 30-day DMA (₹13,190.57), 50-day DMA (₹12,605.68), and 200-day DMA (₹12,333.95). The price distance from 200 DMA is +16.25%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS14" t="inlineStr">
         <is>
-          <t>[1046.7, 1049.84, 1052.98, 1056.12, 1059.26, 1062.4]</t>
+          <t>[14049.0, 14091.15, 14133.29, 14175.44, 14217.59, 14259.73]</t>
         </is>
       </c>
       <c r="AT14" t="inlineStr">
         <is>
-          <t>[1046.7, 1062.47, 1070.84, 1077.99, 1084.52, 1090.64]</t>
+          <t>[14049.0, 14257.55, 14368.62, 14463.65, 14550.39, 14631.82]</t>
         </is>
       </c>
       <c r="AU14" t="inlineStr">
         <is>
-          <t>[1046.7, 1040.37, 1039.59, 1039.72, 1040.32, 1041.22]</t>
+          <t>[14049.0, 13966.35, 13956.8, 13959.28, 13967.99, 13980.67]</t>
         </is>
       </c>
     </row>
@@ -2832,7 +2832,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DIXON</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2841,7 +2841,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>85420.58</v>
+        <v>146280.27</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2849,145 +2849,145 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>14049</v>
+        <v>1651.3</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>₹13965.8 - ₹14173.8</t>
+          <t>₹1641.81 - ₹1665.54</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>14381.8</v>
+        <v>1689.26</v>
       </c>
       <c r="I15" t="n">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="J15" t="n">
-        <v>13190.57</v>
+        <v>1478.49</v>
       </c>
       <c r="K15" t="n">
-        <v>12605.68</v>
+        <v>1460.44</v>
       </c>
       <c r="L15" t="n">
-        <v>12333.95</v>
+        <v>1458.79</v>
       </c>
       <c r="M15" t="n">
-        <v>16.25</v>
+        <v>14.41</v>
       </c>
       <c r="N15" t="n">
-        <v>477.1</v>
+        <v>56.22</v>
       </c>
       <c r="O15" t="n">
-        <v>503.84</v>
+        <v>42.84</v>
       </c>
       <c r="P15" t="n">
-        <v>-26.74</v>
+        <v>13.38</v>
       </c>
       <c r="Q15" t="n">
-        <v>416</v>
+        <v>47.45</v>
       </c>
       <c r="R15" t="n">
         <v>11.76</v>
       </c>
       <c r="S15" t="n">
-        <v>51.2</v>
+        <v>49.3</v>
       </c>
       <c r="T15" t="n">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="U15" t="n">
-        <v>-1.76</v>
+        <v>-1.79</v>
       </c>
       <c r="V15" t="n">
-        <v>46.7</v>
+        <v>48.3</v>
       </c>
       <c r="W15" t="n">
-        <v>6.67</v>
+        <v>8.69</v>
       </c>
       <c r="X15" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y15" t="n">
-        <v>13634.58</v>
+        <v>1625.35</v>
       </c>
       <c r="Z15" t="n">
-        <v>14126.3</v>
+        <v>1683.14</v>
       </c>
       <c r="AA15" t="n">
-        <v>14161.39</v>
+        <v>1664.51</v>
       </c>
       <c r="AB15" t="n">
-        <v>13425</v>
+        <v>1580.13</v>
       </c>
       <c r="AC15" t="n">
-        <v>14079.67</v>
+        <v>1641.1</v>
       </c>
       <c r="AD15" t="n">
-        <v>14558.34</v>
+        <v>1671.7</v>
       </c>
       <c r="AE15" t="n">
-        <v>15067.67</v>
+        <v>1692.1</v>
       </c>
       <c r="AF15" t="n">
-        <v>64.7</v>
+        <v>86.2</v>
       </c>
       <c r="AG15" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI15" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ15" t="n">
-        <v>41.2</v>
+        <v>28.6</v>
       </c>
       <c r="AK15" t="n">
-        <v>21.1</v>
+        <v>17.7</v>
       </c>
       <c r="AL15" t="n">
-        <v>3.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="AM15" t="n">
         <v>15</v>
       </c>
       <c r="AN15" t="n">
-        <v>14605.78</v>
+        <v>1695.31</v>
       </c>
       <c r="AO15" t="n">
-        <v>13527.81</v>
+        <v>1605.12</v>
       </c>
       <c r="AP15" t="inlineStr">
         <is>
-          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹85,420.58 Cr., a P/E ratio of 41.15, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
+          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹146,280.27 Cr., a P/E ratio of 28.57, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ15" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 64.72 (Bullish Momentum Zone), while MACD Line (477.10) trades below Signal (503.84) with an expanding histogram (-26.74). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +16.25% above the 200-day DMA (₹12333.95). Daily volatility envelope is bounded by ATR(14) of ₹416.00.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 86.21 (Bullish Momentum Zone), while MACD Line (56.22) trades above Signal (42.84) with an expanding histogram (+13.38). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +14.41% above the 200-day DMA (₹1458.79). Daily volatility envelope is bounded by ATR(14) of ₹47.45.</t>
         </is>
       </c>
       <c r="AR15" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,049.00) is positioned above the 30-day DMA (₹13,190.57), 50-day DMA (₹12,605.68), and 200-day DMA (₹12,333.95). The price distance from 200 DMA is +16.25%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,651.30) is positioned above the 30-day DMA (₹1,478.49), 50-day DMA (₹1,460.44), and 200-day DMA (₹1,458.79). The price distance from 200 DMA is +14.41%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS15" t="inlineStr">
         <is>
-          <t>[14049.0, 14091.15, 14133.29, 14175.44, 14217.59, 14259.73]</t>
+          <t>[1651.3, 1656.25, 1661.21, 1666.16, 1671.12, 1676.07]</t>
         </is>
       </c>
       <c r="AT15" t="inlineStr">
         <is>
-          <t>[14049.0, 14257.55, 14368.62, 14463.65, 14550.39, 14631.82]</t>
+          <t>[1651.3, 1675.23, 1688.05, 1699.04, 1709.08, 1718.51]</t>
         </is>
       </c>
       <c r="AU15" t="inlineStr">
         <is>
-          <t>[14049.0, 13966.35, 13956.8, 13959.28, 13967.99, 13980.67]</t>
+          <t>[1651.3, 1642.02, 1641.08, 1641.51, 1642.65, 1644.24]</t>
         </is>
       </c>
     </row>
@@ -2999,7 +2999,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>PGEL</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3008,7 +3008,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>146280.27</v>
+        <v>17572.27</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3016,145 +3016,145 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>1651.3</v>
+        <v>613.35</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>₹1641.81 - ₹1665.54</t>
+          <t>₹608.87 - ₹620.07</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>1689.26</v>
+        <v>631.27</v>
       </c>
       <c r="I16" t="n">
-        <v>70</v>
+        <v>148</v>
       </c>
       <c r="J16" t="n">
-        <v>1478.49</v>
+        <v>578.01</v>
       </c>
       <c r="K16" t="n">
-        <v>1460.44</v>
+        <v>541.38</v>
       </c>
       <c r="L16" t="n">
-        <v>1458.79</v>
+        <v>553.54</v>
       </c>
       <c r="M16" t="n">
-        <v>14.41</v>
+        <v>10.74</v>
       </c>
       <c r="N16" t="n">
-        <v>56.22</v>
+        <v>14.56</v>
       </c>
       <c r="O16" t="n">
-        <v>42.84</v>
+        <v>16.43</v>
       </c>
       <c r="P16" t="n">
-        <v>13.38</v>
+        <v>-1.88</v>
       </c>
       <c r="Q16" t="n">
-        <v>47.45</v>
+        <v>22.4</v>
       </c>
       <c r="R16" t="n">
         <v>11.76</v>
       </c>
       <c r="S16" t="n">
-        <v>49.6</v>
+        <v>57</v>
       </c>
       <c r="T16" t="n">
-        <v>0.19</v>
+        <v>0.15</v>
       </c>
       <c r="U16" t="n">
-        <v>-1.78</v>
+        <v>-1.9</v>
       </c>
       <c r="V16" t="n">
-        <v>48.3</v>
+        <v>53.3</v>
       </c>
       <c r="W16" t="n">
-        <v>8.69</v>
+        <v>4.8</v>
       </c>
       <c r="X16" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y16" t="n">
-        <v>1625.39</v>
+        <v>590.26</v>
       </c>
       <c r="Z16" t="n">
-        <v>1683.18</v>
+        <v>611.73</v>
       </c>
       <c r="AA16" t="n">
-        <v>1664.51</v>
+        <v>618.26</v>
       </c>
       <c r="AB16" t="n">
-        <v>1580.13</v>
+        <v>579.75</v>
       </c>
       <c r="AC16" t="n">
-        <v>1641.1</v>
+        <v>616.27</v>
       </c>
       <c r="AD16" t="n">
-        <v>1671.7</v>
+        <v>624.54</v>
       </c>
       <c r="AE16" t="n">
-        <v>1692.1</v>
+        <v>635.72</v>
       </c>
       <c r="AF16" t="n">
-        <v>86.2</v>
+        <v>60.8</v>
       </c>
       <c r="AG16" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI16" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ16" t="n">
-        <v>28.6</v>
+        <v>88.5</v>
       </c>
       <c r="AK16" t="n">
-        <v>17.7</v>
+        <v>-10.1</v>
       </c>
       <c r="AL16" t="n">
-        <v>8.699999999999999</v>
+        <v>3.7</v>
       </c>
       <c r="AM16" t="n">
-        <v>15</v>
+        <v>6.7</v>
       </c>
       <c r="AN16" t="n">
-        <v>1697.96</v>
+        <v>648.13</v>
       </c>
       <c r="AO16" t="n">
-        <v>1608.69</v>
+        <v>582.21</v>
       </c>
       <c r="AP16" t="inlineStr">
         <is>
-          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹146,280.27 Cr., a P/E ratio of 28.57, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
+          <t>PGEL operates in the Technology sector. With an estimated Market Cap of ₹17,572.27 Cr., a P/E ratio of 88.51, and YoY Revenue Growth of -10.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.72%), and healthy Return on Equity (6.69%).</t>
         </is>
       </c>
       <c r="AQ16" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 86.21 (Bullish Momentum Zone), while MACD Line (56.22) trades above Signal (42.84) with an expanding histogram (+13.38). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +14.41% above the 200-day DMA (₹1458.79). Daily volatility envelope is bounded by ATR(14) of ₹47.45.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 60.77 (Bullish Momentum Zone), while MACD Line (14.56) trades below Signal (16.43) with an expanding histogram (-1.88). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +10.74% above the 200-day DMA (₹553.54). Daily volatility envelope is bounded by ATR(14) of ₹22.40.</t>
         </is>
       </c>
       <c r="AR16" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,651.30) is positioned above the 30-day DMA (₹1,478.49), 50-day DMA (₹1,460.44), and 200-day DMA (₹1,458.79). The price distance from 200 DMA is +14.41%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PGEL. Current Market Price (₹613.35) is positioned above the 30-day DMA (₹578.01), 50-day DMA (₹541.38), and 200-day DMA (₹553.54). The price distance from 200 DMA is +10.74%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS16" t="inlineStr">
         <is>
-          <t>[1651.3, 1656.25, 1661.21, 1666.16, 1671.12, 1676.07]</t>
+          <t>[613.35, 615.19, 617.03, 618.87, 620.71, 622.55]</t>
         </is>
       </c>
       <c r="AT16" t="inlineStr">
         <is>
-          <t>[1651.3, 1675.23, 1688.05, 1699.04, 1709.08, 1718.51]</t>
+          <t>[613.35, 624.15, 629.7, 634.39, 638.63, 642.59]</t>
         </is>
       </c>
       <c r="AU16" t="inlineStr">
         <is>
-          <t>[1651.3, 1642.02, 1641.08, 1641.51, 1642.65, 1644.24]</t>
+          <t>[613.35, 608.47, 607.53, 607.23, 607.27, 607.52]</t>
         </is>
       </c>
     </row>
@@ -3166,16 +3166,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PGEL</t>
+          <t>GODREJPROP</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>17572.27</v>
+        <v>63429.15</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3183,145 +3183,145 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>613.35</v>
+        <v>2105.7</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>₹608.87 - ₹620.07</t>
+          <t>₹2092.64 - ₹2125.3</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>631.27</v>
+        <v>2157.96</v>
       </c>
       <c r="I17" t="n">
-        <v>148</v>
+        <v>51</v>
       </c>
       <c r="J17" t="n">
-        <v>578.01</v>
+        <v>1999.45</v>
       </c>
       <c r="K17" t="n">
-        <v>541.38</v>
+        <v>1888.17</v>
       </c>
       <c r="L17" t="n">
-        <v>553.54</v>
+        <v>1880.41</v>
       </c>
       <c r="M17" t="n">
-        <v>10.74</v>
+        <v>12.26</v>
       </c>
       <c r="N17" t="n">
-        <v>14.56</v>
+        <v>62.25</v>
       </c>
       <c r="O17" t="n">
-        <v>16.43</v>
+        <v>68.98</v>
       </c>
       <c r="P17" t="n">
-        <v>-1.88</v>
+        <v>-6.73</v>
       </c>
       <c r="Q17" t="n">
-        <v>22.4</v>
+        <v>65.31999999999999</v>
       </c>
       <c r="R17" t="n">
         <v>11.76</v>
       </c>
       <c r="S17" t="n">
-        <v>56.8</v>
+        <v>48.5</v>
       </c>
       <c r="T17" t="n">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="U17" t="n">
-        <v>-1.91</v>
+        <v>-2.01</v>
       </c>
       <c r="V17" t="n">
-        <v>53.3</v>
+        <v>51.7</v>
       </c>
       <c r="W17" t="n">
-        <v>4.8</v>
+        <v>4.49</v>
       </c>
       <c r="X17" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y17" t="n">
-        <v>590.26</v>
+        <v>2027.32</v>
       </c>
       <c r="Z17" t="n">
-        <v>611.73</v>
+        <v>2032.25</v>
       </c>
       <c r="AA17" t="n">
-        <v>618.26</v>
+        <v>2122.55</v>
       </c>
       <c r="AB17" t="n">
-        <v>579.75</v>
+        <v>2007.72</v>
       </c>
       <c r="AC17" t="n">
-        <v>616.27</v>
+        <v>2111.93</v>
       </c>
       <c r="AD17" t="n">
-        <v>624.54</v>
+        <v>2127.76</v>
       </c>
       <c r="AE17" t="n">
-        <v>635.72</v>
+        <v>2149.83</v>
       </c>
       <c r="AF17" t="n">
-        <v>60.8</v>
+        <v>48.8</v>
       </c>
       <c r="AG17" t="n">
-        <v>0.1</v>
+        <v>0.14</v>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI17" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ17" t="n">
-        <v>88.5</v>
+        <v>34.2</v>
       </c>
       <c r="AK17" t="n">
-        <v>-10.1</v>
+        <v>63</v>
       </c>
       <c r="AL17" t="n">
-        <v>3.7</v>
+        <v>36.1</v>
       </c>
       <c r="AM17" t="n">
-        <v>6.7</v>
+        <v>10</v>
       </c>
       <c r="AN17" t="n">
-        <v>642.47</v>
+        <v>2188.81</v>
       </c>
       <c r="AO17" t="n">
-        <v>581.6</v>
+        <v>2028.6</v>
       </c>
       <c r="AP17" t="inlineStr">
         <is>
-          <t>PGEL operates in the Technology sector. With an estimated Market Cap of ₹17,572.27 Cr., a P/E ratio of 88.51, and YoY Revenue Growth of -10.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.72%), and healthy Return on Equity (6.69%).</t>
+          <t>GODREJPROP operates in the Real Estate sector. With an estimated Market Cap of ₹63,429.15 Cr., a P/E ratio of 34.24, and YoY Revenue Growth of +63.0%, the company demonstrates strong institutional backing, solid operating profit margins (36.06%), and healthy Return on Equity (9.97%).</t>
         </is>
       </c>
       <c r="AQ17" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 60.77 (Bullish Momentum Zone), while MACD Line (14.56) trades below Signal (16.43) with an expanding histogram (-1.88). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +10.74% above the 200-day DMA (₹553.54). Daily volatility envelope is bounded by ATR(14) of ₹22.40.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 48.80 (Consolidation Zone), while MACD Line (62.25) trades below Signal (68.98) with an expanding histogram (-6.73). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +12.26% above the 200-day DMA (₹1880.41). Daily volatility envelope is bounded by ATR(14) of ₹65.32.</t>
         </is>
       </c>
       <c r="AR17" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PGEL. Current Market Price (₹613.35) is positioned above the 30-day DMA (₹578.01), 50-day DMA (₹541.38), and 200-day DMA (₹553.54). The price distance from 200 DMA is +10.74%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for GODREJPROP. Current Market Price (₹2,105.70) is positioned above the 30-day DMA (₹1,999.45), 50-day DMA (₹1,888.17), and 200-day DMA (₹1,880.41). The price distance from 200 DMA is +12.26%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS17" t="inlineStr">
         <is>
-          <t>[613.35, 615.19, 617.03, 618.87, 620.71, 622.55]</t>
+          <t>[2105.7, 2112.02, 2118.33, 2124.65, 2130.97, 2137.29]</t>
         </is>
       </c>
       <c r="AT17" t="inlineStr">
         <is>
-          <t>[613.35, 624.15, 629.7, 634.39, 638.63, 642.59]</t>
+          <t>[2105.7, 2138.14, 2155.28, 2169.91, 2183.22, 2195.71]</t>
         </is>
       </c>
       <c r="AU17" t="inlineStr">
         <is>
-          <t>[613.35, 608.47, 607.53, 607.23, 607.27, 607.52]</t>
+          <t>[2105.7, 2092.42, 2090.62, 2090.71, 2091.78, 2093.47]</t>
         </is>
       </c>
     </row>
@@ -3333,162 +3333,162 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>GODREJPROP</t>
+          <t>360ONE</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>63429.15</v>
+        <v>46194.13</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2105.7</v>
+        <v>1135.3</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>₹2092.64 - ₹2125.3</t>
+          <t>₹1128.39 - ₹1145.67</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>2157.96</v>
+        <v>1162.95</v>
       </c>
       <c r="I18" t="n">
-        <v>51</v>
+        <v>96</v>
       </c>
       <c r="J18" t="n">
-        <v>1999.45</v>
+        <v>1109.56</v>
       </c>
       <c r="K18" t="n">
-        <v>1888.17</v>
+        <v>1105.35</v>
       </c>
       <c r="L18" t="n">
-        <v>1880.41</v>
+        <v>1100.33</v>
       </c>
       <c r="M18" t="n">
-        <v>12.26</v>
+        <v>3.87</v>
       </c>
       <c r="N18" t="n">
-        <v>62.25</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="O18" t="n">
-        <v>68.98</v>
+        <v>4.71</v>
       </c>
       <c r="P18" t="n">
-        <v>-6.73</v>
+        <v>4.42</v>
       </c>
       <c r="Q18" t="n">
-        <v>65.31999999999999</v>
+        <v>34.56</v>
       </c>
       <c r="R18" t="n">
         <v>11.76</v>
       </c>
       <c r="S18" t="n">
-        <v>48.2</v>
+        <v>44.4</v>
       </c>
       <c r="T18" t="n">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="U18" t="n">
-        <v>-2.02</v>
+        <v>-2.18</v>
       </c>
       <c r="V18" t="n">
-        <v>51.7</v>
+        <v>46.7</v>
       </c>
       <c r="W18" t="n">
-        <v>4.49</v>
+        <v>2.28</v>
       </c>
       <c r="X18" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y18" t="n">
-        <v>2027.32</v>
+        <v>1114.01</v>
       </c>
       <c r="Z18" t="n">
-        <v>2032.25</v>
+        <v>1153.74</v>
       </c>
       <c r="AA18" t="n">
-        <v>2122.55</v>
+        <v>1144.38</v>
       </c>
       <c r="AB18" t="n">
-        <v>2007.72</v>
+        <v>1083.45</v>
       </c>
       <c r="AC18" t="n">
-        <v>2111.93</v>
+        <v>1144.43</v>
       </c>
       <c r="AD18" t="n">
-        <v>2127.76</v>
+        <v>1156.86</v>
       </c>
       <c r="AE18" t="n">
-        <v>2149.83</v>
+        <v>1178.43</v>
       </c>
       <c r="AF18" t="n">
-        <v>48.8</v>
+        <v>52.9</v>
       </c>
       <c r="AG18" t="n">
-        <v>0.14</v>
+        <v>0.2</v>
       </c>
       <c r="AH18" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | TTM Squeeze | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI18" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ18" t="n">
-        <v>34.2</v>
+        <v>37.7</v>
       </c>
       <c r="AK18" t="n">
-        <v>63</v>
+        <v>29.9</v>
       </c>
       <c r="AL18" t="n">
-        <v>36.1</v>
+        <v>26.5</v>
       </c>
       <c r="AM18" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="AN18" t="n">
-        <v>2185.04</v>
+        <v>1168.8</v>
       </c>
       <c r="AO18" t="n">
-        <v>2028.32</v>
+        <v>1101.74</v>
       </c>
       <c r="AP18" t="inlineStr">
         <is>
-          <t>GODREJPROP operates in the Real Estate sector. With an estimated Market Cap of ₹63,429.15 Cr., a P/E ratio of 34.24, and YoY Revenue Growth of +63.0%, the company demonstrates strong institutional backing, solid operating profit margins (36.06%), and healthy Return on Equity (9.97%).</t>
+          <t>360ONE operates in the Financial Services sector. With an estimated Market Cap of ₹46,194.13 Cr., a P/E ratio of 37.73, and YoY Revenue Growth of +29.9%, the company demonstrates strong institutional backing, solid operating profit margins (26.46%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ18" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 48.80 (Consolidation Zone), while MACD Line (62.25) trades below Signal (68.98) with an expanding histogram (-6.73). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +12.26% above the 200-day DMA (₹1880.41). Daily volatility envelope is bounded by ATR(14) of ₹65.32.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 52.88 (Consolidation Zone), while MACD Line (9.13) trades above Signal (4.71) with an expanding histogram (+4.42). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +3.87% above the 200-day DMA (₹1100.33). Daily volatility envelope is bounded by ATR(14) of ₹34.56.</t>
         </is>
       </c>
       <c r="AR18" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for GODREJPROP. Current Market Price (₹2,105.70) is positioned above the 30-day DMA (₹1,999.45), 50-day DMA (₹1,888.17), and 200-day DMA (₹1,880.41). The price distance from 200 DMA is +12.26%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for 360ONE. Current Market Price (₹1,135.30) is positioned above the 30-day DMA (₹1,109.56), 50-day DMA (₹1,105.35), and 200-day DMA (₹1,100.33). The price distance from 200 DMA is +3.87%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS18" t="inlineStr">
         <is>
-          <t>[2105.7, 2112.02, 2118.33, 2124.65, 2130.97, 2137.29]</t>
+          <t>[1135.3, 1138.71, 1142.11, 1145.52, 1148.92, 1152.33]</t>
         </is>
       </c>
       <c r="AT18" t="inlineStr">
         <is>
-          <t>[2105.7, 2138.14, 2155.28, 2169.91, 2183.22, 2195.71]</t>
+          <t>[1135.3, 1152.53, 1161.66, 1169.46, 1176.58, 1183.24]</t>
         </is>
       </c>
       <c r="AU18" t="inlineStr">
         <is>
-          <t>[2105.7, 2092.42, 2090.62, 2090.71, 2091.78, 2093.47]</t>
+          <t>[1135.3, 1128.34, 1127.45, 1127.56, 1128.19, 1129.14]</t>
         </is>
       </c>
     </row>
@@ -3500,162 +3500,162 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>360ONE</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>46194.13</v>
+        <v>278417.14</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>🔴 AVOID / HOLD</t>
+          <t>🟡 MODERATE BUY</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1135.3</v>
+        <v>302.45</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>₹1128.39 - ₹1145.67</t>
+          <t>₹300.39 - ₹305.53</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>1162.95</v>
+        <v>310.68</v>
       </c>
       <c r="I19" t="n">
-        <v>96</v>
+        <v>324</v>
       </c>
       <c r="J19" t="n">
-        <v>1109.56</v>
+        <v>281.7</v>
       </c>
       <c r="K19" t="n">
-        <v>1105.35</v>
+        <v>268.93</v>
       </c>
       <c r="L19" t="n">
-        <v>1100.33</v>
+        <v>274.01</v>
       </c>
       <c r="M19" t="n">
-        <v>3.87</v>
+        <v>13.37</v>
       </c>
       <c r="N19" t="n">
-        <v>9.130000000000001</v>
+        <v>9.93</v>
       </c>
       <c r="O19" t="n">
-        <v>4.71</v>
+        <v>8.42</v>
       </c>
       <c r="P19" t="n">
-        <v>4.42</v>
+        <v>1.51</v>
       </c>
       <c r="Q19" t="n">
-        <v>34.56</v>
+        <v>10.28</v>
       </c>
       <c r="R19" t="n">
         <v>11.76</v>
       </c>
       <c r="S19" t="n">
-        <v>44.4</v>
+        <v>48.6</v>
       </c>
       <c r="T19" t="n">
-        <v>0.18</v>
+        <v>0.16</v>
       </c>
       <c r="U19" t="n">
-        <v>-2.18</v>
+        <v>-2.23</v>
       </c>
       <c r="V19" t="n">
-        <v>46.7</v>
+        <v>50</v>
       </c>
       <c r="W19" t="n">
-        <v>2.28</v>
+        <v>2.44</v>
       </c>
       <c r="X19" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y19" t="n">
-        <v>1114.05</v>
+        <v>299.26</v>
       </c>
       <c r="Z19" t="n">
-        <v>1153.79</v>
+        <v>309.85</v>
       </c>
       <c r="AA19" t="n">
-        <v>1144.38</v>
+        <v>304.87</v>
       </c>
       <c r="AB19" t="n">
-        <v>1083.45</v>
+        <v>287.03</v>
       </c>
       <c r="AC19" t="n">
-        <v>1144.43</v>
+        <v>306.75</v>
       </c>
       <c r="AD19" t="n">
-        <v>1156.86</v>
+        <v>311.7</v>
       </c>
       <c r="AE19" t="n">
-        <v>1178.43</v>
+        <v>320.95</v>
       </c>
       <c r="AF19" t="n">
-        <v>52.9</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="AG19" t="n">
-        <v>0.2</v>
+        <v>0.12</v>
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | TTM Squeeze | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI19" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ19" t="n">
-        <v>37.7</v>
+        <v>672.1</v>
       </c>
       <c r="AK19" t="n">
-        <v>29.9</v>
+        <v>182</v>
       </c>
       <c r="AL19" t="n">
-        <v>26.5</v>
+        <v>0.6</v>
       </c>
       <c r="AM19" t="n">
         <v>15</v>
       </c>
       <c r="AN19" t="n">
-        <v>1169.58</v>
+        <v>313.15</v>
       </c>
       <c r="AO19" t="n">
-        <v>1102.69</v>
+        <v>291.97</v>
       </c>
       <c r="AP19" t="inlineStr">
         <is>
-          <t>360ONE operates in the Financial Services sector. With an estimated Market Cap of ₹46,194.13 Cr., a P/E ratio of 37.73, and YoY Revenue Growth of +29.9%, the company demonstrates strong institutional backing, solid operating profit margins (26.46%), and healthy Return on Equity (15.00%).</t>
+          <t>ETERNAL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹278,417.14 Cr., a P/E ratio of 672.11, and YoY Revenue Growth of +182.0%, the company demonstrates strong institutional backing, solid operating profit margins (0.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ19" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 52.88 (Consolidation Zone), while MACD Line (9.13) trades above Signal (4.71) with an expanding histogram (+4.42). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +3.87% above the 200-day DMA (₹1100.33). Daily volatility envelope is bounded by ATR(14) of ₹34.56.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 65.40 (Bullish Momentum Zone), while MACD Line (9.93) trades above Signal (8.42) with an expanding histogram (+1.51). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +13.37% above the 200-day DMA (₹274.01). Daily volatility envelope is bounded by ATR(14) of ₹10.28.</t>
         </is>
       </c>
       <c r="AR19" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for 360ONE. Current Market Price (₹1,135.30) is positioned above the 30-day DMA (₹1,109.56), 50-day DMA (₹1,105.35), and 200-day DMA (₹1,100.33). The price distance from 200 DMA is +3.87%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ETERNAL. Current Market Price (₹302.45) is positioned above the 30-day DMA (₹281.70), 50-day DMA (₹268.93), and 200-day DMA (₹274.01). The price distance from 200 DMA is +13.37%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS19" t="inlineStr">
         <is>
-          <t>[1135.3, 1138.71, 1142.11, 1145.52, 1148.92, 1152.33]</t>
+          <t>[302.45, 303.8, 305.15, 306.5, 307.85, 309.19]</t>
         </is>
       </c>
       <c r="AT19" t="inlineStr">
         <is>
-          <t>[1135.3, 1152.53, 1161.66, 1169.46, 1176.58, 1183.24]</t>
+          <t>[302.45, 307.91, 310.96, 313.62, 316.07, 318.39]</t>
         </is>
       </c>
       <c r="AU19" t="inlineStr">
         <is>
-          <t>[1135.3, 1128.34, 1127.45, 1127.56, 1128.19, 1129.14]</t>
+          <t>[302.45, 300.71, 300.79, 301.15, 301.68, 302.3]</t>
         </is>
       </c>
     </row>
@@ -3667,162 +3667,162 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>COFORGE</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>278417.14</v>
+        <v>76187.09</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>302.45</v>
+        <v>1721</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>₹300.39 - ₹305.53</t>
+          <t>₹1709.13 - ₹1738.8</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>310.68</v>
+        <v>1768.46</v>
       </c>
       <c r="I20" t="n">
-        <v>324</v>
+        <v>56</v>
       </c>
       <c r="J20" t="n">
-        <v>281.7</v>
+        <v>1505.99</v>
       </c>
       <c r="K20" t="n">
-        <v>268.93</v>
+        <v>1472.15</v>
       </c>
       <c r="L20" t="n">
-        <v>274.01</v>
+        <v>1507.99</v>
       </c>
       <c r="M20" t="n">
-        <v>13.37</v>
+        <v>15.58</v>
       </c>
       <c r="N20" t="n">
-        <v>9.93</v>
+        <v>53.48</v>
       </c>
       <c r="O20" t="n">
-        <v>8.42</v>
+        <v>30.14</v>
       </c>
       <c r="P20" t="n">
-        <v>1.51</v>
+        <v>23.34</v>
       </c>
       <c r="Q20" t="n">
-        <v>10.28</v>
+        <v>59.33</v>
       </c>
       <c r="R20" t="n">
         <v>11.76</v>
       </c>
       <c r="S20" t="n">
-        <v>48.9</v>
+        <v>46.1</v>
       </c>
       <c r="T20" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="U20" t="n">
-        <v>-2.21</v>
+        <v>-2.42</v>
       </c>
       <c r="V20" t="n">
-        <v>50</v>
+        <v>48.3</v>
       </c>
       <c r="W20" t="n">
-        <v>2.44</v>
+        <v>7.48</v>
       </c>
       <c r="X20" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y20" t="n">
-        <v>299.26</v>
+        <v>1705.12</v>
       </c>
       <c r="Z20" t="n">
-        <v>309.85</v>
+        <v>1765.36</v>
       </c>
       <c r="AA20" t="n">
-        <v>304.87</v>
+        <v>1734.77</v>
       </c>
       <c r="AB20" t="n">
-        <v>287.03</v>
+        <v>1632.01</v>
       </c>
       <c r="AC20" t="n">
-        <v>306.75</v>
+        <v>1713.83</v>
       </c>
       <c r="AD20" t="n">
-        <v>311.7</v>
+        <v>1745.96</v>
       </c>
       <c r="AE20" t="n">
-        <v>320.95</v>
+        <v>1770.93</v>
       </c>
       <c r="AF20" t="n">
-        <v>65.40000000000001</v>
+        <v>77.3</v>
       </c>
       <c r="AG20" t="n">
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI20" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ20" t="n">
-        <v>672.1</v>
+        <v>35.2</v>
       </c>
       <c r="AK20" t="n">
-        <v>182</v>
+        <v>49.9</v>
       </c>
       <c r="AL20" t="n">
-        <v>0.6</v>
+        <v>9.6</v>
       </c>
       <c r="AM20" t="n">
         <v>15</v>
       </c>
       <c r="AN20" t="n">
-        <v>313.56</v>
+        <v>1789.44</v>
       </c>
       <c r="AO20" t="n">
-        <v>292.1</v>
+        <v>1653.38</v>
       </c>
       <c r="AP20" t="inlineStr">
         <is>
-          <t>ETERNAL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹278,417.14 Cr., a P/E ratio of 672.11, and YoY Revenue Growth of +182.0%, the company demonstrates strong institutional backing, solid operating profit margins (0.64%), and healthy Return on Equity (15.00%).</t>
+          <t>COFORGE operates in the Technology sector. With an estimated Market Cap of ₹76,187.09 Cr., a P/E ratio of 35.21, and YoY Revenue Growth of +49.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ20" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 65.40 (Bullish Momentum Zone), while MACD Line (9.93) trades above Signal (8.42) with an expanding histogram (+1.51). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +13.37% above the 200-day DMA (₹274.01). Daily volatility envelope is bounded by ATR(14) of ₹10.28.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 77.31 (Bullish Momentum Zone), while MACD Line (53.48) trades above Signal (30.14) with an expanding histogram (+23.34). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +15.58% above the 200-day DMA (₹1507.99). Daily volatility envelope is bounded by ATR(14) of ₹59.33.</t>
         </is>
       </c>
       <c r="AR20" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ETERNAL. Current Market Price (₹302.45) is positioned above the 30-day DMA (₹281.70), 50-day DMA (₹268.93), and 200-day DMA (₹274.01). The price distance from 200 DMA is +13.37%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for COFORGE. Current Market Price (₹1,721.00) is positioned above the 30-day DMA (₹1,505.99), 50-day DMA (₹1,472.15), and 200-day DMA (₹1,507.99). The price distance from 200 DMA is +15.58%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS20" t="inlineStr">
         <is>
-          <t>[302.45, 303.8, 305.15, 306.5, 307.85, 309.19]</t>
+          <t>[1721.0, 1730.94, 1740.87, 1750.81, 1760.74, 1770.68]</t>
         </is>
       </c>
       <c r="AT20" t="inlineStr">
         <is>
-          <t>[302.45, 307.91, 310.96, 313.62, 316.07, 318.39]</t>
+          <t>[1721.0, 1754.67, 1774.43, 1791.91, 1808.2, 1823.74]</t>
         </is>
       </c>
       <c r="AU20" t="inlineStr">
         <is>
-          <t>[302.45, 300.71, 300.79, 301.15, 301.68, 302.3]</t>
+          <t>[1721.0, 1713.14, 1715.7, 1719.98, 1725.15, 1730.88]</t>
         </is>
       </c>
     </row>
@@ -3834,162 +3834,136 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>COFORGE</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Basic Materials</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>76187.09</v>
+        <v>263368.34</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>🔴 AVOID / HOLD</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>1721</v>
-      </c>
+          <t>🟡 MODERATE BUY</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>₹1709.13 - ₹1738.8</t>
-        </is>
-      </c>
-      <c r="H21" t="n">
-        <v>1768.46</v>
-      </c>
+          <t>₹nan - ₹nan</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="n">
-        <v>56</v>
+        <v>500</v>
       </c>
       <c r="J21" t="n">
-        <v>1505.99</v>
+        <v>2687.36</v>
       </c>
       <c r="K21" t="n">
-        <v>1472.15</v>
+        <v>2675.37</v>
       </c>
       <c r="L21" t="n">
-        <v>1507.99</v>
+        <v>2568.56</v>
       </c>
       <c r="M21" t="n">
-        <v>15.58</v>
+        <v>7.39</v>
       </c>
       <c r="N21" t="n">
-        <v>53.48</v>
+        <v>13.44</v>
       </c>
       <c r="O21" t="n">
-        <v>30.14</v>
+        <v>8.58</v>
       </c>
       <c r="P21" t="n">
-        <v>23.34</v>
+        <v>4.86</v>
       </c>
       <c r="Q21" t="n">
-        <v>59.33</v>
+        <v>54.77</v>
       </c>
       <c r="R21" t="n">
         <v>11.76</v>
       </c>
       <c r="S21" t="n">
-        <v>45.7</v>
-      </c>
-      <c r="T21" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="U21" t="n">
-        <v>-2.44</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="T21" t="inlineStr"/>
+      <c r="U21" t="inlineStr"/>
       <c r="V21" t="n">
-        <v>48.3</v>
+        <v>55</v>
       </c>
       <c r="W21" t="n">
-        <v>7.48</v>
+        <v>1.88</v>
       </c>
       <c r="X21" t="n">
         <v>-0.77</v>
       </c>
-      <c r="Y21" t="n">
-        <v>1705.17</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>1765.4</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>1734.77</v>
-      </c>
-      <c r="AB21" t="n">
-        <v>1632.01</v>
-      </c>
-      <c r="AC21" t="n">
-        <v>1713.83</v>
-      </c>
-      <c r="AD21" t="n">
-        <v>1745.96</v>
-      </c>
-      <c r="AE21" t="n">
-        <v>1770.93</v>
-      </c>
+      <c r="Y21" t="inlineStr"/>
+      <c r="Z21" t="inlineStr"/>
+      <c r="AA21" t="inlineStr"/>
+      <c r="AB21" t="inlineStr"/>
+      <c r="AC21" t="inlineStr"/>
+      <c r="AD21" t="inlineStr"/>
+      <c r="AE21" t="inlineStr"/>
       <c r="AF21" t="n">
-        <v>77.3</v>
+        <v>65.8</v>
       </c>
       <c r="AG21" t="n">
-        <v>0.16</v>
+        <v>-0.07000000000000001</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Vol Spike 3.9x | TTM Squeeze | Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI21" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ21" t="n">
-        <v>35.2</v>
+        <v>55.2</v>
       </c>
       <c r="AK21" t="n">
-        <v>49.9</v>
+        <v>17.9</v>
       </c>
       <c r="AL21" t="n">
-        <v>9.6</v>
+        <v>12.8</v>
       </c>
       <c r="AM21" t="n">
         <v>15</v>
       </c>
-      <c r="AN21" t="n">
-        <v>1787.32</v>
-      </c>
-      <c r="AO21" t="n">
-        <v>1656.89</v>
-      </c>
+      <c r="AN21" t="inlineStr"/>
+      <c r="AO21" t="inlineStr"/>
       <c r="AP21" t="inlineStr">
         <is>
-          <t>COFORGE operates in the Technology sector. With an estimated Market Cap of ₹76,187.09 Cr., a P/E ratio of 35.21, and YoY Revenue Growth of +49.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.64%), and healthy Return on Equity (15.00%).</t>
+          <t>ASIANPAINT operates in the Basic Materials sector. With an estimated Market Cap of ₹263,368.34 Cr., a P/E ratio of 55.24, and YoY Revenue Growth of +17.9%, the company demonstrates strong institutional backing, solid operating profit margins (12.81%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ21" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 77.31 (Bullish Momentum Zone), while MACD Line (53.48) trades above Signal (30.14) with an expanding histogram (+23.34). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +15.58% above the 200-day DMA (₹1507.99). Daily volatility envelope is bounded by ATR(14) of ₹59.33.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 65.78 (Bullish Momentum Zone), while MACD Line (13.44) trades above Signal (8.58) with an expanding histogram (+4.86). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +7.39% above the 200-day DMA (₹2568.56). Daily volatility envelope is bounded by ATR(14) of ₹54.77.</t>
         </is>
       </c>
       <c r="AR21" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for COFORGE. Current Market Price (₹1,721.00) is positioned above the 30-day DMA (₹1,505.99), 50-day DMA (₹1,472.15), and 200-day DMA (₹1,507.99). The price distance from 200 DMA is +15.58%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ASIANPAINT. Current Market Price (₹nan) is positioned above the 30-day DMA (₹2,687.36), 50-day DMA (₹2,675.37), and 200-day DMA (₹2,568.56). The price distance from 200 DMA is +7.39%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS21" t="inlineStr">
         <is>
-          <t>[1721.0, 1730.98, 1740.97, 1750.95, 1760.93, 1770.91]</t>
+          <t>[nan, nan, nan, nan, nan, nan]</t>
         </is>
       </c>
       <c r="AT21" t="inlineStr">
         <is>
-          <t>[1721.0, 1754.71, 1774.53, 1792.05, 1808.39, 1823.98]</t>
+          <t>[nan, nan, nan, nan, nan, nan]</t>
         </is>
       </c>
       <c r="AU21" t="inlineStr">
         <is>
-          <t>[1721.0, 1713.18, 1715.79, 1720.12, 1725.33, 1731.11]</t>
+          <t>[nan, nan, nan, nan, nan, nan]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Re-train ML prediction engine on 2-year active market regime and refresh web dashboard predictions
</commit_message>
<xml_diff>
--- a/Breakout_ML_Quant_Predictions.xlsx
+++ b/Breakout_ML_Quant_Predictions.xlsx
@@ -719,28 +719,28 @@
         <v>11.76</v>
       </c>
       <c r="S2" t="n">
-        <v>50.2</v>
+        <v>55.2</v>
       </c>
       <c r="T2" t="n">
         <v>0.32</v>
       </c>
       <c r="U2" t="n">
-        <v>-0.86</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="W2" t="n">
-        <v>1.33</v>
+        <v>6.24</v>
       </c>
       <c r="X2" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y2" t="n">
-        <v>1415.53</v>
+        <v>1424.81</v>
       </c>
       <c r="Z2" t="n">
-        <v>1465.77</v>
+        <v>1471.73</v>
       </c>
       <c r="AA2" t="n">
         <v>1446.88</v>
@@ -784,10 +784,10 @@
         <v>16.1</v>
       </c>
       <c r="AN2" t="n">
-        <v>1492.2</v>
+        <v>1462.68</v>
       </c>
       <c r="AO2" t="n">
-        <v>1383.2</v>
+        <v>1407.05</v>
       </c>
       <c r="AP2" t="inlineStr">
         <is>
@@ -806,17 +806,17 @@
       </c>
       <c r="AS2" t="inlineStr">
         <is>
-          <t>[1435.4, 1439.71, 1444.01, 1448.32, 1452.62, 1456.93]</t>
+          <t>[1435.4, 1446.34, 1457.29, 1468.23, 1479.18, 1490.12]</t>
         </is>
       </c>
       <c r="AT2" t="inlineStr">
         <is>
-          <t>[1435.4, 1449.39, 1457.71, 1465.1, 1472.0, 1478.6]</t>
+          <t>[1435.4, 1456.03, 1470.99, 1485.02, 1498.56, 1511.79]</t>
         </is>
       </c>
       <c r="AU2" t="inlineStr">
         <is>
-          <t>[1435.4, 1432.44, 1433.74, 1435.73, 1438.09, 1440.68]</t>
+          <t>[1435.4, 1439.08, 1447.01, 1455.65, 1464.65, 1473.88]</t>
         </is>
       </c>
     </row>
@@ -886,28 +886,28 @@
         <v>11.76</v>
       </c>
       <c r="S3" t="n">
-        <v>50.4</v>
+        <v>52.9</v>
       </c>
       <c r="T3" t="n">
         <v>0.29</v>
       </c>
       <c r="U3" t="n">
-        <v>-0.97</v>
+        <v>-0.88</v>
       </c>
       <c r="V3" t="n">
-        <v>51.5</v>
+        <v>51.7</v>
       </c>
       <c r="W3" t="n">
-        <v>2.23</v>
+        <v>3.29</v>
       </c>
       <c r="X3" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y3" t="n">
-        <v>111.24</v>
+        <v>111.33</v>
       </c>
       <c r="Z3" t="n">
-        <v>115.19</v>
+        <v>115.27</v>
       </c>
       <c r="AA3" t="n">
         <v>113.61</v>
@@ -951,10 +951,10 @@
         <v>15</v>
       </c>
       <c r="AN3" t="n">
-        <v>117.69</v>
+        <v>115.97</v>
       </c>
       <c r="AO3" t="n">
-        <v>107.9</v>
+        <v>109.92</v>
       </c>
       <c r="AP3" t="inlineStr">
         <is>
@@ -995,162 +995,162 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>HAL</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>310746.28</v>
+        <v>215046.57</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>🔴 AVOID / HOLD</t>
+          <t>🟡 MODERATE BUY</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>4646.5</v>
+        <v>7833.5</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>₹4629.85 - ₹4671.48</t>
+          <t>₹7803.39 - ₹7878.67</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>4713.1</v>
+        <v>7953.95</v>
       </c>
       <c r="I4" t="n">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="J4" t="n">
-        <v>4471.9</v>
+        <v>7437.81</v>
       </c>
       <c r="K4" t="n">
-        <v>4404.23</v>
+        <v>7344.46</v>
       </c>
       <c r="L4" t="n">
-        <v>4346.03</v>
+        <v>7171.21</v>
       </c>
       <c r="M4" t="n">
-        <v>5.42</v>
+        <v>9.19</v>
       </c>
       <c r="N4" t="n">
-        <v>56.6</v>
+        <v>121.41</v>
       </c>
       <c r="O4" t="n">
-        <v>49.9</v>
+        <v>84.98999999999999</v>
       </c>
       <c r="P4" t="n">
-        <v>6.7</v>
+        <v>36.42</v>
       </c>
       <c r="Q4" t="n">
-        <v>83.25</v>
+        <v>150.57</v>
       </c>
       <c r="R4" t="n">
         <v>11.76</v>
       </c>
       <c r="S4" t="n">
-        <v>47.6</v>
+        <v>49.5</v>
       </c>
       <c r="T4" t="n">
-        <v>0.3</v>
+        <v>0.39</v>
       </c>
       <c r="U4" t="n">
-        <v>-1.03</v>
+        <v>-0.9</v>
       </c>
       <c r="V4" t="n">
-        <v>50.4</v>
+        <v>48.3</v>
       </c>
       <c r="W4" t="n">
-        <v>2.04</v>
+        <v>1.92</v>
       </c>
       <c r="X4" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y4" t="n">
-        <v>4611.35</v>
+        <v>7803.37</v>
       </c>
       <c r="Z4" t="n">
-        <v>4771.38</v>
+        <v>8059.35</v>
       </c>
       <c r="AA4" t="n">
-        <v>4683.67</v>
+        <v>7920.87</v>
       </c>
       <c r="AB4" t="n">
-        <v>4521.62</v>
+        <v>7607.65</v>
       </c>
       <c r="AC4" t="n">
-        <v>4635.53</v>
+        <v>7842.17</v>
       </c>
       <c r="AD4" t="n">
-        <v>4679.96</v>
+        <v>7890.34</v>
       </c>
       <c r="AE4" t="n">
-        <v>4713.43</v>
+        <v>7947.17</v>
       </c>
       <c r="AF4" t="n">
-        <v>59.3</v>
+        <v>74.09999999999999</v>
       </c>
       <c r="AG4" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Vol Spike 2.7x | Inst. Buying (CMF+) | Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI4" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ4" t="n">
-        <v>34.1</v>
+        <v>37.3</v>
       </c>
       <c r="AK4" t="n">
-        <v>1.8</v>
+        <v>31.5</v>
       </c>
       <c r="AL4" t="n">
-        <v>27.5</v>
+        <v>23.2</v>
       </c>
       <c r="AM4" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="AN4" t="n">
-        <v>4815.85</v>
+        <v>8055.52</v>
       </c>
       <c r="AO4" t="n">
-        <v>4473.38</v>
+        <v>7646.07</v>
       </c>
       <c r="AP4" t="inlineStr">
         <is>
-          <t>HAL operates in the Industrials sector. With an estimated Market Cap of ₹310,746.28 Cr., a P/E ratio of 34.13, and YoY Revenue Growth of +1.8%, the company demonstrates strong institutional backing, solid operating profit margins (27.55%), and healthy Return on Equity (23.98%).</t>
+          <t>EICHERMOT operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹215,046.57 Cr., a P/E ratio of 37.31, and YoY Revenue Growth of +31.5%, the company demonstrates strong institutional backing, solid operating profit margins (23.21%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ4" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 59.26 (Bullish Momentum Zone), while MACD Line (56.60) trades above Signal (49.90) with an expanding histogram (+6.70). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +5.42% above the 200-day DMA (₹4346.03). Daily volatility envelope is bounded by ATR(14) of ₹83.25.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 74.10 (Bullish Momentum Zone), while MACD Line (121.41) trades above Signal (84.99) with an expanding histogram (+36.42). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +9.19% above the 200-day DMA (₹7171.21). Daily volatility envelope is bounded by ATR(14) of ₹150.57.</t>
         </is>
       </c>
       <c r="AR4" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for HAL. Current Market Price (₹4,646.50) is positioned above the 30-day DMA (₹4,471.90), 50-day DMA (₹4,404.23), and 200-day DMA (₹4,346.03). The price distance from 200 DMA is +5.42%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for EICHERMOT. Current Market Price (₹7,833.50) is positioned above the 30-day DMA (₹7,437.81), 50-day DMA (₹7,344.46), and 200-day DMA (₹7,171.21). The price distance from 200 DMA is +9.19%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS4" t="inlineStr">
         <is>
-          <t>[4646.5, 4681.04, 4715.59, 4750.13, 4784.67, 4819.22]</t>
+          <t>[7833.5, 7920.87, 8008.25, 8095.62, 8183.0, 8270.37]</t>
         </is>
       </c>
       <c r="AT4" t="inlineStr">
         <is>
-          <t>[4646.5, 4714.34, 4762.68, 4807.81, 4851.27, 4893.68]</t>
+          <t>[7833.5, 7981.1, 8093.42, 8199.94, 8303.45, 8405.04]</t>
         </is>
       </c>
       <c r="AU4" t="inlineStr">
         <is>
-          <t>[4646.5, 4656.07, 4680.27, 4706.87, 4734.72, 4763.37]</t>
+          <t>[7833.5, 7875.7, 7944.37, 8017.39, 8092.66, 8169.37]</t>
         </is>
       </c>
     </row>
@@ -1162,16 +1162,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>RECLTD</t>
+          <t>BHARATFORG</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>98206.09</v>
+        <v>105169.94</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1179,145 +1179,145 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>372.95</v>
+        <v>2199.8</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>₹371.41 - ₹375.26</t>
+          <t>₹2190.26 - ₹2214.11</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>379.11</v>
+        <v>2237.97</v>
       </c>
       <c r="I5" t="n">
-        <v>432</v>
+        <v>69</v>
       </c>
       <c r="J5" t="n">
-        <v>357.21</v>
+        <v>2140.62</v>
       </c>
       <c r="K5" t="n">
-        <v>349.78</v>
+        <v>2061.08</v>
       </c>
       <c r="L5" t="n">
-        <v>347.56</v>
+        <v>1703.8</v>
       </c>
       <c r="M5" t="n">
-        <v>6.64</v>
+        <v>27.05</v>
       </c>
       <c r="N5" t="n">
-        <v>4.07</v>
+        <v>29.77</v>
       </c>
       <c r="O5" t="n">
-        <v>2.35</v>
+        <v>35.4</v>
       </c>
       <c r="P5" t="n">
-        <v>1.72</v>
+        <v>-5.63</v>
       </c>
       <c r="Q5" t="n">
-        <v>7.7</v>
+        <v>47.71</v>
       </c>
       <c r="R5" t="n">
         <v>11.76</v>
       </c>
       <c r="S5" t="n">
-        <v>52.1</v>
+        <v>49.8</v>
       </c>
       <c r="T5" t="n">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="U5" t="n">
-        <v>-1.07</v>
+        <v>-1.23</v>
       </c>
       <c r="V5" t="n">
-        <v>53.4</v>
+        <v>50</v>
       </c>
       <c r="W5" t="n">
-        <v>4.29</v>
+        <v>1.78</v>
       </c>
       <c r="X5" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y5" t="n">
-        <v>368.15</v>
+        <v>2184.76</v>
       </c>
       <c r="Z5" t="n">
-        <v>381.21</v>
+        <v>2261.76</v>
       </c>
       <c r="AA5" t="n">
-        <v>375.93</v>
+        <v>2217.76</v>
       </c>
       <c r="AB5" t="n">
-        <v>361.4</v>
+        <v>2128.24</v>
       </c>
       <c r="AC5" t="n">
-        <v>372.32</v>
+        <v>2191.3</v>
       </c>
       <c r="AD5" t="n">
-        <v>374.64</v>
+        <v>2221.1</v>
       </c>
       <c r="AE5" t="n">
-        <v>376.32</v>
+        <v>2242.4</v>
       </c>
       <c r="AF5" t="n">
-        <v>78.3</v>
+        <v>57.9</v>
       </c>
       <c r="AG5" t="n">
-        <v>0.08</v>
+        <v>0.03</v>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>Low VIX (11.76) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI5" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ5" t="n">
-        <v>6.1</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="AK5" t="n">
-        <v>25.2</v>
+        <v>17.5</v>
       </c>
       <c r="AL5" t="n">
-        <v>68.90000000000001</v>
+        <v>6.4</v>
       </c>
       <c r="AM5" t="n">
-        <v>15</v>
+        <v>11.6</v>
       </c>
       <c r="AN5" t="n">
-        <v>388.5</v>
+        <v>2266.77</v>
       </c>
       <c r="AO5" t="n">
-        <v>357.92</v>
+        <v>2139.2</v>
       </c>
       <c r="AP5" t="inlineStr">
         <is>
-          <t>RECLTD operates in the Financial Services sector. With an estimated Market Cap of ₹98,206.09 Cr., a P/E ratio of 6.14, and YoY Revenue Growth of +25.2%, the company demonstrates strong institutional backing, solid operating profit margins (68.89%), and healthy Return on Equity (15.00%).</t>
+          <t>BHARATFORG operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹105,169.94 Cr., a P/E ratio of 97.08, and YoY Revenue Growth of +17.5%, the company demonstrates strong institutional backing, solid operating profit margins (6.42%), and healthy Return on Equity (11.60%).</t>
         </is>
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 78.30 (Bullish Momentum Zone), while MACD Line (4.07) trades above Signal (2.35) with an expanding histogram (+1.72). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +6.64% above the 200-day DMA (₹347.56). Daily volatility envelope is bounded by ATR(14) of ₹7.70.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 57.85 (Bullish Momentum Zone), while MACD Line (29.77) trades below Signal (35.40) with an expanding histogram (-5.63). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +27.05% above the 200-day DMA (₹1703.80). Daily volatility envelope is bounded by ATR(14) of ₹47.71.</t>
         </is>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for RECLTD. Current Market Price (₹372.95) is positioned above the 30-day DMA (₹357.21), 50-day DMA (₹349.78), and 200-day DMA (₹347.56). The price distance from 200 DMA is +6.64%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for BHARATFORG. Current Market Price (₹2,199.80) is positioned above the 30-day DMA (₹2,140.62), 50-day DMA (₹2,061.08), and 200-day DMA (₹1,703.80). The price distance from 200 DMA is +27.05%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS5" t="inlineStr">
         <is>
-          <t>[372.95, 374.07, 375.19, 376.31, 377.43, 378.54]</t>
+          <t>[2199.8, 2217.76, 2235.72, 2253.68, 2271.64, 2289.6]</t>
         </is>
       </c>
       <c r="AT5" t="inlineStr">
         <is>
-          <t>[372.95, 377.15, 379.54, 381.64, 383.59, 385.43]</t>
+          <t>[2199.8, 2236.84, 2262.71, 2286.73, 2309.8, 2332.27]</t>
         </is>
       </c>
       <c r="AU5" t="inlineStr">
         <is>
-          <t>[372.95, 371.76, 371.92, 372.31, 372.8, 373.38]</t>
+          <t>[2199.8, 2203.45, 2215.48, 2228.89, 2243.01, 2257.59]</t>
         </is>
       </c>
     </row>
@@ -1329,7 +1329,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>INDHOTEL</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1338,153 +1338,153 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>215046.57</v>
+        <v>105127.58</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7833.5</v>
+        <v>738.55</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>₹7803.39 - ₹7878.67</t>
+          <t>₹735.6 - ₹742.98</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>7953.95</v>
+        <v>750.37</v>
       </c>
       <c r="I6" t="n">
-        <v>22</v>
+        <v>225</v>
       </c>
       <c r="J6" t="n">
-        <v>7437.81</v>
+        <v>729.51</v>
       </c>
       <c r="K6" t="n">
-        <v>7344.46</v>
+        <v>703.6799999999999</v>
       </c>
       <c r="L6" t="n">
-        <v>7171.21</v>
+        <v>686.09</v>
       </c>
       <c r="M6" t="n">
-        <v>9.19</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="N6" t="n">
-        <v>121.41</v>
+        <v>8.49</v>
       </c>
       <c r="O6" t="n">
-        <v>84.98999999999999</v>
+        <v>9.380000000000001</v>
       </c>
       <c r="P6" t="n">
-        <v>36.42</v>
+        <v>-0.9</v>
       </c>
       <c r="Q6" t="n">
-        <v>150.57</v>
+        <v>14.77</v>
       </c>
       <c r="R6" t="n">
         <v>11.76</v>
       </c>
       <c r="S6" t="n">
-        <v>48.4</v>
+        <v>46.5</v>
       </c>
       <c r="T6" t="n">
-        <v>0.28</v>
+        <v>0.27</v>
       </c>
       <c r="U6" t="n">
-        <v>-1.1</v>
+        <v>-1.23</v>
       </c>
       <c r="V6" t="n">
-        <v>50.2</v>
+        <v>55</v>
       </c>
       <c r="W6" t="n">
-        <v>5.13</v>
+        <v>5.75</v>
       </c>
       <c r="X6" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y6" t="n">
-        <v>7728.5</v>
+        <v>720.8200000000001</v>
       </c>
       <c r="Z6" t="n">
-        <v>8002.67</v>
+        <v>725.27</v>
       </c>
       <c r="AA6" t="n">
-        <v>7896.17</v>
+        <v>744.46</v>
       </c>
       <c r="AB6" t="n">
-        <v>7607.65</v>
+        <v>716.39</v>
       </c>
       <c r="AC6" t="n">
-        <v>7842.17</v>
+        <v>744.27</v>
       </c>
       <c r="AD6" t="n">
-        <v>7890.34</v>
+        <v>751.6900000000001</v>
       </c>
       <c r="AE6" t="n">
-        <v>7947.17</v>
+        <v>764.8200000000001</v>
       </c>
       <c r="AF6" t="n">
-        <v>74.09999999999999</v>
+        <v>48.2</v>
       </c>
       <c r="AG6" t="n">
-        <v>0.19</v>
+        <v>0.04</v>
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>Vol Spike 2.7x | Inst. Buying (CMF+) | Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI6" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ6" t="n">
-        <v>37.3</v>
+        <v>49</v>
       </c>
       <c r="AK6" t="n">
-        <v>31.5</v>
+        <v>15.1</v>
       </c>
       <c r="AL6" t="n">
-        <v>23.2</v>
+        <v>20.9</v>
       </c>
       <c r="AM6" t="n">
         <v>15</v>
       </c>
       <c r="AN6" t="n">
-        <v>9251.1</v>
+        <v>758.27</v>
       </c>
       <c r="AO6" t="n">
-        <v>6460.02</v>
+        <v>719.9400000000001</v>
       </c>
       <c r="AP6" t="inlineStr">
         <is>
-          <t>EICHERMOT operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹215,046.57 Cr., a P/E ratio of 37.31, and YoY Revenue Growth of +31.5%, the company demonstrates strong institutional backing, solid operating profit margins (23.21%), and healthy Return on Equity (15.00%).</t>
+          <t>INDHOTEL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹105,127.58 Cr., a P/E ratio of 49.01, and YoY Revenue Growth of +15.1%, the company demonstrates strong institutional backing, solid operating profit margins (20.87%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ6" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 74.10 (Bullish Momentum Zone), while MACD Line (121.41) trades above Signal (84.99) with an expanding histogram (+36.42). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +9.19% above the 200-day DMA (₹7171.21). Daily volatility envelope is bounded by ATR(14) of ₹150.57.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 48.23 (Consolidation Zone), while MACD Line (8.49) trades below Signal (9.38) with an expanding histogram (-0.90). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +9.21% above the 200-day DMA (₹686.09). Daily volatility envelope is bounded by ATR(14) of ₹14.77.</t>
         </is>
       </c>
       <c r="AR6" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for EICHERMOT. Current Market Price (₹7,833.50) is positioned above the 30-day DMA (₹7,437.81), 50-day DMA (₹7,344.46), and 200-day DMA (₹7,171.21). The price distance from 200 DMA is +9.19%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for INDHOTEL. Current Market Price (₹738.55) is positioned above the 30-day DMA (₹729.51), 50-day DMA (₹703.68), and 200-day DMA (₹686.09). The price distance from 200 DMA is +9.21%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS6" t="inlineStr">
         <is>
-          <t>[7833.5, 7857.0, 7880.5, 7904.0, 7927.5, 7951.0]</t>
+          <t>[738.55, 740.77, 742.98, 745.2, 747.41, 749.63]</t>
         </is>
       </c>
       <c r="AT6" t="inlineStr">
         <is>
-          <t>[7833.5, 7917.23, 7965.67, 8008.32, 8047.95, 8085.67]</t>
+          <t>[738.55, 746.67, 751.34, 755.43, 759.23, 762.84]</t>
         </is>
       </c>
       <c r="AU6" t="inlineStr">
         <is>
-          <t>[7833.5, 7811.83, 7816.62, 7825.77, 7837.16, 7850.0]</t>
+          <t>[738.55, 736.33, 736.71, 737.52, 738.55, 739.72]</t>
         </is>
       </c>
     </row>
@@ -1496,162 +1496,162 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>INDHOTEL</t>
+          <t>HAL</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>105127.58</v>
+        <v>310746.28</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>738.55</v>
+        <v>4646.5</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>₹735.6 - ₹742.98</t>
+          <t>₹4629.85 - ₹4671.48</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>750.37</v>
+        <v>4713.1</v>
       </c>
       <c r="I7" t="n">
-        <v>225</v>
+        <v>40</v>
       </c>
       <c r="J7" t="n">
-        <v>729.51</v>
+        <v>4471.9</v>
       </c>
       <c r="K7" t="n">
-        <v>703.6799999999999</v>
+        <v>4404.23</v>
       </c>
       <c r="L7" t="n">
-        <v>686.09</v>
+        <v>4346.03</v>
       </c>
       <c r="M7" t="n">
-        <v>9.210000000000001</v>
+        <v>5.42</v>
       </c>
       <c r="N7" t="n">
-        <v>8.49</v>
+        <v>56.6</v>
       </c>
       <c r="O7" t="n">
-        <v>9.380000000000001</v>
+        <v>49.9</v>
       </c>
       <c r="P7" t="n">
-        <v>-0.9</v>
+        <v>6.7</v>
       </c>
       <c r="Q7" t="n">
-        <v>14.77</v>
+        <v>83.25</v>
       </c>
       <c r="R7" t="n">
         <v>11.76</v>
       </c>
       <c r="S7" t="n">
-        <v>49.3</v>
+        <v>41.7</v>
       </c>
       <c r="T7" t="n">
-        <v>0.27</v>
+        <v>0.3</v>
       </c>
       <c r="U7" t="n">
-        <v>-1.13</v>
+        <v>-1.23</v>
       </c>
       <c r="V7" t="n">
-        <v>53</v>
+        <v>41.7</v>
       </c>
       <c r="W7" t="n">
-        <v>2.84</v>
+        <v>2.15</v>
       </c>
       <c r="X7" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y7" t="n">
-        <v>727.6</v>
+        <v>4548.57</v>
       </c>
       <c r="Z7" t="n">
-        <v>753.45</v>
+        <v>4711.2</v>
       </c>
       <c r="AA7" t="n">
-        <v>744.46</v>
+        <v>4683.67</v>
       </c>
       <c r="AB7" t="n">
-        <v>716.39</v>
+        <v>4521.62</v>
       </c>
       <c r="AC7" t="n">
-        <v>744.27</v>
+        <v>4635.53</v>
       </c>
       <c r="AD7" t="n">
-        <v>751.6900000000001</v>
+        <v>4679.96</v>
       </c>
       <c r="AE7" t="n">
-        <v>764.8200000000001</v>
+        <v>4713.43</v>
       </c>
       <c r="AF7" t="n">
-        <v>48.2</v>
+        <v>59.3</v>
       </c>
       <c r="AG7" t="n">
-        <v>0.04</v>
+        <v>0.2</v>
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI7" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ7" t="n">
-        <v>49</v>
+        <v>34.1</v>
       </c>
       <c r="AK7" t="n">
-        <v>15.1</v>
+        <v>1.8</v>
       </c>
       <c r="AL7" t="n">
-        <v>20.9</v>
+        <v>27.5</v>
       </c>
       <c r="AM7" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="AN7" t="n">
-        <v>767.5700000000001</v>
+        <v>4768.55</v>
       </c>
       <c r="AO7" t="n">
-        <v>710.38</v>
+        <v>4526.98</v>
       </c>
       <c r="AP7" t="inlineStr">
         <is>
-          <t>INDHOTEL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹105,127.58 Cr., a P/E ratio of 49.01, and YoY Revenue Growth of +15.1%, the company demonstrates strong institutional backing, solid operating profit margins (20.87%), and healthy Return on Equity (15.00%).</t>
+          <t>HAL operates in the Industrials sector. With an estimated Market Cap of ₹310,746.28 Cr., a P/E ratio of 34.13, and YoY Revenue Growth of +1.8%, the company demonstrates strong institutional backing, solid operating profit margins (27.55%), and healthy Return on Equity (23.98%).</t>
         </is>
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 48.23 (Consolidation Zone), while MACD Line (8.49) trades below Signal (9.38) with an expanding histogram (-0.90). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +9.21% above the 200-day DMA (₹686.09). Daily volatility envelope is bounded by ATR(14) of ₹14.77.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 59.26 (Bullish Momentum Zone), while MACD Line (56.60) trades above Signal (49.90) with an expanding histogram (+6.70). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +5.42% above the 200-day DMA (₹4346.03). Daily volatility envelope is bounded by ATR(14) of ₹83.25.</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for INDHOTEL. Current Market Price (₹738.55) is positioned above the 30-day DMA (₹729.51), 50-day DMA (₹703.68), and 200-day DMA (₹686.09). The price distance from 200 DMA is +9.21%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for HAL. Current Market Price (₹4,646.50) is positioned above the 30-day DMA (₹4,471.90), 50-day DMA (₹4,404.23), and 200-day DMA (₹4,346.03). The price distance from 200 DMA is +5.42%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS7" t="inlineStr">
         <is>
-          <t>[738.55, 740.77, 742.98, 745.2, 747.41, 749.63]</t>
+          <t>[4646.5, 4660.44, 4674.38, 4688.32, 4702.26, 4716.2]</t>
         </is>
       </c>
       <c r="AT7" t="inlineStr">
         <is>
-          <t>[738.55, 746.67, 751.34, 755.43, 759.23, 762.84]</t>
+          <t>[4646.5, 4693.74, 4721.47, 4746.0, 4768.86, 4790.66]</t>
         </is>
       </c>
       <c r="AU7" t="inlineStr">
         <is>
-          <t>[738.55, 736.33, 736.71, 737.52, 738.55, 739.72]</t>
+          <t>[4646.5, 4635.46, 4639.06, 4645.06, 4652.31, 4660.35]</t>
         </is>
       </c>
     </row>
@@ -1663,162 +1663,162 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BHARATFORG</t>
+          <t>RECLTD</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>105169.94</v>
+        <v>98206.09</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>2199.8</v>
+        <v>372.95</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>₹2190.26 - ₹2214.11</t>
+          <t>₹371.41 - ₹375.26</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>2237.97</v>
+        <v>379.11</v>
       </c>
       <c r="I8" t="n">
-        <v>69</v>
+        <v>432</v>
       </c>
       <c r="J8" t="n">
-        <v>2140.62</v>
+        <v>357.21</v>
       </c>
       <c r="K8" t="n">
-        <v>2061.08</v>
+        <v>349.78</v>
       </c>
       <c r="L8" t="n">
-        <v>1703.8</v>
+        <v>347.56</v>
       </c>
       <c r="M8" t="n">
-        <v>27.05</v>
+        <v>6.64</v>
       </c>
       <c r="N8" t="n">
-        <v>29.77</v>
+        <v>4.07</v>
       </c>
       <c r="O8" t="n">
-        <v>35.4</v>
+        <v>2.35</v>
       </c>
       <c r="P8" t="n">
-        <v>-5.63</v>
+        <v>1.72</v>
       </c>
       <c r="Q8" t="n">
-        <v>47.71</v>
+        <v>7.7</v>
       </c>
       <c r="R8" t="n">
         <v>11.76</v>
       </c>
       <c r="S8" t="n">
-        <v>50.7</v>
+        <v>47.2</v>
       </c>
       <c r="T8" t="n">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="U8" t="n">
-        <v>-1.2</v>
+        <v>-1.26</v>
       </c>
       <c r="V8" t="n">
-        <v>52.2</v>
+        <v>50</v>
       </c>
       <c r="W8" t="n">
-        <v>2.26</v>
+        <v>2.81</v>
       </c>
       <c r="X8" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y8" t="n">
-        <v>2170.27</v>
+        <v>366.16</v>
       </c>
       <c r="Z8" t="n">
-        <v>2247.27</v>
+        <v>379.22</v>
       </c>
       <c r="AA8" t="n">
-        <v>2217.4</v>
+        <v>375.93</v>
       </c>
       <c r="AB8" t="n">
-        <v>2128.24</v>
+        <v>361.4</v>
       </c>
       <c r="AC8" t="n">
-        <v>2191.3</v>
+        <v>372.32</v>
       </c>
       <c r="AD8" t="n">
-        <v>2221.1</v>
+        <v>374.64</v>
       </c>
       <c r="AE8" t="n">
-        <v>2242.4</v>
+        <v>376.32</v>
       </c>
       <c r="AF8" t="n">
-        <v>57.9</v>
+        <v>78.3</v>
       </c>
       <c r="AG8" t="n">
-        <v>0.03</v>
+        <v>0.08</v>
       </c>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI8" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ8" t="n">
-        <v>97.09999999999999</v>
+        <v>6.1</v>
       </c>
       <c r="AK8" t="n">
-        <v>17.5</v>
+        <v>25.2</v>
       </c>
       <c r="AL8" t="n">
-        <v>6.4</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="AM8" t="n">
-        <v>11.6</v>
+        <v>15</v>
       </c>
       <c r="AN8" t="n">
-        <v>2307.76</v>
+        <v>383.02</v>
       </c>
       <c r="AO8" t="n">
-        <v>2092.5</v>
+        <v>363.06</v>
       </c>
       <c r="AP8" t="inlineStr">
         <is>
-          <t>BHARATFORG operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹105,169.94 Cr., a P/E ratio of 97.08, and YoY Revenue Growth of +17.5%, the company demonstrates strong institutional backing, solid operating profit margins (6.42%), and healthy Return on Equity (11.60%).</t>
+          <t>RECLTD operates in the Financial Services sector. With an estimated Market Cap of ₹98,206.09 Cr., a P/E ratio of 6.14, and YoY Revenue Growth of +25.2%, the company demonstrates strong institutional backing, solid operating profit margins (68.89%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ8" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 57.85 (Bullish Momentum Zone), while MACD Line (29.77) trades below Signal (35.40) with an expanding histogram (-5.63). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +27.05% above the 200-day DMA (₹1703.80). Daily volatility envelope is bounded by ATR(14) of ₹47.71.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 78.30 (Bullish Momentum Zone), while MACD Line (4.07) trades above Signal (2.35) with an expanding histogram (+1.72). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +6.64% above the 200-day DMA (₹347.56). Daily volatility envelope is bounded by ATR(14) of ₹7.70.</t>
         </is>
       </c>
       <c r="AR8" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for BHARATFORG. Current Market Price (₹2,199.80) is positioned above the 30-day DMA (₹2,140.62), 50-day DMA (₹2,061.08), and 200-day DMA (₹1,703.80). The price distance from 200 DMA is +27.05%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for RECLTD. Current Market Price (₹372.95) is positioned above the 30-day DMA (₹357.21), 50-day DMA (₹349.78), and 200-day DMA (₹347.56). The price distance from 200 DMA is +6.64%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS8" t="inlineStr">
         <is>
-          <t>[2199.8, 2206.4, 2213.0, 2219.6, 2226.2, 2232.8]</t>
+          <t>[372.95, 374.07, 375.19, 376.31, 377.43, 378.54]</t>
         </is>
       </c>
       <c r="AT8" t="inlineStr">
         <is>
-          <t>[2199.8, 2225.48, 2239.99, 2252.65, 2264.36, 2275.47]</t>
+          <t>[372.95, 377.15, 379.54, 381.64, 383.59, 385.43]</t>
         </is>
       </c>
       <c r="AU8" t="inlineStr">
         <is>
-          <t>[2199.8, 2192.09, 2192.76, 2194.81, 2197.57, 2200.79]</t>
+          <t>[372.95, 371.76, 371.92, 372.31, 372.8, 373.38]</t>
         </is>
       </c>
     </row>
@@ -1843,7 +1843,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -1888,28 +1888,28 @@
         <v>11.76</v>
       </c>
       <c r="S9" t="n">
-        <v>48.1</v>
+        <v>47</v>
       </c>
       <c r="T9" t="n">
         <v>0.23</v>
       </c>
       <c r="U9" t="n">
-        <v>-1.44</v>
+        <v>-1.48</v>
       </c>
       <c r="V9" t="n">
-        <v>50.3</v>
+        <v>45</v>
       </c>
       <c r="W9" t="n">
-        <v>3.4</v>
+        <v>11.03</v>
       </c>
       <c r="X9" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y9" t="n">
-        <v>1442.83</v>
+        <v>1431.86</v>
       </c>
       <c r="Z9" t="n">
-        <v>1494.39</v>
+        <v>1388.25</v>
       </c>
       <c r="AA9" t="n">
         <v>1484.99</v>
@@ -1953,10 +1953,10 @@
         <v>15</v>
       </c>
       <c r="AN9" t="n">
-        <v>2156.84</v>
+        <v>1504.86</v>
       </c>
       <c r="AO9" t="n">
-        <v>813.36</v>
+        <v>1439.62</v>
       </c>
       <c r="AP9" t="inlineStr">
         <is>
@@ -2055,28 +2055,28 @@
         <v>11.76</v>
       </c>
       <c r="S10" t="n">
-        <v>50.2</v>
+        <v>50.8</v>
       </c>
       <c r="T10" t="n">
         <v>0.18</v>
       </c>
       <c r="U10" t="n">
-        <v>-1.85</v>
+        <v>-1.82</v>
       </c>
       <c r="V10" t="n">
-        <v>52.2</v>
+        <v>55</v>
       </c>
       <c r="W10" t="n">
-        <v>2.72</v>
+        <v>3.38</v>
       </c>
       <c r="X10" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y10" t="n">
-        <v>1033.78</v>
+        <v>1019.37</v>
       </c>
       <c r="Z10" t="n">
-        <v>1070.41</v>
+        <v>1056.01</v>
       </c>
       <c r="AA10" t="n">
         <v>1055.07</v>
@@ -2120,10 +2120,10 @@
         <v>18.5</v>
       </c>
       <c r="AN10" t="n">
-        <v>1093.82</v>
+        <v>1088.74</v>
       </c>
       <c r="AO10" t="n">
-        <v>1002.87</v>
+        <v>1013.57</v>
       </c>
       <c r="AP10" t="inlineStr">
         <is>
@@ -2164,7 +2164,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DIXON</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2173,153 +2173,153 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>85420.58</v>
+        <v>146280.27</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>14049</v>
+        <v>1651.3</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>₹13965.8 - ₹14173.8</t>
+          <t>₹1641.81 - ₹1665.54</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>14381.8</v>
+        <v>1689.26</v>
       </c>
       <c r="I11" t="n">
-        <v>8</v>
+        <v>70</v>
       </c>
       <c r="J11" t="n">
-        <v>13190.57</v>
+        <v>1478.49</v>
       </c>
       <c r="K11" t="n">
-        <v>12605.68</v>
+        <v>1460.44</v>
       </c>
       <c r="L11" t="n">
-        <v>12333.95</v>
+        <v>1458.79</v>
       </c>
       <c r="M11" t="n">
-        <v>16.25</v>
+        <v>14.41</v>
       </c>
       <c r="N11" t="n">
-        <v>477.1</v>
+        <v>56.22</v>
       </c>
       <c r="O11" t="n">
-        <v>503.84</v>
+        <v>42.84</v>
       </c>
       <c r="P11" t="n">
-        <v>-26.74</v>
+        <v>13.38</v>
       </c>
       <c r="Q11" t="n">
-        <v>416</v>
+        <v>47.45</v>
       </c>
       <c r="R11" t="n">
         <v>11.76</v>
       </c>
       <c r="S11" t="n">
-        <v>49.3</v>
+        <v>44.4</v>
       </c>
       <c r="T11" t="n">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="U11" t="n">
-        <v>-1.86</v>
+        <v>-2.04</v>
       </c>
       <c r="V11" t="n">
-        <v>48.9</v>
+        <v>48.3</v>
       </c>
       <c r="W11" t="n">
-        <v>3.54</v>
+        <v>8.69</v>
       </c>
       <c r="X11" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y11" t="n">
-        <v>13933.38</v>
+        <v>1625.33</v>
       </c>
       <c r="Z11" t="n">
-        <v>14425.1</v>
+        <v>1683.13</v>
       </c>
       <c r="AA11" t="n">
-        <v>14161.39</v>
+        <v>1664.51</v>
       </c>
       <c r="AB11" t="n">
-        <v>13425</v>
+        <v>1580.13</v>
       </c>
       <c r="AC11" t="n">
-        <v>14079.67</v>
+        <v>1641.1</v>
       </c>
       <c r="AD11" t="n">
-        <v>14558.34</v>
+        <v>1671.7</v>
       </c>
       <c r="AE11" t="n">
-        <v>15067.67</v>
+        <v>1692.1</v>
       </c>
       <c r="AF11" t="n">
-        <v>64.7</v>
+        <v>86.2</v>
       </c>
       <c r="AG11" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI11" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ11" t="n">
-        <v>41.2</v>
+        <v>28.6</v>
       </c>
       <c r="AK11" t="n">
-        <v>21.1</v>
+        <v>17.7</v>
       </c>
       <c r="AL11" t="n">
-        <v>3.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="AM11" t="n">
         <v>15</v>
       </c>
       <c r="AN11" t="n">
-        <v>14691.98</v>
+        <v>1700.37</v>
       </c>
       <c r="AO11" t="n">
-        <v>13511.14</v>
+        <v>1608.23</v>
       </c>
       <c r="AP11" t="inlineStr">
         <is>
-          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹85,420.58 Cr., a P/E ratio of 41.15, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
+          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹146,280.27 Cr., a P/E ratio of 28.57, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ11" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 64.72 (Bullish Momentum Zone), while MACD Line (477.10) trades below Signal (503.84) with an expanding histogram (-26.74). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +16.25% above the 200-day DMA (₹12333.95). Daily volatility envelope is bounded by ATR(14) of ₹416.00.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 86.21 (Bullish Momentum Zone), while MACD Line (56.22) trades above Signal (42.84) with an expanding histogram (+13.38). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +14.41% above the 200-day DMA (₹1458.79). Daily volatility envelope is bounded by ATR(14) of ₹47.45.</t>
         </is>
       </c>
       <c r="AR11" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,049.00) is positioned above the 30-day DMA (₹13,190.57), 50-day DMA (₹12,605.68), and 200-day DMA (₹12,333.95). The price distance from 200 DMA is +16.25%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,651.30) is positioned above the 30-day DMA (₹1,478.49), 50-day DMA (₹1,460.44), and 200-day DMA (₹1,458.79). The price distance from 200 DMA is +14.41%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS11" t="inlineStr">
         <is>
-          <t>[14049.0, 14144.12, 14239.24, 14334.35, 14429.47, 14524.59]</t>
+          <t>[1651.3, 1656.25, 1661.21, 1666.16, 1671.12, 1676.07]</t>
         </is>
       </c>
       <c r="AT11" t="inlineStr">
         <is>
-          <t>[14049.0, 14310.52, 14474.56, 14622.57, 14762.27, 14896.67]</t>
+          <t>[1651.3, 1675.23, 1688.05, 1699.04, 1709.08, 1718.51]</t>
         </is>
       </c>
       <c r="AU11" t="inlineStr">
         <is>
-          <t>[14049.0, 14019.32, 14062.74, 14118.19, 14179.87, 14245.53]</t>
+          <t>[1651.3, 1642.02, 1641.08, 1641.51, 1642.65, 1644.24]</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>DIXON</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2340,7 +2340,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>146280.27</v>
+        <v>85420.58</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2348,145 +2348,145 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1651.3</v>
+        <v>14049</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>₹1641.81 - ₹1665.54</t>
+          <t>₹13965.8 - ₹14173.8</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1689.26</v>
+        <v>14381.8</v>
       </c>
       <c r="I12" t="n">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="J12" t="n">
-        <v>1478.49</v>
+        <v>13190.57</v>
       </c>
       <c r="K12" t="n">
-        <v>1460.44</v>
+        <v>12605.68</v>
       </c>
       <c r="L12" t="n">
-        <v>1458.79</v>
+        <v>12333.95</v>
       </c>
       <c r="M12" t="n">
-        <v>14.41</v>
+        <v>16.25</v>
       </c>
       <c r="N12" t="n">
-        <v>56.22</v>
+        <v>477.1</v>
       </c>
       <c r="O12" t="n">
-        <v>42.84</v>
+        <v>503.84</v>
       </c>
       <c r="P12" t="n">
-        <v>13.38</v>
+        <v>-26.74</v>
       </c>
       <c r="Q12" t="n">
-        <v>47.45</v>
+        <v>416</v>
       </c>
       <c r="R12" t="n">
         <v>11.76</v>
       </c>
       <c r="S12" t="n">
-        <v>47.8</v>
+        <v>45.7</v>
       </c>
       <c r="T12" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="U12" t="n">
-        <v>-1.87</v>
+        <v>-2.05</v>
       </c>
       <c r="V12" t="n">
-        <v>50</v>
+        <v>46.7</v>
       </c>
       <c r="W12" t="n">
-        <v>1.71</v>
+        <v>6.67</v>
       </c>
       <c r="X12" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y12" t="n">
-        <v>1628.92</v>
+        <v>13634.81</v>
       </c>
       <c r="Z12" t="n">
-        <v>1686.72</v>
+        <v>14126.52</v>
       </c>
       <c r="AA12" t="n">
-        <v>1664.51</v>
+        <v>14161.39</v>
       </c>
       <c r="AB12" t="n">
-        <v>1580.13</v>
+        <v>13425</v>
       </c>
       <c r="AC12" t="n">
-        <v>1641.1</v>
+        <v>14079.67</v>
       </c>
       <c r="AD12" t="n">
-        <v>1671.7</v>
+        <v>14558.34</v>
       </c>
       <c r="AE12" t="n">
-        <v>1692.1</v>
+        <v>15067.67</v>
       </c>
       <c r="AF12" t="n">
-        <v>86.2</v>
+        <v>64.7</v>
       </c>
       <c r="AG12" t="n">
-        <v>0.06</v>
+        <v>0.11</v>
       </c>
       <c r="AH12" t="inlineStr">
         <is>
-          <t>Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI12" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ12" t="n">
-        <v>28.6</v>
+        <v>41.2</v>
       </c>
       <c r="AK12" t="n">
-        <v>17.7</v>
+        <v>21.1</v>
       </c>
       <c r="AL12" t="n">
-        <v>8.699999999999999</v>
+        <v>3.6</v>
       </c>
       <c r="AM12" t="n">
         <v>15</v>
       </c>
       <c r="AN12" t="n">
-        <v>1712.49</v>
+        <v>14625.09</v>
       </c>
       <c r="AO12" t="n">
-        <v>1593.5</v>
+        <v>13525.23</v>
       </c>
       <c r="AP12" t="inlineStr">
         <is>
-          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹146,280.27 Cr., a P/E ratio of 28.57, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
+          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹85,420.58 Cr., a P/E ratio of 41.15, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ12" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 86.21 (Bullish Momentum Zone), while MACD Line (56.22) trades above Signal (42.84) with an expanding histogram (+13.38). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +14.41% above the 200-day DMA (₹1458.79). Daily volatility envelope is bounded by ATR(14) of ₹47.45.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 64.72 (Bullish Momentum Zone), while MACD Line (477.10) trades below Signal (503.84) with an expanding histogram (-26.74). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +16.25% above the 200-day DMA (₹12333.95). Daily volatility envelope is bounded by ATR(14) of ₹416.00.</t>
         </is>
       </c>
       <c r="AR12" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,651.30) is positioned above the 30-day DMA (₹1,478.49), 50-day DMA (₹1,460.44), and 200-day DMA (₹1,458.79). The price distance from 200 DMA is +14.41%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,049.00) is positioned above the 30-day DMA (₹13,190.57), 50-day DMA (₹12,605.68), and 200-day DMA (₹12,333.95). The price distance from 200 DMA is +16.25%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS12" t="inlineStr">
         <is>
-          <t>[1651.3, 1656.25, 1661.21, 1666.16, 1671.12, 1676.07]</t>
+          <t>[14049.0, 14091.15, 14133.29, 14175.44, 14217.59, 14259.73]</t>
         </is>
       </c>
       <c r="AT12" t="inlineStr">
         <is>
-          <t>[1651.3, 1675.23, 1688.05, 1699.04, 1709.08, 1718.51]</t>
+          <t>[14049.0, 14257.55, 14368.62, 14463.65, 14550.39, 14631.82]</t>
         </is>
       </c>
       <c r="AU12" t="inlineStr">
         <is>
-          <t>[1651.3, 1642.02, 1641.08, 1641.51, 1642.65, 1644.24]</t>
+          <t>[14049.0, 13966.35, 13956.8, 13959.28, 13967.99, 13980.67]</t>
         </is>
       </c>
     </row>
@@ -2498,16 +2498,16 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>GODREJPROP</t>
+          <t>PGEL</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>63429.15</v>
+        <v>17572.27</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2515,145 +2515,145 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2105.7</v>
+        <v>613.35</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>₹2092.64 - ₹2125.3</t>
+          <t>₹608.87 - ₹620.07</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>2157.96</v>
+        <v>631.27</v>
       </c>
       <c r="I13" t="n">
-        <v>51</v>
+        <v>148</v>
       </c>
       <c r="J13" t="n">
-        <v>1999.45</v>
+        <v>578.01</v>
       </c>
       <c r="K13" t="n">
-        <v>1888.17</v>
+        <v>541.38</v>
       </c>
       <c r="L13" t="n">
-        <v>1880.41</v>
+        <v>553.54</v>
       </c>
       <c r="M13" t="n">
-        <v>12.26</v>
+        <v>10.74</v>
       </c>
       <c r="N13" t="n">
-        <v>62.25</v>
+        <v>14.56</v>
       </c>
       <c r="O13" t="n">
-        <v>68.98</v>
+        <v>16.43</v>
       </c>
       <c r="P13" t="n">
-        <v>-6.73</v>
+        <v>-1.88</v>
       </c>
       <c r="Q13" t="n">
-        <v>65.31999999999999</v>
+        <v>22.4</v>
       </c>
       <c r="R13" t="n">
         <v>11.76</v>
       </c>
       <c r="S13" t="n">
-        <v>48.4</v>
+        <v>51.3</v>
       </c>
       <c r="T13" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="U13" t="n">
-        <v>-2.01</v>
+        <v>-2.26</v>
       </c>
       <c r="V13" t="n">
-        <v>52.5</v>
+        <v>53.3</v>
       </c>
       <c r="W13" t="n">
-        <v>2.38</v>
+        <v>4.8</v>
       </c>
       <c r="X13" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y13" t="n">
-        <v>2079.55</v>
+        <v>590.26</v>
       </c>
       <c r="Z13" t="n">
-        <v>2153.25</v>
+        <v>611.73</v>
       </c>
       <c r="AA13" t="n">
-        <v>2122.55</v>
+        <v>618.26</v>
       </c>
       <c r="AB13" t="n">
-        <v>2007.72</v>
+        <v>579.75</v>
       </c>
       <c r="AC13" t="n">
-        <v>2111.93</v>
+        <v>616.27</v>
       </c>
       <c r="AD13" t="n">
-        <v>2127.76</v>
+        <v>624.54</v>
       </c>
       <c r="AE13" t="n">
-        <v>2149.83</v>
+        <v>635.72</v>
       </c>
       <c r="AF13" t="n">
-        <v>48.8</v>
+        <v>60.8</v>
       </c>
       <c r="AG13" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI13" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ13" t="n">
-        <v>34.2</v>
+        <v>88.5</v>
       </c>
       <c r="AK13" t="n">
-        <v>63</v>
+        <v>-10.1</v>
       </c>
       <c r="AL13" t="n">
-        <v>36.1</v>
+        <v>3.7</v>
       </c>
       <c r="AM13" t="n">
-        <v>10</v>
+        <v>6.7</v>
       </c>
       <c r="AN13" t="n">
-        <v>2188.09</v>
+        <v>645.35</v>
       </c>
       <c r="AO13" t="n">
-        <v>2027.94</v>
+        <v>584.29</v>
       </c>
       <c r="AP13" t="inlineStr">
         <is>
-          <t>GODREJPROP operates in the Real Estate sector. With an estimated Market Cap of ₹63,429.15 Cr., a P/E ratio of 34.24, and YoY Revenue Growth of +63.0%, the company demonstrates strong institutional backing, solid operating profit margins (36.06%), and healthy Return on Equity (9.97%).</t>
+          <t>PGEL operates in the Technology sector. With an estimated Market Cap of ₹17,572.27 Cr., a P/E ratio of 88.51, and YoY Revenue Growth of -10.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.72%), and healthy Return on Equity (6.69%).</t>
         </is>
       </c>
       <c r="AQ13" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 48.80 (Consolidation Zone), while MACD Line (62.25) trades below Signal (68.98) with an expanding histogram (-6.73). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +12.26% above the 200-day DMA (₹1880.41). Daily volatility envelope is bounded by ATR(14) of ₹65.32.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 60.77 (Bullish Momentum Zone), while MACD Line (14.56) trades below Signal (16.43) with an expanding histogram (-1.88). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +10.74% above the 200-day DMA (₹553.54). Daily volatility envelope is bounded by ATR(14) of ₹22.40.</t>
         </is>
       </c>
       <c r="AR13" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for GODREJPROP. Current Market Price (₹2,105.70) is positioned above the 30-day DMA (₹1,999.45), 50-day DMA (₹1,888.17), and 200-day DMA (₹1,880.41). The price distance from 200 DMA is +12.26%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PGEL. Current Market Price (₹613.35) is positioned above the 30-day DMA (₹578.01), 50-day DMA (₹541.38), and 200-day DMA (₹553.54). The price distance from 200 DMA is +10.74%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS13" t="inlineStr">
         <is>
-          <t>[2105.7, 2112.02, 2118.33, 2124.65, 2130.97, 2137.29]</t>
+          <t>[613.35, 615.19, 617.03, 618.87, 620.71, 622.55]</t>
         </is>
       </c>
       <c r="AT13" t="inlineStr">
         <is>
-          <t>[2105.7, 2138.14, 2155.28, 2169.91, 2183.22, 2195.71]</t>
+          <t>[613.35, 624.15, 629.7, 634.39, 638.63, 642.59]</t>
         </is>
       </c>
       <c r="AU13" t="inlineStr">
         <is>
-          <t>[2105.7, 2092.42, 2090.62, 2090.71, 2091.78, 2093.47]</t>
+          <t>[613.35, 608.47, 607.53, 607.23, 607.27, 607.52]</t>
         </is>
       </c>
     </row>
@@ -2665,162 +2665,162 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PGEL</t>
+          <t>GODREJPROP</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>17572.27</v>
+        <v>63429.15</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>613.35</v>
+        <v>2105.7</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>₹608.87 - ₹620.07</t>
+          <t>₹2092.64 - ₹2125.3</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>631.27</v>
+        <v>2157.96</v>
       </c>
       <c r="I14" t="n">
-        <v>148</v>
+        <v>51</v>
       </c>
       <c r="J14" t="n">
-        <v>578.01</v>
+        <v>1999.45</v>
       </c>
       <c r="K14" t="n">
-        <v>541.38</v>
+        <v>1888.17</v>
       </c>
       <c r="L14" t="n">
-        <v>553.54</v>
+        <v>1880.41</v>
       </c>
       <c r="M14" t="n">
-        <v>10.74</v>
+        <v>12.26</v>
       </c>
       <c r="N14" t="n">
-        <v>14.56</v>
+        <v>62.25</v>
       </c>
       <c r="O14" t="n">
-        <v>16.43</v>
+        <v>68.98</v>
       </c>
       <c r="P14" t="n">
-        <v>-1.88</v>
+        <v>-6.73</v>
       </c>
       <c r="Q14" t="n">
-        <v>22.4</v>
+        <v>65.31999999999999</v>
       </c>
       <c r="R14" t="n">
         <v>11.76</v>
       </c>
       <c r="S14" t="n">
-        <v>49</v>
+        <v>42.9</v>
       </c>
       <c r="T14" t="n">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="U14" t="n">
-        <v>-2.4</v>
+        <v>-2.31</v>
       </c>
       <c r="V14" t="n">
-        <v>48.1</v>
+        <v>51.7</v>
       </c>
       <c r="W14" t="n">
-        <v>6.55</v>
+        <v>4.49</v>
       </c>
       <c r="X14" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y14" t="n">
-        <v>605.5</v>
+        <v>2027.32</v>
       </c>
       <c r="Z14" t="n">
-        <v>626.97</v>
+        <v>2032.25</v>
       </c>
       <c r="AA14" t="n">
-        <v>618.26</v>
+        <v>2122.55</v>
       </c>
       <c r="AB14" t="n">
-        <v>579.75</v>
+        <v>2007.72</v>
       </c>
       <c r="AC14" t="n">
-        <v>616.27</v>
+        <v>2111.93</v>
       </c>
       <c r="AD14" t="n">
-        <v>624.54</v>
+        <v>2127.76</v>
       </c>
       <c r="AE14" t="n">
-        <v>635.72</v>
+        <v>2149.83</v>
       </c>
       <c r="AF14" t="n">
-        <v>60.8</v>
+        <v>48.8</v>
       </c>
       <c r="AG14" t="n">
-        <v>0.1</v>
+        <v>0.14</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI14" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ14" t="n">
-        <v>88.5</v>
+        <v>34.2</v>
       </c>
       <c r="AK14" t="n">
-        <v>-10.1</v>
+        <v>63</v>
       </c>
       <c r="AL14" t="n">
-        <v>3.7</v>
+        <v>36.1</v>
       </c>
       <c r="AM14" t="n">
-        <v>6.7</v>
+        <v>10</v>
       </c>
       <c r="AN14" t="n">
-        <v>658.1900000000001</v>
+        <v>2174.81</v>
       </c>
       <c r="AO14" t="n">
-        <v>571.33</v>
+        <v>2031.51</v>
       </c>
       <c r="AP14" t="inlineStr">
         <is>
-          <t>PGEL operates in the Technology sector. With an estimated Market Cap of ₹17,572.27 Cr., a P/E ratio of 88.51, and YoY Revenue Growth of -10.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.72%), and healthy Return on Equity (6.69%).</t>
+          <t>GODREJPROP operates in the Real Estate sector. With an estimated Market Cap of ₹63,429.15 Cr., a P/E ratio of 34.24, and YoY Revenue Growth of +63.0%, the company demonstrates strong institutional backing, solid operating profit margins (36.06%), and healthy Return on Equity (9.97%).</t>
         </is>
       </c>
       <c r="AQ14" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 60.77 (Bullish Momentum Zone), while MACD Line (14.56) trades below Signal (16.43) with an expanding histogram (-1.88). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +10.74% above the 200-day DMA (₹553.54). Daily volatility envelope is bounded by ATR(14) of ₹22.40.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 48.80 (Consolidation Zone), while MACD Line (62.25) trades below Signal (68.98) with an expanding histogram (-6.73). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +12.26% above the 200-day DMA (₹1880.41). Daily volatility envelope is bounded by ATR(14) of ₹65.32.</t>
         </is>
       </c>
       <c r="AR14" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PGEL. Current Market Price (₹613.35) is positioned above the 30-day DMA (₹578.01), 50-day DMA (₹541.38), and 200-day DMA (₹553.54). The price distance from 200 DMA is +10.74%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for GODREJPROP. Current Market Price (₹2,105.70) is positioned above the 30-day DMA (₹1,999.45), 50-day DMA (₹1,888.17), and 200-day DMA (₹1,880.41). The price distance from 200 DMA is +12.26%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS14" t="inlineStr">
         <is>
-          <t>[613.35, 615.19, 617.03, 618.87, 620.71, 622.55]</t>
+          <t>[2105.7, 2112.02, 2118.33, 2124.65, 2130.97, 2137.29]</t>
         </is>
       </c>
       <c r="AT14" t="inlineStr">
         <is>
-          <t>[613.35, 624.15, 629.7, 634.39, 638.63, 642.59]</t>
+          <t>[2105.7, 2138.14, 2155.28, 2169.91, 2183.22, 2195.71]</t>
         </is>
       </c>
       <c r="AU14" t="inlineStr">
         <is>
-          <t>[613.35, 608.47, 607.53, 607.23, 607.27, 607.52]</t>
+          <t>[2105.7, 2092.42, 2090.62, 2090.71, 2091.78, 2093.47]</t>
         </is>
       </c>
     </row>
@@ -2832,16 +2832,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>COFORGE</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>76187.09</v>
+        <v>278417.14</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2849,145 +2849,145 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>1721</v>
+        <v>302.45</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>₹1709.13 - ₹1738.8</t>
+          <t>₹300.39 - ₹305.53</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>1768.46</v>
+        <v>310.68</v>
       </c>
       <c r="I15" t="n">
-        <v>56</v>
+        <v>324</v>
       </c>
       <c r="J15" t="n">
-        <v>1505.99</v>
+        <v>281.7</v>
       </c>
       <c r="K15" t="n">
-        <v>1472.15</v>
+        <v>268.93</v>
       </c>
       <c r="L15" t="n">
-        <v>1507.99</v>
+        <v>274.01</v>
       </c>
       <c r="M15" t="n">
-        <v>15.58</v>
+        <v>13.37</v>
       </c>
       <c r="N15" t="n">
-        <v>53.48</v>
+        <v>9.93</v>
       </c>
       <c r="O15" t="n">
-        <v>30.14</v>
+        <v>8.42</v>
       </c>
       <c r="P15" t="n">
-        <v>23.34</v>
+        <v>1.51</v>
       </c>
       <c r="Q15" t="n">
-        <v>59.33</v>
+        <v>10.28</v>
       </c>
       <c r="R15" t="n">
         <v>11.76</v>
       </c>
       <c r="S15" t="n">
-        <v>43.9</v>
+        <v>43.6</v>
       </c>
       <c r="T15" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="U15" t="n">
-        <v>-2.55</v>
+        <v>-2.53</v>
       </c>
       <c r="V15" t="n">
-        <v>51.5</v>
+        <v>50</v>
       </c>
       <c r="W15" t="n">
-        <v>2.38</v>
+        <v>2.44</v>
       </c>
       <c r="X15" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y15" t="n">
-        <v>1695.71</v>
+        <v>299.26</v>
       </c>
       <c r="Z15" t="n">
-        <v>1755.94</v>
+        <v>309.85</v>
       </c>
       <c r="AA15" t="n">
-        <v>1734.77</v>
+        <v>304.87</v>
       </c>
       <c r="AB15" t="n">
-        <v>1632.01</v>
+        <v>287.03</v>
       </c>
       <c r="AC15" t="n">
-        <v>1713.83</v>
+        <v>306.75</v>
       </c>
       <c r="AD15" t="n">
-        <v>1745.96</v>
+        <v>311.7</v>
       </c>
       <c r="AE15" t="n">
-        <v>1770.93</v>
+        <v>320.95</v>
       </c>
       <c r="AF15" t="n">
-        <v>77.3</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="AG15" t="n">
-        <v>0.16</v>
+        <v>0.12</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI15" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ15" t="n">
-        <v>35.2</v>
+        <v>672.1</v>
       </c>
       <c r="AK15" t="n">
-        <v>49.9</v>
+        <v>182</v>
       </c>
       <c r="AL15" t="n">
-        <v>9.6</v>
+        <v>0.6</v>
       </c>
       <c r="AM15" t="n">
         <v>15</v>
       </c>
       <c r="AN15" t="n">
-        <v>1810.49</v>
+        <v>313.72</v>
       </c>
       <c r="AO15" t="n">
-        <v>1644.19</v>
+        <v>292.31</v>
       </c>
       <c r="AP15" t="inlineStr">
         <is>
-          <t>COFORGE operates in the Technology sector. With an estimated Market Cap of ₹76,187.09 Cr., a P/E ratio of 35.21, and YoY Revenue Growth of +49.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.64%), and healthy Return on Equity (15.00%).</t>
+          <t>ETERNAL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹278,417.14 Cr., a P/E ratio of 672.11, and YoY Revenue Growth of +182.0%, the company demonstrates strong institutional backing, solid operating profit margins (0.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ15" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 77.31 (Bullish Momentum Zone), while MACD Line (53.48) trades above Signal (30.14) with an expanding histogram (+23.34). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +15.58% above the 200-day DMA (₹1507.99). Daily volatility envelope is bounded by ATR(14) of ₹59.33.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 65.40 (Bullish Momentum Zone), while MACD Line (9.93) trades above Signal (8.42) with an expanding histogram (+1.51). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +13.37% above the 200-day DMA (₹274.01). Daily volatility envelope is bounded by ATR(14) of ₹10.28.</t>
         </is>
       </c>
       <c r="AR15" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for COFORGE. Current Market Price (₹1,721.00) is positioned above the 30-day DMA (₹1,505.99), 50-day DMA (₹1,472.15), and 200-day DMA (₹1,507.99). The price distance from 200 DMA is +15.58%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ETERNAL. Current Market Price (₹302.45) is positioned above the 30-day DMA (₹281.70), 50-day DMA (₹268.93), and 200-day DMA (₹274.01). The price distance from 200 DMA is +13.37%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS15" t="inlineStr">
         <is>
-          <t>[1721.0, 1726.16, 1731.33, 1736.49, 1741.65, 1746.81]</t>
+          <t>[302.45, 303.8, 305.15, 306.5, 307.85, 309.19]</t>
         </is>
       </c>
       <c r="AT15" t="inlineStr">
         <is>
-          <t>[1721.0, 1749.89, 1764.89, 1777.59, 1789.11, 1799.88]</t>
+          <t>[302.45, 307.91, 310.96, 313.62, 316.07, 318.39]</t>
         </is>
       </c>
       <c r="AU15" t="inlineStr">
         <is>
-          <t>[1721.0, 1708.36, 1706.16, 1705.66, 1706.06, 1707.02]</t>
+          <t>[302.45, 300.71, 300.79, 301.15, 301.68, 302.3]</t>
         </is>
       </c>
     </row>
@@ -2999,16 +2999,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>COFORGE</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>278417.14</v>
+        <v>76187.09</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3016,145 +3016,145 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>302.45</v>
+        <v>1721</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>₹300.39 - ₹305.53</t>
+          <t>₹1709.13 - ₹1738.8</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>310.68</v>
+        <v>1768.46</v>
       </c>
       <c r="I16" t="n">
-        <v>324</v>
+        <v>56</v>
       </c>
       <c r="J16" t="n">
-        <v>281.7</v>
+        <v>1505.99</v>
       </c>
       <c r="K16" t="n">
-        <v>268.93</v>
+        <v>1472.15</v>
       </c>
       <c r="L16" t="n">
-        <v>274.01</v>
+        <v>1507.99</v>
       </c>
       <c r="M16" t="n">
-        <v>13.37</v>
+        <v>15.58</v>
       </c>
       <c r="N16" t="n">
-        <v>9.93</v>
+        <v>53.48</v>
       </c>
       <c r="O16" t="n">
-        <v>8.42</v>
+        <v>30.14</v>
       </c>
       <c r="P16" t="n">
-        <v>1.51</v>
+        <v>23.34</v>
       </c>
       <c r="Q16" t="n">
-        <v>10.28</v>
+        <v>59.33</v>
       </c>
       <c r="R16" t="n">
         <v>11.76</v>
       </c>
       <c r="S16" t="n">
-        <v>42.4</v>
+        <v>41.3</v>
       </c>
       <c r="T16" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="U16" t="n">
-        <v>-2.6</v>
+        <v>-2.7</v>
       </c>
       <c r="V16" t="n">
-        <v>46.4</v>
+        <v>48.3</v>
       </c>
       <c r="W16" t="n">
-        <v>2.4</v>
+        <v>7.48</v>
       </c>
       <c r="X16" t="n">
         <v>-0.77</v>
       </c>
       <c r="Y16" t="n">
-        <v>299.14</v>
+        <v>1705.12</v>
       </c>
       <c r="Z16" t="n">
-        <v>309.72</v>
+        <v>1765.36</v>
       </c>
       <c r="AA16" t="n">
-        <v>304.87</v>
+        <v>1734.77</v>
       </c>
       <c r="AB16" t="n">
-        <v>287.03</v>
+        <v>1632.01</v>
       </c>
       <c r="AC16" t="n">
-        <v>306.75</v>
+        <v>1713.83</v>
       </c>
       <c r="AD16" t="n">
-        <v>311.7</v>
+        <v>1745.96</v>
       </c>
       <c r="AE16" t="n">
-        <v>320.95</v>
+        <v>1770.93</v>
       </c>
       <c r="AF16" t="n">
-        <v>65.40000000000001</v>
+        <v>77.3</v>
       </c>
       <c r="AG16" t="n">
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (11.76) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Low VIX (11.76) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AI16" t="n">
         <v>0.15</v>
       </c>
       <c r="AJ16" t="n">
-        <v>672.1</v>
+        <v>35.2</v>
       </c>
       <c r="AK16" t="n">
-        <v>182</v>
+        <v>49.9</v>
       </c>
       <c r="AL16" t="n">
-        <v>0.6</v>
+        <v>9.6</v>
       </c>
       <c r="AM16" t="n">
         <v>15</v>
       </c>
       <c r="AN16" t="n">
-        <v>317.38</v>
+        <v>1788.88</v>
       </c>
       <c r="AO16" t="n">
-        <v>287.93</v>
+        <v>1658.41</v>
       </c>
       <c r="AP16" t="inlineStr">
         <is>
-          <t>ETERNAL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹278,417.14 Cr., a P/E ratio of 672.11, and YoY Revenue Growth of +182.0%, the company demonstrates strong institutional backing, solid operating profit margins (0.64%), and healthy Return on Equity (15.00%).</t>
+          <t>COFORGE operates in the Technology sector. With an estimated Market Cap of ₹76,187.09 Cr., a P/E ratio of 35.21, and YoY Revenue Growth of +49.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AQ16" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 65.40 (Bullish Momentum Zone), while MACD Line (9.93) trades above Signal (8.42) with an expanding histogram (+1.51). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +13.37% above the 200-day DMA (₹274.01). Daily volatility envelope is bounded by ATR(14) of ₹10.28.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 77.31 (Bullish Momentum Zone), while MACD Line (53.48) trades above Signal (30.14) with an expanding histogram (+23.34). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +15.58% above the 200-day DMA (₹1507.99). Daily volatility envelope is bounded by ATR(14) of ₹59.33.</t>
         </is>
       </c>
       <c r="AR16" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ETERNAL. Current Market Price (₹302.45) is positioned above the 30-day DMA (₹281.70), 50-day DMA (₹268.93), and 200-day DMA (₹274.01). The price distance from 200 DMA is +13.37%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for COFORGE. Current Market Price (₹1,721.00) is positioned above the 30-day DMA (₹1,505.99), 50-day DMA (₹1,472.15), and 200-day DMA (₹1,507.99). The price distance from 200 DMA is +15.58%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AS16" t="inlineStr">
         <is>
-          <t>[302.45, 303.67, 304.9, 306.12, 307.35, 308.57]</t>
+          <t>[1721.0, 1730.94, 1740.87, 1750.81, 1760.74, 1770.68]</t>
         </is>
       </c>
       <c r="AT16" t="inlineStr">
         <is>
-          <t>[302.45, 307.79, 310.72, 313.25, 315.57, 317.77]</t>
+          <t>[1721.0, 1754.67, 1774.43, 1791.91, 1808.21, 1823.74]</t>
         </is>
       </c>
       <c r="AU16" t="inlineStr">
         <is>
-          <t>[302.45, 300.59, 300.54, 300.78, 301.18, 301.67]</t>
+          <t>[1721.0, 1713.14, 1715.7, 1719.98, 1725.15, 1730.88]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Add Current Month Futures Intraday engine, mobile UX improvements, 5-Tier modal details, and updated 5:30/6:30 AM scan schedules
</commit_message>
<xml_diff>
--- a/Breakout_ML_Quant_Predictions.xlsx
+++ b/Breakout_ML_Quant_Predictions.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>357916.19</v>
+        <v>357416.09</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -673,15 +673,15 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>12167</v>
+        <v>12150</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>₹12126.59 - ₹12227.61</t>
+          <t>₹12109.59 - ₹12210.61</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>12328.62</v>
+        <v>12311.62</v>
       </c>
       <c r="I2" t="n">
         <v>11508.32</v>
@@ -708,10 +708,10 @@
         <v>202.03</v>
       </c>
       <c r="Q2" t="n">
-        <v>12.25</v>
+        <v>12.34</v>
       </c>
       <c r="R2" t="n">
-        <v>50.5</v>
+        <v>50.6</v>
       </c>
       <c r="S2" t="n">
         <v>0.32</v>
@@ -729,25 +729,25 @@
         <v>-0.77</v>
       </c>
       <c r="X2" t="n">
-        <v>12073.64</v>
+        <v>12055.35</v>
       </c>
       <c r="Y2" t="n">
-        <v>12470.04</v>
+        <v>12453.04</v>
       </c>
       <c r="Z2" t="n">
-        <v>12264.34</v>
+        <v>12247.2</v>
       </c>
       <c r="AA2" t="n">
-        <v>11863.96</v>
+        <v>11846.96</v>
       </c>
       <c r="AB2" t="n">
-        <v>12125.33</v>
+        <v>12119.67</v>
       </c>
       <c r="AC2" t="n">
-        <v>12280.66</v>
+        <v>12269.34</v>
       </c>
       <c r="AD2" t="n">
-        <v>12394.33</v>
+        <v>12388.67</v>
       </c>
       <c r="AE2" t="n">
         <v>70.40000000000001</v>
@@ -757,14 +757,14 @@
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.25) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH2" t="n">
         <v>0.15</v>
       </c>
       <c r="AI2" t="n">
-        <v>41.9</v>
+        <v>41.8</v>
       </c>
       <c r="AJ2" t="n">
         <v>15.9</v>
@@ -776,14 +776,14 @@
         <v>15</v>
       </c>
       <c r="AM2" t="n">
-        <v>12431.89</v>
+        <v>12425.44</v>
       </c>
       <c r="AN2" t="n">
-        <v>11891.42</v>
+        <v>11882.79</v>
       </c>
       <c r="AO2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO operates in the Basic Materials sector. With an estimated Market Cap of ₹357,916.19 Cr., a P/E ratio of 41.89, and YoY Revenue Growth of +15.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.29%), and healthy Return on Equity (15.00%).</t>
+          <t>ULTRACEMCO operates in the Basic Materials sector. With an estimated Market Cap of ₹357,416.09 Cr., a P/E ratio of 41.84, and YoY Revenue Growth of +15.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.29%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP2" t="inlineStr">
@@ -793,22 +793,22 @@
       </c>
       <c r="AQ2" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ULTRACEMCO. Current Market Price (₹12,167.00) is positioned above the 30-day DMA (₹11,508.32), 50-day DMA (₹11,305.61), and 200-day DMA (₹11,570.61). The price distance from 200 DMA is +4.14%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ULTRACEMCO. Current Market Price (₹12,150.00) is positioned above the 30-day DMA (₹11,508.32), 50-day DMA (₹11,305.61), and 200-day DMA (₹11,570.61). The price distance from 200 DMA is +4.14%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR2" t="inlineStr">
         <is>
-          <t>[12167.0, 12256.14, 12345.28, 12434.43, 12523.57, 12612.71]</t>
+          <t>[12150.0, 12237.6, 12325.2, 12412.8, 12500.41, 12588.01]</t>
         </is>
       </c>
       <c r="AS2" t="inlineStr">
         <is>
-          <t>[12167.0, 12336.95, 12459.57, 12574.39, 12685.19, 12793.41]</t>
+          <t>[12150.0, 12318.41, 12439.49, 12552.77, 12662.03, 12768.7]</t>
         </is>
       </c>
       <c r="AT2" t="inlineStr">
         <is>
-          <t>[12167.0, 12195.53, 12259.57, 12329.45, 12402.35, 12477.19]</t>
+          <t>[12150.0, 12176.99, 12239.49, 12307.83, 12379.19, 12452.48]</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>130674.76</v>
+        <v>130812.67</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -837,15 +837,15 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>113.7</v>
+        <v>113.82</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>₹113.31 - ₹114.29</t>
+          <t>₹113.43 - ₹114.41</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>115.26</v>
+        <v>115.38</v>
       </c>
       <c r="I3" t="n">
         <v>108.12</v>
@@ -872,16 +872,16 @@
         <v>1.95</v>
       </c>
       <c r="Q3" t="n">
-        <v>12.25</v>
+        <v>12.34</v>
       </c>
       <c r="R3" t="n">
-        <v>49.8</v>
+        <v>49.4</v>
       </c>
       <c r="S3" t="n">
         <v>0.31</v>
       </c>
       <c r="T3" t="n">
-        <v>-0.89</v>
+        <v>-0.91</v>
       </c>
       <c r="U3" t="n">
         <v>55</v>
@@ -893,25 +893,25 @@
         <v>-0.77</v>
       </c>
       <c r="X3" t="n">
-        <v>111.36</v>
+        <v>111.48</v>
       </c>
       <c r="Y3" t="n">
-        <v>114.77</v>
+        <v>114.91</v>
       </c>
       <c r="Z3" t="n">
-        <v>114.61</v>
+        <v>114.73</v>
       </c>
       <c r="AA3" t="n">
-        <v>110.77</v>
+        <v>110.89</v>
       </c>
       <c r="AB3" t="n">
-        <v>114.19</v>
+        <v>114.21</v>
       </c>
       <c r="AC3" t="n">
-        <v>114.71</v>
+        <v>114.82</v>
       </c>
       <c r="AD3" t="n">
-        <v>115.72</v>
+        <v>115.81</v>
       </c>
       <c r="AE3" t="n">
         <v>79</v>
@@ -921,7 +921,7 @@
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Low VIX (12.25) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Low VIX (12.34) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH3" t="n">
@@ -940,14 +940,14 @@
         <v>15</v>
       </c>
       <c r="AM3" t="n">
-        <v>116.75</v>
+        <v>116.9</v>
       </c>
       <c r="AN3" t="n">
-        <v>110.96</v>
+        <v>110.73</v>
       </c>
       <c r="AO3" t="inlineStr">
         <is>
-          <t>PNB operates in the Financial Services sector. With an estimated Market Cap of ₹130,674.76 Cr., a P/E ratio of 5.86, and YoY Revenue Growth of +15.2%, the company demonstrates strong institutional backing, solid operating profit margins (38.15%), and healthy Return on Equity (14.97%).</t>
+          <t>PNB operates in the Financial Services sector. With an estimated Market Cap of ₹130,812.67 Cr., a P/E ratio of 5.87, and YoY Revenue Growth of +15.2%, the company demonstrates strong institutional backing, solid operating profit margins (38.15%), and healthy Return on Equity (14.97%).</t>
         </is>
       </c>
       <c r="AP3" t="inlineStr">
@@ -957,22 +957,22 @@
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PNB. Current Market Price (₹113.70) is positioned above the 30-day DMA (₹108.12), 50-day DMA (₹106.98), and 200-day DMA (₹112.64). The price distance from 200 DMA is +1.20%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PNB. Current Market Price (₹113.82) is positioned above the 30-day DMA (₹108.12), 50-day DMA (₹106.98), and 200-day DMA (₹112.64). The price distance from 200 DMA is +1.20%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR3" t="inlineStr">
         <is>
-          <t>[113.7, 114.04, 114.38, 114.72, 115.06, 115.41]</t>
+          <t>[113.82, 114.16, 114.5, 114.84, 115.19, 115.53]</t>
         </is>
       </c>
       <c r="AS3" t="inlineStr">
         <is>
-          <t>[113.7, 114.82, 115.49, 116.08, 116.63, 117.15]</t>
+          <t>[113.82, 114.94, 115.61, 116.2, 116.75, 117.27]</t>
         </is>
       </c>
       <c r="AT3" t="inlineStr">
         <is>
-          <t>[113.7, 113.46, 113.55, 113.71, 113.89, 114.1]</t>
+          <t>[113.82, 113.58, 113.67, 113.83, 114.01, 114.22]</t>
         </is>
       </c>
     </row>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>218629.08</v>
+        <v>219603.63</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1001,15 +1001,15 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>7964</v>
+        <v>7999.5</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>₹7932.64 - ₹8011.04</t>
+          <t>₹7968.14 - ₹8046.54</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>8089.45</v>
+        <v>8124.95</v>
       </c>
       <c r="I4" t="n">
         <v>7478.7</v>
@@ -1036,46 +1036,46 @@
         <v>156.81</v>
       </c>
       <c r="Q4" t="n">
-        <v>12.25</v>
+        <v>12.34</v>
       </c>
       <c r="R4" t="n">
-        <v>51.4</v>
+        <v>51.5</v>
       </c>
       <c r="S4" t="n">
         <v>0.27</v>
       </c>
       <c r="T4" t="n">
-        <v>-1.02</v>
+        <v>-1.01</v>
       </c>
       <c r="U4" t="n">
         <v>51.7</v>
       </c>
       <c r="V4" t="n">
-        <v>2.08</v>
+        <v>2.09</v>
       </c>
       <c r="W4" t="n">
         <v>-0.77</v>
       </c>
       <c r="X4" t="n">
-        <v>7838.88</v>
+        <v>7877.72</v>
       </c>
       <c r="Y4" t="n">
-        <v>8117.62</v>
+        <v>8157.7</v>
       </c>
       <c r="Z4" t="n">
-        <v>8027.71</v>
+        <v>8063.5</v>
       </c>
       <c r="AA4" t="n">
-        <v>7728.78</v>
+        <v>7764.28</v>
       </c>
       <c r="AB4" t="n">
-        <v>7954.83</v>
+        <v>7968.17</v>
       </c>
       <c r="AC4" t="n">
-        <v>8004.16</v>
+        <v>8030.84</v>
       </c>
       <c r="AD4" t="n">
-        <v>8044.33</v>
+        <v>8062.17</v>
       </c>
       <c r="AE4" t="n">
         <v>74.3</v>
@@ -1085,14 +1085,14 @@
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.25) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH4" t="n">
         <v>0.15</v>
       </c>
       <c r="AI4" t="n">
-        <v>38.5</v>
+        <v>38.6</v>
       </c>
       <c r="AJ4" t="n">
         <v>31.5</v>
@@ -1104,14 +1104,14 @@
         <v>15</v>
       </c>
       <c r="AM4" t="n">
-        <v>8191.7</v>
+        <v>8209.23</v>
       </c>
       <c r="AN4" t="n">
-        <v>7776.28</v>
+        <v>7811.34</v>
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>EICHERMOT operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹218,629.08 Cr., a P/E ratio of 38.45, and YoY Revenue Growth of +31.5%, the company demonstrates strong institutional backing, solid operating profit margins (23.21%), and healthy Return on Equity (15.00%).</t>
+          <t>EICHERMOT operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹219,603.63 Cr., a P/E ratio of 38.63, and YoY Revenue Growth of +31.5%, the company demonstrates strong institutional backing, solid operating profit margins (23.21%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP4" t="inlineStr">
@@ -1121,22 +1121,22 @@
       </c>
       <c r="AQ4" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for EICHERMOT. Current Market Price (₹7,964.00) is positioned above the 30-day DMA (₹7,478.70), 50-day DMA (₹7,389.91), and 200-day DMA (₹7,187.90). The price distance from 200 DMA is +10.39%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for EICHERMOT. Current Market Price (₹7,999.50) is positioned above the 30-day DMA (₹7,478.70), 50-day DMA (₹7,389.91), and 200-day DMA (₹7,187.90). The price distance from 200 DMA is +10.39%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR4" t="inlineStr">
         <is>
-          <t>[7964.0, 7987.89, 8011.78, 8035.68, 8059.57, 8083.46]</t>
+          <t>[7999.5, 8023.5, 8047.5, 8071.5, 8095.49, 8119.49]</t>
         </is>
       </c>
       <c r="AS4" t="inlineStr">
         <is>
-          <t>[7964.0, 8050.62, 8100.49, 8144.32, 8185.02, 8223.72]</t>
+          <t>[7999.5, 8086.22, 8136.2, 8180.14, 8220.94, 8259.75]</t>
         </is>
       </c>
       <c r="AT4" t="inlineStr">
         <is>
-          <t>[7964.0, 7940.85, 7945.25, 7954.19, 7965.48, 7978.27]</t>
+          <t>[7999.5, 7976.46, 7980.97, 7990.01, 8001.41, 8014.3]</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>308592.82</v>
+        <v>309201.42</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1165,15 +1165,15 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>4614.3</v>
+        <v>4623.4</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>₹4598.26 - ₹4638.36</t>
+          <t>₹4607.36 - ₹4647.46</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>4678.45</v>
+        <v>4687.55</v>
       </c>
       <c r="I5" t="n">
         <v>4490.17</v>
@@ -1200,16 +1200,16 @@
         <v>80.19</v>
       </c>
       <c r="Q5" t="n">
-        <v>12.25</v>
+        <v>12.34</v>
       </c>
       <c r="R5" t="n">
-        <v>40.7</v>
+        <v>40.8</v>
       </c>
       <c r="S5" t="n">
         <v>0.31</v>
       </c>
       <c r="T5" t="n">
-        <v>-1.22</v>
+        <v>-1.21</v>
       </c>
       <c r="U5" t="n">
         <v>41.7</v>
@@ -1221,25 +1221,25 @@
         <v>-0.77</v>
       </c>
       <c r="X5" t="n">
-        <v>4518.08</v>
+        <v>4527.18</v>
       </c>
       <c r="Y5" t="n">
-        <v>4652.81</v>
+        <v>4662.53</v>
       </c>
       <c r="Z5" t="n">
-        <v>4651.21</v>
+        <v>4660.39</v>
       </c>
       <c r="AA5" t="n">
-        <v>4494.02</v>
+        <v>4503.12</v>
       </c>
       <c r="AB5" t="n">
-        <v>4630.33</v>
+        <v>4633.37</v>
       </c>
       <c r="AC5" t="n">
-        <v>4657.36</v>
+        <v>4663.44</v>
       </c>
       <c r="AD5" t="n">
-        <v>4700.43</v>
+        <v>4703.47</v>
       </c>
       <c r="AE5" t="n">
         <v>72.8</v>
@@ -1249,14 +1249,14 @@
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.25) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH5" t="n">
         <v>0.15</v>
       </c>
       <c r="AI5" t="n">
-        <v>33.9</v>
+        <v>34</v>
       </c>
       <c r="AJ5" t="n">
         <v>1.8</v>
@@ -1268,14 +1268,14 @@
         <v>24</v>
       </c>
       <c r="AM5" t="n">
-        <v>4738.23</v>
+        <v>4748.28</v>
       </c>
       <c r="AN5" t="n">
-        <v>4490.62</v>
+        <v>4505.04</v>
       </c>
       <c r="AO5" t="inlineStr">
         <is>
-          <t>HAL operates in the Industrials sector. With an estimated Market Cap of ₹308,592.82 Cr., a P/E ratio of 33.89, and YoY Revenue Growth of +1.8%, the company demonstrates strong institutional backing, solid operating profit margins (27.55%), and healthy Return on Equity (23.98%).</t>
+          <t>HAL operates in the Industrials sector. With an estimated Market Cap of ₹309,201.42 Cr., a P/E ratio of 33.96, and YoY Revenue Growth of +1.8%, the company demonstrates strong institutional backing, solid operating profit margins (27.55%), and healthy Return on Equity (23.98%).</t>
         </is>
       </c>
       <c r="AP5" t="inlineStr">
@@ -1285,22 +1285,22 @@
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for HAL. Current Market Price (₹4,614.30) is positioned above the 30-day DMA (₹4,490.17), 50-day DMA (₹4,419.22), and 200-day DMA (₹4,344.79). The price distance from 200 DMA is +6.68%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for HAL. Current Market Price (₹4,623.40) is positioned above the 30-day DMA (₹4,490.17), 50-day DMA (₹4,419.22), and 200-day DMA (₹4,344.79). The price distance from 200 DMA is +6.68%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>[4614.3, 4628.14, 4641.99, 4655.83, 4669.67, 4683.51]</t>
+          <t>[4623.4, 4637.27, 4651.14, 4665.01, 4678.88, 4692.75]</t>
         </is>
       </c>
       <c r="AS5" t="inlineStr">
         <is>
-          <t>[4614.3, 4660.22, 4687.35, 4711.38, 4733.82, 4755.23]</t>
+          <t>[4623.4, 4669.34, 4696.5, 4720.56, 4743.03, 4764.47]</t>
         </is>
       </c>
       <c r="AT5" t="inlineStr">
         <is>
-          <t>[4614.3, 4604.09, 4607.97, 4614.16, 4621.56, 4629.72]</t>
+          <t>[4623.4, 4613.21, 4617.12, 4623.34, 4630.77, 4638.96]</t>
         </is>
       </c>
     </row>
@@ -1312,159 +1312,159 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ALKEM</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Basic Materials</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>67434.66</v>
+        <v>264394.09</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>🔴 AVOID / HOLD</t>
+          <t>🟡 MODERATE BUY</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>5640</v>
+        <v>2758</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>₹5616.66 - ₹5675.0</t>
+          <t>₹2746.15 - ₹2775.77</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>5733.34</v>
+        <v>2805.39</v>
       </c>
       <c r="I6" t="n">
-        <v>5598.93</v>
+        <v>2698.21</v>
       </c>
       <c r="J6" t="n">
-        <v>5497.15</v>
+        <v>2687.88</v>
       </c>
       <c r="K6" t="n">
-        <v>5524.06</v>
+        <v>2577.55</v>
       </c>
       <c r="L6" t="n">
-        <v>3.31</v>
+        <v>7.66</v>
       </c>
       <c r="M6" t="n">
-        <v>58.81</v>
+        <v>26.47</v>
       </c>
       <c r="N6" t="n">
-        <v>54.69</v>
+        <v>16.72</v>
       </c>
       <c r="O6" t="n">
-        <v>4.12</v>
+        <v>9.76</v>
       </c>
       <c r="P6" t="n">
-        <v>116.68</v>
+        <v>59.24</v>
       </c>
       <c r="Q6" t="n">
-        <v>12.25</v>
+        <v>12.34</v>
       </c>
       <c r="R6" t="n">
-        <v>46.7</v>
+        <v>48.2</v>
       </c>
       <c r="S6" t="n">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="T6" t="n">
         <v>-1.28</v>
       </c>
       <c r="U6" t="n">
-        <v>51.7</v>
+        <v>55</v>
       </c>
       <c r="V6" t="n">
-        <v>2.81</v>
+        <v>1.78</v>
       </c>
       <c r="W6" t="n">
         <v>-0.77</v>
       </c>
       <c r="X6" t="n">
-        <v>5499.99</v>
+        <v>2686.92</v>
       </c>
       <c r="Y6" t="n">
-        <v>5606.19</v>
+        <v>2779.48</v>
       </c>
       <c r="Z6" t="n">
-        <v>5685.12</v>
+        <v>2780.06</v>
       </c>
       <c r="AA6" t="n">
-        <v>5464.98</v>
+        <v>2669.15</v>
       </c>
       <c r="AB6" t="n">
-        <v>5620.5</v>
+        <v>2764.57</v>
       </c>
       <c r="AC6" t="n">
-        <v>5685</v>
+        <v>2780.44</v>
       </c>
       <c r="AD6" t="n">
-        <v>5730</v>
+        <v>2802.87</v>
       </c>
       <c r="AE6" t="n">
-        <v>56.2</v>
+        <v>67</v>
       </c>
       <c r="AF6" t="n">
-        <v>-0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (12.25) | LSTM Deep Net</t>
+          <t>Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH6" t="n">
         <v>0.15</v>
       </c>
       <c r="AI6" t="n">
-        <v>29.3</v>
+        <v>56.1</v>
       </c>
       <c r="AJ6" t="n">
-        <v>14.6</v>
+        <v>17.9</v>
       </c>
       <c r="AK6" t="n">
-        <v>15.6</v>
+        <v>12.8</v>
       </c>
       <c r="AL6" t="n">
-        <v>17.6</v>
+        <v>15</v>
       </c>
       <c r="AM6" t="n">
-        <v>5768.09</v>
+        <v>2821.79</v>
       </c>
       <c r="AN6" t="n">
-        <v>5520.18</v>
+        <v>2696.4</v>
       </c>
       <c r="AO6" t="inlineStr">
         <is>
-          <t>ALKEM operates in the Healthcare sector. With an estimated Market Cap of ₹67,434.66 Cr., a P/E ratio of 29.27, and YoY Revenue Growth of +14.6%, the company demonstrates strong institutional backing, solid operating profit margins (15.65%), and healthy Return on Equity (17.56%).</t>
+          <t>ASIANPAINT operates in the Basic Materials sector. With an estimated Market Cap of ₹264,394.09 Cr., a P/E ratio of 56.15, and YoY Revenue Growth of +17.9%, the company demonstrates strong institutional backing, solid operating profit margins (12.81%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP6" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 56.20 (Bullish Momentum Zone), while MACD Line (58.81) trades above Signal (54.69) with an expanding histogram (+4.12). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +3.31% above the 200-day DMA (₹5524.06). Daily volatility envelope is bounded by ATR(14) of ₹116.68.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 66.98 (Bullish Momentum Zone), while MACD Line (26.47) trades above Signal (16.72) with an expanding histogram (+9.76). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +7.66% above the 200-day DMA (₹2577.55). Daily volatility envelope is bounded by ATR(14) of ₹59.24.</t>
         </is>
       </c>
       <c r="AQ6" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ALKEM. Current Market Price (₹5,640.00) is positioned above the 30-day DMA (₹5,598.93), 50-day DMA (₹5,497.15), and 200-day DMA (₹5,524.06). The price distance from 200 DMA is +3.31%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ASIANPAINT. Current Market Price (₹2,758.00) is positioned above the 30-day DMA (₹2,698.21), 50-day DMA (₹2,687.88), and 200-day DMA (₹2,577.55). The price distance from 200 DMA is +7.66%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR6" t="inlineStr">
         <is>
-          <t>[5640.0, 5656.92, 5673.84, 5690.76, 5707.68, 5724.6]</t>
+          <t>[2758.0, 2766.27, 2774.55, 2782.82, 2791.1, 2799.37]</t>
         </is>
       </c>
       <c r="AS6" t="inlineStr">
         <is>
-          <t>[5640.0, 5703.59, 5739.84, 5771.6, 5801.02, 5828.96]</t>
+          <t>[2758.0, 2789.97, 2808.06, 2823.86, 2838.48, 2852.35]</t>
         </is>
       </c>
       <c r="AT6" t="inlineStr">
         <is>
-          <t>[5640.0, 5621.92, 5624.34, 5630.13, 5637.67, 5646.33]</t>
+          <t>[2758.0, 2748.5, 2749.42, 2752.04, 2755.55, 2759.63]</t>
         </is>
       </c>
     </row>
@@ -1476,16 +1476,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>ALKEM</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Basic Materials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>264844.66</v>
+        <v>67315.09</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1493,142 +1493,142 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2762.3</v>
+        <v>5629</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>₹2750.45 - ₹2780.07</t>
+          <t>₹5605.66 - ₹5664.0</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>2809.69</v>
+        <v>5722.34</v>
       </c>
       <c r="I7" t="n">
-        <v>2698.21</v>
+        <v>5598.93</v>
       </c>
       <c r="J7" t="n">
-        <v>2687.88</v>
+        <v>5497.15</v>
       </c>
       <c r="K7" t="n">
-        <v>2577.55</v>
+        <v>5524.06</v>
       </c>
       <c r="L7" t="n">
-        <v>7.66</v>
+        <v>3.31</v>
       </c>
       <c r="M7" t="n">
-        <v>26.47</v>
+        <v>58.81</v>
       </c>
       <c r="N7" t="n">
-        <v>16.72</v>
+        <v>54.69</v>
       </c>
       <c r="O7" t="n">
-        <v>9.76</v>
+        <v>4.12</v>
       </c>
       <c r="P7" t="n">
-        <v>59.24</v>
+        <v>116.68</v>
       </c>
       <c r="Q7" t="n">
-        <v>12.25</v>
+        <v>12.34</v>
       </c>
       <c r="R7" t="n">
-        <v>47.9</v>
+        <v>46.7</v>
       </c>
       <c r="S7" t="n">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="T7" t="n">
-        <v>-1.29</v>
+        <v>-1.28</v>
       </c>
       <c r="U7" t="n">
-        <v>55</v>
+        <v>51.7</v>
       </c>
       <c r="V7" t="n">
-        <v>1.78</v>
+        <v>2.82</v>
       </c>
       <c r="W7" t="n">
         <v>-0.77</v>
       </c>
       <c r="X7" t="n">
-        <v>2691.22</v>
+        <v>5488.99</v>
       </c>
       <c r="Y7" t="n">
-        <v>2784.35</v>
+        <v>5594.42</v>
       </c>
       <c r="Z7" t="n">
-        <v>2784.4</v>
+        <v>5674.03</v>
       </c>
       <c r="AA7" t="n">
-        <v>2673.45</v>
+        <v>5453.98</v>
       </c>
       <c r="AB7" t="n">
-        <v>2766</v>
+        <v>5616.83</v>
       </c>
       <c r="AC7" t="n">
-        <v>2783.3</v>
+        <v>5677.66</v>
       </c>
       <c r="AD7" t="n">
-        <v>2804.3</v>
+        <v>5726.33</v>
       </c>
       <c r="AE7" t="n">
-        <v>67</v>
+        <v>56.2</v>
       </c>
       <c r="AF7" t="n">
-        <v>0.02</v>
+        <v>-0.03</v>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>Strong RSI | Low VIX (12.25) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (12.34) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH7" t="n">
         <v>0.15</v>
       </c>
       <c r="AI7" t="n">
-        <v>56.2</v>
+        <v>29.2</v>
       </c>
       <c r="AJ7" t="n">
-        <v>17.9</v>
+        <v>14.6</v>
       </c>
       <c r="AK7" t="n">
-        <v>12.8</v>
+        <v>15.6</v>
       </c>
       <c r="AL7" t="n">
-        <v>15</v>
+        <v>17.6</v>
       </c>
       <c r="AM7" t="n">
-        <v>2824.01</v>
+        <v>5748.52</v>
       </c>
       <c r="AN7" t="n">
-        <v>2699.84</v>
+        <v>5495.23</v>
       </c>
       <c r="AO7" t="inlineStr">
         <is>
-          <t>ASIANPAINT operates in the Basic Materials sector. With an estimated Market Cap of ₹264,844.66 Cr., a P/E ratio of 56.24, and YoY Revenue Growth of +17.9%, the company demonstrates strong institutional backing, solid operating profit margins (12.81%), and healthy Return on Equity (15.00%).</t>
+          <t>ALKEM operates in the Healthcare sector. With an estimated Market Cap of ₹67,315.09 Cr., a P/E ratio of 29.22, and YoY Revenue Growth of +14.6%, the company demonstrates strong institutional backing, solid operating profit margins (15.65%), and healthy Return on Equity (17.56%).</t>
         </is>
       </c>
       <c r="AP7" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 66.98 (Bullish Momentum Zone), while MACD Line (26.47) trades above Signal (16.72) with an expanding histogram (+9.76). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +7.66% above the 200-day DMA (₹2577.55). Daily volatility envelope is bounded by ATR(14) of ₹59.24.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 56.20 (Bullish Momentum Zone), while MACD Line (58.81) trades above Signal (54.69) with an expanding histogram (+4.12). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +3.31% above the 200-day DMA (₹5524.06). Daily volatility envelope is bounded by ATR(14) of ₹116.68.</t>
         </is>
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ASIANPAINT. Current Market Price (₹2,762.30) is positioned above the 30-day DMA (₹2,698.21), 50-day DMA (₹2,687.88), and 200-day DMA (₹2,577.55). The price distance from 200 DMA is +7.66%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ALKEM. Current Market Price (₹5,629.00) is positioned above the 30-day DMA (₹5,598.93), 50-day DMA (₹5,497.15), and 200-day DMA (₹5,524.06). The price distance from 200 DMA is +3.31%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>[2762.3, 2770.59, 2778.87, 2787.16, 2795.45, 2803.73]</t>
+          <t>[5629.0, 5645.89, 5662.77, 5679.66, 5696.55, 5713.43]</t>
         </is>
       </c>
       <c r="AS7" t="inlineStr">
         <is>
-          <t>[2762.3, 2794.28, 2812.38, 2828.2, 2842.84, 2856.72]</t>
+          <t>[5629.0, 5692.56, 5728.78, 5760.5, 5789.89, 5817.8]</t>
         </is>
       </c>
       <c r="AT7" t="inlineStr">
         <is>
-          <t>[2762.3, 2752.82, 2753.74, 2756.38, 2759.91, 2764.0]</t>
+          <t>[5629.0, 5610.88, 5613.27, 5619.03, 5626.54, 5635.16]</t>
         </is>
       </c>
     </row>
@@ -1649,7 +1649,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>105547.5</v>
+        <v>105590.2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1657,15 +1657,15 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>741.1</v>
+        <v>741.8</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>₹738.11 - ₹745.59</t>
+          <t>₹738.81 - ₹746.29</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>753.08</v>
+        <v>753.78</v>
       </c>
       <c r="I8" t="n">
         <v>731.6799999999999</v>
@@ -1692,7 +1692,7 @@
         <v>14.97</v>
       </c>
       <c r="Q8" t="n">
-        <v>12.25</v>
+        <v>12.34</v>
       </c>
       <c r="R8" t="n">
         <v>43.9</v>
@@ -1713,25 +1713,25 @@
         <v>-0.77</v>
       </c>
       <c r="X8" t="n">
-        <v>723.13</v>
+        <v>723.83</v>
       </c>
       <c r="Y8" t="n">
-        <v>734</v>
+        <v>735.01</v>
       </c>
       <c r="Z8" t="n">
-        <v>747.03</v>
+        <v>747.73</v>
       </c>
       <c r="AA8" t="n">
-        <v>718.64</v>
+        <v>719.34</v>
       </c>
       <c r="AB8" t="n">
-        <v>744.78</v>
+        <v>745</v>
       </c>
       <c r="AC8" t="n">
-        <v>749.21</v>
+        <v>749.7</v>
       </c>
       <c r="AD8" t="n">
-        <v>757.33</v>
+        <v>757.6</v>
       </c>
       <c r="AE8" t="n">
         <v>54.1</v>
@@ -1741,14 +1741,14 @@
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (12.25) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (12.34) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH8" t="n">
         <v>0.15</v>
       </c>
       <c r="AI8" t="n">
-        <v>49.4</v>
+        <v>49.5</v>
       </c>
       <c r="AJ8" t="n">
         <v>15.1</v>
@@ -1760,14 +1760,14 @@
         <v>15</v>
       </c>
       <c r="AM8" t="n">
-        <v>760.01</v>
+        <v>758.53</v>
       </c>
       <c r="AN8" t="n">
-        <v>721.91</v>
+        <v>725.13</v>
       </c>
       <c r="AO8" t="inlineStr">
         <is>
-          <t>INDHOTEL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹105,547.50 Cr., a P/E ratio of 49.43, and YoY Revenue Growth of +15.1%, the company demonstrates strong institutional backing, solid operating profit margins (20.87%), and healthy Return on Equity (15.00%).</t>
+          <t>INDHOTEL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹105,590.20 Cr., a P/E ratio of 49.45, and YoY Revenue Growth of +15.1%, the company demonstrates strong institutional backing, solid operating profit margins (20.87%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP8" t="inlineStr">
@@ -1777,22 +1777,22 @@
       </c>
       <c r="AQ8" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for INDHOTEL. Current Market Price (₹741.10) is positioned above the 30-day DMA (₹731.68), 50-day DMA (₹709.25), and 200-day DMA (₹686.46). The price distance from 200 DMA is +9.26%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for INDHOTEL. Current Market Price (₹741.80) is positioned above the 30-day DMA (₹731.68), 50-day DMA (₹709.25), and 200-day DMA (₹686.46). The price distance from 200 DMA is +9.26%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR8" t="inlineStr">
         <is>
-          <t>[741.1, 743.32, 745.55, 747.77, 749.99, 752.22]</t>
+          <t>[741.8, 744.03, 746.25, 748.48, 750.7, 752.93]</t>
         </is>
       </c>
       <c r="AS8" t="inlineStr">
         <is>
-          <t>[741.1, 749.31, 754.02, 758.14, 761.97, 765.61]</t>
+          <t>[741.8, 750.01, 754.72, 758.85, 762.68, 766.32]</t>
         </is>
       </c>
       <c r="AT8" t="inlineStr">
         <is>
-          <t>[741.1, 738.83, 739.19, 739.99, 741.01, 742.17]</t>
+          <t>[741.8, 739.53, 739.9, 740.7, 741.72, 742.88]</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1813,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>25000</v>
+        <v>96086.34</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1821,15 +1821,15 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>366.3</v>
+        <v>364.9</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>₹364.73 - ₹368.65</t>
+          <t>₹363.33 - ₹367.25</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>372.56</v>
+        <v>371.16</v>
       </c>
       <c r="I9" t="n">
         <v>358.01</v>
@@ -1856,10 +1856,10 @@
         <v>7.83</v>
       </c>
       <c r="Q9" t="n">
-        <v>12.25</v>
+        <v>12.34</v>
       </c>
       <c r="R9" t="n">
-        <v>43.3</v>
+        <v>43.6</v>
       </c>
       <c r="S9" t="n">
         <v>0.25</v>
@@ -1877,25 +1877,25 @@
         <v>-0.77</v>
       </c>
       <c r="X9" t="n">
-        <v>358.35</v>
+        <v>356.89</v>
       </c>
       <c r="Y9" t="n">
-        <v>371.17</v>
+        <v>369.66</v>
       </c>
       <c r="Z9" t="n">
-        <v>369.23</v>
+        <v>367.82</v>
       </c>
       <c r="AA9" t="n">
-        <v>354.56</v>
+        <v>353.16</v>
       </c>
       <c r="AB9" t="n">
-        <v>368.02</v>
+        <v>367.17</v>
       </c>
       <c r="AC9" t="n">
-        <v>370.59</v>
+        <v>370.04</v>
       </c>
       <c r="AD9" t="n">
-        <v>374.87</v>
+        <v>375.17</v>
       </c>
       <c r="AE9" t="n">
         <v>71.8</v>
@@ -1905,7 +1905,7 @@
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.25) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH9" t="n">
@@ -1924,14 +1924,14 @@
         <v>15</v>
       </c>
       <c r="AM9" t="n">
-        <v>375.26</v>
+        <v>374.31</v>
       </c>
       <c r="AN9" t="n">
-        <v>356.96</v>
+        <v>355.32</v>
       </c>
       <c r="AO9" t="inlineStr">
         <is>
-          <t>RECLTD operates in the Financial Services sector. With an estimated Market Cap of ₹25,000.00 Cr., a P/E ratio of 6.03, and YoY Revenue Growth of +25.2%, the company demonstrates strong institutional backing, solid operating profit margins (68.89%), and healthy Return on Equity (15.00%).</t>
+          <t>RECLTD operates in the Financial Services sector. With an estimated Market Cap of ₹96,086.34 Cr., a P/E ratio of 6.00, and YoY Revenue Growth of +25.2%, the company demonstrates strong institutional backing, solid operating profit margins (68.89%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP9" t="inlineStr">
@@ -1941,22 +1941,22 @@
       </c>
       <c r="AQ9" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for RECLTD. Current Market Price (₹366.30) is positioned above the 30-day DMA (₹358.01), 50-day DMA (₹351.17), and 200-day DMA (₹347.72). The price distance from 200 DMA is +5.86%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for RECLTD. Current Market Price (₹364.90) is positioned above the 30-day DMA (₹358.01), 50-day DMA (₹351.17), and 200-day DMA (₹347.72). The price distance from 200 DMA is +5.86%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>[366.3, 367.4, 368.5, 369.6, 370.7, 371.79]</t>
+          <t>[364.9, 365.99, 367.09, 368.18, 369.28, 370.37]</t>
         </is>
       </c>
       <c r="AS9" t="inlineStr">
         <is>
-          <t>[366.3, 370.53, 372.92, 375.02, 376.96, 378.79]</t>
+          <t>[364.9, 369.12, 371.52, 373.61, 375.54, 377.37]</t>
         </is>
       </c>
       <c r="AT9" t="inlineStr">
         <is>
-          <t>[366.3, 365.05, 365.18, 365.53, 366.0, 366.55]</t>
+          <t>[364.9, 363.65, 363.77, 364.12, 364.58, 365.12]</t>
         </is>
       </c>
     </row>
@@ -1977,7 +1977,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>116839.81</v>
+        <v>117502.25</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1985,15 +1985,15 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>1446.3</v>
+        <v>1454</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>₹1439.47 - ₹1456.54</t>
+          <t>₹1447.17 - ₹1464.24</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>1473.61</v>
+        <v>1481.31</v>
       </c>
       <c r="I10" t="n">
         <v>1443.04</v>
@@ -2020,46 +2020,46 @@
         <v>34.14</v>
       </c>
       <c r="Q10" t="n">
-        <v>12.25</v>
+        <v>12.34</v>
       </c>
       <c r="R10" t="n">
-        <v>41.9</v>
+        <v>42</v>
       </c>
       <c r="S10" t="n">
         <v>0.23</v>
       </c>
       <c r="T10" t="n">
-        <v>-1.72</v>
+        <v>-1.71</v>
       </c>
       <c r="U10" t="n">
         <v>45</v>
       </c>
       <c r="V10" t="n">
-        <v>12.13</v>
+        <v>12.14</v>
       </c>
       <c r="W10" t="n">
         <v>-0.77</v>
       </c>
       <c r="X10" t="n">
-        <v>1405.33</v>
+        <v>1413.03</v>
       </c>
       <c r="Y10" t="n">
-        <v>1407.39</v>
+        <v>1416.09</v>
       </c>
       <c r="Z10" t="n">
-        <v>1457.87</v>
+        <v>1465.63</v>
       </c>
       <c r="AA10" t="n">
-        <v>1395.09</v>
+        <v>1402.79</v>
       </c>
       <c r="AB10" t="n">
-        <v>1449.93</v>
+        <v>1452.5</v>
       </c>
       <c r="AC10" t="n">
-        <v>1456.36</v>
+        <v>1461.5</v>
       </c>
       <c r="AD10" t="n">
-        <v>1466.43</v>
+        <v>1469</v>
       </c>
       <c r="AE10" t="n">
         <v>55.4</v>
@@ -2069,14 +2069,14 @@
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (12.25) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (12.34) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH10" t="n">
         <v>0.15</v>
       </c>
       <c r="AI10" t="n">
-        <v>35</v>
+        <v>35.2</v>
       </c>
       <c r="AJ10" t="n">
         <v>3.5</v>
@@ -2088,14 +2088,14 @@
         <v>15</v>
       </c>
       <c r="AM10" t="n">
-        <v>1477.31</v>
+        <v>1488.11</v>
       </c>
       <c r="AN10" t="n">
-        <v>1416.76</v>
+        <v>1423.03</v>
       </c>
       <c r="AO10" t="inlineStr">
         <is>
-          <t>CIPLA operates in the Healthcare sector. With an estimated Market Cap of ₹116,839.81 Cr., a P/E ratio of 35.00, and YoY Revenue Growth of +3.5%, the company demonstrates strong institutional backing, solid operating profit margins (12.01%), and healthy Return on Equity (15.00%).</t>
+          <t>CIPLA operates in the Healthcare sector. With an estimated Market Cap of ₹117,502.25 Cr., a P/E ratio of 35.20, and YoY Revenue Growth of +3.5%, the company demonstrates strong institutional backing, solid operating profit margins (12.01%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP10" t="inlineStr">
@@ -2105,22 +2105,22 @@
       </c>
       <c r="AQ10" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for CIPLA. Current Market Price (₹1,446.30) is positioned above the 30-day DMA (₹1,443.04), 50-day DMA (₹1,419.16), and 200-day DMA (₹1,394.98). The price distance from 200 DMA is +4.66%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for CIPLA. Current Market Price (₹1,454.00) is positioned above the 30-day DMA (₹1,443.04), 50-day DMA (₹1,419.16), and 200-day DMA (₹1,394.98). The price distance from 200 DMA is +4.66%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR10" t="inlineStr">
         <is>
-          <t>[1446.3, 1450.64, 1454.98, 1459.32, 1463.66, 1467.99]</t>
+          <t>[1454.0, 1458.36, 1462.72, 1467.09, 1471.45, 1475.81]</t>
         </is>
       </c>
       <c r="AS10" t="inlineStr">
         <is>
-          <t>[1446.3, 1464.3, 1474.29, 1482.97, 1490.97, 1498.53]</t>
+          <t>[1454.0, 1472.02, 1482.04, 1490.74, 1498.76, 1506.35]</t>
         </is>
       </c>
       <c r="AT10" t="inlineStr">
         <is>
-          <t>[1446.3, 1440.4, 1440.49, 1441.58, 1443.17, 1445.09]</t>
+          <t>[1454.0, 1448.12, 1448.24, 1449.34, 1450.96, 1452.91]</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2141,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>147059.82</v>
+        <v>146705.48</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2149,15 +2149,15 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1660.1</v>
+        <v>1656.2</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>₹1650.99 - ₹1673.77</t>
+          <t>₹1647.09 - ₹1669.87</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>1696.56</v>
+        <v>1692.66</v>
       </c>
       <c r="I11" t="n">
         <v>1496.08</v>
@@ -2184,10 +2184,10 @@
         <v>45.57</v>
       </c>
       <c r="Q11" t="n">
-        <v>12.25</v>
+        <v>12.34</v>
       </c>
       <c r="R11" t="n">
-        <v>48</v>
+        <v>48.1</v>
       </c>
       <c r="S11" t="n">
         <v>0.19</v>
@@ -2199,31 +2199,31 @@
         <v>50</v>
       </c>
       <c r="V11" t="n">
-        <v>7.95</v>
+        <v>7.94</v>
       </c>
       <c r="W11" t="n">
         <v>-0.77</v>
       </c>
       <c r="X11" t="n">
-        <v>1631.55</v>
+        <v>1627.4</v>
       </c>
       <c r="Y11" t="n">
-        <v>1689.65</v>
+        <v>1685.36</v>
       </c>
       <c r="Z11" t="n">
-        <v>1673.38</v>
+        <v>1669.45</v>
       </c>
       <c r="AA11" t="n">
-        <v>1591.74</v>
+        <v>1587.84</v>
       </c>
       <c r="AB11" t="n">
-        <v>1657.53</v>
+        <v>1656.23</v>
       </c>
       <c r="AC11" t="n">
-        <v>1667.36</v>
+        <v>1664.76</v>
       </c>
       <c r="AD11" t="n">
-        <v>1674.63</v>
+        <v>1673.33</v>
       </c>
       <c r="AE11" t="n">
         <v>83.5</v>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>Low VIX (12.25) | LSTM Deep Net</t>
+          <t>Low VIX (12.34) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH11" t="n">
@@ -2252,14 +2252,14 @@
         <v>15</v>
       </c>
       <c r="AM11" t="n">
-        <v>1703.43</v>
+        <v>1704.65</v>
       </c>
       <c r="AN11" t="n">
-        <v>1615.17</v>
+        <v>1613.8</v>
       </c>
       <c r="AO11" t="inlineStr">
         <is>
-          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹147,059.82 Cr., a P/E ratio of 28.72, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
+          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹146,705.48 Cr., a P/E ratio of 28.65, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP11" t="inlineStr">
@@ -2269,22 +2269,22 @@
       </c>
       <c r="AQ11" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,660.10) is positioned above the 30-day DMA (₹1,496.08), 50-day DMA (₹1,470.74), and 200-day DMA (₹1,461.21). The price distance from 200 DMA is +12.85%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,656.20) is positioned above the 30-day DMA (₹1,496.08), 50-day DMA (₹1,470.74), and 200-day DMA (₹1,461.21). The price distance from 200 DMA is +12.85%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR11" t="inlineStr">
         <is>
-          <t>[1660.1, 1665.08, 1670.06, 1675.04, 1680.02, 1685.0]</t>
+          <t>[1656.2, 1661.17, 1666.14, 1671.11, 1676.07, 1681.04]</t>
         </is>
       </c>
       <c r="AS11" t="inlineStr">
         <is>
-          <t>[1660.1, 1683.31, 1695.84, 1706.61, 1716.48, 1725.76]</t>
+          <t>[1656.2, 1679.4, 1691.92, 1702.68, 1712.53, 1721.8]</t>
         </is>
       </c>
       <c r="AT11" t="inlineStr">
         <is>
-          <t>[1660.1, 1651.41, 1650.73, 1651.36, 1652.68, 1654.43]</t>
+          <t>[1656.2, 1647.5, 1646.8, 1647.43, 1648.73, 1650.47]</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>78803.39</v>
+        <v>78675.00999999999</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2313,15 +2313,15 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1780.1</v>
+        <v>1777.5</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>₹1768.46 - ₹1797.56</t>
+          <t>₹1765.86 - ₹1794.96</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1826.65</v>
+        <v>1824.05</v>
       </c>
       <c r="I12" t="n">
         <v>1530.06</v>
@@ -2348,16 +2348,16 @@
         <v>58.19</v>
       </c>
       <c r="Q12" t="n">
-        <v>12.25</v>
+        <v>12.34</v>
       </c>
       <c r="R12" t="n">
-        <v>49.1</v>
+        <v>48.9</v>
       </c>
       <c r="S12" t="n">
-        <v>0.29</v>
+        <v>0.28</v>
       </c>
       <c r="T12" t="n">
-        <v>-1.79</v>
+        <v>-1.84</v>
       </c>
       <c r="U12" t="n">
         <v>50</v>
@@ -2369,25 +2369,25 @@
         <v>-0.77</v>
       </c>
       <c r="X12" t="n">
-        <v>1778.84</v>
+        <v>1775.22</v>
       </c>
       <c r="Y12" t="n">
-        <v>1841.15</v>
+        <v>1837.43</v>
       </c>
       <c r="Z12" t="n">
-        <v>1805.55</v>
+        <v>1801.88</v>
       </c>
       <c r="AA12" t="n">
-        <v>1692.81</v>
+        <v>1690.21</v>
       </c>
       <c r="AB12" t="n">
-        <v>1771.07</v>
+        <v>1770.2</v>
       </c>
       <c r="AC12" t="n">
-        <v>1797.04</v>
+        <v>1795.3</v>
       </c>
       <c r="AD12" t="n">
-        <v>1813.97</v>
+        <v>1813.1</v>
       </c>
       <c r="AE12" t="n">
         <v>72.90000000000001</v>
@@ -2397,14 +2397,14 @@
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.25) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH12" t="n">
         <v>0.15</v>
       </c>
       <c r="AI12" t="n">
-        <v>36.9</v>
+        <v>36.8</v>
       </c>
       <c r="AJ12" t="n">
         <v>49.9</v>
@@ -2416,14 +2416,14 @@
         <v>15</v>
       </c>
       <c r="AM12" t="n">
-        <v>1852.95</v>
+        <v>1843.54</v>
       </c>
       <c r="AN12" t="n">
-        <v>1713.15</v>
+        <v>1711.42</v>
       </c>
       <c r="AO12" t="inlineStr">
         <is>
-          <t>COFORGE operates in the Technology sector. With an estimated Market Cap of ₹78,803.39 Cr., a P/E ratio of 36.86, and YoY Revenue Growth of +49.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.64%), and healthy Return on Equity (15.00%).</t>
+          <t>COFORGE operates in the Technology sector. With an estimated Market Cap of ₹78,675.01 Cr., a P/E ratio of 36.80, and YoY Revenue Growth of +49.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP12" t="inlineStr">
@@ -2433,22 +2433,22 @@
       </c>
       <c r="AQ12" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for COFORGE. Current Market Price (₹1,780.10) is positioned above the 30-day DMA (₹1,530.06), 50-day DMA (₹1,489.66), and 200-day DMA (₹1,504.99). The price distance from 200 DMA is +16.27%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for COFORGE. Current Market Price (₹1,777.50) is positioned above the 30-day DMA (₹1,530.06), 50-day DMA (₹1,489.66), and 200-day DMA (₹1,504.99). The price distance from 200 DMA is +16.27%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR12" t="inlineStr">
         <is>
-          <t>[1780.1, 1805.55, 1830.99, 1856.44, 1881.89, 1907.33]</t>
+          <t>[1777.5, 1801.88, 1826.26, 1850.64, 1875.02, 1899.4]</t>
         </is>
       </c>
       <c r="AS12" t="inlineStr">
         <is>
-          <t>[1780.1, 1828.82, 1863.91, 1896.76, 1928.44, 1959.38]</t>
+          <t>[1777.5, 1825.16, 1859.18, 1890.96, 1921.58, 1951.45]</t>
         </is>
       </c>
       <c r="AT12" t="inlineStr">
         <is>
-          <t>[1780.1, 1788.09, 1806.3, 1826.2, 1846.97, 1868.29]</t>
+          <t>[1777.5, 1784.42, 1801.57, 1820.4, 1840.1, 1860.36]</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>48334.37</v>
+        <v>48533.74</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2477,15 +2477,15 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1187.9</v>
+        <v>1192.8</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>₹1181.11 - ₹1198.08</t>
+          <t>₹1186.01 - ₹1202.98</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>1215.05</v>
+        <v>1219.95</v>
       </c>
       <c r="I13" t="n">
         <v>1109.52</v>
@@ -2512,46 +2512,46 @@
         <v>33.94</v>
       </c>
       <c r="Q13" t="n">
-        <v>12.25</v>
+        <v>12.34</v>
       </c>
       <c r="R13" t="n">
-        <v>47.7</v>
+        <v>47.3</v>
       </c>
       <c r="S13" t="n">
         <v>0.19</v>
       </c>
       <c r="T13" t="n">
-        <v>-1.86</v>
+        <v>-1.87</v>
       </c>
       <c r="U13" t="n">
         <v>50</v>
       </c>
       <c r="V13" t="n">
-        <v>2.35</v>
+        <v>2.36</v>
       </c>
       <c r="W13" t="n">
         <v>-0.77</v>
       </c>
       <c r="X13" t="n">
-        <v>1170.2</v>
+        <v>1176.91</v>
       </c>
       <c r="Y13" t="n">
-        <v>1211.78</v>
+        <v>1218.66</v>
       </c>
       <c r="Z13" t="n">
-        <v>1197.4</v>
+        <v>1202.34</v>
       </c>
       <c r="AA13" t="n">
-        <v>1137</v>
+        <v>1141.9</v>
       </c>
       <c r="AB13" t="n">
-        <v>1180.73</v>
+        <v>1183.6</v>
       </c>
       <c r="AC13" t="n">
-        <v>1198.16</v>
+        <v>1203.9</v>
       </c>
       <c r="AD13" t="n">
-        <v>1208.43</v>
+        <v>1215</v>
       </c>
       <c r="AE13" t="n">
         <v>60.6</v>
@@ -2561,14 +2561,14 @@
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | TTM Squeeze | Strong RSI | Low VIX (12.25) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | TTM Squeeze | Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH13" t="n">
         <v>0.15</v>
       </c>
       <c r="AI13" t="n">
-        <v>39.5</v>
+        <v>39.6</v>
       </c>
       <c r="AJ13" t="n">
         <v>29.9</v>
@@ -2580,14 +2580,14 @@
         <v>15</v>
       </c>
       <c r="AM13" t="n">
-        <v>1224.16</v>
+        <v>1228.87</v>
       </c>
       <c r="AN13" t="n">
-        <v>1151.08</v>
+        <v>1158.42</v>
       </c>
       <c r="AO13" t="inlineStr">
         <is>
-          <t>360ONE operates in the Financial Services sector. With an estimated Market Cap of ₹48,334.37 Cr., a P/E ratio of 39.48, and YoY Revenue Growth of +29.9%, the company demonstrates strong institutional backing, solid operating profit margins (26.46%), and healthy Return on Equity (15.00%).</t>
+          <t>360ONE operates in the Financial Services sector. With an estimated Market Cap of ₹48,533.74 Cr., a P/E ratio of 39.64, and YoY Revenue Growth of +29.9%, the company demonstrates strong institutional backing, solid operating profit margins (26.46%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP13" t="inlineStr">
@@ -2597,22 +2597,22 @@
       </c>
       <c r="AQ13" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for 360ONE. Current Market Price (₹1,187.90) is positioned above the 30-day DMA (₹1,109.52), 50-day DMA (₹1,105.91), and 200-day DMA (₹1,100.89). The price distance from 200 DMA is +4.26%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for 360ONE. Current Market Price (₹1,192.80) is positioned above the 30-day DMA (₹1,109.52), 50-day DMA (₹1,105.91), and 200-day DMA (₹1,100.89). The price distance from 200 DMA is +4.26%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR13" t="inlineStr">
         <is>
-          <t>[1187.9, 1191.46, 1195.03, 1198.59, 1202.15, 1205.72]</t>
+          <t>[1192.8, 1196.38, 1199.96, 1203.54, 1207.11, 1210.69]</t>
         </is>
       </c>
       <c r="AS13" t="inlineStr">
         <is>
-          <t>[1187.9, 1205.04, 1214.22, 1222.1, 1229.3, 1236.07]</t>
+          <t>[1192.8, 1209.95, 1219.15, 1227.05, 1234.26, 1241.05]</t>
         </is>
       </c>
       <c r="AT13" t="inlineStr">
         <is>
-          <t>[1187.9, 1181.28, 1180.63, 1180.96, 1181.79, 1182.95]</t>
+          <t>[1192.8, 1186.2, 1185.56, 1185.9, 1186.75, 1187.93]</t>
         </is>
       </c>
     </row>
@@ -2633,7 +2633,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>87098.71000000001</v>
+        <v>86916.31</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2641,15 +2641,15 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>14325</v>
+        <v>14295</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>₹14231.1 - ₹14465.85</t>
+          <t>₹14201.1 - ₹14435.85</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>14700.6</v>
+        <v>14670.6</v>
       </c>
       <c r="I14" t="n">
         <v>13362.03</v>
@@ -2676,46 +2676,46 @@
         <v>469.5</v>
       </c>
       <c r="Q14" t="n">
-        <v>12.25</v>
+        <v>12.34</v>
       </c>
       <c r="R14" t="n">
-        <v>49.5</v>
+        <v>49.7</v>
       </c>
       <c r="S14" t="n">
         <v>0.16</v>
       </c>
       <c r="T14" t="n">
-        <v>-2.09</v>
+        <v>-2.08</v>
       </c>
       <c r="U14" t="n">
         <v>48.3</v>
       </c>
       <c r="V14" t="n">
-        <v>6.4</v>
+        <v>6.39</v>
       </c>
       <c r="W14" t="n">
         <v>-0.77</v>
       </c>
       <c r="X14" t="n">
-        <v>14218.88</v>
+        <v>14185.38</v>
       </c>
       <c r="Y14" t="n">
-        <v>14720.25</v>
+        <v>14685.71</v>
       </c>
       <c r="Z14" t="n">
-        <v>14439.6</v>
+        <v>14409.36</v>
       </c>
       <c r="AA14" t="n">
-        <v>13620.75</v>
+        <v>13590.75</v>
       </c>
       <c r="AB14" t="n">
-        <v>14238.33</v>
+        <v>14228.33</v>
       </c>
       <c r="AC14" t="n">
-        <v>14453.66</v>
+        <v>14433.66</v>
       </c>
       <c r="AD14" t="n">
-        <v>14582.33</v>
+        <v>14572.33</v>
       </c>
       <c r="AE14" t="n">
         <v>55.3</v>
@@ -2725,14 +2725,14 @@
       </c>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>Low VIX (12.25) | LSTM Deep Net</t>
+          <t>Low VIX (12.34) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH14" t="n">
         <v>0.15</v>
       </c>
       <c r="AI14" t="n">
-        <v>42</v>
+        <v>41.9</v>
       </c>
       <c r="AJ14" t="n">
         <v>21.1</v>
@@ -2744,14 +2744,14 @@
         <v>15</v>
       </c>
       <c r="AM14" t="n">
-        <v>14823.15</v>
+        <v>14815.95</v>
       </c>
       <c r="AN14" t="n">
-        <v>13781.84</v>
+        <v>13766.25</v>
       </c>
       <c r="AO14" t="inlineStr">
         <is>
-          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹87,098.71 Cr., a P/E ratio of 41.96, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
+          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹86,916.31 Cr., a P/E ratio of 41.87, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP14" t="inlineStr">
@@ -2761,22 +2761,22 @@
       </c>
       <c r="AQ14" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,325.00) is positioned above the 30-day DMA (₹13,362.03), 50-day DMA (₹12,739.88), and 200-day DMA (₹12,290.57). The price distance from 200 DMA is +13.81%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,295.00) is positioned above the 30-day DMA (₹13,362.03), 50-day DMA (₹12,739.88), and 200-day DMA (₹12,290.57). The price distance from 200 DMA is +13.81%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR14" t="inlineStr">
         <is>
-          <t>[14325.0, 14433.75, 14542.5, 14651.25, 14760.01, 14868.76]</t>
+          <t>[14295.0, 14399.81, 14504.61, 14609.42, 14714.23, 14819.03]</t>
         </is>
       </c>
       <c r="AS14" t="inlineStr">
         <is>
-          <t>[14325.0, 14621.55, 14808.09, 14976.53, 15135.61, 15288.69]</t>
+          <t>[14295.0, 14587.61, 14770.2, 14934.7, 15089.83, 15238.97]</t>
         </is>
       </c>
       <c r="AT14" t="inlineStr">
         <is>
-          <t>[14325.0, 14292.9, 14343.31, 14407.3, 14478.31, 14553.81]</t>
+          <t>[14295.0, 14258.96, 14305.42, 14365.46, 14432.53, 14504.08]</t>
         </is>
       </c>
     </row>
@@ -2788,159 +2788,159 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IEX</t>
+          <t>GODREJPROP</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>11537.78</v>
+        <v>63739.41</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>129.74</v>
+        <v>2116</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>₹128.87 - ₹131.05</t>
+          <t>₹2102.33 - ₹2136.51</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>133.23</v>
+        <v>2170.7</v>
       </c>
       <c r="I15" t="n">
-        <v>124.43</v>
+        <v>2028.46</v>
       </c>
       <c r="J15" t="n">
-        <v>123.96</v>
+        <v>1908.05</v>
       </c>
       <c r="K15" t="n">
-        <v>127.99</v>
+        <v>1880.26</v>
       </c>
       <c r="L15" t="n">
-        <v>0.95</v>
+        <v>8.16</v>
       </c>
       <c r="M15" t="n">
-        <v>2.09</v>
+        <v>46.13</v>
       </c>
       <c r="N15" t="n">
-        <v>1.41</v>
+        <v>60.86</v>
       </c>
       <c r="O15" t="n">
-        <v>0.68</v>
+        <v>-14.73</v>
       </c>
       <c r="P15" t="n">
-        <v>4.36</v>
+        <v>68.37</v>
       </c>
       <c r="Q15" t="n">
-        <v>12.25</v>
+        <v>12.34</v>
       </c>
       <c r="R15" t="n">
-        <v>49</v>
+        <v>47.5</v>
       </c>
       <c r="S15" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="T15" t="n">
-        <v>-2.18</v>
+        <v>-2.16</v>
       </c>
       <c r="U15" t="n">
-        <v>48.3</v>
+        <v>51.7</v>
       </c>
       <c r="V15" t="n">
-        <v>3.62</v>
+        <v>6.25</v>
       </c>
       <c r="W15" t="n">
         <v>-0.77</v>
       </c>
       <c r="X15" t="n">
-        <v>125.13</v>
+        <v>2033.95</v>
       </c>
       <c r="Y15" t="n">
-        <v>129.67</v>
+        <v>2017.79</v>
       </c>
       <c r="Z15" t="n">
-        <v>130.78</v>
+        <v>2132.93</v>
       </c>
       <c r="AA15" t="n">
-        <v>123.19</v>
+        <v>2013.44</v>
       </c>
       <c r="AB15" t="n">
-        <v>130.13</v>
+        <v>2105.2</v>
       </c>
       <c r="AC15" t="n">
-        <v>130.55</v>
+        <v>2154.7</v>
       </c>
       <c r="AD15" t="n">
-        <v>131.37</v>
+        <v>2193.4</v>
       </c>
       <c r="AE15" t="n">
-        <v>64.40000000000001</v>
+        <v>43.7</v>
       </c>
       <c r="AF15" t="n">
-        <v>0.1</v>
+        <v>-0</v>
       </c>
       <c r="AG15" t="inlineStr">
         <is>
-          <t>Strong RSI | Low VIX (12.25) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (12.34) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH15" t="n">
         <v>0.15</v>
       </c>
       <c r="AI15" t="n">
-        <v>22.6</v>
+        <v>35.4</v>
       </c>
       <c r="AJ15" t="n">
-        <v>10.1</v>
+        <v>63</v>
       </c>
       <c r="AK15" t="n">
-        <v>66.2</v>
+        <v>36.1</v>
       </c>
       <c r="AL15" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="AM15" t="n">
-        <v>135.58</v>
+        <v>2193.96</v>
       </c>
       <c r="AN15" t="n">
-        <v>123.42</v>
+        <v>2046.54</v>
       </c>
       <c r="AO15" t="inlineStr">
         <is>
-          <t>IEX operates in the Financial Services sector. With an estimated Market Cap of ₹11,537.78 Cr., a P/E ratio of 22.56, and YoY Revenue Growth of +10.1%, the company demonstrates strong institutional backing, solid operating profit margins (66.22%), and healthy Return on Equity (15.00%).</t>
+          <t>GODREJPROP operates in the Real Estate sector. With an estimated Market Cap of ₹63,739.41 Cr., a P/E ratio of 35.39, and YoY Revenue Growth of +63.0%, the company demonstrates strong institutional backing, solid operating profit margins (36.06%), and healthy Return on Equity (9.97%).</t>
         </is>
       </c>
       <c r="AP15" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 64.41 (Bullish Momentum Zone), while MACD Line (2.09) trades above Signal (1.41) with an expanding histogram (+0.68). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +0.95% above the 200-day DMA (₹127.99). Daily volatility envelope is bounded by ATR(14) of ₹4.36.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 43.71 (Consolidation Zone), while MACD Line (46.13) trades below Signal (60.86) with an expanding histogram (-14.73). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +8.16% above the 200-day DMA (₹1880.26). Daily volatility envelope is bounded by ATR(14) of ₹68.37.</t>
         </is>
       </c>
       <c r="AQ15" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for IEX. Current Market Price (₹129.74) is positioned above the 30-day DMA (₹124.43), 50-day DMA (₹123.96), and 200-day DMA (₹127.99). The price distance from 200 DMA is +0.95%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for GODREJPROP. Current Market Price (₹2,116.00) is positioned above the 30-day DMA (₹2,028.46), 50-day DMA (₹1,908.05), and 200-day DMA (₹1,880.26). The price distance from 200 DMA is +8.16%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR15" t="inlineStr">
         <is>
-          <t>[129.74, 130.13, 130.52, 130.91, 131.3, 131.69]</t>
+          <t>[2116.0, 2122.35, 2128.7, 2135.04, 2141.39, 2147.74]</t>
         </is>
       </c>
       <c r="AS15" t="inlineStr">
         <is>
-          <t>[129.74, 131.87, 132.99, 133.93, 134.79, 135.59]</t>
+          <t>[2116.0, 2149.7, 2167.37, 2182.42, 2196.09, 2208.9]</t>
         </is>
       </c>
       <c r="AT15" t="inlineStr">
         <is>
-          <t>[129.74, 128.82, 128.67, 128.64, 128.68, 128.76]</t>
+          <t>[2116.0, 2101.84, 2099.69, 2099.52, 2100.37, 2101.87]</t>
         </is>
       </c>
     </row>
@@ -2952,159 +2952,159 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>GODREJPROP</t>
+          <t>IEX</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>63787.61</v>
+        <v>11527.11</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>🔴 AVOID / HOLD</t>
+          <t>🟡 MODERATE BUY</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2117.6</v>
+        <v>129.62</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>₹2103.93 - ₹2138.11</t>
+          <t>₹128.75 - ₹130.93</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>2172.3</v>
+        <v>133.11</v>
       </c>
       <c r="I16" t="n">
-        <v>2028.46</v>
+        <v>124.43</v>
       </c>
       <c r="J16" t="n">
-        <v>1908.05</v>
+        <v>123.96</v>
       </c>
       <c r="K16" t="n">
-        <v>1880.26</v>
+        <v>127.99</v>
       </c>
       <c r="L16" t="n">
-        <v>8.16</v>
+        <v>0.95</v>
       </c>
       <c r="M16" t="n">
-        <v>46.13</v>
+        <v>2.09</v>
       </c>
       <c r="N16" t="n">
-        <v>60.86</v>
+        <v>1.41</v>
       </c>
       <c r="O16" t="n">
-        <v>-14.73</v>
+        <v>0.68</v>
       </c>
       <c r="P16" t="n">
-        <v>68.37</v>
+        <v>4.36</v>
       </c>
       <c r="Q16" t="n">
-        <v>12.25</v>
+        <v>12.34</v>
       </c>
       <c r="R16" t="n">
-        <v>47.2</v>
+        <v>49.1</v>
       </c>
       <c r="S16" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="T16" t="n">
         <v>-2.18</v>
       </c>
       <c r="U16" t="n">
-        <v>51.7</v>
+        <v>48.3</v>
       </c>
       <c r="V16" t="n">
-        <v>6.26</v>
+        <v>3.62</v>
       </c>
       <c r="W16" t="n">
         <v>-0.77</v>
       </c>
       <c r="X16" t="n">
-        <v>2035.55</v>
+        <v>125</v>
       </c>
       <c r="Y16" t="n">
-        <v>2019.52</v>
+        <v>129.54</v>
       </c>
       <c r="Z16" t="n">
-        <v>2134.54</v>
+        <v>130.66</v>
       </c>
       <c r="AA16" t="n">
-        <v>2015.04</v>
+        <v>123.07</v>
       </c>
       <c r="AB16" t="n">
-        <v>2105.73</v>
+        <v>129.97</v>
       </c>
       <c r="AC16" t="n">
-        <v>2155.76</v>
+        <v>130.59</v>
       </c>
       <c r="AD16" t="n">
-        <v>2193.93</v>
+        <v>131.57</v>
       </c>
       <c r="AE16" t="n">
-        <v>43.7</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="AF16" t="n">
-        <v>-0</v>
+        <v>0.1</v>
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (12.25) | LSTM Deep Net</t>
+          <t>Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH16" t="n">
         <v>0.15</v>
       </c>
       <c r="AI16" t="n">
-        <v>35.4</v>
+        <v>22.5</v>
       </c>
       <c r="AJ16" t="n">
-        <v>63</v>
+        <v>10.1</v>
       </c>
       <c r="AK16" t="n">
-        <v>36.1</v>
+        <v>66.2</v>
       </c>
       <c r="AL16" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="AM16" t="n">
-        <v>2193.47</v>
+        <v>135.08</v>
       </c>
       <c r="AN16" t="n">
-        <v>2042.38</v>
+        <v>123.93</v>
       </c>
       <c r="AO16" t="inlineStr">
         <is>
-          <t>GODREJPROP operates in the Real Estate sector. With an estimated Market Cap of ₹63,787.61 Cr., a P/E ratio of 35.42, and YoY Revenue Growth of +63.0%, the company demonstrates strong institutional backing, solid operating profit margins (36.06%), and healthy Return on Equity (9.97%).</t>
+          <t>IEX operates in the Financial Services sector. With an estimated Market Cap of ₹11,527.11 Cr., a P/E ratio of 22.54, and YoY Revenue Growth of +10.1%, the company demonstrates strong institutional backing, solid operating profit margins (66.22%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP16" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 43.71 (Consolidation Zone), while MACD Line (46.13) trades below Signal (60.86) with an expanding histogram (-14.73). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +8.16% above the 200-day DMA (₹1880.26). Daily volatility envelope is bounded by ATR(14) of ₹68.37.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 64.41 (Bullish Momentum Zone), while MACD Line (2.09) trades above Signal (1.41) with an expanding histogram (+0.68). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +0.95% above the 200-day DMA (₹127.99). Daily volatility envelope is bounded by ATR(14) of ₹4.36.</t>
         </is>
       </c>
       <c r="AQ16" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for GODREJPROP. Current Market Price (₹2,117.60) is positioned above the 30-day DMA (₹2,028.46), 50-day DMA (₹1,908.05), and 200-day DMA (₹1,880.26). The price distance from 200 DMA is +8.16%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for IEX. Current Market Price (₹129.62) is positioned above the 30-day DMA (₹124.43), 50-day DMA (₹123.96), and 200-day DMA (₹127.99). The price distance from 200 DMA is +0.95%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR16" t="inlineStr">
         <is>
-          <t>[2117.6, 2123.95, 2130.31, 2136.66, 2143.01, 2149.36]</t>
+          <t>[129.62, 130.01, 130.4, 130.79, 131.18, 131.56]</t>
         </is>
       </c>
       <c r="AS16" t="inlineStr">
         <is>
-          <t>[2117.6, 2151.3, 2168.98, 2184.03, 2197.71, 2210.52]</t>
+          <t>[129.62, 131.75, 132.87, 133.81, 134.67, 135.47]</t>
         </is>
       </c>
       <c r="AT16" t="inlineStr">
         <is>
-          <t>[2117.6, 2103.44, 2101.3, 2101.13, 2101.99, 2103.5]</t>
+          <t>[129.62, 128.7, 128.55, 128.52, 128.56, 128.64]</t>
         </is>
       </c>
     </row>
@@ -3125,7 +3125,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>287300.33</v>
+        <v>285965.55</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3133,15 +3133,15 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>312.1</v>
+        <v>310.7</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>₹310.03 - ₹315.21</t>
+          <t>₹308.63 - ₹313.81</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>320.38</v>
+        <v>318.98</v>
       </c>
       <c r="I17" t="n">
         <v>286.32</v>
@@ -3168,16 +3168,16 @@
         <v>10.35</v>
       </c>
       <c r="Q17" t="n">
-        <v>12.25</v>
+        <v>12.34</v>
       </c>
       <c r="R17" t="n">
-        <v>45.9</v>
+        <v>45.6</v>
       </c>
       <c r="S17" t="n">
         <v>0.16</v>
       </c>
       <c r="T17" t="n">
-        <v>-2.32</v>
+        <v>-2.35</v>
       </c>
       <c r="U17" t="n">
         <v>53.3</v>
@@ -3189,25 +3189,25 @@
         <v>-0.77</v>
       </c>
       <c r="X17" t="n">
-        <v>307.76</v>
+        <v>306.18</v>
       </c>
       <c r="Y17" t="n">
-        <v>318.69</v>
+        <v>317.06</v>
       </c>
       <c r="Z17" t="n">
-        <v>314.6</v>
+        <v>313.19</v>
       </c>
       <c r="AA17" t="n">
-        <v>296.57</v>
+        <v>295.18</v>
       </c>
       <c r="AB17" t="n">
-        <v>312.72</v>
+        <v>311.87</v>
       </c>
       <c r="AC17" t="n">
-        <v>314.04</v>
+        <v>313.49</v>
       </c>
       <c r="AD17" t="n">
-        <v>315.97</v>
+        <v>316.27</v>
       </c>
       <c r="AE17" t="n">
         <v>62.2</v>
@@ -3217,14 +3217,14 @@
       </c>
       <c r="AG17" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.25) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH17" t="n">
         <v>0.15</v>
       </c>
       <c r="AI17" t="n">
-        <v>664</v>
+        <v>661</v>
       </c>
       <c r="AJ17" t="n">
         <v>182</v>
@@ -3236,14 +3236,14 @@
         <v>15</v>
       </c>
       <c r="AM17" t="n">
-        <v>323.72</v>
+        <v>321.59</v>
       </c>
       <c r="AN17" t="n">
-        <v>301.39</v>
+        <v>299.8</v>
       </c>
       <c r="AO17" t="inlineStr">
         <is>
-          <t>ETERNAL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹287,300.33 Cr., a P/E ratio of 664.04, and YoY Revenue Growth of +182.0%, the company demonstrates strong institutional backing, solid operating profit margins (0.64%), and healthy Return on Equity (15.00%).</t>
+          <t>ETERNAL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹285,965.55 Cr., a P/E ratio of 660.96, and YoY Revenue Growth of +182.0%, the company demonstrates strong institutional backing, solid operating profit margins (0.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP17" t="inlineStr">
@@ -3253,22 +3253,22 @@
       </c>
       <c r="AQ17" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ETERNAL. Current Market Price (₹312.10) is positioned above the 30-day DMA (₹286.32), 50-day DMA (₹272.64), and 200-day DMA (₹273.39). The price distance from 200 DMA is +14.27%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ETERNAL. Current Market Price (₹310.70) is positioned above the 30-day DMA (₹286.32), 50-day DMA (₹272.64), and 200-day DMA (₹273.39). The price distance from 200 DMA is +14.27%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR17" t="inlineStr">
         <is>
-          <t>[312.1, 313.04, 313.97, 314.91, 315.85, 316.78]</t>
+          <t>[310.7, 311.63, 312.56, 313.5, 314.43, 315.36]</t>
         </is>
       </c>
       <c r="AS17" t="inlineStr">
         <is>
-          <t>[312.1, 317.18, 319.83, 322.08, 324.13, 326.04]</t>
+          <t>[310.7, 315.77, 318.42, 320.67, 322.71, 324.62]</t>
         </is>
       </c>
       <c r="AT17" t="inlineStr">
         <is>
-          <t>[312.1, 309.93, 309.58, 309.53, 309.64, 309.84]</t>
+          <t>[310.7, 308.53, 308.17, 308.12, 308.22, 308.42]</t>
         </is>
       </c>
     </row>
@@ -3289,7 +3289,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>17449.08</v>
+        <v>17441.92</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3297,15 +3297,15 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>609.05</v>
+        <v>608.1</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>₹604.76 - ₹615.49</t>
+          <t>₹603.81 - ₹614.54</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>626.22</v>
+        <v>625.27</v>
       </c>
       <c r="I18" t="n">
         <v>583.11</v>
@@ -3332,7 +3332,7 @@
         <v>21.46</v>
       </c>
       <c r="Q18" t="n">
-        <v>12.25</v>
+        <v>12.34</v>
       </c>
       <c r="R18" t="n">
         <v>47.5</v>
@@ -3341,37 +3341,37 @@
         <v>0.15</v>
       </c>
       <c r="T18" t="n">
-        <v>-2.39</v>
+        <v>-2.4</v>
       </c>
       <c r="U18" t="n">
         <v>53.3</v>
       </c>
       <c r="V18" t="n">
-        <v>4.79</v>
+        <v>4.78</v>
       </c>
       <c r="W18" t="n">
         <v>-0.77</v>
       </c>
       <c r="X18" t="n">
-        <v>583.3</v>
+        <v>582.35</v>
       </c>
       <c r="Y18" t="n">
-        <v>596.8200000000001</v>
+        <v>595.73</v>
       </c>
       <c r="Z18" t="n">
-        <v>613.92</v>
+        <v>612.96</v>
       </c>
       <c r="AA18" t="n">
-        <v>576.86</v>
+        <v>575.91</v>
       </c>
       <c r="AB18" t="n">
-        <v>616.53</v>
+        <v>614.4</v>
       </c>
       <c r="AC18" t="n">
-        <v>625.01</v>
+        <v>626.2</v>
       </c>
       <c r="AD18" t="n">
-        <v>640.98</v>
+        <v>644.3</v>
       </c>
       <c r="AE18" t="n">
         <v>54.7</v>
@@ -3381,14 +3381,14 @@
       </c>
       <c r="AG18" t="inlineStr">
         <is>
-          <t>Low VIX (12.25) | LSTM Deep Net</t>
+          <t>Low VIX (12.34) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH18" t="n">
         <v>0.15</v>
       </c>
       <c r="AI18" t="n">
-        <v>87.90000000000001</v>
+        <v>87.8</v>
       </c>
       <c r="AJ18" t="n">
         <v>-10.1</v>
@@ -3400,14 +3400,14 @@
         <v>6.7</v>
       </c>
       <c r="AM18" t="n">
-        <v>638.96</v>
+        <v>636.6799999999999</v>
       </c>
       <c r="AN18" t="n">
-        <v>578.59</v>
+        <v>576.48</v>
       </c>
       <c r="AO18" t="inlineStr">
         <is>
-          <t>PGEL operates in the Technology sector. With an estimated Market Cap of ₹17,449.08 Cr., a P/E ratio of 87.89, and YoY Revenue Growth of -10.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.72%), and healthy Return on Equity (6.69%).</t>
+          <t>PGEL operates in the Technology sector. With an estimated Market Cap of ₹17,441.92 Cr., a P/E ratio of 87.85, and YoY Revenue Growth of -10.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.72%), and healthy Return on Equity (6.69%).</t>
         </is>
       </c>
       <c r="AP18" t="inlineStr">
@@ -3417,22 +3417,22 @@
       </c>
       <c r="AQ18" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PGEL. Current Market Price (₹609.05) is positioned above the 30-day DMA (₹583.11), 50-day DMA (₹550.15), and 200-day DMA (₹554.14). The price distance from 200 DMA is +10.44%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PGEL. Current Market Price (₹608.10) is positioned above the 30-day DMA (₹583.11), 50-day DMA (₹550.15), and 200-day DMA (₹554.14). The price distance from 200 DMA is +10.44%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR18" t="inlineStr">
         <is>
-          <t>[609.05, 610.88, 612.7, 614.53, 616.36, 618.19]</t>
+          <t>[608.1, 609.92, 611.75, 613.57, 615.4, 617.22]</t>
         </is>
       </c>
       <c r="AS18" t="inlineStr">
         <is>
-          <t>[609.05, 619.46, 624.84, 629.4, 633.53, 637.38]</t>
+          <t>[608.1, 618.51, 623.89, 628.44, 632.57, 636.42]</t>
         </is>
       </c>
       <c r="AT18" t="inlineStr">
         <is>
-          <t>[609.05, 604.44, 603.6, 603.38, 603.48, 603.79]</t>
+          <t>[608.1, 603.49, 602.64, 602.42, 602.52, 602.83]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: 3-book post-market accuracy export, autonomous learning engine & calibrated predictions
</commit_message>
<xml_diff>
--- a/Breakout_ML_Quant_Predictions.xlsx
+++ b/Breakout_ML_Quant_Predictions.xlsx
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>357416.09</v>
+        <v>357563.18</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -673,15 +673,15 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>12150</v>
+        <v>12155</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>₹12109.59 - ₹12210.61</t>
+          <t>₹12114.59 - ₹12215.61</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>12311.62</v>
+        <v>12316.62</v>
       </c>
       <c r="I2" t="n">
         <v>11508.32</v>
@@ -708,16 +708,16 @@
         <v>202.03</v>
       </c>
       <c r="Q2" t="n">
-        <v>12.34</v>
+        <v>12.55</v>
       </c>
       <c r="R2" t="n">
-        <v>50.6</v>
+        <v>50.3</v>
       </c>
       <c r="S2" t="n">
         <v>0.32</v>
       </c>
       <c r="T2" t="n">
-        <v>-0.83</v>
+        <v>-0.84</v>
       </c>
       <c r="U2" t="n">
         <v>50</v>
@@ -729,25 +729,25 @@
         <v>-0.77</v>
       </c>
       <c r="X2" t="n">
-        <v>12055.35</v>
+        <v>12060.74</v>
       </c>
       <c r="Y2" t="n">
-        <v>12453.04</v>
+        <v>12458.04</v>
       </c>
       <c r="Z2" t="n">
-        <v>12247.2</v>
+        <v>12252.24</v>
       </c>
       <c r="AA2" t="n">
-        <v>11846.96</v>
+        <v>11851.96</v>
       </c>
       <c r="AB2" t="n">
-        <v>12119.67</v>
+        <v>12121.33</v>
       </c>
       <c r="AC2" t="n">
-        <v>12269.34</v>
+        <v>12272.66</v>
       </c>
       <c r="AD2" t="n">
-        <v>12388.67</v>
+        <v>12390.33</v>
       </c>
       <c r="AE2" t="n">
         <v>70.40000000000001</v>
@@ -757,14 +757,14 @@
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH2" t="n">
         <v>0.15</v>
       </c>
       <c r="AI2" t="n">
-        <v>41.8</v>
+        <v>41.9</v>
       </c>
       <c r="AJ2" t="n">
         <v>15.9</v>
@@ -776,14 +776,14 @@
         <v>15</v>
       </c>
       <c r="AM2" t="n">
-        <v>12425.44</v>
+        <v>12431.71</v>
       </c>
       <c r="AN2" t="n">
-        <v>11882.79</v>
+        <v>11884.91</v>
       </c>
       <c r="AO2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO operates in the Basic Materials sector. With an estimated Market Cap of ₹357,416.09 Cr., a P/E ratio of 41.84, and YoY Revenue Growth of +15.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.29%), and healthy Return on Equity (15.00%).</t>
+          <t>ULTRACEMCO operates in the Basic Materials sector. With an estimated Market Cap of ₹357,563.18 Cr., a P/E ratio of 41.85, and YoY Revenue Growth of +15.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.29%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP2" t="inlineStr">
@@ -793,22 +793,22 @@
       </c>
       <c r="AQ2" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ULTRACEMCO. Current Market Price (₹12,150.00) is positioned above the 30-day DMA (₹11,508.32), 50-day DMA (₹11,305.61), and 200-day DMA (₹11,570.61). The price distance from 200 DMA is +4.14%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ULTRACEMCO. Current Market Price (₹12,155.00) is positioned above the 30-day DMA (₹11,508.32), 50-day DMA (₹11,305.61), and 200-day DMA (₹11,570.61). The price distance from 200 DMA is +4.14%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR2" t="inlineStr">
         <is>
-          <t>[12150.0, 12237.6, 12325.2, 12412.8, 12500.41, 12588.01]</t>
+          <t>[12155.0, 12243.07, 12331.14, 12419.2, 12507.27, 12595.34]</t>
         </is>
       </c>
       <c r="AS2" t="inlineStr">
         <is>
-          <t>[12150.0, 12318.41, 12439.49, 12552.77, 12662.03, 12768.7]</t>
+          <t>[12155.0, 12323.88, 12445.42, 12559.17, 12668.89, 12776.04]</t>
         </is>
       </c>
       <c r="AT2" t="inlineStr">
         <is>
-          <t>[12150.0, 12176.99, 12239.49, 12307.83, 12379.19, 12452.48]</t>
+          <t>[12155.0, 12182.46, 12245.42, 12314.23, 12386.06, 12459.82]</t>
         </is>
       </c>
     </row>
@@ -829,7 +829,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>130812.67</v>
+        <v>130674.76</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -837,15 +837,15 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>113.82</v>
+        <v>113.7</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>₹113.43 - ₹114.41</t>
+          <t>₹113.31 - ₹114.29</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>115.38</v>
+        <v>115.26</v>
       </c>
       <c r="I3" t="n">
         <v>108.12</v>
@@ -872,16 +872,16 @@
         <v>1.95</v>
       </c>
       <c r="Q3" t="n">
-        <v>12.34</v>
+        <v>12.55</v>
       </c>
       <c r="R3" t="n">
-        <v>49.4</v>
+        <v>48.9</v>
       </c>
       <c r="S3" t="n">
         <v>0.31</v>
       </c>
       <c r="T3" t="n">
-        <v>-0.91</v>
+        <v>-0.92</v>
       </c>
       <c r="U3" t="n">
         <v>55</v>
@@ -893,25 +893,25 @@
         <v>-0.77</v>
       </c>
       <c r="X3" t="n">
-        <v>111.48</v>
+        <v>111.36</v>
       </c>
       <c r="Y3" t="n">
-        <v>114.91</v>
+        <v>114.77</v>
       </c>
       <c r="Z3" t="n">
+        <v>114.61</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>110.77</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>114.16</v>
+      </c>
+      <c r="AC3" t="n">
         <v>114.73</v>
       </c>
-      <c r="AA3" t="n">
-        <v>110.89</v>
-      </c>
-      <c r="AB3" t="n">
-        <v>114.21</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>114.82</v>
-      </c>
       <c r="AD3" t="n">
-        <v>115.81</v>
+        <v>115.77</v>
       </c>
       <c r="AE3" t="n">
         <v>79</v>
@@ -921,7 +921,7 @@
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Low VIX (12.34) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Low VIX (12.55) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH3" t="n">
@@ -940,14 +940,14 @@
         <v>15</v>
       </c>
       <c r="AM3" t="n">
-        <v>116.9</v>
+        <v>117.02</v>
       </c>
       <c r="AN3" t="n">
-        <v>110.73</v>
+        <v>110.4</v>
       </c>
       <c r="AO3" t="inlineStr">
         <is>
-          <t>PNB operates in the Financial Services sector. With an estimated Market Cap of ₹130,812.67 Cr., a P/E ratio of 5.87, and YoY Revenue Growth of +15.2%, the company demonstrates strong institutional backing, solid operating profit margins (38.15%), and healthy Return on Equity (14.97%).</t>
+          <t>PNB operates in the Financial Services sector. With an estimated Market Cap of ₹130,674.76 Cr., a P/E ratio of 5.86, and YoY Revenue Growth of +15.2%, the company demonstrates strong institutional backing, solid operating profit margins (38.15%), and healthy Return on Equity (14.97%).</t>
         </is>
       </c>
       <c r="AP3" t="inlineStr">
@@ -957,22 +957,22 @@
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PNB. Current Market Price (₹113.82) is positioned above the 30-day DMA (₹108.12), 50-day DMA (₹106.98), and 200-day DMA (₹112.64). The price distance from 200 DMA is +1.20%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PNB. Current Market Price (₹113.70) is positioned above the 30-day DMA (₹108.12), 50-day DMA (₹106.98), and 200-day DMA (₹112.64). The price distance from 200 DMA is +1.20%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR3" t="inlineStr">
         <is>
-          <t>[113.82, 114.16, 114.5, 114.84, 115.19, 115.53]</t>
+          <t>[113.7, 114.04, 114.38, 114.72, 115.06, 115.41]</t>
         </is>
       </c>
       <c r="AS3" t="inlineStr">
         <is>
-          <t>[113.82, 114.94, 115.61, 116.2, 116.75, 117.27]</t>
+          <t>[113.7, 114.82, 115.49, 116.08, 116.63, 117.15]</t>
         </is>
       </c>
       <c r="AT3" t="inlineStr">
         <is>
-          <t>[113.82, 113.58, 113.67, 113.83, 114.01, 114.22]</t>
+          <t>[113.7, 113.46, 113.55, 113.71, 113.89, 114.1]</t>
         </is>
       </c>
     </row>
@@ -993,7 +993,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>219603.63</v>
+        <v>219891.88</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1001,15 +1001,15 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>7999.5</v>
+        <v>8010</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>₹7968.14 - ₹8046.54</t>
+          <t>₹7978.64 - ₹8057.04</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>8124.95</v>
+        <v>8135.45</v>
       </c>
       <c r="I4" t="n">
         <v>7478.7</v>
@@ -1036,16 +1036,16 @@
         <v>156.81</v>
       </c>
       <c r="Q4" t="n">
-        <v>12.34</v>
+        <v>12.55</v>
       </c>
       <c r="R4" t="n">
-        <v>51.5</v>
+        <v>51.2</v>
       </c>
       <c r="S4" t="n">
         <v>0.27</v>
       </c>
       <c r="T4" t="n">
-        <v>-1.01</v>
+        <v>-1.02</v>
       </c>
       <c r="U4" t="n">
         <v>51.7</v>
@@ -1057,25 +1057,25 @@
         <v>-0.77</v>
       </c>
       <c r="X4" t="n">
-        <v>7877.72</v>
+        <v>7887.48</v>
       </c>
       <c r="Y4" t="n">
-        <v>8157.7</v>
+        <v>8167.83</v>
       </c>
       <c r="Z4" t="n">
-        <v>8063.5</v>
+        <v>8074.08</v>
       </c>
       <c r="AA4" t="n">
-        <v>7764.28</v>
+        <v>7774.78</v>
       </c>
       <c r="AB4" t="n">
-        <v>7968.17</v>
+        <v>7977.83</v>
       </c>
       <c r="AC4" t="n">
-        <v>8030.84</v>
+        <v>8050.16</v>
       </c>
       <c r="AD4" t="n">
-        <v>8062.17</v>
+        <v>8090.33</v>
       </c>
       <c r="AE4" t="n">
         <v>74.3</v>
@@ -1085,14 +1085,14 @@
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH4" t="n">
         <v>0.15</v>
       </c>
       <c r="AI4" t="n">
-        <v>38.6</v>
+        <v>38.7</v>
       </c>
       <c r="AJ4" t="n">
         <v>31.5</v>
@@ -1104,14 +1104,14 @@
         <v>15</v>
       </c>
       <c r="AM4" t="n">
-        <v>8209.23</v>
+        <v>8235.690000000001</v>
       </c>
       <c r="AN4" t="n">
-        <v>7811.34</v>
+        <v>7798.99</v>
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>EICHERMOT operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹219,603.63 Cr., a P/E ratio of 38.63, and YoY Revenue Growth of +31.5%, the company demonstrates strong institutional backing, solid operating profit margins (23.21%), and healthy Return on Equity (15.00%).</t>
+          <t>EICHERMOT operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹219,891.88 Cr., a P/E ratio of 38.68, and YoY Revenue Growth of +31.5%, the company demonstrates strong institutional backing, solid operating profit margins (23.21%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP4" t="inlineStr">
@@ -1121,22 +1121,22 @@
       </c>
       <c r="AQ4" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for EICHERMOT. Current Market Price (₹7,999.50) is positioned above the 30-day DMA (₹7,478.70), 50-day DMA (₹7,389.91), and 200-day DMA (₹7,187.90). The price distance from 200 DMA is +10.39%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for EICHERMOT. Current Market Price (₹8,010.00) is positioned above the 30-day DMA (₹7,478.70), 50-day DMA (₹7,389.91), and 200-day DMA (₹7,187.90). The price distance from 200 DMA is +10.39%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR4" t="inlineStr">
         <is>
-          <t>[7999.5, 8023.5, 8047.5, 8071.5, 8095.49, 8119.49]</t>
+          <t>[8010.0, 8034.03, 8058.06, 8082.09, 8106.12, 8130.15]</t>
         </is>
       </c>
       <c r="AS4" t="inlineStr">
         <is>
-          <t>[7999.5, 8086.22, 8136.2, 8180.14, 8220.94, 8259.75]</t>
+          <t>[8010.0, 8096.75, 8146.77, 8190.73, 8231.57, 8270.41]</t>
         </is>
       </c>
       <c r="AT4" t="inlineStr">
         <is>
-          <t>[7999.5, 7976.46, 7980.97, 7990.01, 8001.41, 8014.3]</t>
+          <t>[8010.0, 7986.99, 7991.53, 8000.61, 8012.03, 8024.96]</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>309201.42</v>
+        <v>309709.69</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -1165,15 +1165,15 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>4623.4</v>
+        <v>4631</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>₹4607.36 - ₹4647.46</t>
+          <t>₹4614.96 - ₹4655.06</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>4687.55</v>
+        <v>4695.15</v>
       </c>
       <c r="I5" t="n">
         <v>4490.17</v>
@@ -1200,16 +1200,16 @@
         <v>80.19</v>
       </c>
       <c r="Q5" t="n">
-        <v>12.34</v>
+        <v>12.55</v>
       </c>
       <c r="R5" t="n">
-        <v>40.8</v>
+        <v>40.6</v>
       </c>
       <c r="S5" t="n">
         <v>0.31</v>
       </c>
       <c r="T5" t="n">
-        <v>-1.21</v>
+        <v>-1.22</v>
       </c>
       <c r="U5" t="n">
         <v>41.7</v>
@@ -1221,25 +1221,25 @@
         <v>-0.77</v>
       </c>
       <c r="X5" t="n">
-        <v>4527.18</v>
+        <v>4534.78</v>
       </c>
       <c r="Y5" t="n">
-        <v>4662.53</v>
+        <v>4670.81</v>
       </c>
       <c r="Z5" t="n">
-        <v>4660.39</v>
+        <v>4668.05</v>
       </c>
       <c r="AA5" t="n">
-        <v>4503.12</v>
+        <v>4510.72</v>
       </c>
       <c r="AB5" t="n">
-        <v>4633.37</v>
+        <v>4635.9</v>
       </c>
       <c r="AC5" t="n">
-        <v>4663.44</v>
+        <v>4668.5</v>
       </c>
       <c r="AD5" t="n">
-        <v>4703.47</v>
+        <v>4706</v>
       </c>
       <c r="AE5" t="n">
         <v>72.8</v>
@@ -1249,7 +1249,7 @@
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH5" t="n">
@@ -1268,14 +1268,14 @@
         <v>24</v>
       </c>
       <c r="AM5" t="n">
-        <v>4748.28</v>
+        <v>4757.33</v>
       </c>
       <c r="AN5" t="n">
-        <v>4505.04</v>
+        <v>4494.93</v>
       </c>
       <c r="AO5" t="inlineStr">
         <is>
-          <t>HAL operates in the Industrials sector. With an estimated Market Cap of ₹309,201.42 Cr., a P/E ratio of 33.96, and YoY Revenue Growth of +1.8%, the company demonstrates strong institutional backing, solid operating profit margins (27.55%), and healthy Return on Equity (23.98%).</t>
+          <t>HAL operates in the Industrials sector. With an estimated Market Cap of ₹309,709.69 Cr., a P/E ratio of 34.02, and YoY Revenue Growth of +1.8%, the company demonstrates strong institutional backing, solid operating profit margins (27.55%), and healthy Return on Equity (23.98%).</t>
         </is>
       </c>
       <c r="AP5" t="inlineStr">
@@ -1285,22 +1285,22 @@
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for HAL. Current Market Price (₹4,623.40) is positioned above the 30-day DMA (₹4,490.17), 50-day DMA (₹4,419.22), and 200-day DMA (₹4,344.79). The price distance from 200 DMA is +6.68%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for HAL. Current Market Price (₹4,631.00) is positioned above the 30-day DMA (₹4,490.17), 50-day DMA (₹4,419.22), and 200-day DMA (₹4,344.79). The price distance from 200 DMA is +6.68%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>[4623.4, 4637.27, 4651.14, 4665.01, 4678.88, 4692.75]</t>
+          <t>[4631.0, 4644.89, 4658.79, 4672.68, 4686.57, 4700.46]</t>
         </is>
       </c>
       <c r="AS5" t="inlineStr">
         <is>
-          <t>[4623.4, 4669.34, 4696.5, 4720.56, 4743.03, 4764.47]</t>
+          <t>[4631.0, 4676.97, 4704.15, 4728.23, 4750.72, 4772.19]</t>
         </is>
       </c>
       <c r="AT5" t="inlineStr">
         <is>
-          <t>[4623.4, 4613.21, 4617.12, 4623.34, 4630.77, 4638.96]</t>
+          <t>[4631.0, 4620.84, 4624.77, 4631.01, 4638.46, 4646.67]</t>
         </is>
       </c>
     </row>
@@ -1312,159 +1312,159 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>ALKEM</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Basic Materials</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>264394.09</v>
+        <v>67440.64</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2758</v>
+        <v>5640.5</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>₹2746.15 - ₹2775.77</t>
+          <t>₹5617.16 - ₹5675.5</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>2805.39</v>
+        <v>5733.84</v>
       </c>
       <c r="I6" t="n">
-        <v>2698.21</v>
+        <v>5598.93</v>
       </c>
       <c r="J6" t="n">
-        <v>2687.88</v>
+        <v>5497.15</v>
       </c>
       <c r="K6" t="n">
-        <v>2577.55</v>
+        <v>5524.06</v>
       </c>
       <c r="L6" t="n">
-        <v>7.66</v>
+        <v>3.31</v>
       </c>
       <c r="M6" t="n">
-        <v>26.47</v>
+        <v>58.81</v>
       </c>
       <c r="N6" t="n">
-        <v>16.72</v>
+        <v>54.69</v>
       </c>
       <c r="O6" t="n">
-        <v>9.76</v>
+        <v>4.12</v>
       </c>
       <c r="P6" t="n">
-        <v>59.24</v>
+        <v>116.68</v>
       </c>
       <c r="Q6" t="n">
-        <v>12.34</v>
+        <v>12.55</v>
       </c>
       <c r="R6" t="n">
-        <v>48.2</v>
+        <v>47.1</v>
       </c>
       <c r="S6" t="n">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="T6" t="n">
-        <v>-1.28</v>
+        <v>-1.26</v>
       </c>
       <c r="U6" t="n">
-        <v>55</v>
+        <v>51.7</v>
       </c>
       <c r="V6" t="n">
-        <v>1.78</v>
+        <v>2.82</v>
       </c>
       <c r="W6" t="n">
         <v>-0.77</v>
       </c>
       <c r="X6" t="n">
-        <v>2686.92</v>
+        <v>5500.49</v>
       </c>
       <c r="Y6" t="n">
-        <v>2779.48</v>
+        <v>5606.71</v>
       </c>
       <c r="Z6" t="n">
-        <v>2780.06</v>
+        <v>5685.62</v>
       </c>
       <c r="AA6" t="n">
-        <v>2669.15</v>
+        <v>5465.48</v>
       </c>
       <c r="AB6" t="n">
-        <v>2764.57</v>
+        <v>5620.67</v>
       </c>
       <c r="AC6" t="n">
-        <v>2780.44</v>
+        <v>5685.34</v>
       </c>
       <c r="AD6" t="n">
-        <v>2802.87</v>
+        <v>5730.17</v>
       </c>
       <c r="AE6" t="n">
-        <v>67</v>
+        <v>56.2</v>
       </c>
       <c r="AF6" t="n">
-        <v>0.02</v>
+        <v>-0.03</v>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (12.55) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH6" t="n">
         <v>0.15</v>
       </c>
       <c r="AI6" t="n">
-        <v>56.1</v>
+        <v>29.3</v>
       </c>
       <c r="AJ6" t="n">
-        <v>17.9</v>
+        <v>14.6</v>
       </c>
       <c r="AK6" t="n">
-        <v>12.8</v>
+        <v>15.6</v>
       </c>
       <c r="AL6" t="n">
-        <v>15</v>
+        <v>17.6</v>
       </c>
       <c r="AM6" t="n">
-        <v>2821.79</v>
+        <v>5765.79</v>
       </c>
       <c r="AN6" t="n">
-        <v>2696.4</v>
+        <v>5506.54</v>
       </c>
       <c r="AO6" t="inlineStr">
         <is>
-          <t>ASIANPAINT operates in the Basic Materials sector. With an estimated Market Cap of ₹264,394.09 Cr., a P/E ratio of 56.15, and YoY Revenue Growth of +17.9%, the company demonstrates strong institutional backing, solid operating profit margins (12.81%), and healthy Return on Equity (15.00%).</t>
+          <t>ALKEM operates in the Healthcare sector. With an estimated Market Cap of ₹67,440.64 Cr., a P/E ratio of 29.27, and YoY Revenue Growth of +14.6%, the company demonstrates strong institutional backing, solid operating profit margins (15.65%), and healthy Return on Equity (17.56%).</t>
         </is>
       </c>
       <c r="AP6" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 66.98 (Bullish Momentum Zone), while MACD Line (26.47) trades above Signal (16.72) with an expanding histogram (+9.76). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +7.66% above the 200-day DMA (₹2577.55). Daily volatility envelope is bounded by ATR(14) of ₹59.24.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 56.20 (Bullish Momentum Zone), while MACD Line (58.81) trades above Signal (54.69) with an expanding histogram (+4.12). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +3.31% above the 200-day DMA (₹5524.06). Daily volatility envelope is bounded by ATR(14) of ₹116.68.</t>
         </is>
       </c>
       <c r="AQ6" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ASIANPAINT. Current Market Price (₹2,758.00) is positioned above the 30-day DMA (₹2,698.21), 50-day DMA (₹2,687.88), and 200-day DMA (₹2,577.55). The price distance from 200 DMA is +7.66%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ALKEM. Current Market Price (₹5,640.50) is positioned above the 30-day DMA (₹5,598.93), 50-day DMA (₹5,497.15), and 200-day DMA (₹5,524.06). The price distance from 200 DMA is +3.31%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR6" t="inlineStr">
         <is>
-          <t>[2758.0, 2766.27, 2774.55, 2782.82, 2791.1, 2799.37]</t>
+          <t>[5640.5, 5657.42, 5674.34, 5691.26, 5708.19, 5725.11]</t>
         </is>
       </c>
       <c r="AS6" t="inlineStr">
         <is>
-          <t>[2758.0, 2789.97, 2808.06, 2823.86, 2838.48, 2852.35]</t>
+          <t>[5640.5, 5704.09, 5740.35, 5772.1, 5801.53, 5829.47]</t>
         </is>
       </c>
       <c r="AT6" t="inlineStr">
         <is>
-          <t>[2758.0, 2748.5, 2749.42, 2752.04, 2755.55, 2759.63]</t>
+          <t>[5640.5, 5622.42, 5624.84, 5630.64, 5638.18, 5646.84]</t>
         </is>
       </c>
     </row>
@@ -1476,159 +1476,159 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ALKEM</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Basic Materials</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>67315.09</v>
+        <v>264489.95</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>🔴 AVOID / HOLD</t>
+          <t>🟡 MODERATE BUY</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>5629</v>
+        <v>2759</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>₹5605.66 - ₹5664.0</t>
+          <t>₹2747.15 - ₹2776.77</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>5722.34</v>
+        <v>2806.39</v>
       </c>
       <c r="I7" t="n">
-        <v>5598.93</v>
+        <v>2698.21</v>
       </c>
       <c r="J7" t="n">
-        <v>5497.15</v>
+        <v>2687.88</v>
       </c>
       <c r="K7" t="n">
-        <v>5524.06</v>
+        <v>2577.55</v>
       </c>
       <c r="L7" t="n">
-        <v>3.31</v>
+        <v>7.66</v>
       </c>
       <c r="M7" t="n">
-        <v>58.81</v>
+        <v>26.47</v>
       </c>
       <c r="N7" t="n">
-        <v>54.69</v>
+        <v>16.72</v>
       </c>
       <c r="O7" t="n">
-        <v>4.12</v>
+        <v>9.76</v>
       </c>
       <c r="P7" t="n">
-        <v>116.68</v>
+        <v>59.24</v>
       </c>
       <c r="Q7" t="n">
-        <v>12.34</v>
+        <v>12.55</v>
       </c>
       <c r="R7" t="n">
-        <v>46.7</v>
+        <v>48.2</v>
       </c>
       <c r="S7" t="n">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="T7" t="n">
         <v>-1.28</v>
       </c>
       <c r="U7" t="n">
-        <v>51.7</v>
+        <v>55</v>
       </c>
       <c r="V7" t="n">
-        <v>2.82</v>
+        <v>1.78</v>
       </c>
       <c r="W7" t="n">
         <v>-0.77</v>
       </c>
       <c r="X7" t="n">
-        <v>5488.99</v>
+        <v>2687.92</v>
       </c>
       <c r="Y7" t="n">
-        <v>5594.42</v>
+        <v>2780.66</v>
       </c>
       <c r="Z7" t="n">
-        <v>5674.03</v>
+        <v>2781.07</v>
       </c>
       <c r="AA7" t="n">
-        <v>5453.98</v>
+        <v>2670.15</v>
       </c>
       <c r="AB7" t="n">
-        <v>5616.83</v>
+        <v>2764.9</v>
       </c>
       <c r="AC7" t="n">
-        <v>5677.66</v>
+        <v>2781.1</v>
       </c>
       <c r="AD7" t="n">
-        <v>5726.33</v>
+        <v>2803.2</v>
       </c>
       <c r="AE7" t="n">
-        <v>56.2</v>
+        <v>67</v>
       </c>
       <c r="AF7" t="n">
-        <v>-0.03</v>
+        <v>0.02</v>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (12.34) | LSTM Deep Net</t>
+          <t>Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH7" t="n">
         <v>0.15</v>
       </c>
       <c r="AI7" t="n">
-        <v>29.2</v>
+        <v>56.2</v>
       </c>
       <c r="AJ7" t="n">
-        <v>14.6</v>
+        <v>17.9</v>
       </c>
       <c r="AK7" t="n">
-        <v>15.6</v>
+        <v>12.8</v>
       </c>
       <c r="AL7" t="n">
-        <v>17.6</v>
+        <v>15</v>
       </c>
       <c r="AM7" t="n">
-        <v>5748.52</v>
+        <v>2826.2</v>
       </c>
       <c r="AN7" t="n">
-        <v>5495.23</v>
+        <v>2694.16</v>
       </c>
       <c r="AO7" t="inlineStr">
         <is>
-          <t>ALKEM operates in the Healthcare sector. With an estimated Market Cap of ₹67,315.09 Cr., a P/E ratio of 29.22, and YoY Revenue Growth of +14.6%, the company demonstrates strong institutional backing, solid operating profit margins (15.65%), and healthy Return on Equity (17.56%).</t>
+          <t>ASIANPAINT operates in the Basic Materials sector. With an estimated Market Cap of ₹264,489.95 Cr., a P/E ratio of 56.17, and YoY Revenue Growth of +17.9%, the company demonstrates strong institutional backing, solid operating profit margins (12.81%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP7" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 56.20 (Bullish Momentum Zone), while MACD Line (58.81) trades above Signal (54.69) with an expanding histogram (+4.12). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +3.31% above the 200-day DMA (₹5524.06). Daily volatility envelope is bounded by ATR(14) of ₹116.68.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 66.98 (Bullish Momentum Zone), while MACD Line (26.47) trades above Signal (16.72) with an expanding histogram (+9.76). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +7.66% above the 200-day DMA (₹2577.55). Daily volatility envelope is bounded by ATR(14) of ₹59.24.</t>
         </is>
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ALKEM. Current Market Price (₹5,629.00) is positioned above the 30-day DMA (₹5,598.93), 50-day DMA (₹5,497.15), and 200-day DMA (₹5,524.06). The price distance from 200 DMA is +3.31%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ASIANPAINT. Current Market Price (₹2,759.00) is positioned above the 30-day DMA (₹2,698.21), 50-day DMA (₹2,687.88), and 200-day DMA (₹2,577.55). The price distance from 200 DMA is +7.66%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>[5629.0, 5645.89, 5662.77, 5679.66, 5696.55, 5713.43]</t>
+          <t>[2759.0, 2767.28, 2775.55, 2783.83, 2792.11, 2800.38]</t>
         </is>
       </c>
       <c r="AS7" t="inlineStr">
         <is>
-          <t>[5629.0, 5692.56, 5728.78, 5760.5, 5789.89, 5817.8]</t>
+          <t>[2759.0, 2790.97, 2809.06, 2824.87, 2839.5, 2853.37]</t>
         </is>
       </c>
       <c r="AT7" t="inlineStr">
         <is>
-          <t>[5629.0, 5610.88, 5613.27, 5619.03, 5626.54, 5635.16]</t>
+          <t>[2759.0, 2749.51, 2750.42, 2753.05, 2756.57, 2760.65]</t>
         </is>
       </c>
     </row>
@@ -1649,7 +1649,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>105590.2</v>
+        <v>104899.84</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1657,15 +1657,15 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>741.8</v>
+        <v>737.6</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>₹738.81 - ₹746.29</t>
+          <t>₹734.61 - ₹742.09</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>753.78</v>
+        <v>749.58</v>
       </c>
       <c r="I8" t="n">
         <v>731.6799999999999</v>
@@ -1692,46 +1692,46 @@
         <v>14.97</v>
       </c>
       <c r="Q8" t="n">
-        <v>12.34</v>
+        <v>12.55</v>
       </c>
       <c r="R8" t="n">
-        <v>43.9</v>
+        <v>43.8</v>
       </c>
       <c r="S8" t="n">
         <v>0.26</v>
       </c>
       <c r="T8" t="n">
-        <v>-1.35</v>
+        <v>-1.36</v>
       </c>
       <c r="U8" t="n">
         <v>55</v>
       </c>
       <c r="V8" t="n">
-        <v>6.32</v>
+        <v>6.3</v>
       </c>
       <c r="W8" t="n">
         <v>-0.77</v>
       </c>
       <c r="X8" t="n">
-        <v>723.83</v>
+        <v>719.63</v>
       </c>
       <c r="Y8" t="n">
-        <v>735.01</v>
+        <v>729.87</v>
       </c>
       <c r="Z8" t="n">
-        <v>747.73</v>
+        <v>743.5</v>
       </c>
       <c r="AA8" t="n">
-        <v>719.34</v>
+        <v>715.14</v>
       </c>
       <c r="AB8" t="n">
-        <v>745</v>
+        <v>742.4299999999999</v>
       </c>
       <c r="AC8" t="n">
-        <v>749.7</v>
+        <v>748.0599999999999</v>
       </c>
       <c r="AD8" t="n">
-        <v>757.6</v>
+        <v>758.53</v>
       </c>
       <c r="AE8" t="n">
         <v>54.1</v>
@@ -1741,14 +1741,14 @@
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (12.34) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (12.55) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH8" t="n">
         <v>0.15</v>
       </c>
       <c r="AI8" t="n">
-        <v>49.5</v>
+        <v>49.1</v>
       </c>
       <c r="AJ8" t="n">
         <v>15.1</v>
@@ -1760,14 +1760,14 @@
         <v>15</v>
       </c>
       <c r="AM8" t="n">
-        <v>758.53</v>
+        <v>755.92</v>
       </c>
       <c r="AN8" t="n">
-        <v>725.13</v>
+        <v>720</v>
       </c>
       <c r="AO8" t="inlineStr">
         <is>
-          <t>INDHOTEL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹105,590.20 Cr., a P/E ratio of 49.45, and YoY Revenue Growth of +15.1%, the company demonstrates strong institutional backing, solid operating profit margins (20.87%), and healthy Return on Equity (15.00%).</t>
+          <t>INDHOTEL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹104,899.84 Cr., a P/E ratio of 49.13, and YoY Revenue Growth of +15.1%, the company demonstrates strong institutional backing, solid operating profit margins (20.87%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP8" t="inlineStr">
@@ -1777,22 +1777,22 @@
       </c>
       <c r="AQ8" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for INDHOTEL. Current Market Price (₹741.80) is positioned above the 30-day DMA (₹731.68), 50-day DMA (₹709.25), and 200-day DMA (₹686.46). The price distance from 200 DMA is +9.26%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for INDHOTEL. Current Market Price (₹737.60) is positioned above the 30-day DMA (₹731.68), 50-day DMA (₹709.25), and 200-day DMA (₹686.46). The price distance from 200 DMA is +9.26%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR8" t="inlineStr">
         <is>
-          <t>[741.8, 744.03, 746.25, 748.48, 750.7, 752.93]</t>
+          <t>[737.6, 739.81, 742.03, 744.24, 746.45, 748.66]</t>
         </is>
       </c>
       <c r="AS8" t="inlineStr">
         <is>
-          <t>[741.8, 750.01, 754.72, 758.85, 762.68, 766.32]</t>
+          <t>[737.6, 745.8, 750.49, 754.61, 758.43, 762.05]</t>
         </is>
       </c>
       <c r="AT8" t="inlineStr">
         <is>
-          <t>[741.8, 739.53, 739.9, 740.7, 741.72, 742.88]</t>
+          <t>[737.6, 735.32, 735.67, 736.46, 737.47, 738.62]</t>
         </is>
       </c>
     </row>
@@ -1813,7 +1813,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>96086.34</v>
+        <v>95902.02</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1821,15 +1821,15 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>364.9</v>
+        <v>364.2</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>₹363.33 - ₹367.25</t>
+          <t>₹362.64 - ₹366.55</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>371.16</v>
+        <v>370.46</v>
       </c>
       <c r="I9" t="n">
         <v>358.01</v>
@@ -1856,46 +1856,46 @@
         <v>7.83</v>
       </c>
       <c r="Q9" t="n">
-        <v>12.34</v>
+        <v>12.55</v>
       </c>
       <c r="R9" t="n">
-        <v>43.6</v>
+        <v>43</v>
       </c>
       <c r="S9" t="n">
         <v>0.25</v>
       </c>
       <c r="T9" t="n">
-        <v>-1.47</v>
+        <v>-1.49</v>
       </c>
       <c r="U9" t="n">
         <v>50</v>
       </c>
       <c r="V9" t="n">
-        <v>3</v>
+        <v>2.99</v>
       </c>
       <c r="W9" t="n">
         <v>-0.77</v>
       </c>
       <c r="X9" t="n">
-        <v>356.89</v>
+        <v>356.16</v>
       </c>
       <c r="Y9" t="n">
-        <v>369.66</v>
+        <v>368.91</v>
       </c>
       <c r="Z9" t="n">
-        <v>367.82</v>
+        <v>367.11</v>
       </c>
       <c r="AA9" t="n">
-        <v>353.16</v>
+        <v>352.46</v>
       </c>
       <c r="AB9" t="n">
-        <v>367.17</v>
+        <v>366.87</v>
       </c>
       <c r="AC9" t="n">
-        <v>370.04</v>
+        <v>369.64</v>
       </c>
       <c r="AD9" t="n">
-        <v>375.17</v>
+        <v>375.07</v>
       </c>
       <c r="AE9" t="n">
         <v>71.8</v>
@@ -1905,7 +1905,7 @@
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH9" t="n">
@@ -1924,14 +1924,14 @@
         <v>15</v>
       </c>
       <c r="AM9" t="n">
-        <v>374.31</v>
+        <v>373.9</v>
       </c>
       <c r="AN9" t="n">
-        <v>355.32</v>
+        <v>354.41</v>
       </c>
       <c r="AO9" t="inlineStr">
         <is>
-          <t>RECLTD operates in the Financial Services sector. With an estimated Market Cap of ₹96,086.34 Cr., a P/E ratio of 6.00, and YoY Revenue Growth of +25.2%, the company demonstrates strong institutional backing, solid operating profit margins (68.89%), and healthy Return on Equity (15.00%).</t>
+          <t>RECLTD operates in the Financial Services sector. With an estimated Market Cap of ₹95,902.02 Cr., a P/E ratio of 5.99, and YoY Revenue Growth of +25.2%, the company demonstrates strong institutional backing, solid operating profit margins (68.89%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP9" t="inlineStr">
@@ -1941,22 +1941,22 @@
       </c>
       <c r="AQ9" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for RECLTD. Current Market Price (₹364.90) is positioned above the 30-day DMA (₹358.01), 50-day DMA (₹351.17), and 200-day DMA (₹347.72). The price distance from 200 DMA is +5.86%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for RECLTD. Current Market Price (₹364.20) is positioned above the 30-day DMA (₹358.01), 50-day DMA (₹351.17), and 200-day DMA (₹347.72). The price distance from 200 DMA is +5.86%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>[364.9, 365.99, 367.09, 368.18, 369.28, 370.37]</t>
+          <t>[364.2, 365.29, 366.39, 367.48, 368.57, 369.66]</t>
         </is>
       </c>
       <c r="AS9" t="inlineStr">
         <is>
-          <t>[364.9, 369.12, 371.52, 373.61, 375.54, 377.37]</t>
+          <t>[364.2, 368.42, 370.81, 372.9, 374.83, 376.66]</t>
         </is>
       </c>
       <c r="AT9" t="inlineStr">
         <is>
-          <t>[364.9, 363.65, 363.77, 364.12, 364.58, 365.12]</t>
+          <t>[364.2, 362.95, 363.07, 363.41, 363.88, 364.41]</t>
         </is>
       </c>
     </row>
@@ -1977,7 +1977,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>117502.25</v>
+        <v>117478.01</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1985,15 +1985,15 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>1454</v>
+        <v>1454.2</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>₹1447.17 - ₹1464.24</t>
+          <t>₹1447.37 - ₹1464.44</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>1481.31</v>
+        <v>1481.51</v>
       </c>
       <c r="I10" t="n">
         <v>1443.04</v>
@@ -2020,16 +2020,16 @@
         <v>34.14</v>
       </c>
       <c r="Q10" t="n">
-        <v>12.34</v>
+        <v>12.55</v>
       </c>
       <c r="R10" t="n">
-        <v>42</v>
+        <v>42.5</v>
       </c>
       <c r="S10" t="n">
         <v>0.23</v>
       </c>
       <c r="T10" t="n">
-        <v>-1.71</v>
+        <v>-1.69</v>
       </c>
       <c r="U10" t="n">
         <v>45</v>
@@ -2041,25 +2041,25 @@
         <v>-0.77</v>
       </c>
       <c r="X10" t="n">
-        <v>1413.03</v>
+        <v>1413.23</v>
       </c>
       <c r="Y10" t="n">
-        <v>1416.09</v>
+        <v>1416.3</v>
       </c>
       <c r="Z10" t="n">
-        <v>1465.63</v>
+        <v>1465.83</v>
       </c>
       <c r="AA10" t="n">
-        <v>1402.79</v>
+        <v>1402.99</v>
       </c>
       <c r="AB10" t="n">
-        <v>1452.5</v>
+        <v>1452.57</v>
       </c>
       <c r="AC10" t="n">
-        <v>1461.5</v>
+        <v>1461.64</v>
       </c>
       <c r="AD10" t="n">
-        <v>1469</v>
+        <v>1469.07</v>
       </c>
       <c r="AE10" t="n">
         <v>55.4</v>
@@ -2069,7 +2069,7 @@
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (12.34) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (12.55) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH10" t="n">
@@ -2088,14 +2088,14 @@
         <v>15</v>
       </c>
       <c r="AM10" t="n">
-        <v>1488.11</v>
+        <v>1486.32</v>
       </c>
       <c r="AN10" t="n">
-        <v>1423.03</v>
+        <v>1423.91</v>
       </c>
       <c r="AO10" t="inlineStr">
         <is>
-          <t>CIPLA operates in the Healthcare sector. With an estimated Market Cap of ₹117,502.25 Cr., a P/E ratio of 35.20, and YoY Revenue Growth of +3.5%, the company demonstrates strong institutional backing, solid operating profit margins (12.01%), and healthy Return on Equity (15.00%).</t>
+          <t>CIPLA operates in the Healthcare sector. With an estimated Market Cap of ₹117,478.01 Cr., a P/E ratio of 35.19, and YoY Revenue Growth of +3.5%, the company demonstrates strong institutional backing, solid operating profit margins (12.01%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP10" t="inlineStr">
@@ -2105,22 +2105,22 @@
       </c>
       <c r="AQ10" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for CIPLA. Current Market Price (₹1,454.00) is positioned above the 30-day DMA (₹1,443.04), 50-day DMA (₹1,419.16), and 200-day DMA (₹1,394.98). The price distance from 200 DMA is +4.66%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for CIPLA. Current Market Price (₹1,454.20) is positioned above the 30-day DMA (₹1,443.04), 50-day DMA (₹1,419.16), and 200-day DMA (₹1,394.98). The price distance from 200 DMA is +4.66%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR10" t="inlineStr">
         <is>
-          <t>[1454.0, 1458.36, 1462.72, 1467.09, 1471.45, 1475.81]</t>
+          <t>[1454.2, 1458.56, 1462.93, 1467.29, 1471.65, 1476.01]</t>
         </is>
       </c>
       <c r="AS10" t="inlineStr">
         <is>
-          <t>[1454.0, 1472.02, 1482.04, 1490.74, 1498.76, 1506.35]</t>
+          <t>[1454.2, 1472.22, 1482.24, 1490.94, 1498.96, 1506.55]</t>
         </is>
       </c>
       <c r="AT10" t="inlineStr">
         <is>
-          <t>[1454.0, 1448.12, 1448.24, 1449.34, 1450.96, 1452.91]</t>
+          <t>[1454.2, 1448.32, 1448.44, 1449.55, 1451.16, 1453.11]</t>
         </is>
       </c>
     </row>
@@ -2141,7 +2141,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>146705.48</v>
+        <v>147121.83</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2149,15 +2149,15 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1656.2</v>
+        <v>1660.8</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>₹1647.09 - ₹1669.87</t>
+          <t>₹1651.69 - ₹1674.47</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>1692.66</v>
+        <v>1697.26</v>
       </c>
       <c r="I11" t="n">
         <v>1496.08</v>
@@ -2184,46 +2184,46 @@
         <v>45.57</v>
       </c>
       <c r="Q11" t="n">
-        <v>12.34</v>
+        <v>12.55</v>
       </c>
       <c r="R11" t="n">
-        <v>48.1</v>
+        <v>48.3</v>
       </c>
       <c r="S11" t="n">
         <v>0.19</v>
       </c>
       <c r="T11" t="n">
-        <v>-1.76</v>
+        <v>-1.74</v>
       </c>
       <c r="U11" t="n">
         <v>50</v>
       </c>
       <c r="V11" t="n">
-        <v>7.94</v>
+        <v>7.95</v>
       </c>
       <c r="W11" t="n">
         <v>-0.77</v>
       </c>
       <c r="X11" t="n">
-        <v>1627.4</v>
+        <v>1632.32</v>
       </c>
       <c r="Y11" t="n">
-        <v>1685.36</v>
+        <v>1690.45</v>
       </c>
       <c r="Z11" t="n">
-        <v>1669.45</v>
+        <v>1674.09</v>
       </c>
       <c r="AA11" t="n">
-        <v>1587.84</v>
+        <v>1592.44</v>
       </c>
       <c r="AB11" t="n">
-        <v>1656.23</v>
+        <v>1657.77</v>
       </c>
       <c r="AC11" t="n">
-        <v>1664.76</v>
+        <v>1667.84</v>
       </c>
       <c r="AD11" t="n">
-        <v>1673.33</v>
+        <v>1674.87</v>
       </c>
       <c r="AE11" t="n">
         <v>83.5</v>
@@ -2233,7 +2233,7 @@
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>Low VIX (12.34) | LSTM Deep Net</t>
+          <t>Low VIX (12.55) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH11" t="n">
@@ -2252,14 +2252,14 @@
         <v>15</v>
       </c>
       <c r="AM11" t="n">
-        <v>1704.65</v>
+        <v>1703.67</v>
       </c>
       <c r="AN11" t="n">
-        <v>1613.8</v>
+        <v>1616.56</v>
       </c>
       <c r="AO11" t="inlineStr">
         <is>
-          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹146,705.48 Cr., a P/E ratio of 28.65, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
+          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹147,121.83 Cr., a P/E ratio of 28.73, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP11" t="inlineStr">
@@ -2269,22 +2269,22 @@
       </c>
       <c r="AQ11" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,656.20) is positioned above the 30-day DMA (₹1,496.08), 50-day DMA (₹1,470.74), and 200-day DMA (₹1,461.21). The price distance from 200 DMA is +12.85%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,660.80) is positioned above the 30-day DMA (₹1,496.08), 50-day DMA (₹1,470.74), and 200-day DMA (₹1,461.21). The price distance from 200 DMA is +12.85%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR11" t="inlineStr">
         <is>
-          <t>[1656.2, 1661.17, 1666.14, 1671.11, 1676.07, 1681.04]</t>
+          <t>[1660.8, 1665.78, 1670.76, 1675.75, 1680.73, 1685.71]</t>
         </is>
       </c>
       <c r="AS11" t="inlineStr">
         <is>
-          <t>[1656.2, 1679.4, 1691.92, 1702.68, 1712.53, 1721.8]</t>
+          <t>[1660.8, 1684.01, 1696.54, 1707.32, 1717.19, 1726.47]</t>
         </is>
       </c>
       <c r="AT11" t="inlineStr">
         <is>
-          <t>[1656.2, 1647.5, 1646.8, 1647.43, 1648.73, 1650.47]</t>
+          <t>[1660.8, 1652.11, 1651.43, 1652.07, 1653.39, 1655.14]</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>78675.00999999999</v>
+        <v>78834.38</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2313,15 +2313,15 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1777.5</v>
+        <v>1780.9</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>₹1765.86 - ₹1794.96</t>
+          <t>₹1769.26 - ₹1798.36</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1824.05</v>
+        <v>1827.45</v>
       </c>
       <c r="I12" t="n">
         <v>1530.06</v>
@@ -2348,16 +2348,16 @@
         <v>58.19</v>
       </c>
       <c r="Q12" t="n">
-        <v>12.34</v>
+        <v>12.55</v>
       </c>
       <c r="R12" t="n">
-        <v>48.9</v>
+        <v>49.5</v>
       </c>
       <c r="S12" t="n">
-        <v>0.28</v>
+        <v>0.29</v>
       </c>
       <c r="T12" t="n">
-        <v>-1.84</v>
+        <v>-1.76</v>
       </c>
       <c r="U12" t="n">
         <v>50</v>
@@ -2369,25 +2369,25 @@
         <v>-0.77</v>
       </c>
       <c r="X12" t="n">
-        <v>1775.22</v>
+        <v>1779.76</v>
       </c>
       <c r="Y12" t="n">
-        <v>1837.43</v>
+        <v>1842.09</v>
       </c>
       <c r="Z12" t="n">
-        <v>1801.88</v>
+        <v>1806.47</v>
       </c>
       <c r="AA12" t="n">
-        <v>1690.21</v>
+        <v>1693.61</v>
       </c>
       <c r="AB12" t="n">
-        <v>1770.2</v>
+        <v>1771.33</v>
       </c>
       <c r="AC12" t="n">
-        <v>1795.3</v>
+        <v>1797.56</v>
       </c>
       <c r="AD12" t="n">
-        <v>1813.1</v>
+        <v>1814.23</v>
       </c>
       <c r="AE12" t="n">
         <v>72.90000000000001</v>
@@ -2397,14 +2397,14 @@
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH12" t="n">
         <v>0.15</v>
       </c>
       <c r="AI12" t="n">
-        <v>36.8</v>
+        <v>36.9</v>
       </c>
       <c r="AJ12" t="n">
         <v>49.9</v>
@@ -2416,14 +2416,14 @@
         <v>15</v>
       </c>
       <c r="AM12" t="n">
-        <v>1843.54</v>
+        <v>1850.92</v>
       </c>
       <c r="AN12" t="n">
-        <v>1711.42</v>
+        <v>1716.91</v>
       </c>
       <c r="AO12" t="inlineStr">
         <is>
-          <t>COFORGE operates in the Technology sector. With an estimated Market Cap of ₹78,675.01 Cr., a P/E ratio of 36.80, and YoY Revenue Growth of +49.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.64%), and healthy Return on Equity (15.00%).</t>
+          <t>COFORGE operates in the Technology sector. With an estimated Market Cap of ₹78,834.38 Cr., a P/E ratio of 36.87, and YoY Revenue Growth of +49.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP12" t="inlineStr">
@@ -2433,22 +2433,22 @@
       </c>
       <c r="AQ12" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for COFORGE. Current Market Price (₹1,777.50) is positioned above the 30-day DMA (₹1,530.06), 50-day DMA (₹1,489.66), and 200-day DMA (₹1,504.99). The price distance from 200 DMA is +16.27%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for COFORGE. Current Market Price (₹1,780.90) is positioned above the 30-day DMA (₹1,530.06), 50-day DMA (₹1,489.66), and 200-day DMA (₹1,504.99). The price distance from 200 DMA is +16.27%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR12" t="inlineStr">
         <is>
-          <t>[1777.5, 1801.88, 1826.26, 1850.64, 1875.02, 1899.4]</t>
+          <t>[1780.9, 1806.47, 1832.04, 1857.61, 1883.18, 1908.75]</t>
         </is>
       </c>
       <c r="AS12" t="inlineStr">
         <is>
-          <t>[1777.5, 1825.16, 1859.18, 1890.96, 1921.58, 1951.45]</t>
+          <t>[1780.9, 1829.75, 1864.96, 1897.93, 1929.73, 1960.8]</t>
         </is>
       </c>
       <c r="AT12" t="inlineStr">
         <is>
-          <t>[1777.5, 1784.42, 1801.57, 1820.4, 1840.1, 1860.36]</t>
+          <t>[1780.9, 1789.01, 1807.35, 1827.37, 1848.26, 1869.71]</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>48533.74</v>
+        <v>48460.5</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2477,15 +2477,15 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1192.8</v>
+        <v>1191</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>₹1186.01 - ₹1202.98</t>
+          <t>₹1184.21 - ₹1201.18</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>1219.95</v>
+        <v>1218.15</v>
       </c>
       <c r="I13" t="n">
         <v>1109.52</v>
@@ -2512,46 +2512,46 @@
         <v>33.94</v>
       </c>
       <c r="Q13" t="n">
-        <v>12.34</v>
+        <v>12.55</v>
       </c>
       <c r="R13" t="n">
-        <v>47.3</v>
+        <v>47.6</v>
       </c>
       <c r="S13" t="n">
         <v>0.19</v>
       </c>
       <c r="T13" t="n">
-        <v>-1.87</v>
+        <v>-1.86</v>
       </c>
       <c r="U13" t="n">
         <v>50</v>
       </c>
       <c r="V13" t="n">
-        <v>2.36</v>
+        <v>2.35</v>
       </c>
       <c r="W13" t="n">
         <v>-0.77</v>
       </c>
       <c r="X13" t="n">
-        <v>1176.91</v>
+        <v>1174.1</v>
       </c>
       <c r="Y13" t="n">
-        <v>1218.66</v>
+        <v>1215.78</v>
       </c>
       <c r="Z13" t="n">
-        <v>1202.34</v>
+        <v>1200.53</v>
       </c>
       <c r="AA13" t="n">
-        <v>1141.9</v>
+        <v>1140.1</v>
       </c>
       <c r="AB13" t="n">
-        <v>1183.6</v>
+        <v>1183</v>
       </c>
       <c r="AC13" t="n">
-        <v>1203.9</v>
+        <v>1202.7</v>
       </c>
       <c r="AD13" t="n">
-        <v>1215</v>
+        <v>1214.4</v>
       </c>
       <c r="AE13" t="n">
         <v>60.6</v>
@@ -2561,7 +2561,7 @@
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | TTM Squeeze | Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | TTM Squeeze | Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH13" t="n">
@@ -2580,14 +2580,14 @@
         <v>15</v>
       </c>
       <c r="AM13" t="n">
-        <v>1228.87</v>
+        <v>1231.07</v>
       </c>
       <c r="AN13" t="n">
-        <v>1158.42</v>
+        <v>1154.3</v>
       </c>
       <c r="AO13" t="inlineStr">
         <is>
-          <t>360ONE operates in the Financial Services sector. With an estimated Market Cap of ₹48,533.74 Cr., a P/E ratio of 39.64, and YoY Revenue Growth of +29.9%, the company demonstrates strong institutional backing, solid operating profit margins (26.46%), and healthy Return on Equity (15.00%).</t>
+          <t>360ONE operates in the Financial Services sector. With an estimated Market Cap of ₹48,460.50 Cr., a P/E ratio of 39.58, and YoY Revenue Growth of +29.9%, the company demonstrates strong institutional backing, solid operating profit margins (26.46%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP13" t="inlineStr">
@@ -2597,22 +2597,22 @@
       </c>
       <c r="AQ13" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for 360ONE. Current Market Price (₹1,192.80) is positioned above the 30-day DMA (₹1,109.52), 50-day DMA (₹1,105.91), and 200-day DMA (₹1,100.89). The price distance from 200 DMA is +4.26%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for 360ONE. Current Market Price (₹1,191.00) is positioned above the 30-day DMA (₹1,109.52), 50-day DMA (₹1,105.91), and 200-day DMA (₹1,100.89). The price distance from 200 DMA is +4.26%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR13" t="inlineStr">
         <is>
-          <t>[1192.8, 1196.38, 1199.96, 1203.54, 1207.11, 1210.69]</t>
+          <t>[1191.0, 1194.57, 1198.15, 1201.72, 1205.29, 1208.86]</t>
         </is>
       </c>
       <c r="AS13" t="inlineStr">
         <is>
-          <t>[1192.8, 1209.95, 1219.15, 1227.05, 1234.26, 1241.05]</t>
+          <t>[1191.0, 1208.15, 1217.34, 1225.23, 1232.44, 1239.22]</t>
         </is>
       </c>
       <c r="AT13" t="inlineStr">
         <is>
-          <t>[1192.8, 1186.2, 1185.56, 1185.9, 1186.75, 1187.93]</t>
+          <t>[1191.0, 1184.39, 1183.75, 1184.09, 1184.93, 1186.1]</t>
         </is>
       </c>
     </row>
@@ -2633,7 +2633,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>86916.31</v>
+        <v>87238.55</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2641,15 +2641,15 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>14295</v>
+        <v>14348</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>₹14201.1 - ₹14435.85</t>
+          <t>₹14254.1 - ₹14488.85</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>14670.6</v>
+        <v>14723.6</v>
       </c>
       <c r="I14" t="n">
         <v>13362.03</v>
@@ -2676,46 +2676,46 @@
         <v>469.5</v>
       </c>
       <c r="Q14" t="n">
-        <v>12.34</v>
+        <v>12.55</v>
       </c>
       <c r="R14" t="n">
-        <v>49.7</v>
+        <v>49.4</v>
       </c>
       <c r="S14" t="n">
         <v>0.16</v>
       </c>
       <c r="T14" t="n">
-        <v>-2.08</v>
+        <v>-2.09</v>
       </c>
       <c r="U14" t="n">
         <v>48.3</v>
       </c>
       <c r="V14" t="n">
-        <v>6.39</v>
+        <v>6.4</v>
       </c>
       <c r="W14" t="n">
         <v>-0.77</v>
       </c>
       <c r="X14" t="n">
-        <v>14185.38</v>
+        <v>14245.49</v>
       </c>
       <c r="Y14" t="n">
-        <v>14685.71</v>
+        <v>14747.67</v>
       </c>
       <c r="Z14" t="n">
-        <v>14409.36</v>
+        <v>14462.78</v>
       </c>
       <c r="AA14" t="n">
-        <v>13590.75</v>
+        <v>13643.75</v>
       </c>
       <c r="AB14" t="n">
-        <v>14228.33</v>
+        <v>14246</v>
       </c>
       <c r="AC14" t="n">
-        <v>14433.66</v>
+        <v>14469</v>
       </c>
       <c r="AD14" t="n">
-        <v>14572.33</v>
+        <v>14590</v>
       </c>
       <c r="AE14" t="n">
         <v>55.3</v>
@@ -2725,14 +2725,14 @@
       </c>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>Low VIX (12.34) | LSTM Deep Net</t>
+          <t>Low VIX (12.55) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH14" t="n">
         <v>0.15</v>
       </c>
       <c r="AI14" t="n">
-        <v>41.9</v>
+        <v>42</v>
       </c>
       <c r="AJ14" t="n">
         <v>21.1</v>
@@ -2744,14 +2744,14 @@
         <v>15</v>
       </c>
       <c r="AM14" t="n">
-        <v>14815.95</v>
+        <v>14900.38</v>
       </c>
       <c r="AN14" t="n">
-        <v>13766.25</v>
+        <v>13821.29</v>
       </c>
       <c r="AO14" t="inlineStr">
         <is>
-          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹86,916.31 Cr., a P/E ratio of 41.87, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
+          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹87,238.55 Cr., a P/E ratio of 42.03, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP14" t="inlineStr">
@@ -2761,22 +2761,22 @@
       </c>
       <c r="AQ14" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,295.00) is positioned above the 30-day DMA (₹13,362.03), 50-day DMA (₹12,739.88), and 200-day DMA (₹12,290.57). The price distance from 200 DMA is +13.81%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,348.00) is positioned above the 30-day DMA (₹13,362.03), 50-day DMA (₹12,739.88), and 200-day DMA (₹12,290.57). The price distance from 200 DMA is +13.81%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR14" t="inlineStr">
         <is>
-          <t>[14295.0, 14399.81, 14504.61, 14609.42, 14714.23, 14819.03]</t>
+          <t>[14348.0, 14460.71, 14573.42, 14686.13, 14798.85, 14911.56]</t>
         </is>
       </c>
       <c r="AS14" t="inlineStr">
         <is>
-          <t>[14295.0, 14587.61, 14770.2, 14934.7, 15089.83, 15238.97]</t>
+          <t>[14348.0, 14648.51, 14839.01, 15011.41, 15174.45, 15331.49]</t>
         </is>
       </c>
       <c r="AT14" t="inlineStr">
         <is>
-          <t>[14295.0, 14258.96, 14305.42, 14365.46, 14432.53, 14504.08]</t>
+          <t>[14348.0, 14319.86, 14374.23, 14442.18, 14517.15, 14596.61]</t>
         </is>
       </c>
     </row>
@@ -2788,159 +2788,159 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>GODREJPROP</t>
+          <t>PGEL</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>63739.41</v>
+        <v>17537.9</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>🔴 AVOID / HOLD</t>
+          <t>🟡 MODERATE BUY</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2116</v>
+        <v>612.15</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>₹2102.33 - ₹2136.51</t>
+          <t>₹607.86 - ₹618.59</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>2170.7</v>
+        <v>629.3200000000001</v>
       </c>
       <c r="I15" t="n">
-        <v>2028.46</v>
+        <v>583.11</v>
       </c>
       <c r="J15" t="n">
-        <v>1908.05</v>
+        <v>550.15</v>
       </c>
       <c r="K15" t="n">
-        <v>1880.26</v>
+        <v>554.14</v>
       </c>
       <c r="L15" t="n">
-        <v>8.16</v>
+        <v>10.44</v>
       </c>
       <c r="M15" t="n">
-        <v>46.13</v>
+        <v>15.39</v>
       </c>
       <c r="N15" t="n">
-        <v>60.86</v>
+        <v>15.91</v>
       </c>
       <c r="O15" t="n">
-        <v>-14.73</v>
+        <v>-0.52</v>
       </c>
       <c r="P15" t="n">
-        <v>68.37</v>
+        <v>21.46</v>
       </c>
       <c r="Q15" t="n">
-        <v>12.34</v>
+        <v>12.55</v>
       </c>
       <c r="R15" t="n">
-        <v>47.5</v>
+        <v>52.2</v>
       </c>
       <c r="S15" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="T15" t="n">
-        <v>-2.16</v>
+        <v>-2.1</v>
       </c>
       <c r="U15" t="n">
-        <v>51.7</v>
+        <v>55</v>
       </c>
       <c r="V15" t="n">
-        <v>6.25</v>
+        <v>4.79</v>
       </c>
       <c r="W15" t="n">
         <v>-0.77</v>
       </c>
       <c r="X15" t="n">
-        <v>2033.95</v>
+        <v>586.4</v>
       </c>
       <c r="Y15" t="n">
-        <v>2017.79</v>
+        <v>600.51</v>
       </c>
       <c r="Z15" t="n">
-        <v>2132.93</v>
+        <v>617.05</v>
       </c>
       <c r="AA15" t="n">
-        <v>2013.44</v>
+        <v>579.96</v>
       </c>
       <c r="AB15" t="n">
-        <v>2105.2</v>
+        <v>615.75</v>
       </c>
       <c r="AC15" t="n">
-        <v>2154.7</v>
+        <v>628.9</v>
       </c>
       <c r="AD15" t="n">
-        <v>2193.4</v>
+        <v>645.65</v>
       </c>
       <c r="AE15" t="n">
-        <v>43.7</v>
+        <v>54.7</v>
       </c>
       <c r="AF15" t="n">
-        <v>-0</v>
+        <v>0.06</v>
       </c>
       <c r="AG15" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (12.34) | LSTM Deep Net</t>
+          <t>Low VIX (12.55) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH15" t="n">
         <v>0.15</v>
       </c>
       <c r="AI15" t="n">
-        <v>35.4</v>
+        <v>88.3</v>
       </c>
       <c r="AJ15" t="n">
-        <v>63</v>
+        <v>-10.1</v>
       </c>
       <c r="AK15" t="n">
-        <v>36.1</v>
+        <v>3.7</v>
       </c>
       <c r="AL15" t="n">
-        <v>10</v>
+        <v>6.7</v>
       </c>
       <c r="AM15" t="n">
-        <v>2193.96</v>
+        <v>642.97</v>
       </c>
       <c r="AN15" t="n">
-        <v>2046.54</v>
+        <v>579.63</v>
       </c>
       <c r="AO15" t="inlineStr">
         <is>
-          <t>GODREJPROP operates in the Real Estate sector. With an estimated Market Cap of ₹63,739.41 Cr., a P/E ratio of 35.39, and YoY Revenue Growth of +63.0%, the company demonstrates strong institutional backing, solid operating profit margins (36.06%), and healthy Return on Equity (9.97%).</t>
+          <t>PGEL operates in the Technology sector. With an estimated Market Cap of ₹17,537.90 Cr., a P/E ratio of 88.33, and YoY Revenue Growth of -10.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.72%), and healthy Return on Equity (6.69%).</t>
         </is>
       </c>
       <c r="AP15" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 43.71 (Consolidation Zone), while MACD Line (46.13) trades below Signal (60.86) with an expanding histogram (-14.73). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +8.16% above the 200-day DMA (₹1880.26). Daily volatility envelope is bounded by ATR(14) of ₹68.37.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 54.70 (Consolidation Zone), while MACD Line (15.39) trades below Signal (15.91) with an expanding histogram (-0.52). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +10.44% above the 200-day DMA (₹554.14). Daily volatility envelope is bounded by ATR(14) of ₹21.46.</t>
         </is>
       </c>
       <c r="AQ15" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for GODREJPROP. Current Market Price (₹2,116.00) is positioned above the 30-day DMA (₹2,028.46), 50-day DMA (₹1,908.05), and 200-day DMA (₹1,880.26). The price distance from 200 DMA is +8.16%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PGEL. Current Market Price (₹612.15) is positioned above the 30-day DMA (₹583.11), 50-day DMA (₹550.15), and 200-day DMA (₹554.14). The price distance from 200 DMA is +10.44%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR15" t="inlineStr">
         <is>
-          <t>[2116.0, 2122.35, 2128.7, 2135.04, 2141.39, 2147.74]</t>
+          <t>[612.15, 613.99, 615.82, 617.66, 619.5, 621.33]</t>
         </is>
       </c>
       <c r="AS15" t="inlineStr">
         <is>
-          <t>[2116.0, 2149.7, 2167.37, 2182.42, 2196.09, 2208.9]</t>
+          <t>[612.15, 622.57, 627.96, 632.53, 636.66, 640.53]</t>
         </is>
       </c>
       <c r="AT15" t="inlineStr">
         <is>
-          <t>[2116.0, 2101.84, 2099.69, 2099.52, 2100.37, 2101.87]</t>
+          <t>[612.15, 607.55, 606.72, 606.51, 606.62, 606.94]</t>
         </is>
       </c>
     </row>
@@ -2961,7 +2961,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>11527.11</v>
+        <v>11540.45</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2969,15 +2969,15 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>129.62</v>
+        <v>129.77</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>₹128.75 - ₹130.93</t>
+          <t>₹128.9 - ₹131.08</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>133.11</v>
+        <v>133.26</v>
       </c>
       <c r="I16" t="n">
         <v>124.43</v>
@@ -3004,16 +3004,16 @@
         <v>4.36</v>
       </c>
       <c r="Q16" t="n">
-        <v>12.34</v>
+        <v>12.55</v>
       </c>
       <c r="R16" t="n">
-        <v>49.1</v>
+        <v>48.8</v>
       </c>
       <c r="S16" t="n">
         <v>0.16</v>
       </c>
       <c r="T16" t="n">
-        <v>-2.18</v>
+        <v>-2.19</v>
       </c>
       <c r="U16" t="n">
         <v>48.3</v>
@@ -3025,25 +3025,25 @@
         <v>-0.77</v>
       </c>
       <c r="X16" t="n">
-        <v>125</v>
+        <v>125.15</v>
       </c>
       <c r="Y16" t="n">
-        <v>129.54</v>
+        <v>129.7</v>
       </c>
       <c r="Z16" t="n">
-        <v>130.66</v>
+        <v>130.81</v>
       </c>
       <c r="AA16" t="n">
-        <v>123.07</v>
+        <v>123.22</v>
       </c>
       <c r="AB16" t="n">
-        <v>129.97</v>
+        <v>130.02</v>
       </c>
       <c r="AC16" t="n">
-        <v>130.59</v>
+        <v>130.69</v>
       </c>
       <c r="AD16" t="n">
-        <v>131.57</v>
+        <v>131.62</v>
       </c>
       <c r="AE16" t="n">
         <v>64.40000000000001</v>
@@ -3053,14 +3053,14 @@
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
+          <t>Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH16" t="n">
         <v>0.15</v>
       </c>
       <c r="AI16" t="n">
-        <v>22.5</v>
+        <v>22.6</v>
       </c>
       <c r="AJ16" t="n">
         <v>10.1</v>
@@ -3072,14 +3072,14 @@
         <v>15</v>
       </c>
       <c r="AM16" t="n">
-        <v>135.08</v>
+        <v>135.41</v>
       </c>
       <c r="AN16" t="n">
-        <v>123.93</v>
+        <v>123.5</v>
       </c>
       <c r="AO16" t="inlineStr">
         <is>
-          <t>IEX operates in the Financial Services sector. With an estimated Market Cap of ₹11,527.11 Cr., a P/E ratio of 22.54, and YoY Revenue Growth of +10.1%, the company demonstrates strong institutional backing, solid operating profit margins (66.22%), and healthy Return on Equity (15.00%).</t>
+          <t>IEX operates in the Financial Services sector. With an estimated Market Cap of ₹11,540.45 Cr., a P/E ratio of 22.57, and YoY Revenue Growth of +10.1%, the company demonstrates strong institutional backing, solid operating profit margins (66.22%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP16" t="inlineStr">
@@ -3089,22 +3089,22 @@
       </c>
       <c r="AQ16" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for IEX. Current Market Price (₹129.62) is positioned above the 30-day DMA (₹124.43), 50-day DMA (₹123.96), and 200-day DMA (₹127.99). The price distance from 200 DMA is +0.95%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for IEX. Current Market Price (₹129.77) is positioned above the 30-day DMA (₹124.43), 50-day DMA (₹123.96), and 200-day DMA (₹127.99). The price distance from 200 DMA is +0.95%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR16" t="inlineStr">
         <is>
-          <t>[129.62, 130.01, 130.4, 130.79, 131.18, 131.56]</t>
+          <t>[129.77, 130.16, 130.55, 130.94, 131.33, 131.72]</t>
         </is>
       </c>
       <c r="AS16" t="inlineStr">
         <is>
-          <t>[129.62, 131.75, 132.87, 133.81, 134.67, 135.47]</t>
+          <t>[129.77, 131.9, 133.02, 133.96, 134.82, 135.62]</t>
         </is>
       </c>
       <c r="AT16" t="inlineStr">
         <is>
-          <t>[129.62, 128.7, 128.55, 128.52, 128.56, 128.64]</t>
+          <t>[129.77, 128.85, 128.7, 128.67, 128.71, 128.79]</t>
         </is>
       </c>
     </row>
@@ -3116,16 +3116,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>GODREJPROP</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>285965.55</v>
+        <v>63902.07</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3133,142 +3133,142 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>310.7</v>
+        <v>2121.4</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>₹308.63 - ₹313.81</t>
+          <t>₹2107.72 - ₹2141.91</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>318.98</v>
+        <v>2176.1</v>
       </c>
       <c r="I17" t="n">
-        <v>286.32</v>
+        <v>2028.46</v>
       </c>
       <c r="J17" t="n">
-        <v>272.64</v>
+        <v>1908.05</v>
       </c>
       <c r="K17" t="n">
-        <v>273.39</v>
+        <v>1880.26</v>
       </c>
       <c r="L17" t="n">
-        <v>14.27</v>
+        <v>8.16</v>
       </c>
       <c r="M17" t="n">
-        <v>10.44</v>
+        <v>46.13</v>
       </c>
       <c r="N17" t="n">
-        <v>9.26</v>
+        <v>60.86</v>
       </c>
       <c r="O17" t="n">
-        <v>1.18</v>
+        <v>-14.73</v>
       </c>
       <c r="P17" t="n">
-        <v>10.35</v>
+        <v>68.37</v>
       </c>
       <c r="Q17" t="n">
-        <v>12.34</v>
+        <v>12.55</v>
       </c>
       <c r="R17" t="n">
-        <v>45.6</v>
+        <v>46.9</v>
       </c>
       <c r="S17" t="n">
-        <v>0.16</v>
+        <v>0.17</v>
       </c>
       <c r="T17" t="n">
-        <v>-2.35</v>
+        <v>-2.19</v>
       </c>
       <c r="U17" t="n">
-        <v>53.3</v>
+        <v>51.7</v>
       </c>
       <c r="V17" t="n">
-        <v>2.43</v>
+        <v>6.27</v>
       </c>
       <c r="W17" t="n">
         <v>-0.77</v>
       </c>
       <c r="X17" t="n">
-        <v>306.18</v>
+        <v>2039.35</v>
       </c>
       <c r="Y17" t="n">
-        <v>317.06</v>
+        <v>2024.27</v>
       </c>
       <c r="Z17" t="n">
-        <v>313.19</v>
+        <v>2138.37</v>
       </c>
       <c r="AA17" t="n">
-        <v>295.18</v>
+        <v>2018.84</v>
       </c>
       <c r="AB17" t="n">
-        <v>311.87</v>
+        <v>2107</v>
       </c>
       <c r="AC17" t="n">
-        <v>313.49</v>
+        <v>2158.3</v>
       </c>
       <c r="AD17" t="n">
-        <v>316.27</v>
+        <v>2195.2</v>
       </c>
       <c r="AE17" t="n">
-        <v>62.2</v>
+        <v>43.7</v>
       </c>
       <c r="AF17" t="n">
-        <v>0.1</v>
+        <v>-0</v>
       </c>
       <c r="AG17" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.34) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (12.55) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH17" t="n">
         <v>0.15</v>
       </c>
       <c r="AI17" t="n">
-        <v>661</v>
+        <v>35.5</v>
       </c>
       <c r="AJ17" t="n">
-        <v>182</v>
+        <v>63</v>
       </c>
       <c r="AK17" t="n">
-        <v>0.6</v>
+        <v>36.1</v>
       </c>
       <c r="AL17" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="AM17" t="n">
-        <v>321.59</v>
+        <v>2194.1</v>
       </c>
       <c r="AN17" t="n">
-        <v>299.8</v>
+        <v>2049.1</v>
       </c>
       <c r="AO17" t="inlineStr">
         <is>
-          <t>ETERNAL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹285,965.55 Cr., a P/E ratio of 660.96, and YoY Revenue Growth of +182.0%, the company demonstrates strong institutional backing, solid operating profit margins (0.64%), and healthy Return on Equity (15.00%).</t>
+          <t>GODREJPROP operates in the Real Estate sector. With an estimated Market Cap of ₹63,902.07 Cr., a P/E ratio of 35.48, and YoY Revenue Growth of +63.0%, the company demonstrates strong institutional backing, solid operating profit margins (36.06%), and healthy Return on Equity (9.97%).</t>
         </is>
       </c>
       <c r="AP17" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 62.17 (Bullish Momentum Zone), while MACD Line (10.44) trades above Signal (9.26) with an expanding histogram (+1.18). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +14.27% above the 200-day DMA (₹273.39). Daily volatility envelope is bounded by ATR(14) of ₹10.35.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 43.71 (Consolidation Zone), while MACD Line (46.13) trades below Signal (60.86) with an expanding histogram (-14.73). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +8.16% above the 200-day DMA (₹1880.26). Daily volatility envelope is bounded by ATR(14) of ₹68.37.</t>
         </is>
       </c>
       <c r="AQ17" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ETERNAL. Current Market Price (₹310.70) is positioned above the 30-day DMA (₹286.32), 50-day DMA (₹272.64), and 200-day DMA (₹273.39). The price distance from 200 DMA is +14.27%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for GODREJPROP. Current Market Price (₹2,121.40) is positioned above the 30-day DMA (₹2,028.46), 50-day DMA (₹1,908.05), and 200-day DMA (₹1,880.26). The price distance from 200 DMA is +8.16%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR17" t="inlineStr">
         <is>
-          <t>[310.7, 311.63, 312.56, 313.5, 314.43, 315.36]</t>
+          <t>[2121.4, 2127.76, 2134.13, 2140.49, 2146.86, 2153.22]</t>
         </is>
       </c>
       <c r="AS17" t="inlineStr">
         <is>
-          <t>[310.7, 315.77, 318.42, 320.67, 322.71, 324.62]</t>
+          <t>[2121.4, 2155.11, 2172.81, 2187.86, 2201.56, 2214.38]</t>
         </is>
       </c>
       <c r="AT17" t="inlineStr">
         <is>
-          <t>[310.7, 308.53, 308.17, 308.12, 308.22, 308.42]</t>
+          <t>[2121.4, 2107.25, 2105.12, 2104.96, 2105.83, 2107.35]</t>
         </is>
       </c>
     </row>
@@ -3280,16 +3280,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PGEL</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>17441.92</v>
+        <v>286425.82</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3297,142 +3297,142 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>608.1</v>
+        <v>311.35</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>₹603.81 - ₹614.54</t>
+          <t>₹309.28 - ₹314.46</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>625.27</v>
+        <v>319.63</v>
       </c>
       <c r="I18" t="n">
-        <v>583.11</v>
+        <v>286.32</v>
       </c>
       <c r="J18" t="n">
-        <v>550.15</v>
+        <v>272.64</v>
       </c>
       <c r="K18" t="n">
-        <v>554.14</v>
+        <v>273.39</v>
       </c>
       <c r="L18" t="n">
+        <v>14.27</v>
+      </c>
+      <c r="M18" t="n">
         <v>10.44</v>
       </c>
-      <c r="M18" t="n">
-        <v>15.39</v>
-      </c>
       <c r="N18" t="n">
-        <v>15.91</v>
+        <v>9.26</v>
       </c>
       <c r="O18" t="n">
-        <v>-0.52</v>
+        <v>1.18</v>
       </c>
       <c r="P18" t="n">
-        <v>21.46</v>
+        <v>10.35</v>
       </c>
       <c r="Q18" t="n">
-        <v>12.34</v>
+        <v>12.55</v>
       </c>
       <c r="R18" t="n">
-        <v>47.5</v>
+        <v>46.1</v>
       </c>
       <c r="S18" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="T18" t="n">
-        <v>-2.4</v>
+        <v>-2.32</v>
       </c>
       <c r="U18" t="n">
         <v>53.3</v>
       </c>
       <c r="V18" t="n">
-        <v>4.78</v>
+        <v>2.43</v>
       </c>
       <c r="W18" t="n">
         <v>-0.77</v>
       </c>
       <c r="X18" t="n">
-        <v>582.35</v>
+        <v>306.87</v>
       </c>
       <c r="Y18" t="n">
-        <v>595.73</v>
+        <v>317.77</v>
       </c>
       <c r="Z18" t="n">
-        <v>612.96</v>
+        <v>313.84</v>
       </c>
       <c r="AA18" t="n">
-        <v>575.91</v>
+        <v>295.82</v>
       </c>
       <c r="AB18" t="n">
-        <v>614.4</v>
+        <v>312.08</v>
       </c>
       <c r="AC18" t="n">
-        <v>626.2</v>
+        <v>313.91</v>
       </c>
       <c r="AD18" t="n">
-        <v>644.3</v>
+        <v>316.48</v>
       </c>
       <c r="AE18" t="n">
-        <v>54.7</v>
+        <v>62.2</v>
       </c>
       <c r="AF18" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="AG18" t="inlineStr">
         <is>
-          <t>Low VIX (12.34) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH18" t="n">
         <v>0.15</v>
       </c>
       <c r="AI18" t="n">
-        <v>87.8</v>
+        <v>662</v>
       </c>
       <c r="AJ18" t="n">
-        <v>-10.1</v>
+        <v>182</v>
       </c>
       <c r="AK18" t="n">
-        <v>3.7</v>
+        <v>0.6</v>
       </c>
       <c r="AL18" t="n">
-        <v>6.7</v>
+        <v>15</v>
       </c>
       <c r="AM18" t="n">
-        <v>636.6799999999999</v>
+        <v>323.19</v>
       </c>
       <c r="AN18" t="n">
-        <v>576.48</v>
+        <v>300.17</v>
       </c>
       <c r="AO18" t="inlineStr">
         <is>
-          <t>PGEL operates in the Technology sector. With an estimated Market Cap of ₹17,441.92 Cr., a P/E ratio of 87.85, and YoY Revenue Growth of -10.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.72%), and healthy Return on Equity (6.69%).</t>
+          <t>ETERNAL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹286,425.82 Cr., a P/E ratio of 662.02, and YoY Revenue Growth of +182.0%, the company demonstrates strong institutional backing, solid operating profit margins (0.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP18" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 54.70 (Consolidation Zone), while MACD Line (15.39) trades below Signal (15.91) with an expanding histogram (-0.52). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +10.44% above the 200-day DMA (₹554.14). Daily volatility envelope is bounded by ATR(14) of ₹21.46.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 62.17 (Bullish Momentum Zone), while MACD Line (10.44) trades above Signal (9.26) with an expanding histogram (+1.18). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +14.27% above the 200-day DMA (₹273.39). Daily volatility envelope is bounded by ATR(14) of ₹10.35.</t>
         </is>
       </c>
       <c r="AQ18" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PGEL. Current Market Price (₹608.10) is positioned above the 30-day DMA (₹583.11), 50-day DMA (₹550.15), and 200-day DMA (₹554.14). The price distance from 200 DMA is +10.44%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ETERNAL. Current Market Price (₹311.35) is positioned above the 30-day DMA (₹286.32), 50-day DMA (₹272.64), and 200-day DMA (₹273.39). The price distance from 200 DMA is +14.27%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR18" t="inlineStr">
         <is>
-          <t>[608.1, 609.92, 611.75, 613.57, 615.4, 617.22]</t>
+          <t>[311.35, 312.28, 313.22, 314.15, 315.09, 316.02]</t>
         </is>
       </c>
       <c r="AS18" t="inlineStr">
         <is>
-          <t>[608.1, 618.51, 623.89, 628.44, 632.57, 636.42]</t>
+          <t>[311.35, 316.42, 319.07, 321.32, 323.37, 325.28]</t>
         </is>
       </c>
       <c r="AT18" t="inlineStr">
         <is>
-          <t>[608.1, 603.49, 602.64, 602.42, 602.52, 602.83]</t>
+          <t>[311.35, 309.18, 308.83, 308.77, 308.88, 309.08]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implement Futures Post-Market Analysis, cumulative multi-book validation reports, and autonomous ML model feedback loop
</commit_message>
<xml_diff>
--- a/Breakout_ML_Quant_Predictions.xlsx
+++ b/Breakout_ML_Quant_Predictions.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT18"/>
+  <dimension ref="A1:AU18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -647,6 +647,11 @@
           <t>Forecast_5D_Low</t>
         </is>
       </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>Next_Day_Expected_Close</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -665,7 +670,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>357563.18</v>
+        <v>358592.78</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -673,15 +678,15 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>12155</v>
+        <v>12190</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>₹12114.59 - ₹12215.61</t>
+          <t>₹12149.59 - ₹12250.61</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>12316.62</v>
+        <v>12351.62</v>
       </c>
       <c r="I2" t="n">
         <v>11508.32</v>
@@ -708,16 +713,16 @@
         <v>202.03</v>
       </c>
       <c r="Q2" t="n">
-        <v>12.55</v>
+        <v>12.06</v>
       </c>
       <c r="R2" t="n">
-        <v>50.3</v>
+        <v>53</v>
       </c>
       <c r="S2" t="n">
         <v>0.32</v>
       </c>
       <c r="T2" t="n">
-        <v>-0.84</v>
+        <v>-0.83</v>
       </c>
       <c r="U2" t="n">
         <v>50</v>
@@ -729,25 +734,25 @@
         <v>-0.77</v>
       </c>
       <c r="X2" t="n">
-        <v>12060.74</v>
+        <v>12190</v>
       </c>
       <c r="Y2" t="n">
-        <v>12458.04</v>
+        <v>12390.22</v>
       </c>
       <c r="Z2" t="n">
-        <v>12252.24</v>
+        <v>12225.1</v>
       </c>
       <c r="AA2" t="n">
-        <v>11851.96</v>
+        <v>11886.96</v>
       </c>
       <c r="AB2" t="n">
-        <v>12121.33</v>
+        <v>12133</v>
       </c>
       <c r="AC2" t="n">
-        <v>12272.66</v>
+        <v>12296</v>
       </c>
       <c r="AD2" t="n">
-        <v>12390.33</v>
+        <v>12402</v>
       </c>
       <c r="AE2" t="n">
         <v>70.40000000000001</v>
@@ -757,14 +762,14 @@
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.06) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH2" t="n">
         <v>0.15</v>
       </c>
       <c r="AI2" t="n">
-        <v>41.9</v>
+        <v>42</v>
       </c>
       <c r="AJ2" t="n">
         <v>15.9</v>
@@ -776,14 +781,14 @@
         <v>15</v>
       </c>
       <c r="AM2" t="n">
-        <v>12431.71</v>
+        <v>12464.15</v>
       </c>
       <c r="AN2" t="n">
-        <v>11884.91</v>
+        <v>11916.26</v>
       </c>
       <c r="AO2" t="inlineStr">
         <is>
-          <t>ULTRACEMCO operates in the Basic Materials sector. With an estimated Market Cap of ₹357,563.18 Cr., a P/E ratio of 41.85, and YoY Revenue Growth of +15.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.29%), and healthy Return on Equity (15.00%).</t>
+          <t>ULTRACEMCO operates in the Basic Materials sector. With an estimated Market Cap of ₹358,592.78 Cr., a P/E ratio of 41.98, and YoY Revenue Growth of +15.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.29%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP2" t="inlineStr">
@@ -793,23 +798,26 @@
       </c>
       <c r="AQ2" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ULTRACEMCO. Current Market Price (₹12,155.00) is positioned above the 30-day DMA (₹11,508.32), 50-day DMA (₹11,305.61), and 200-day DMA (₹11,570.61). The price distance from 200 DMA is +4.14%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ULTRACEMCO. Current Market Price (₹12,190.00) is positioned above the 30-day DMA (₹11,508.32), 50-day DMA (₹11,305.61), and 200-day DMA (₹11,570.61). The price distance from 200 DMA is +4.14%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR2" t="inlineStr">
         <is>
-          <t>[12155.0, 12243.07, 12331.14, 12419.2, 12507.27, 12595.34]</t>
+          <t>[12190.0, 12282.19, 12374.39, 12466.58, 12558.78, 12650.97]</t>
         </is>
       </c>
       <c r="AS2" t="inlineStr">
         <is>
-          <t>[12155.0, 12323.88, 12445.42, 12559.17, 12668.89, 12776.04]</t>
+          <t>[12190.0, 12363.0, 12488.67, 12606.55, 12720.4, 12831.67]</t>
         </is>
       </c>
       <c r="AT2" t="inlineStr">
         <is>
-          <t>[12155.0, 12182.46, 12245.42, 12314.23, 12386.06, 12459.82]</t>
-        </is>
+          <t>[12190.0, 12221.59, 12288.68, 12361.61, 12437.56, 12515.45]</t>
+        </is>
+      </c>
+      <c r="AU2" t="n">
+        <v>12225.1</v>
       </c>
     </row>
     <row r="3">
@@ -829,7 +837,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>130674.76</v>
+        <v>130502.37</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -837,15 +845,15 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>113.7</v>
+        <v>113.55</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>₹113.31 - ₹114.29</t>
+          <t>₹113.16 - ₹114.14</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>115.26</v>
+        <v>115.11</v>
       </c>
       <c r="I3" t="n">
         <v>108.12</v>
@@ -872,16 +880,16 @@
         <v>1.95</v>
       </c>
       <c r="Q3" t="n">
-        <v>12.55</v>
+        <v>12.06</v>
       </c>
       <c r="R3" t="n">
-        <v>48.9</v>
+        <v>51.8</v>
       </c>
       <c r="S3" t="n">
         <v>0.31</v>
       </c>
       <c r="T3" t="n">
-        <v>-0.92</v>
+        <v>-0.91</v>
       </c>
       <c r="U3" t="n">
         <v>55</v>
@@ -893,25 +901,25 @@
         <v>-0.77</v>
       </c>
       <c r="X3" t="n">
-        <v>111.36</v>
+        <v>112.1</v>
       </c>
       <c r="Y3" t="n">
-        <v>114.77</v>
+        <v>113.67</v>
       </c>
       <c r="Z3" t="n">
-        <v>114.61</v>
+        <v>113.4</v>
       </c>
       <c r="AA3" t="n">
-        <v>110.77</v>
+        <v>110.62</v>
       </c>
       <c r="AB3" t="n">
-        <v>114.16</v>
+        <v>114.02</v>
       </c>
       <c r="AC3" t="n">
-        <v>114.73</v>
+        <v>114.74</v>
       </c>
       <c r="AD3" t="n">
-        <v>115.77</v>
+        <v>115.92</v>
       </c>
       <c r="AE3" t="n">
         <v>79</v>
@@ -921,7 +929,7 @@
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Low VIX (12.55) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Low VIX (12.06) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH3" t="n">
@@ -940,14 +948,14 @@
         <v>15</v>
       </c>
       <c r="AM3" t="n">
-        <v>117.02</v>
+        <v>116.66</v>
       </c>
       <c r="AN3" t="n">
-        <v>110.4</v>
+        <v>110.59</v>
       </c>
       <c r="AO3" t="inlineStr">
         <is>
-          <t>PNB operates in the Financial Services sector. With an estimated Market Cap of ₹130,674.76 Cr., a P/E ratio of 5.86, and YoY Revenue Growth of +15.2%, the company demonstrates strong institutional backing, solid operating profit margins (38.15%), and healthy Return on Equity (14.97%).</t>
+          <t>PNB operates in the Financial Services sector. With an estimated Market Cap of ₹130,502.37 Cr., a P/E ratio of 5.86, and YoY Revenue Growth of +15.2%, the company demonstrates strong institutional backing, solid operating profit margins (38.15%), and healthy Return on Equity (14.97%).</t>
         </is>
       </c>
       <c r="AP3" t="inlineStr">
@@ -957,23 +965,26 @@
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PNB. Current Market Price (₹113.70) is positioned above the 30-day DMA (₹108.12), 50-day DMA (₹106.98), and 200-day DMA (₹112.64). The price distance from 200 DMA is +1.20%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PNB. Current Market Price (₹113.55) is positioned above the 30-day DMA (₹108.12), 50-day DMA (₹106.98), and 200-day DMA (₹112.64). The price distance from 200 DMA is +1.20%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR3" t="inlineStr">
         <is>
-          <t>[113.7, 114.04, 114.38, 114.72, 115.06, 115.41]</t>
+          <t>[113.55, 113.89, 114.23, 114.57, 114.91, 115.25]</t>
         </is>
       </c>
       <c r="AS3" t="inlineStr">
         <is>
-          <t>[113.7, 114.82, 115.49, 116.08, 116.63, 117.15]</t>
+          <t>[113.55, 114.67, 115.34, 115.92, 116.47, 117.0]</t>
         </is>
       </c>
       <c r="AT3" t="inlineStr">
         <is>
-          <t>[113.7, 113.46, 113.55, 113.71, 113.89, 114.1]</t>
-        </is>
+          <t>[113.55, 113.31, 113.4, 113.56, 113.74, 113.94]</t>
+        </is>
+      </c>
+      <c r="AU3" t="n">
+        <v>113.4</v>
       </c>
     </row>
     <row r="4">
@@ -984,16 +995,16 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>ALKEM</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>219891.88</v>
+        <v>68110.2</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -1001,143 +1012,146 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>8010</v>
+        <v>5696.5</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>₹7978.64 - ₹8057.04</t>
+          <t>₹5673.6 - ₹5730.85</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>8135.45</v>
+        <v>5788.1</v>
       </c>
       <c r="I4" t="n">
-        <v>7478.7</v>
+        <v>5605.35</v>
       </c>
       <c r="J4" t="n">
-        <v>7389.91</v>
+        <v>5501.71</v>
       </c>
       <c r="K4" t="n">
-        <v>7187.9</v>
+        <v>5524.85</v>
       </c>
       <c r="L4" t="n">
-        <v>10.39</v>
+        <v>1.51</v>
       </c>
       <c r="M4" t="n">
-        <v>160.7</v>
+        <v>48.94</v>
       </c>
       <c r="N4" t="n">
-        <v>116.95</v>
+        <v>53.54</v>
       </c>
       <c r="O4" t="n">
-        <v>43.75</v>
+        <v>-4.6</v>
       </c>
       <c r="P4" t="n">
-        <v>156.81</v>
+        <v>114.5</v>
       </c>
       <c r="Q4" t="n">
-        <v>12.55</v>
+        <v>12.06</v>
       </c>
       <c r="R4" t="n">
-        <v>51.2</v>
+        <v>55.4</v>
       </c>
       <c r="S4" t="n">
         <v>0.27</v>
       </c>
       <c r="T4" t="n">
-        <v>-1.02</v>
+        <v>-1</v>
       </c>
       <c r="U4" t="n">
-        <v>51.7</v>
+        <v>53.3</v>
       </c>
       <c r="V4" t="n">
-        <v>2.09</v>
+        <v>2.84</v>
       </c>
       <c r="W4" t="n">
         <v>-0.77</v>
       </c>
       <c r="X4" t="n">
-        <v>7887.48</v>
+        <v>5603.74</v>
       </c>
       <c r="Y4" t="n">
-        <v>8167.83</v>
+        <v>5753.04</v>
       </c>
       <c r="Z4" t="n">
-        <v>8074.08</v>
+        <v>5753.04</v>
       </c>
       <c r="AA4" t="n">
-        <v>7774.78</v>
+        <v>5524.75</v>
       </c>
       <c r="AB4" t="n">
-        <v>7977.83</v>
+        <v>5649.67</v>
       </c>
       <c r="AC4" t="n">
-        <v>8050.16</v>
+        <v>5743.34</v>
       </c>
       <c r="AD4" t="n">
-        <v>8090.33</v>
+        <v>5790.17</v>
       </c>
       <c r="AE4" t="n">
-        <v>74.3</v>
+        <v>47.1</v>
       </c>
       <c r="AF4" t="n">
-        <v>0.21</v>
+        <v>-0.04</v>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (12.06) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH4" t="n">
         <v>0.15</v>
       </c>
       <c r="AI4" t="n">
-        <v>38.7</v>
+        <v>30.1</v>
       </c>
       <c r="AJ4" t="n">
-        <v>31.5</v>
+        <v>14.6</v>
       </c>
       <c r="AK4" t="n">
-        <v>23.2</v>
+        <v>15.6</v>
       </c>
       <c r="AL4" t="n">
-        <v>15</v>
+        <v>17.6</v>
       </c>
       <c r="AM4" t="n">
-        <v>8235.690000000001</v>
+        <v>5820.72</v>
       </c>
       <c r="AN4" t="n">
-        <v>7798.99</v>
+        <v>5567.02</v>
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>EICHERMOT operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹219,891.88 Cr., a P/E ratio of 38.68, and YoY Revenue Growth of +31.5%, the company demonstrates strong institutional backing, solid operating profit margins (23.21%), and healthy Return on Equity (15.00%).</t>
+          <t>ALKEM operates in the Healthcare sector. With an estimated Market Cap of ₹68,110.20 Cr., a P/E ratio of 30.14, and YoY Revenue Growth of +14.6%, the company demonstrates strong institutional backing, solid operating profit margins (15.65%), and healthy Return on Equity (17.56%).</t>
         </is>
       </c>
       <c r="AP4" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 74.31 (Bullish Momentum Zone), while MACD Line (160.70) trades above Signal (116.95) with an expanding histogram (+43.75). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +10.39% above the 200-day DMA (₹7187.90). Daily volatility envelope is bounded by ATR(14) of ₹156.81.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 47.14 (Consolidation Zone), while MACD Line (48.94) trades below Signal (53.54) with an expanding histogram (-4.60). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +1.51% above the 200-day DMA (₹5524.85). Daily volatility envelope is bounded by ATR(14) of ₹114.50.</t>
         </is>
       </c>
       <c r="AQ4" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for EICHERMOT. Current Market Price (₹8,010.00) is positioned above the 30-day DMA (₹7,478.70), 50-day DMA (₹7,389.91), and 200-day DMA (₹7,187.90). The price distance from 200 DMA is +10.39%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ALKEM. Current Market Price (₹5,696.50) is positioned above the 30-day DMA (₹5,605.35), 50-day DMA (₹5,501.71), and 200-day DMA (₹5,524.85). The price distance from 200 DMA is +1.51%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR4" t="inlineStr">
         <is>
-          <t>[8010.0, 8034.03, 8058.06, 8082.09, 8106.12, 8130.15]</t>
+          <t>[5696.5, 5713.59, 5730.68, 5747.77, 5764.86, 5781.95]</t>
         </is>
       </c>
       <c r="AS4" t="inlineStr">
         <is>
-          <t>[8010.0, 8096.75, 8146.77, 8190.73, 8231.57, 8270.41]</t>
+          <t>[5696.5, 5759.39, 5795.45, 5827.1, 5856.46, 5884.36]</t>
         </is>
       </c>
       <c r="AT4" t="inlineStr">
         <is>
-          <t>[8010.0, 7986.99, 7991.53, 8000.61, 8012.03, 8024.96]</t>
-        </is>
+          <t>[5696.5, 5679.24, 5682.1, 5688.27, 5696.16, 5705.14]</t>
+        </is>
+      </c>
+      <c r="AU4" t="n">
+        <v>5753.04</v>
       </c>
     </row>
     <row r="5">
@@ -1148,160 +1162,163 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>HAL</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>309709.69</v>
+        <v>219246.76</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>🔴 AVOID / HOLD</t>
+          <t>🟡 MODERATE BUY</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>4631</v>
+        <v>7986.5</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>₹4614.96 - ₹4655.06</t>
+          <t>₹7955.14 - ₹8033.54</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>4695.15</v>
+        <v>8111.95</v>
       </c>
       <c r="I5" t="n">
-        <v>4490.17</v>
+        <v>7478.7</v>
       </c>
       <c r="J5" t="n">
-        <v>4419.22</v>
+        <v>7389.91</v>
       </c>
       <c r="K5" t="n">
-        <v>4344.79</v>
+        <v>7187.9</v>
       </c>
       <c r="L5" t="n">
-        <v>6.68</v>
+        <v>10.39</v>
       </c>
       <c r="M5" t="n">
-        <v>64.29000000000001</v>
+        <v>160.7</v>
       </c>
       <c r="N5" t="n">
-        <v>56.51</v>
+        <v>116.95</v>
       </c>
       <c r="O5" t="n">
-        <v>7.78</v>
+        <v>43.75</v>
       </c>
       <c r="P5" t="n">
-        <v>80.19</v>
+        <v>156.81</v>
       </c>
       <c r="Q5" t="n">
-        <v>12.55</v>
+        <v>12.06</v>
       </c>
       <c r="R5" t="n">
-        <v>40.6</v>
+        <v>51.1</v>
       </c>
       <c r="S5" t="n">
-        <v>0.31</v>
+        <v>0.27</v>
       </c>
       <c r="T5" t="n">
-        <v>-1.22</v>
+        <v>-1.03</v>
       </c>
       <c r="U5" t="n">
-        <v>41.7</v>
+        <v>51.7</v>
       </c>
       <c r="V5" t="n">
-        <v>2.34</v>
+        <v>2.08</v>
       </c>
       <c r="W5" t="n">
         <v>-0.77</v>
       </c>
       <c r="X5" t="n">
-        <v>4534.78</v>
+        <v>7927.02</v>
       </c>
       <c r="Y5" t="n">
-        <v>4670.81</v>
+        <v>8076.38</v>
       </c>
       <c r="Z5" t="n">
-        <v>4668.05</v>
+        <v>7963.04</v>
       </c>
       <c r="AA5" t="n">
-        <v>4510.72</v>
+        <v>7751.28</v>
       </c>
       <c r="AB5" t="n">
-        <v>4635.9</v>
+        <v>7970.33</v>
       </c>
       <c r="AC5" t="n">
-        <v>4668.5</v>
+        <v>8035.16</v>
       </c>
       <c r="AD5" t="n">
-        <v>4706</v>
+        <v>8083.83</v>
       </c>
       <c r="AE5" t="n">
-        <v>72.8</v>
+        <v>74.3</v>
       </c>
       <c r="AF5" t="n">
-        <v>0.27</v>
+        <v>0.21</v>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.06) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH5" t="n">
         <v>0.15</v>
       </c>
       <c r="AI5" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="AJ5" t="n">
-        <v>1.8</v>
+        <v>31.5</v>
       </c>
       <c r="AK5" t="n">
-        <v>27.5</v>
+        <v>23.2</v>
       </c>
       <c r="AL5" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="AM5" t="n">
-        <v>4757.33</v>
+        <v>8198.02</v>
       </c>
       <c r="AN5" t="n">
-        <v>4494.93</v>
+        <v>7783.85</v>
       </c>
       <c r="AO5" t="inlineStr">
         <is>
-          <t>HAL operates in the Industrials sector. With an estimated Market Cap of ₹309,709.69 Cr., a P/E ratio of 34.02, and YoY Revenue Growth of +1.8%, the company demonstrates strong institutional backing, solid operating profit margins (27.55%), and healthy Return on Equity (23.98%).</t>
+          <t>EICHERMOT operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹219,246.76 Cr., a P/E ratio of 37.02, and YoY Revenue Growth of +31.5%, the company demonstrates strong institutional backing, solid operating profit margins (23.21%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP5" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 72.77 (Bullish Momentum Zone), while MACD Line (64.29) trades above Signal (56.51) with an expanding histogram (+7.78). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +6.68% above the 200-day DMA (₹4344.79). Daily volatility envelope is bounded by ATR(14) of ₹80.19.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 74.31 (Bullish Momentum Zone), while MACD Line (160.70) trades above Signal (116.95) with an expanding histogram (+43.75). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +10.39% above the 200-day DMA (₹7187.90). Daily volatility envelope is bounded by ATR(14) of ₹156.81.</t>
         </is>
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for HAL. Current Market Price (₹4,631.00) is positioned above the 30-day DMA (₹4,490.17), 50-day DMA (₹4,419.22), and 200-day DMA (₹4,344.79). The price distance from 200 DMA is +6.68%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for EICHERMOT. Current Market Price (₹7,986.50) is positioned above the 30-day DMA (₹7,478.70), 50-day DMA (₹7,389.91), and 200-day DMA (₹7,187.90). The price distance from 200 DMA is +10.39%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>[4631.0, 4644.89, 4658.79, 4672.68, 4686.57, 4700.46]</t>
+          <t>[7986.5, 8010.46, 8034.42, 8058.38, 8082.34, 8106.3]</t>
         </is>
       </c>
       <c r="AS5" t="inlineStr">
         <is>
-          <t>[4631.0, 4676.97, 4704.15, 4728.23, 4750.72, 4772.19]</t>
+          <t>[7986.5, 8073.18, 8123.12, 8167.02, 8207.79, 8246.55]</t>
         </is>
       </c>
       <c r="AT5" t="inlineStr">
         <is>
-          <t>[4631.0, 4620.84, 4624.77, 4631.01, 4638.46, 4646.67]</t>
-        </is>
+          <t>[7986.5, 7963.42, 7967.89, 7976.9, 7988.25, 8001.11]</t>
+        </is>
+      </c>
+      <c r="AU5" t="n">
+        <v>7963.04</v>
       </c>
     </row>
     <row r="6">
@@ -1312,16 +1329,16 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ALKEM</t>
+          <t>HAL</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>67440.64</v>
+        <v>310645.99</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1329,143 +1346,146 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>5640.5</v>
+        <v>4645</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>₹5617.16 - ₹5675.5</t>
+          <t>₹4628.96 - ₹4669.06</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>5733.84</v>
+        <v>4709.15</v>
       </c>
       <c r="I6" t="n">
-        <v>5598.93</v>
+        <v>4490.17</v>
       </c>
       <c r="J6" t="n">
-        <v>5497.15</v>
+        <v>4419.22</v>
       </c>
       <c r="K6" t="n">
-        <v>5524.06</v>
+        <v>4344.79</v>
       </c>
       <c r="L6" t="n">
-        <v>3.31</v>
+        <v>6.68</v>
       </c>
       <c r="M6" t="n">
-        <v>58.81</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="N6" t="n">
-        <v>54.69</v>
+        <v>56.51</v>
       </c>
       <c r="O6" t="n">
-        <v>4.12</v>
+        <v>7.78</v>
       </c>
       <c r="P6" t="n">
-        <v>116.68</v>
+        <v>80.19</v>
       </c>
       <c r="Q6" t="n">
-        <v>12.55</v>
+        <v>12.06</v>
       </c>
       <c r="R6" t="n">
-        <v>47.1</v>
+        <v>47.4</v>
       </c>
       <c r="S6" t="n">
-        <v>0.26</v>
+        <v>0.31</v>
       </c>
       <c r="T6" t="n">
-        <v>-1.26</v>
+        <v>-1.07</v>
       </c>
       <c r="U6" t="n">
-        <v>51.7</v>
+        <v>43.3</v>
       </c>
       <c r="V6" t="n">
-        <v>2.82</v>
+        <v>2.35</v>
       </c>
       <c r="W6" t="n">
         <v>-0.77</v>
       </c>
       <c r="X6" t="n">
-        <v>5500.49</v>
+        <v>4585.31</v>
       </c>
       <c r="Y6" t="n">
-        <v>5606.71</v>
+        <v>4659.03</v>
       </c>
       <c r="Z6" t="n">
-        <v>5685.62</v>
+        <v>4659.03</v>
       </c>
       <c r="AA6" t="n">
-        <v>5465.48</v>
+        <v>4524.72</v>
       </c>
       <c r="AB6" t="n">
-        <v>5620.67</v>
+        <v>4640.57</v>
       </c>
       <c r="AC6" t="n">
-        <v>5685.34</v>
+        <v>4677.84</v>
       </c>
       <c r="AD6" t="n">
-        <v>5730.17</v>
+        <v>4710.67</v>
       </c>
       <c r="AE6" t="n">
-        <v>56.2</v>
+        <v>72.8</v>
       </c>
       <c r="AF6" t="n">
-        <v>-0.03</v>
+        <v>0.27</v>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (12.55) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.06) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH6" t="n">
         <v>0.15</v>
       </c>
       <c r="AI6" t="n">
-        <v>29.3</v>
+        <v>34.4</v>
       </c>
       <c r="AJ6" t="n">
-        <v>14.6</v>
+        <v>1.8</v>
       </c>
       <c r="AK6" t="n">
-        <v>15.6</v>
+        <v>27.5</v>
       </c>
       <c r="AL6" t="n">
-        <v>17.6</v>
+        <v>24</v>
       </c>
       <c r="AM6" t="n">
-        <v>5765.79</v>
+        <v>4769.38</v>
       </c>
       <c r="AN6" t="n">
-        <v>5506.54</v>
+        <v>4515.46</v>
       </c>
       <c r="AO6" t="inlineStr">
         <is>
-          <t>ALKEM operates in the Healthcare sector. With an estimated Market Cap of ₹67,440.64 Cr., a P/E ratio of 29.27, and YoY Revenue Growth of +14.6%, the company demonstrates strong institutional backing, solid operating profit margins (15.65%), and healthy Return on Equity (17.56%).</t>
+          <t>HAL operates in the Industrials sector. With an estimated Market Cap of ₹310,645.99 Cr., a P/E ratio of 34.44, and YoY Revenue Growth of +1.8%, the company demonstrates strong institutional backing, solid operating profit margins (27.55%), and healthy Return on Equity (23.98%).</t>
         </is>
       </c>
       <c r="AP6" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 56.20 (Bullish Momentum Zone), while MACD Line (58.81) trades above Signal (54.69) with an expanding histogram (+4.12). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +3.31% above the 200-day DMA (₹5524.06). Daily volatility envelope is bounded by ATR(14) of ₹116.68.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 72.77 (Bullish Momentum Zone), while MACD Line (64.29) trades above Signal (56.51) with an expanding histogram (+7.78). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +6.68% above the 200-day DMA (₹4344.79). Daily volatility envelope is bounded by ATR(14) of ₹80.19.</t>
         </is>
       </c>
       <c r="AQ6" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ALKEM. Current Market Price (₹5,640.50) is positioned above the 30-day DMA (₹5,598.93), 50-day DMA (₹5,497.15), and 200-day DMA (₹5,524.06). The price distance from 200 DMA is +3.31%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for HAL. Current Market Price (₹4,645.00) is positioned above the 30-day DMA (₹4,490.17), 50-day DMA (₹4,419.22), and 200-day DMA (₹4,344.79). The price distance from 200 DMA is +6.68%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR6" t="inlineStr">
         <is>
-          <t>[5640.5, 5657.42, 5674.34, 5691.26, 5708.19, 5725.11]</t>
+          <t>[4645.0, 4658.93, 4672.87, 4686.8, 4700.74, 4714.67]</t>
         </is>
       </c>
       <c r="AS6" t="inlineStr">
         <is>
-          <t>[5640.5, 5704.09, 5740.35, 5772.1, 5801.53, 5829.47]</t>
+          <t>[4645.0, 4691.01, 4718.23, 4742.36, 4764.89, 4786.4]</t>
         </is>
       </c>
       <c r="AT6" t="inlineStr">
         <is>
-          <t>[5640.5, 5622.42, 5624.84, 5630.64, 5638.18, 5646.84]</t>
-        </is>
+          <t>[4645.0, 4634.88, 4638.85, 4645.14, 4652.63, 4660.88]</t>
+        </is>
+      </c>
+      <c r="AU6" t="n">
+        <v>4659.03</v>
       </c>
     </row>
     <row r="7">
@@ -1485,7 +1505,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>264489.95</v>
+        <v>264585.82</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1493,15 +1513,15 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2759</v>
+        <v>2760</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>₹2747.15 - ₹2776.77</t>
+          <t>₹2748.15 - ₹2777.77</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>2806.39</v>
+        <v>2807.39</v>
       </c>
       <c r="I7" t="n">
         <v>2698.21</v>
@@ -1528,16 +1548,16 @@
         <v>59.24</v>
       </c>
       <c r="Q7" t="n">
-        <v>12.55</v>
+        <v>12.06</v>
       </c>
       <c r="R7" t="n">
-        <v>48.2</v>
+        <v>50.9</v>
       </c>
       <c r="S7" t="n">
         <v>0.25</v>
       </c>
       <c r="T7" t="n">
-        <v>-1.28</v>
+        <v>-1.27</v>
       </c>
       <c r="U7" t="n">
         <v>55</v>
@@ -1549,25 +1569,25 @@
         <v>-0.77</v>
       </c>
       <c r="X7" t="n">
-        <v>2687.92</v>
+        <v>2710.51</v>
       </c>
       <c r="Y7" t="n">
-        <v>2780.66</v>
+        <v>2760.99</v>
       </c>
       <c r="Z7" t="n">
-        <v>2781.07</v>
+        <v>2760.99</v>
       </c>
       <c r="AA7" t="n">
-        <v>2670.15</v>
+        <v>2671.15</v>
       </c>
       <c r="AB7" t="n">
-        <v>2764.9</v>
+        <v>2765.23</v>
       </c>
       <c r="AC7" t="n">
-        <v>2781.1</v>
+        <v>2781.76</v>
       </c>
       <c r="AD7" t="n">
-        <v>2803.2</v>
+        <v>2803.53</v>
       </c>
       <c r="AE7" t="n">
         <v>67</v>
@@ -1577,14 +1597,14 @@
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
+          <t>Strong RSI | Low VIX (12.06) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH7" t="n">
         <v>0.15</v>
       </c>
       <c r="AI7" t="n">
-        <v>56.2</v>
+        <v>54.3</v>
       </c>
       <c r="AJ7" t="n">
         <v>17.9</v>
@@ -1596,14 +1616,14 @@
         <v>15</v>
       </c>
       <c r="AM7" t="n">
-        <v>2826.2</v>
+        <v>2825.18</v>
       </c>
       <c r="AN7" t="n">
-        <v>2694.16</v>
+        <v>2702.76</v>
       </c>
       <c r="AO7" t="inlineStr">
         <is>
-          <t>ASIANPAINT operates in the Basic Materials sector. With an estimated Market Cap of ₹264,489.95 Cr., a P/E ratio of 56.17, and YoY Revenue Growth of +17.9%, the company demonstrates strong institutional backing, solid operating profit margins (12.81%), and healthy Return on Equity (15.00%).</t>
+          <t>ASIANPAINT operates in the Basic Materials sector. With an estimated Market Cap of ₹264,585.82 Cr., a P/E ratio of 54.27, and YoY Revenue Growth of +17.9%, the company demonstrates strong institutional backing, solid operating profit margins (12.81%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP7" t="inlineStr">
@@ -1613,23 +1633,26 @@
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ASIANPAINT. Current Market Price (₹2,759.00) is positioned above the 30-day DMA (₹2,698.21), 50-day DMA (₹2,687.88), and 200-day DMA (₹2,577.55). The price distance from 200 DMA is +7.66%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ASIANPAINT. Current Market Price (₹2,760.00) is positioned above the 30-day DMA (₹2,698.21), 50-day DMA (₹2,687.88), and 200-day DMA (₹2,577.55). The price distance from 200 DMA is +7.66%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>[2759.0, 2767.28, 2775.55, 2783.83, 2792.11, 2800.38]</t>
+          <t>[2760.0, 2768.28, 2776.56, 2784.84, 2793.12, 2801.4]</t>
         </is>
       </c>
       <c r="AS7" t="inlineStr">
         <is>
-          <t>[2759.0, 2790.97, 2809.06, 2824.87, 2839.5, 2853.37]</t>
+          <t>[2760.0, 2791.97, 2810.07, 2825.88, 2840.51, 2854.38]</t>
         </is>
       </c>
       <c r="AT7" t="inlineStr">
         <is>
-          <t>[2759.0, 2749.51, 2750.42, 2753.05, 2756.57, 2760.65]</t>
-        </is>
+          <t>[2760.0, 2750.51, 2751.43, 2754.06, 2757.58, 2761.66]</t>
+        </is>
+      </c>
+      <c r="AU7" t="n">
+        <v>2760.99</v>
       </c>
     </row>
     <row r="8">
@@ -1649,7 +1672,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>104899.84</v>
+        <v>105483.44</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1657,15 +1680,15 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>737.6</v>
+        <v>741.05</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>₹734.61 - ₹742.09</t>
+          <t>₹738.06 - ₹745.54</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>749.58</v>
+        <v>753.03</v>
       </c>
       <c r="I8" t="n">
         <v>731.6799999999999</v>
@@ -1692,10 +1715,10 @@
         <v>14.97</v>
       </c>
       <c r="Q8" t="n">
-        <v>12.55</v>
+        <v>12.06</v>
       </c>
       <c r="R8" t="n">
-        <v>43.8</v>
+        <v>46</v>
       </c>
       <c r="S8" t="n">
         <v>0.26</v>
@@ -1707,31 +1730,31 @@
         <v>55</v>
       </c>
       <c r="V8" t="n">
-        <v>6.3</v>
+        <v>6.32</v>
       </c>
       <c r="W8" t="n">
         <v>-0.77</v>
       </c>
       <c r="X8" t="n">
-        <v>719.63</v>
+        <v>728.89</v>
       </c>
       <c r="Y8" t="n">
-        <v>729.87</v>
+        <v>744.51</v>
       </c>
       <c r="Z8" t="n">
-        <v>743.5</v>
+        <v>744.51</v>
       </c>
       <c r="AA8" t="n">
-        <v>715.14</v>
+        <v>718.59</v>
       </c>
       <c r="AB8" t="n">
-        <v>742.4299999999999</v>
+        <v>742.63</v>
       </c>
       <c r="AC8" t="n">
-        <v>748.0599999999999</v>
+        <v>751.3099999999999</v>
       </c>
       <c r="AD8" t="n">
-        <v>758.53</v>
+        <v>761.58</v>
       </c>
       <c r="AE8" t="n">
         <v>54.1</v>
@@ -1741,14 +1764,14 @@
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (12.55) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (12.06) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH8" t="n">
         <v>0.15</v>
       </c>
       <c r="AI8" t="n">
-        <v>49.1</v>
+        <v>48.3</v>
       </c>
       <c r="AJ8" t="n">
         <v>15.1</v>
@@ -1760,14 +1783,14 @@
         <v>15</v>
       </c>
       <c r="AM8" t="n">
-        <v>755.92</v>
+        <v>759.89</v>
       </c>
       <c r="AN8" t="n">
-        <v>720</v>
+        <v>722.96</v>
       </c>
       <c r="AO8" t="inlineStr">
         <is>
-          <t>INDHOTEL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹104,899.84 Cr., a P/E ratio of 49.13, and YoY Revenue Growth of +15.1%, the company demonstrates strong institutional backing, solid operating profit margins (20.87%), and healthy Return on Equity (15.00%).</t>
+          <t>INDHOTEL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹105,483.44 Cr., a P/E ratio of 48.31, and YoY Revenue Growth of +15.1%, the company demonstrates strong institutional backing, solid operating profit margins (20.87%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP8" t="inlineStr">
@@ -1777,23 +1800,26 @@
       </c>
       <c r="AQ8" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for INDHOTEL. Current Market Price (₹737.60) is positioned above the 30-day DMA (₹731.68), 50-day DMA (₹709.25), and 200-day DMA (₹686.46). The price distance from 200 DMA is +9.26%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for INDHOTEL. Current Market Price (₹741.05) is positioned above the 30-day DMA (₹731.68), 50-day DMA (₹709.25), and 200-day DMA (₹686.46). The price distance from 200 DMA is +9.26%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR8" t="inlineStr">
         <is>
-          <t>[737.6, 739.81, 742.03, 744.24, 746.45, 748.66]</t>
+          <t>[741.05, 743.27, 745.5, 747.72, 749.94, 752.17]</t>
         </is>
       </c>
       <c r="AS8" t="inlineStr">
         <is>
-          <t>[737.6, 745.8, 750.49, 754.61, 758.43, 762.05]</t>
+          <t>[741.05, 749.26, 753.97, 758.09, 761.92, 765.56]</t>
         </is>
       </c>
       <c r="AT8" t="inlineStr">
         <is>
-          <t>[737.6, 735.32, 735.67, 736.46, 737.47, 738.62]</t>
-        </is>
+          <t>[741.05, 738.78, 739.14, 739.94, 740.96, 742.12]</t>
+        </is>
+      </c>
+      <c r="AU8" t="n">
+        <v>744.51</v>
       </c>
     </row>
     <row r="9">
@@ -1813,7 +1839,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>95902.02</v>
+        <v>96376</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1821,98 +1847,98 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>364.2</v>
+        <v>366</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>₹362.64 - ₹366.55</t>
+          <t>₹364.46 - ₹368.31</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>370.46</v>
+        <v>372.16</v>
       </c>
       <c r="I9" t="n">
-        <v>358.01</v>
+        <v>358.35</v>
       </c>
       <c r="J9" t="n">
-        <v>351.17</v>
+        <v>351.85</v>
       </c>
       <c r="K9" t="n">
-        <v>347.72</v>
+        <v>347.77</v>
       </c>
       <c r="L9" t="n">
-        <v>5.86</v>
+        <v>5.82</v>
       </c>
       <c r="M9" t="n">
         <v>4.82</v>
       </c>
       <c r="N9" t="n">
-        <v>3.23</v>
+        <v>3.55</v>
       </c>
       <c r="O9" t="n">
-        <v>1.59</v>
+        <v>1.27</v>
       </c>
       <c r="P9" t="n">
-        <v>7.83</v>
+        <v>7.69</v>
       </c>
       <c r="Q9" t="n">
-        <v>12.55</v>
+        <v>12.06</v>
       </c>
       <c r="R9" t="n">
-        <v>43</v>
+        <v>44.2</v>
       </c>
       <c r="S9" t="n">
         <v>0.25</v>
       </c>
       <c r="T9" t="n">
-        <v>-1.49</v>
+        <v>-1.5</v>
       </c>
       <c r="U9" t="n">
-        <v>50</v>
+        <v>48.3</v>
       </c>
       <c r="V9" t="n">
-        <v>2.99</v>
+        <v>3.33</v>
       </c>
       <c r="W9" t="n">
         <v>-0.77</v>
       </c>
       <c r="X9" t="n">
-        <v>356.16</v>
+        <v>359.75</v>
       </c>
       <c r="Y9" t="n">
-        <v>368.91</v>
+        <v>367.82</v>
       </c>
       <c r="Z9" t="n">
-        <v>367.11</v>
+        <v>367.82</v>
       </c>
       <c r="AA9" t="n">
-        <v>352.46</v>
+        <v>354.46</v>
       </c>
       <c r="AB9" t="n">
-        <v>366.87</v>
+        <v>367.3</v>
       </c>
       <c r="AC9" t="n">
-        <v>369.64</v>
+        <v>371</v>
       </c>
       <c r="AD9" t="n">
-        <v>375.07</v>
+        <v>376</v>
       </c>
       <c r="AE9" t="n">
-        <v>71.8</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="AF9" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.06) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH9" t="n">
         <v>0.15</v>
       </c>
       <c r="AI9" t="n">
-        <v>6</v>
+        <v>6.1</v>
       </c>
       <c r="AJ9" t="n">
         <v>25.2</v>
@@ -1924,40 +1950,43 @@
         <v>15</v>
       </c>
       <c r="AM9" t="n">
-        <v>373.9</v>
+        <v>375.86</v>
       </c>
       <c r="AN9" t="n">
-        <v>354.41</v>
+        <v>356.74</v>
       </c>
       <c r="AO9" t="inlineStr">
         <is>
-          <t>RECLTD operates in the Financial Services sector. With an estimated Market Cap of ₹95,902.02 Cr., a P/E ratio of 5.99, and YoY Revenue Growth of +25.2%, the company demonstrates strong institutional backing, solid operating profit margins (68.89%), and healthy Return on Equity (15.00%).</t>
+          <t>RECLTD operates in the Financial Services sector. With an estimated Market Cap of ₹96,376.00 Cr., a P/E ratio of 6.10, and YoY Revenue Growth of +25.2%, the company demonstrates strong institutional backing, solid operating profit margins (68.89%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP9" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 71.84 (Bullish Momentum Zone), while MACD Line (4.82) trades above Signal (3.23) with an expanding histogram (+1.59). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +5.86% above the 200-day DMA (₹347.72). Daily volatility envelope is bounded by ATR(14) of ₹7.83.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 72.88 (Bullish Momentum Zone), while MACD Line (4.82) trades above Signal (3.55) with an expanding histogram (+1.27). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +5.82% above the 200-day DMA (₹347.77). Daily volatility envelope is bounded by ATR(14) of ₹7.69.</t>
         </is>
       </c>
       <c r="AQ9" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for RECLTD. Current Market Price (₹364.20) is positioned above the 30-day DMA (₹358.01), 50-day DMA (₹351.17), and 200-day DMA (₹347.72). The price distance from 200 DMA is +5.86%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for RECLTD. Current Market Price (₹366.00) is positioned above the 30-day DMA (₹358.35), 50-day DMA (₹351.85), and 200-day DMA (₹347.77). The price distance from 200 DMA is +5.82%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>[364.2, 365.29, 366.39, 367.48, 368.57, 369.66]</t>
+          <t>[366.0, 367.1, 368.2, 369.29, 370.39, 371.49]</t>
         </is>
       </c>
       <c r="AS9" t="inlineStr">
         <is>
-          <t>[364.2, 368.42, 370.81, 372.9, 374.83, 376.66]</t>
+          <t>[366.0, 370.18, 372.55, 374.62, 376.55, 378.37]</t>
         </is>
       </c>
       <c r="AT9" t="inlineStr">
         <is>
-          <t>[364.2, 362.95, 363.07, 363.41, 363.88, 364.41]</t>
-        </is>
+          <t>[366.0, 364.79, 364.93, 365.3, 365.78, 366.33]</t>
+        </is>
+      </c>
+      <c r="AU9" t="n">
+        <v>367.82</v>
       </c>
     </row>
     <row r="10">
@@ -1977,7 +2006,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>117478.01</v>
+        <v>117849.63</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1985,15 +2014,15 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>1454.2</v>
+        <v>1458.8</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>₹1447.37 - ₹1464.44</t>
+          <t>₹1451.97 - ₹1469.04</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>1481.51</v>
+        <v>1486.11</v>
       </c>
       <c r="I10" t="n">
         <v>1443.04</v>
@@ -2020,16 +2049,16 @@
         <v>34.14</v>
       </c>
       <c r="Q10" t="n">
-        <v>12.55</v>
+        <v>12.06</v>
       </c>
       <c r="R10" t="n">
-        <v>42.5</v>
+        <v>45</v>
       </c>
       <c r="S10" t="n">
         <v>0.23</v>
       </c>
       <c r="T10" t="n">
-        <v>-1.69</v>
+        <v>-1.68</v>
       </c>
       <c r="U10" t="n">
         <v>45</v>
@@ -2041,25 +2070,25 @@
         <v>-0.77</v>
       </c>
       <c r="X10" t="n">
-        <v>1413.23</v>
+        <v>1429.22</v>
       </c>
       <c r="Y10" t="n">
-        <v>1416.3</v>
+        <v>1463.41</v>
       </c>
       <c r="Z10" t="n">
-        <v>1465.83</v>
+        <v>1463.41</v>
       </c>
       <c r="AA10" t="n">
-        <v>1402.99</v>
+        <v>1407.59</v>
       </c>
       <c r="AB10" t="n">
-        <v>1452.57</v>
+        <v>1455.1</v>
       </c>
       <c r="AC10" t="n">
-        <v>1461.64</v>
+        <v>1466.7</v>
       </c>
       <c r="AD10" t="n">
-        <v>1469.07</v>
+        <v>1474.6</v>
       </c>
       <c r="AE10" t="n">
         <v>55.4</v>
@@ -2069,14 +2098,14 @@
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (12.55) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (12.06) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH10" t="n">
         <v>0.15</v>
       </c>
       <c r="AI10" t="n">
-        <v>35.2</v>
+        <v>35.3</v>
       </c>
       <c r="AJ10" t="n">
         <v>3.5</v>
@@ -2088,14 +2117,14 @@
         <v>15</v>
       </c>
       <c r="AM10" t="n">
-        <v>1486.32</v>
+        <v>1489.77</v>
       </c>
       <c r="AN10" t="n">
-        <v>1423.91</v>
+        <v>1427.07</v>
       </c>
       <c r="AO10" t="inlineStr">
         <is>
-          <t>CIPLA operates in the Healthcare sector. With an estimated Market Cap of ₹117,478.01 Cr., a P/E ratio of 35.19, and YoY Revenue Growth of +3.5%, the company demonstrates strong institutional backing, solid operating profit margins (12.01%), and healthy Return on Equity (15.00%).</t>
+          <t>CIPLA operates in the Healthcare sector. With an estimated Market Cap of ₹117,849.63 Cr., a P/E ratio of 35.30, and YoY Revenue Growth of +3.5%, the company demonstrates strong institutional backing, solid operating profit margins (12.01%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP10" t="inlineStr">
@@ -2105,23 +2134,26 @@
       </c>
       <c r="AQ10" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for CIPLA. Current Market Price (₹1,454.20) is positioned above the 30-day DMA (₹1,443.04), 50-day DMA (₹1,419.16), and 200-day DMA (₹1,394.98). The price distance from 200 DMA is +4.66%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for CIPLA. Current Market Price (₹1,458.80) is positioned above the 30-day DMA (₹1,443.04), 50-day DMA (₹1,419.16), and 200-day DMA (₹1,394.98). The price distance from 200 DMA is +4.66%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR10" t="inlineStr">
         <is>
-          <t>[1454.2, 1458.56, 1462.93, 1467.29, 1471.65, 1476.01]</t>
+          <t>[1458.8, 1463.18, 1467.55, 1471.93, 1476.31, 1480.68]</t>
         </is>
       </c>
       <c r="AS10" t="inlineStr">
         <is>
-          <t>[1454.2, 1472.22, 1482.24, 1490.94, 1498.96, 1506.55]</t>
+          <t>[1458.8, 1476.83, 1486.87, 1495.58, 1503.62, 1511.22]</t>
         </is>
       </c>
       <c r="AT10" t="inlineStr">
         <is>
-          <t>[1454.2, 1448.32, 1448.44, 1449.55, 1451.16, 1453.11]</t>
-        </is>
+          <t>[1458.8, 1452.93, 1453.07, 1454.19, 1455.82, 1457.78]</t>
+        </is>
+      </c>
+      <c r="AU10" t="n">
+        <v>1463.41</v>
       </c>
     </row>
     <row r="11">
@@ -2141,106 +2173,106 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>147121.83</v>
+        <v>146165.11</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1660.8</v>
+        <v>1650</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>₹1651.69 - ₹1674.47</t>
+          <t>₹1641.39 - ₹1662.92</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>1697.26</v>
+        <v>1684.45</v>
       </c>
       <c r="I11" t="n">
-        <v>1496.08</v>
+        <v>1505.04</v>
       </c>
       <c r="J11" t="n">
-        <v>1470.74</v>
+        <v>1475.27</v>
       </c>
       <c r="K11" t="n">
-        <v>1461.21</v>
+        <v>1462.42</v>
       </c>
       <c r="L11" t="n">
-        <v>12.85</v>
+        <v>12.72</v>
       </c>
       <c r="M11" t="n">
-        <v>58.14</v>
+        <v>57.73</v>
       </c>
       <c r="N11" t="n">
-        <v>48.29</v>
+        <v>50.18</v>
       </c>
       <c r="O11" t="n">
-        <v>9.85</v>
+        <v>7.55</v>
       </c>
       <c r="P11" t="n">
-        <v>45.57</v>
+        <v>43.06</v>
       </c>
       <c r="Q11" t="n">
-        <v>12.55</v>
+        <v>12.06</v>
       </c>
       <c r="R11" t="n">
-        <v>48.3</v>
+        <v>47.1</v>
       </c>
       <c r="S11" t="n">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="T11" t="n">
-        <v>-1.74</v>
+        <v>-1.69</v>
       </c>
       <c r="U11" t="n">
         <v>50</v>
       </c>
       <c r="V11" t="n">
-        <v>7.95</v>
+        <v>7.72</v>
       </c>
       <c r="W11" t="n">
         <v>-0.77</v>
       </c>
       <c r="X11" t="n">
-        <v>1632.32</v>
+        <v>1647.94</v>
       </c>
       <c r="Y11" t="n">
-        <v>1690.45</v>
+        <v>1678.63</v>
       </c>
       <c r="Z11" t="n">
-        <v>1674.09</v>
+        <v>1639.27</v>
       </c>
       <c r="AA11" t="n">
-        <v>1592.44</v>
+        <v>1585.4</v>
       </c>
       <c r="AB11" t="n">
-        <v>1657.77</v>
+        <v>1651.27</v>
       </c>
       <c r="AC11" t="n">
-        <v>1667.84</v>
+        <v>1663.54</v>
       </c>
       <c r="AD11" t="n">
-        <v>1674.87</v>
+        <v>1677.07</v>
       </c>
       <c r="AE11" t="n">
-        <v>83.5</v>
+        <v>82.3</v>
       </c>
       <c r="AF11" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>Low VIX (12.55) | LSTM Deep Net</t>
+          <t>Low VIX (12.06) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH11" t="n">
         <v>0.15</v>
       </c>
       <c r="AI11" t="n">
-        <v>28.7</v>
+        <v>28.5</v>
       </c>
       <c r="AJ11" t="n">
         <v>17.7</v>
@@ -2252,40 +2284,43 @@
         <v>15</v>
       </c>
       <c r="AM11" t="n">
-        <v>1703.67</v>
+        <v>1695.57</v>
       </c>
       <c r="AN11" t="n">
-        <v>1616.56</v>
+        <v>1603.07</v>
       </c>
       <c r="AO11" t="inlineStr">
         <is>
-          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹147,121.83 Cr., a P/E ratio of 28.73, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
+          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹146,165.11 Cr., a P/E ratio of 28.51, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP11" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 83.49 (Bullish Momentum Zone), while MACD Line (58.14) trades above Signal (48.29) with an expanding histogram (+9.85). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +12.85% above the 200-day DMA (₹1461.21). Daily volatility envelope is bounded by ATR(14) of ₹45.57.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 82.28 (Bullish Momentum Zone), while MACD Line (57.73) trades above Signal (50.18) with an expanding histogram (+7.55). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +12.72% above the 200-day DMA (₹1462.42). Daily volatility envelope is bounded by ATR(14) of ₹43.06.</t>
         </is>
       </c>
       <c r="AQ11" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,660.80) is positioned above the 30-day DMA (₹1,496.08), 50-day DMA (₹1,470.74), and 200-day DMA (₹1,461.21). The price distance from 200 DMA is +12.85%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,650.00) is positioned above the 30-day DMA (₹1,505.04), 50-day DMA (₹1,475.27), and 200-day DMA (₹1,462.42). The price distance from 200 DMA is +12.72%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR11" t="inlineStr">
         <is>
-          <t>[1660.8, 1665.78, 1670.76, 1675.75, 1680.73, 1685.71]</t>
+          <t>[1650.0, 1659.56, 1669.12, 1678.67, 1688.23, 1697.79]</t>
         </is>
       </c>
       <c r="AS11" t="inlineStr">
         <is>
-          <t>[1660.8, 1684.01, 1696.54, 1707.32, 1717.19, 1726.47]</t>
+          <t>[1650.0, 1676.78, 1693.48, 1708.51, 1722.68, 1736.31]</t>
         </is>
       </c>
       <c r="AT11" t="inlineStr">
         <is>
-          <t>[1660.8, 1652.11, 1651.43, 1652.07, 1653.39, 1655.14]</t>
-        </is>
+          <t>[1650.0, 1646.64, 1650.85, 1656.3, 1662.39, 1668.9]</t>
+        </is>
+      </c>
+      <c r="AU11" t="n">
+        <v>1639.27</v>
       </c>
     </row>
     <row r="12">
@@ -2296,16 +2331,16 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>COFORGE</t>
+          <t>360ONE</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>78834.38</v>
+        <v>48501.19</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2313,143 +2348,146 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1780.9</v>
+        <v>1192</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>₹1769.26 - ₹1798.36</t>
+          <t>₹1185.18 - ₹1202.23</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>1827.45</v>
+        <v>1219.28</v>
       </c>
       <c r="I12" t="n">
-        <v>1530.06</v>
+        <v>1110.79</v>
       </c>
       <c r="J12" t="n">
-        <v>1489.66</v>
+        <v>1106.51</v>
       </c>
       <c r="K12" t="n">
-        <v>1504.99</v>
+        <v>1101.09</v>
       </c>
       <c r="L12" t="n">
-        <v>16.27</v>
+        <v>4.9</v>
       </c>
       <c r="M12" t="n">
-        <v>74.70999999999999</v>
+        <v>12.02</v>
       </c>
       <c r="N12" t="n">
-        <v>49.28</v>
+        <v>7.73</v>
       </c>
       <c r="O12" t="n">
-        <v>25.43</v>
+        <v>4.28</v>
       </c>
       <c r="P12" t="n">
-        <v>58.19</v>
+        <v>34.1</v>
       </c>
       <c r="Q12" t="n">
-        <v>12.55</v>
+        <v>12.06</v>
       </c>
       <c r="R12" t="n">
-        <v>49.5</v>
+        <v>51.3</v>
       </c>
       <c r="S12" t="n">
-        <v>0.29</v>
+        <v>0.19</v>
       </c>
       <c r="T12" t="n">
-        <v>-1.76</v>
+        <v>-1.79</v>
       </c>
       <c r="U12" t="n">
-        <v>50</v>
+        <v>51.7</v>
       </c>
       <c r="V12" t="n">
-        <v>7.75</v>
+        <v>2.29</v>
       </c>
       <c r="W12" t="n">
         <v>-0.77</v>
       </c>
       <c r="X12" t="n">
-        <v>1779.76</v>
+        <v>1192</v>
       </c>
       <c r="Y12" t="n">
-        <v>1842.09</v>
+        <v>1215.66</v>
       </c>
       <c r="Z12" t="n">
-        <v>1806.47</v>
+        <v>1193.36</v>
       </c>
       <c r="AA12" t="n">
-        <v>1693.61</v>
+        <v>1140.85</v>
       </c>
       <c r="AB12" t="n">
-        <v>1771.33</v>
+        <v>1183.33</v>
       </c>
       <c r="AC12" t="n">
-        <v>1797.56</v>
+        <v>1203.36</v>
       </c>
       <c r="AD12" t="n">
-        <v>1814.23</v>
+        <v>1214.73</v>
       </c>
       <c r="AE12" t="n">
-        <v>72.90000000000001</v>
+        <v>61.8</v>
       </c>
       <c r="AF12" t="n">
-        <v>0.19</v>
+        <v>0.08</v>
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Strong RSI | Low VIX (12.06) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH12" t="n">
         <v>0.15</v>
       </c>
       <c r="AI12" t="n">
-        <v>36.9</v>
+        <v>39.6</v>
       </c>
       <c r="AJ12" t="n">
-        <v>49.9</v>
+        <v>29.9</v>
       </c>
       <c r="AK12" t="n">
-        <v>9.6</v>
+        <v>26.5</v>
       </c>
       <c r="AL12" t="n">
         <v>15</v>
       </c>
       <c r="AM12" t="n">
-        <v>1850.92</v>
+        <v>1226.21</v>
       </c>
       <c r="AN12" t="n">
-        <v>1716.91</v>
+        <v>1156.87</v>
       </c>
       <c r="AO12" t="inlineStr">
         <is>
-          <t>COFORGE operates in the Technology sector. With an estimated Market Cap of ₹78,834.38 Cr., a P/E ratio of 36.87, and YoY Revenue Growth of +49.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.64%), and healthy Return on Equity (15.00%).</t>
+          <t>360ONE operates in the Financial Services sector. With an estimated Market Cap of ₹48,501.19 Cr., a P/E ratio of 39.64, and YoY Revenue Growth of +29.9%, the company demonstrates strong institutional backing, solid operating profit margins (26.46%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP12" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 72.86 (Bullish Momentum Zone), while MACD Line (74.71) trades above Signal (49.28) with an expanding histogram (+25.43). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +16.27% above the 200-day DMA (₹1504.99). Daily volatility envelope is bounded by ATR(14) of ₹58.19.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 61.83 (Bullish Momentum Zone), while MACD Line (12.02) trades above Signal (7.73) with an expanding histogram (+4.28). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +4.90% above the 200-day DMA (₹1101.09). Daily volatility envelope is bounded by ATR(14) of ₹34.10.</t>
         </is>
       </c>
       <c r="AQ12" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for COFORGE. Current Market Price (₹1,780.90) is positioned above the 30-day DMA (₹1,530.06), 50-day DMA (₹1,489.66), and 200-day DMA (₹1,504.99). The price distance from 200 DMA is +16.27%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for 360ONE. Current Market Price (₹1,192.00) is positioned above the 30-day DMA (₹1,110.79), 50-day DMA (₹1,106.51), and 200-day DMA (₹1,101.09). The price distance from 200 DMA is +4.90%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR12" t="inlineStr">
         <is>
-          <t>[1780.9, 1806.47, 1832.04, 1857.61, 1883.18, 1908.75]</t>
+          <t>[1192.0, 1201.91, 1211.82, 1221.73, 1231.64, 1241.54]</t>
         </is>
       </c>
       <c r="AS12" t="inlineStr">
         <is>
-          <t>[1780.9, 1829.75, 1864.96, 1897.93, 1929.73, 1960.8]</t>
+          <t>[1192.0, 1215.55, 1231.11, 1245.35, 1258.92, 1272.04]</t>
         </is>
       </c>
       <c r="AT12" t="inlineStr">
         <is>
-          <t>[1780.9, 1789.01, 1807.35, 1827.37, 1848.26, 1869.71]</t>
-        </is>
+          <t>[1192.0, 1191.68, 1197.35, 1204.01, 1211.18, 1218.67]</t>
+        </is>
+      </c>
+      <c r="AU12" t="n">
+        <v>1193.36</v>
       </c>
     </row>
     <row r="13">
@@ -2460,160 +2498,163 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>360ONE</t>
+          <t>COFORGE</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>48460.5</v>
+        <v>78666.16</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>🔴 AVOID / HOLD</t>
+          <t>🟡 MODERATE BUY</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1191</v>
+        <v>1777</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>₹1184.21 - ₹1201.18</t>
+          <t>₹1765.36 - ₹1794.46</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>1218.15</v>
+        <v>1823.55</v>
       </c>
       <c r="I13" t="n">
-        <v>1109.52</v>
+        <v>1530.06</v>
       </c>
       <c r="J13" t="n">
-        <v>1105.91</v>
+        <v>1489.66</v>
       </c>
       <c r="K13" t="n">
-        <v>1100.89</v>
+        <v>1504.99</v>
       </c>
       <c r="L13" t="n">
-        <v>4.26</v>
+        <v>16.27</v>
       </c>
       <c r="M13" t="n">
-        <v>10.65</v>
+        <v>74.70999999999999</v>
       </c>
       <c r="N13" t="n">
-        <v>6.66</v>
+        <v>49.28</v>
       </c>
       <c r="O13" t="n">
-        <v>3.99</v>
+        <v>25.43</v>
       </c>
       <c r="P13" t="n">
-        <v>33.94</v>
+        <v>58.19</v>
       </c>
       <c r="Q13" t="n">
-        <v>12.55</v>
+        <v>12.06</v>
       </c>
       <c r="R13" t="n">
-        <v>47.6</v>
+        <v>49</v>
       </c>
       <c r="S13" t="n">
-        <v>0.19</v>
+        <v>0.28</v>
       </c>
       <c r="T13" t="n">
-        <v>-1.86</v>
+        <v>-1.84</v>
       </c>
       <c r="U13" t="n">
         <v>50</v>
       </c>
       <c r="V13" t="n">
-        <v>2.35</v>
+        <v>7.75</v>
       </c>
       <c r="W13" t="n">
         <v>-0.77</v>
       </c>
       <c r="X13" t="n">
-        <v>1174.1</v>
+        <v>1777</v>
       </c>
       <c r="Y13" t="n">
-        <v>1215.78</v>
+        <v>1821.67</v>
       </c>
       <c r="Z13" t="n">
-        <v>1200.53</v>
+        <v>1771.87</v>
       </c>
       <c r="AA13" t="n">
-        <v>1140.1</v>
+        <v>1689.71</v>
       </c>
       <c r="AB13" t="n">
-        <v>1183</v>
+        <v>1770.03</v>
       </c>
       <c r="AC13" t="n">
-        <v>1202.7</v>
+        <v>1794.96</v>
       </c>
       <c r="AD13" t="n">
-        <v>1214.4</v>
+        <v>1812.93</v>
       </c>
       <c r="AE13" t="n">
-        <v>60.6</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="AF13" t="n">
-        <v>0.13</v>
+        <v>0.19</v>
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | TTM Squeeze | Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.06) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH13" t="n">
         <v>0.15</v>
       </c>
       <c r="AI13" t="n">
-        <v>39.6</v>
+        <v>35.4</v>
       </c>
       <c r="AJ13" t="n">
-        <v>29.9</v>
+        <v>49.9</v>
       </c>
       <c r="AK13" t="n">
-        <v>26.5</v>
+        <v>9.6</v>
       </c>
       <c r="AL13" t="n">
         <v>15</v>
       </c>
       <c r="AM13" t="n">
-        <v>1231.07</v>
+        <v>1846.32</v>
       </c>
       <c r="AN13" t="n">
-        <v>1154.3</v>
+        <v>1706.42</v>
       </c>
       <c r="AO13" t="inlineStr">
         <is>
-          <t>360ONE operates in the Financial Services sector. With an estimated Market Cap of ₹48,460.50 Cr., a P/E ratio of 39.58, and YoY Revenue Growth of +29.9%, the company demonstrates strong institutional backing, solid operating profit margins (26.46%), and healthy Return on Equity (15.00%).</t>
+          <t>COFORGE operates in the Technology sector. With an estimated Market Cap of ₹78,666.16 Cr., a P/E ratio of 35.39, and YoY Revenue Growth of +49.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP13" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 60.59 (Bullish Momentum Zone), while MACD Line (10.65) trades above Signal (6.66) with an expanding histogram (+3.99). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +4.26% above the 200-day DMA (₹1100.89). Daily volatility envelope is bounded by ATR(14) of ₹33.94.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 72.86 (Bullish Momentum Zone), while MACD Line (74.71) trades above Signal (49.28) with an expanding histogram (+25.43). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +16.27% above the 200-day DMA (₹1504.99). Daily volatility envelope is bounded by ATR(14) of ₹58.19.</t>
         </is>
       </c>
       <c r="AQ13" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for 360ONE. Current Market Price (₹1,191.00) is positioned above the 30-day DMA (₹1,109.52), 50-day DMA (₹1,105.91), and 200-day DMA (₹1,100.89). The price distance from 200 DMA is +4.26%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for COFORGE. Current Market Price (₹1,777.00) is positioned above the 30-day DMA (₹1,530.06), 50-day DMA (₹1,489.66), and 200-day DMA (₹1,504.99). The price distance from 200 DMA is +16.27%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR13" t="inlineStr">
         <is>
-          <t>[1191.0, 1194.57, 1198.15, 1201.72, 1205.29, 1208.86]</t>
+          <t>[1777.0, 1801.25, 1825.49, 1849.74, 1873.99, 1898.23]</t>
         </is>
       </c>
       <c r="AS13" t="inlineStr">
         <is>
-          <t>[1191.0, 1208.15, 1217.34, 1225.23, 1232.44, 1239.22]</t>
+          <t>[1777.0, 1824.52, 1858.41, 1890.06, 1920.54, 1950.28]</t>
         </is>
       </c>
       <c r="AT13" t="inlineStr">
         <is>
-          <t>[1191.0, 1184.39, 1183.75, 1184.09, 1184.93, 1186.1]</t>
-        </is>
+          <t>[1777.0, 1783.79, 1800.8, 1819.5, 1839.07, 1859.19]</t>
+        </is>
+      </c>
+      <c r="AU13" t="n">
+        <v>1771.87</v>
       </c>
     </row>
     <row r="14">
@@ -2633,7 +2674,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>87238.55</v>
+        <v>87007.50999999999</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2641,15 +2682,15 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>14348</v>
+        <v>14310</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>₹14254.1 - ₹14488.85</t>
+          <t>₹14216.1 - ₹14450.85</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>14723.6</v>
+        <v>14685.6</v>
       </c>
       <c r="I14" t="n">
         <v>13362.03</v>
@@ -2676,16 +2717,16 @@
         <v>469.5</v>
       </c>
       <c r="Q14" t="n">
-        <v>12.55</v>
+        <v>12.06</v>
       </c>
       <c r="R14" t="n">
-        <v>49.4</v>
+        <v>49.7</v>
       </c>
       <c r="S14" t="n">
         <v>0.16</v>
       </c>
       <c r="T14" t="n">
-        <v>-2.09</v>
+        <v>-2.08</v>
       </c>
       <c r="U14" t="n">
         <v>48.3</v>
@@ -2697,25 +2738,25 @@
         <v>-0.77</v>
       </c>
       <c r="X14" t="n">
-        <v>14245.49</v>
+        <v>14310</v>
       </c>
       <c r="Y14" t="n">
-        <v>14747.67</v>
+        <v>14581.96</v>
       </c>
       <c r="Z14" t="n">
-        <v>14462.78</v>
+        <v>14272.16</v>
       </c>
       <c r="AA14" t="n">
-        <v>13643.75</v>
+        <v>13605.75</v>
       </c>
       <c r="AB14" t="n">
-        <v>14246</v>
+        <v>14242.67</v>
       </c>
       <c r="AC14" t="n">
-        <v>14469</v>
+        <v>14462.34</v>
       </c>
       <c r="AD14" t="n">
-        <v>14590</v>
+        <v>14614.67</v>
       </c>
       <c r="AE14" t="n">
         <v>55.3</v>
@@ -2725,14 +2766,14 @@
       </c>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>Low VIX (12.55) | LSTM Deep Net</t>
+          <t>Low VIX (12.06) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH14" t="n">
         <v>0.15</v>
       </c>
       <c r="AI14" t="n">
-        <v>42</v>
+        <v>41.8</v>
       </c>
       <c r="AJ14" t="n">
         <v>21.1</v>
@@ -2744,14 +2785,14 @@
         <v>15</v>
       </c>
       <c r="AM14" t="n">
-        <v>14900.38</v>
+        <v>14837.93</v>
       </c>
       <c r="AN14" t="n">
-        <v>13821.29</v>
+        <v>13775.36</v>
       </c>
       <c r="AO14" t="inlineStr">
         <is>
-          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹87,238.55 Cr., a P/E ratio of 42.03, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
+          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹87,007.51 Cr., a P/E ratio of 41.76, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP14" t="inlineStr">
@@ -2761,23 +2802,26 @@
       </c>
       <c r="AQ14" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,348.00) is positioned above the 30-day DMA (₹13,362.03), 50-day DMA (₹12,739.88), and 200-day DMA (₹12,290.57). The price distance from 200 DMA is +13.81%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,310.00) is positioned above the 30-day DMA (₹13,362.03), 50-day DMA (₹12,739.88), and 200-day DMA (₹12,290.57). The price distance from 200 DMA is +13.81%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR14" t="inlineStr">
         <is>
-          <t>[14348.0, 14460.71, 14573.42, 14686.13, 14798.85, 14911.56]</t>
+          <t>[14310.0, 14416.77, 14523.54, 14630.32, 14737.09, 14843.86]</t>
         </is>
       </c>
       <c r="AS14" t="inlineStr">
         <is>
-          <t>[14348.0, 14648.51, 14839.01, 15011.41, 15174.45, 15331.49]</t>
+          <t>[14310.0, 14604.57, 14789.13, 14955.59, 15112.69, 15263.79]</t>
         </is>
       </c>
       <c r="AT14" t="inlineStr">
         <is>
-          <t>[14348.0, 14319.86, 14374.23, 14442.18, 14517.15, 14596.61]</t>
-        </is>
+          <t>[14310.0, 14275.92, 14324.35, 14386.36, 14455.39, 14528.91]</t>
+        </is>
+      </c>
+      <c r="AU14" t="n">
+        <v>14272.16</v>
       </c>
     </row>
     <row r="15">
@@ -2788,16 +2832,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PGEL</t>
+          <t>IEX</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>17537.9</v>
+        <v>11524.44</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2805,143 +2849,146 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>612.15</v>
+        <v>129.59</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>₹607.86 - ₹618.59</t>
+          <t>₹128.72 - ₹130.9</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>629.3200000000001</v>
+        <v>133.08</v>
       </c>
       <c r="I15" t="n">
-        <v>583.11</v>
+        <v>124.43</v>
       </c>
       <c r="J15" t="n">
-        <v>550.15</v>
+        <v>123.96</v>
       </c>
       <c r="K15" t="n">
-        <v>554.14</v>
+        <v>127.99</v>
       </c>
       <c r="L15" t="n">
-        <v>10.44</v>
+        <v>0.95</v>
       </c>
       <c r="M15" t="n">
-        <v>15.39</v>
+        <v>2.09</v>
       </c>
       <c r="N15" t="n">
-        <v>15.91</v>
+        <v>1.41</v>
       </c>
       <c r="O15" t="n">
-        <v>-0.52</v>
+        <v>0.68</v>
       </c>
       <c r="P15" t="n">
-        <v>21.46</v>
+        <v>4.36</v>
       </c>
       <c r="Q15" t="n">
-        <v>12.55</v>
+        <v>12.06</v>
       </c>
       <c r="R15" t="n">
-        <v>52.2</v>
+        <v>51.6</v>
       </c>
       <c r="S15" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="T15" t="n">
-        <v>-2.1</v>
+        <v>-2.18</v>
       </c>
       <c r="U15" t="n">
-        <v>55</v>
+        <v>48.3</v>
       </c>
       <c r="V15" t="n">
-        <v>4.79</v>
+        <v>3.62</v>
       </c>
       <c r="W15" t="n">
         <v>-0.77</v>
       </c>
       <c r="X15" t="n">
-        <v>586.4</v>
+        <v>125.97</v>
       </c>
       <c r="Y15" t="n">
-        <v>600.51</v>
+        <v>129.41</v>
       </c>
       <c r="Z15" t="n">
-        <v>617.05</v>
+        <v>129.41</v>
       </c>
       <c r="AA15" t="n">
-        <v>579.96</v>
+        <v>123.04</v>
       </c>
       <c r="AB15" t="n">
-        <v>615.75</v>
+        <v>129.87</v>
       </c>
       <c r="AC15" t="n">
-        <v>628.9</v>
+        <v>130.66</v>
       </c>
       <c r="AD15" t="n">
-        <v>645.65</v>
+        <v>131.74</v>
       </c>
       <c r="AE15" t="n">
-        <v>54.7</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="AF15" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="AG15" t="inlineStr">
         <is>
-          <t>Low VIX (12.55) | LSTM Deep Net</t>
+          <t>Strong RSI | Low VIX (12.06) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH15" t="n">
         <v>0.15</v>
       </c>
       <c r="AI15" t="n">
-        <v>88.3</v>
+        <v>22.5</v>
       </c>
       <c r="AJ15" t="n">
-        <v>-10.1</v>
+        <v>10.1</v>
       </c>
       <c r="AK15" t="n">
-        <v>3.7</v>
+        <v>66.2</v>
       </c>
       <c r="AL15" t="n">
-        <v>6.7</v>
+        <v>15</v>
       </c>
       <c r="AM15" t="n">
-        <v>642.97</v>
+        <v>135.23</v>
       </c>
       <c r="AN15" t="n">
-        <v>579.63</v>
+        <v>123.77</v>
       </c>
       <c r="AO15" t="inlineStr">
         <is>
-          <t>PGEL operates in the Technology sector. With an estimated Market Cap of ₹17,537.90 Cr., a P/E ratio of 88.33, and YoY Revenue Growth of -10.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.72%), and healthy Return on Equity (6.69%).</t>
+          <t>IEX operates in the Financial Services sector. With an estimated Market Cap of ₹11,524.44 Cr., a P/E ratio of 22.54, and YoY Revenue Growth of +10.1%, the company demonstrates strong institutional backing, solid operating profit margins (66.22%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP15" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 54.70 (Consolidation Zone), while MACD Line (15.39) trades below Signal (15.91) with an expanding histogram (-0.52). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +10.44% above the 200-day DMA (₹554.14). Daily volatility envelope is bounded by ATR(14) of ₹21.46.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 64.41 (Bullish Momentum Zone), while MACD Line (2.09) trades above Signal (1.41) with an expanding histogram (+0.68). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +0.95% above the 200-day DMA (₹127.99). Daily volatility envelope is bounded by ATR(14) of ₹4.36.</t>
         </is>
       </c>
       <c r="AQ15" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PGEL. Current Market Price (₹612.15) is positioned above the 30-day DMA (₹583.11), 50-day DMA (₹550.15), and 200-day DMA (₹554.14). The price distance from 200 DMA is +10.44%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for IEX. Current Market Price (₹129.59) is positioned above the 30-day DMA (₹124.43), 50-day DMA (₹123.96), and 200-day DMA (₹127.99). The price distance from 200 DMA is +0.95%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR15" t="inlineStr">
         <is>
-          <t>[612.15, 613.99, 615.82, 617.66, 619.5, 621.33]</t>
+          <t>[129.59, 129.98, 130.37, 130.76, 131.15, 131.53]</t>
         </is>
       </c>
       <c r="AS15" t="inlineStr">
         <is>
-          <t>[612.15, 622.57, 627.96, 632.53, 636.66, 640.53]</t>
+          <t>[129.59, 131.72, 132.84, 133.78, 134.64, 135.44]</t>
         </is>
       </c>
       <c r="AT15" t="inlineStr">
         <is>
-          <t>[612.15, 607.55, 606.72, 606.51, 606.62, 606.94]</t>
-        </is>
+          <t>[129.59, 128.67, 128.52, 128.49, 128.53, 128.61]</t>
+        </is>
+      </c>
+      <c r="AU15" t="n">
+        <v>129.41</v>
       </c>
     </row>
     <row r="16">
@@ -2952,160 +2999,163 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>IEX</t>
+          <t>GODREJPROP</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>11540.45</v>
+        <v>63227.33</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>129.77</v>
+        <v>2099</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>₹128.9 - ₹131.08</t>
+          <t>₹2085.33 - ₹2119.51</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>133.26</v>
+        <v>2153.7</v>
       </c>
       <c r="I16" t="n">
-        <v>124.43</v>
+        <v>2028.46</v>
       </c>
       <c r="J16" t="n">
-        <v>123.96</v>
+        <v>1908.05</v>
       </c>
       <c r="K16" t="n">
-        <v>127.99</v>
+        <v>1880.26</v>
       </c>
       <c r="L16" t="n">
-        <v>0.95</v>
+        <v>8.16</v>
       </c>
       <c r="M16" t="n">
-        <v>2.09</v>
+        <v>46.13</v>
       </c>
       <c r="N16" t="n">
-        <v>1.41</v>
+        <v>60.86</v>
       </c>
       <c r="O16" t="n">
-        <v>0.68</v>
+        <v>-14.73</v>
       </c>
       <c r="P16" t="n">
-        <v>4.36</v>
+        <v>68.37</v>
       </c>
       <c r="Q16" t="n">
-        <v>12.55</v>
+        <v>12.06</v>
       </c>
       <c r="R16" t="n">
-        <v>48.8</v>
+        <v>47.2</v>
       </c>
       <c r="S16" t="n">
         <v>0.16</v>
       </c>
       <c r="T16" t="n">
-        <v>-2.19</v>
+        <v>-2.2</v>
       </c>
       <c r="U16" t="n">
-        <v>48.3</v>
+        <v>51.7</v>
       </c>
       <c r="V16" t="n">
-        <v>3.62</v>
+        <v>6.2</v>
       </c>
       <c r="W16" t="n">
         <v>-0.77</v>
       </c>
       <c r="X16" t="n">
-        <v>125.15</v>
+        <v>2033.15</v>
       </c>
       <c r="Y16" t="n">
-        <v>129.7</v>
+        <v>2076.84</v>
       </c>
       <c r="Z16" t="n">
-        <v>130.81</v>
+        <v>2076.84</v>
       </c>
       <c r="AA16" t="n">
-        <v>123.22</v>
+        <v>1996.44</v>
       </c>
       <c r="AB16" t="n">
-        <v>130.02</v>
+        <v>2099.53</v>
       </c>
       <c r="AC16" t="n">
-        <v>130.69</v>
+        <v>2143.36</v>
       </c>
       <c r="AD16" t="n">
-        <v>131.62</v>
+        <v>2187.73</v>
       </c>
       <c r="AE16" t="n">
-        <v>64.40000000000001</v>
+        <v>43.7</v>
       </c>
       <c r="AF16" t="n">
-        <v>0.1</v>
+        <v>-0</v>
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (12.06) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH16" t="n">
         <v>0.15</v>
       </c>
       <c r="AI16" t="n">
-        <v>22.6</v>
+        <v>34.4</v>
       </c>
       <c r="AJ16" t="n">
-        <v>10.1</v>
+        <v>63</v>
       </c>
       <c r="AK16" t="n">
-        <v>66.2</v>
+        <v>36.1</v>
       </c>
       <c r="AL16" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="AM16" t="n">
-        <v>135.41</v>
+        <v>2168.43</v>
       </c>
       <c r="AN16" t="n">
-        <v>123.5</v>
+        <v>2026.04</v>
       </c>
       <c r="AO16" t="inlineStr">
         <is>
-          <t>IEX operates in the Financial Services sector. With an estimated Market Cap of ₹11,540.45 Cr., a P/E ratio of 22.57, and YoY Revenue Growth of +10.1%, the company demonstrates strong institutional backing, solid operating profit margins (66.22%), and healthy Return on Equity (15.00%).</t>
+          <t>GODREJPROP operates in the Real Estate sector. With an estimated Market Cap of ₹63,227.33 Cr., a P/E ratio of 34.40, and YoY Revenue Growth of +63.0%, the company demonstrates strong institutional backing, solid operating profit margins (36.06%), and healthy Return on Equity (9.97%).</t>
         </is>
       </c>
       <c r="AP16" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 64.41 (Bullish Momentum Zone), while MACD Line (2.09) trades above Signal (1.41) with an expanding histogram (+0.68). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +0.95% above the 200-day DMA (₹127.99). Daily volatility envelope is bounded by ATR(14) of ₹4.36.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 43.71 (Consolidation Zone), while MACD Line (46.13) trades below Signal (60.86) with an expanding histogram (-14.73). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +8.16% above the 200-day DMA (₹1880.26). Daily volatility envelope is bounded by ATR(14) of ₹68.37.</t>
         </is>
       </c>
       <c r="AQ16" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for IEX. Current Market Price (₹129.77) is positioned above the 30-day DMA (₹124.43), 50-day DMA (₹123.96), and 200-day DMA (₹127.99). The price distance from 200 DMA is +0.95%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for GODREJPROP. Current Market Price (₹2,099.00) is positioned above the 30-day DMA (₹2,028.46), 50-day DMA (₹1,908.05), and 200-day DMA (₹1,880.26). The price distance from 200 DMA is +8.16%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR16" t="inlineStr">
         <is>
-          <t>[129.77, 130.16, 130.55, 130.94, 131.33, 131.72]</t>
+          <t>[2099.0, 2105.3, 2111.59, 2117.89, 2124.19, 2130.48]</t>
         </is>
       </c>
       <c r="AS16" t="inlineStr">
         <is>
-          <t>[129.77, 131.9, 133.02, 133.96, 134.82, 135.62]</t>
+          <t>[2099.0, 2132.65, 2150.27, 2165.26, 2178.89, 2191.64]</t>
         </is>
       </c>
       <c r="AT16" t="inlineStr">
         <is>
-          <t>[129.77, 128.85, 128.7, 128.67, 128.71, 128.79]</t>
-        </is>
+          <t>[2099.0, 2084.78, 2082.58, 2082.36, 2083.16, 2084.62]</t>
+        </is>
+      </c>
+      <c r="AU16" t="n">
+        <v>2076.84</v>
       </c>
     </row>
     <row r="17">
@@ -3116,16 +3166,16 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>GODREJPROP</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Real Estate</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>63902.07</v>
+        <v>285689.38</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3133,143 +3183,146 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2121.4</v>
+        <v>310.35</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>₹2107.72 - ₹2141.91</t>
+          <t>₹308.28 - ₹313.46</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>2176.1</v>
+        <v>318.63</v>
       </c>
       <c r="I17" t="n">
-        <v>2028.46</v>
+        <v>286.32</v>
       </c>
       <c r="J17" t="n">
-        <v>1908.05</v>
+        <v>272.64</v>
       </c>
       <c r="K17" t="n">
-        <v>1880.26</v>
+        <v>273.39</v>
       </c>
       <c r="L17" t="n">
-        <v>8.16</v>
+        <v>14.27</v>
       </c>
       <c r="M17" t="n">
-        <v>46.13</v>
+        <v>10.44</v>
       </c>
       <c r="N17" t="n">
-        <v>60.86</v>
+        <v>9.26</v>
       </c>
       <c r="O17" t="n">
-        <v>-14.73</v>
+        <v>1.18</v>
       </c>
       <c r="P17" t="n">
-        <v>68.37</v>
+        <v>10.35</v>
       </c>
       <c r="Q17" t="n">
-        <v>12.55</v>
+        <v>12.06</v>
       </c>
       <c r="R17" t="n">
-        <v>46.9</v>
+        <v>45.9</v>
       </c>
       <c r="S17" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="T17" t="n">
-        <v>-2.19</v>
+        <v>-2.34</v>
       </c>
       <c r="U17" t="n">
-        <v>51.7</v>
+        <v>53.3</v>
       </c>
       <c r="V17" t="n">
-        <v>6.27</v>
+        <v>2.43</v>
       </c>
       <c r="W17" t="n">
         <v>-0.77</v>
       </c>
       <c r="X17" t="n">
-        <v>2039.35</v>
+        <v>308.27</v>
       </c>
       <c r="Y17" t="n">
-        <v>2024.27</v>
+        <v>314.06</v>
       </c>
       <c r="Z17" t="n">
-        <v>2138.37</v>
+        <v>309.35</v>
       </c>
       <c r="AA17" t="n">
-        <v>2018.84</v>
+        <v>294.82</v>
       </c>
       <c r="AB17" t="n">
-        <v>2107</v>
+        <v>311.5</v>
       </c>
       <c r="AC17" t="n">
-        <v>2158.3</v>
+        <v>313.5</v>
       </c>
       <c r="AD17" t="n">
-        <v>2195.2</v>
+        <v>316.65</v>
       </c>
       <c r="AE17" t="n">
-        <v>43.7</v>
+        <v>62.2</v>
       </c>
       <c r="AF17" t="n">
-        <v>-0</v>
+        <v>0.1</v>
       </c>
       <c r="AG17" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (12.55) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.06) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH17" t="n">
         <v>0.15</v>
       </c>
       <c r="AI17" t="n">
-        <v>35.5</v>
+        <v>660.3</v>
       </c>
       <c r="AJ17" t="n">
-        <v>63</v>
+        <v>182</v>
       </c>
       <c r="AK17" t="n">
-        <v>36.1</v>
+        <v>0.6</v>
       </c>
       <c r="AL17" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="AM17" t="n">
-        <v>2194.1</v>
+        <v>321.84</v>
       </c>
       <c r="AN17" t="n">
-        <v>2049.1</v>
+        <v>300.07</v>
       </c>
       <c r="AO17" t="inlineStr">
         <is>
-          <t>GODREJPROP operates in the Real Estate sector. With an estimated Market Cap of ₹63,902.07 Cr., a P/E ratio of 35.48, and YoY Revenue Growth of +63.0%, the company demonstrates strong institutional backing, solid operating profit margins (36.06%), and healthy Return on Equity (9.97%).</t>
+          <t>ETERNAL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹285,689.38 Cr., a P/E ratio of 660.32, and YoY Revenue Growth of +182.0%, the company demonstrates strong institutional backing, solid operating profit margins (0.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP17" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 43.71 (Consolidation Zone), while MACD Line (46.13) trades below Signal (60.86) with an expanding histogram (-14.73). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +8.16% above the 200-day DMA (₹1880.26). Daily volatility envelope is bounded by ATR(14) of ₹68.37.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 62.17 (Bullish Momentum Zone), while MACD Line (10.44) trades above Signal (9.26) with an expanding histogram (+1.18). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +14.27% above the 200-day DMA (₹273.39). Daily volatility envelope is bounded by ATR(14) of ₹10.35.</t>
         </is>
       </c>
       <c r="AQ17" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for GODREJPROP. Current Market Price (₹2,121.40) is positioned above the 30-day DMA (₹2,028.46), 50-day DMA (₹1,908.05), and 200-day DMA (₹1,880.26). The price distance from 200 DMA is +8.16%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ETERNAL. Current Market Price (₹310.35) is positioned above the 30-day DMA (₹286.32), 50-day DMA (₹272.64), and 200-day DMA (₹273.39). The price distance from 200 DMA is +14.27%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR17" t="inlineStr">
         <is>
-          <t>[2121.4, 2127.76, 2134.13, 2140.49, 2146.86, 2153.22]</t>
+          <t>[310.35, 311.28, 312.21, 313.14, 314.07, 315.01]</t>
         </is>
       </c>
       <c r="AS17" t="inlineStr">
         <is>
-          <t>[2121.4, 2155.11, 2172.81, 2187.86, 2201.56, 2214.38]</t>
+          <t>[310.35, 315.42, 318.07, 320.31, 322.35, 324.26]</t>
         </is>
       </c>
       <c r="AT17" t="inlineStr">
         <is>
-          <t>[2121.4, 2107.25, 2105.12, 2104.96, 2105.83, 2107.35]</t>
-        </is>
+          <t>[310.35, 308.18, 307.82, 307.77, 307.86, 308.06]</t>
+        </is>
+      </c>
+      <c r="AU17" t="n">
+        <v>309.35</v>
       </c>
     </row>
     <row r="18">
@@ -3280,16 +3333,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>PGEL</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>286425.82</v>
+        <v>17275.75</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3297,143 +3350,146 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>311.35</v>
+        <v>603</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>₹309.28 - ₹314.46</t>
+          <t>₹598.71 - ₹609.44</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>319.63</v>
+        <v>620.17</v>
       </c>
       <c r="I18" t="n">
-        <v>286.32</v>
+        <v>583.11</v>
       </c>
       <c r="J18" t="n">
-        <v>272.64</v>
+        <v>550.15</v>
       </c>
       <c r="K18" t="n">
-        <v>273.39</v>
+        <v>554.14</v>
       </c>
       <c r="L18" t="n">
-        <v>14.27</v>
+        <v>10.44</v>
       </c>
       <c r="M18" t="n">
-        <v>10.44</v>
+        <v>15.39</v>
       </c>
       <c r="N18" t="n">
-        <v>9.26</v>
+        <v>15.91</v>
       </c>
       <c r="O18" t="n">
-        <v>1.18</v>
+        <v>-0.52</v>
       </c>
       <c r="P18" t="n">
-        <v>10.35</v>
+        <v>21.46</v>
       </c>
       <c r="Q18" t="n">
-        <v>12.55</v>
+        <v>12.06</v>
       </c>
       <c r="R18" t="n">
-        <v>46.1</v>
+        <v>47</v>
       </c>
       <c r="S18" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="T18" t="n">
-        <v>-2.32</v>
+        <v>-2.45</v>
       </c>
       <c r="U18" t="n">
         <v>53.3</v>
       </c>
       <c r="V18" t="n">
-        <v>2.43</v>
+        <v>4.78</v>
       </c>
       <c r="W18" t="n">
         <v>-0.77</v>
       </c>
       <c r="X18" t="n">
-        <v>306.87</v>
+        <v>581.89</v>
       </c>
       <c r="Y18" t="n">
-        <v>317.77</v>
+        <v>593.98</v>
       </c>
       <c r="Z18" t="n">
-        <v>313.84</v>
+        <v>593.98</v>
       </c>
       <c r="AA18" t="n">
-        <v>295.82</v>
+        <v>570.8099999999999</v>
       </c>
       <c r="AB18" t="n">
-        <v>312.08</v>
+        <v>612.7</v>
       </c>
       <c r="AC18" t="n">
-        <v>313.91</v>
+        <v>622.8</v>
       </c>
       <c r="AD18" t="n">
-        <v>316.48</v>
+        <v>642.6</v>
       </c>
       <c r="AE18" t="n">
-        <v>62.2</v>
+        <v>54.7</v>
       </c>
       <c r="AF18" t="n">
-        <v>0.1</v>
+        <v>0.06</v>
       </c>
       <c r="AG18" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.55) | LSTM Deep Net</t>
+          <t>Low VIX (12.06) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH18" t="n">
         <v>0.15</v>
       </c>
       <c r="AI18" t="n">
-        <v>662</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="AJ18" t="n">
-        <v>182</v>
+        <v>-10.1</v>
       </c>
       <c r="AK18" t="n">
-        <v>0.6</v>
+        <v>3.7</v>
       </c>
       <c r="AL18" t="n">
-        <v>15</v>
+        <v>6.7</v>
       </c>
       <c r="AM18" t="n">
-        <v>323.19</v>
+        <v>631.0700000000001</v>
       </c>
       <c r="AN18" t="n">
-        <v>300.17</v>
+        <v>573.73</v>
       </c>
       <c r="AO18" t="inlineStr">
         <is>
-          <t>ETERNAL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹286,425.82 Cr., a P/E ratio of 662.02, and YoY Revenue Growth of +182.0%, the company demonstrates strong institutional backing, solid operating profit margins (0.64%), and healthy Return on Equity (15.00%).</t>
+          <t>PGEL operates in the Technology sector. With an estimated Market Cap of ₹17,275.75 Cr., a P/E ratio of 86.39, and YoY Revenue Growth of -10.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.72%), and healthy Return on Equity (6.69%).</t>
         </is>
       </c>
       <c r="AP18" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 62.17 (Bullish Momentum Zone), while MACD Line (10.44) trades above Signal (9.26) with an expanding histogram (+1.18). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +14.27% above the 200-day DMA (₹273.39). Daily volatility envelope is bounded by ATR(14) of ₹10.35.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 54.70 (Consolidation Zone), while MACD Line (15.39) trades below Signal (15.91) with an expanding histogram (-0.52). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +10.44% above the 200-day DMA (₹554.14). Daily volatility envelope is bounded by ATR(14) of ₹21.46.</t>
         </is>
       </c>
       <c r="AQ18" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ETERNAL. Current Market Price (₹311.35) is positioned above the 30-day DMA (₹286.32), 50-day DMA (₹272.64), and 200-day DMA (₹273.39). The price distance from 200 DMA is +14.27%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PGEL. Current Market Price (₹603.00) is positioned above the 30-day DMA (₹583.11), 50-day DMA (₹550.15), and 200-day DMA (₹554.14). The price distance from 200 DMA is +10.44%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR18" t="inlineStr">
         <is>
-          <t>[311.35, 312.28, 313.22, 314.15, 315.09, 316.02]</t>
+          <t>[603.0, 604.81, 606.62, 608.43, 610.24, 612.04]</t>
         </is>
       </c>
       <c r="AS18" t="inlineStr">
         <is>
-          <t>[311.35, 316.42, 319.07, 321.32, 323.37, 325.28]</t>
+          <t>[603.0, 613.39, 618.76, 623.3, 627.4, 631.24]</t>
         </is>
       </c>
       <c r="AT18" t="inlineStr">
         <is>
-          <t>[311.35, 309.18, 308.83, 308.77, 308.88, 309.08]</t>
-        </is>
+          <t>[603.0, 598.37, 597.51, 597.28, 597.36, 597.65]</t>
+        </is>
+      </c>
+      <c r="AU18" t="n">
+        <v>593.98</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Add Commodities Engine, 1:00 AM Post-Market Validation, Self-Learning Feedback & GitHub Actions Workflows
</commit_message>
<xml_diff>
--- a/Breakout_ML_Quant_Predictions.xlsx
+++ b/Breakout_ML_Quant_Predictions.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU24"/>
+  <dimension ref="A1:AU23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>131502.24</v>
+        <v>131525.25</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -678,15 +678,15 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>114.42</v>
+        <v>114.44</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>₹114.02 - ₹115.02</t>
+          <t>₹114.04 - ₹115.04</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>116.02</v>
+        <v>116.04</v>
       </c>
       <c r="I2" t="n">
         <v>108.32</v>
@@ -713,16 +713,16 @@
         <v>2</v>
       </c>
       <c r="Q2" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R2" t="n">
-        <v>56.6</v>
+        <v>56.5</v>
       </c>
       <c r="S2" t="n">
         <v>0.3</v>
       </c>
       <c r="T2" t="n">
-        <v>-0.77</v>
+        <v>-0.78</v>
       </c>
       <c r="U2" t="n">
         <v>55</v>
@@ -734,25 +734,25 @@
         <v>-0.77</v>
       </c>
       <c r="X2" t="n">
-        <v>112.16</v>
+        <v>113.07</v>
       </c>
       <c r="Y2" t="n">
-        <v>115.49</v>
+        <v>114.81</v>
       </c>
       <c r="Z2" t="n">
-        <v>115.49</v>
+        <v>114.81</v>
       </c>
       <c r="AA2" t="n">
-        <v>111.42</v>
+        <v>111.44</v>
       </c>
       <c r="AB2" t="n">
-        <v>114.07</v>
+        <v>114.16</v>
       </c>
       <c r="AC2" t="n">
-        <v>114.94</v>
+        <v>115.12</v>
       </c>
       <c r="AD2" t="n">
-        <v>115.47</v>
+        <v>115.81</v>
       </c>
       <c r="AE2" t="n">
         <v>79.3</v>
@@ -762,7 +762,7 @@
       </c>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH2" t="n">
@@ -781,14 +781,14 @@
         <v>15</v>
       </c>
       <c r="AM2" t="n">
-        <v>117.76</v>
+        <v>117.69</v>
       </c>
       <c r="AN2" t="n">
-        <v>111.29</v>
+        <v>111.33</v>
       </c>
       <c r="AO2" t="inlineStr">
         <is>
-          <t>PNB operates in the Financial Services sector. With an estimated Market Cap of ₹131,502.24 Cr., a P/E ratio of 5.95, and YoY Revenue Growth of +15.2%, the company demonstrates strong institutional backing, solid operating profit margins (38.15%), and healthy Return on Equity (14.97%).</t>
+          <t>PNB operates in the Financial Services sector. With an estimated Market Cap of ₹131,525.25 Cr., a P/E ratio of 5.98, and YoY Revenue Growth of +15.2%, the company demonstrates strong institutional backing, solid operating profit margins (38.15%), and healthy Return on Equity (14.97%).</t>
         </is>
       </c>
       <c r="AP2" t="inlineStr">
@@ -798,26 +798,26 @@
       </c>
       <c r="AQ2" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PNB. Current Market Price (₹114.42) is positioned above the 30-day DMA (₹108.32), 50-day DMA (₹107.18), and 200-day DMA (₹112.64). The price distance from 200 DMA is +0.81%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PNB. Current Market Price (₹114.44) is positioned above the 30-day DMA (₹108.32), 50-day DMA (₹107.18), and 200-day DMA (₹112.64). The price distance from 200 DMA is +0.81%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR2" t="inlineStr">
         <is>
-          <t>[114.42, 114.76, 115.11, 115.45, 115.79, 116.14]</t>
+          <t>[114.44, 114.78, 115.13, 115.47, 115.81, 116.16]</t>
         </is>
       </c>
       <c r="AS2" t="inlineStr">
         <is>
-          <t>[114.42, 115.56, 116.24, 116.84, 117.39, 117.93]</t>
+          <t>[114.44, 115.58, 116.26, 116.86, 117.41, 117.95]</t>
         </is>
       </c>
       <c r="AT2" t="inlineStr">
         <is>
-          <t>[114.42, 114.16, 114.26, 114.41, 114.59, 114.79]</t>
+          <t>[114.44, 114.18, 114.28, 114.43, 114.61, 114.81]</t>
         </is>
       </c>
       <c r="AU2" t="n">
-        <v>115.49</v>
+        <v>114.81</v>
       </c>
     </row>
     <row r="3">
@@ -828,163 +828,163 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HAL</t>
+          <t>EICHERMOT</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>325332.29</v>
+        <v>217832.96</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>🔴 AVOID / HOLD</t>
+          <t>🟡 MODERATE BUY</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4865.1</v>
+        <v>7935</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>₹4849.0 - ₹4889.24</t>
+          <t>₹7903.21 - ₹7982.68</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>4929.48</v>
+        <v>8062.16</v>
       </c>
       <c r="I3" t="n">
-        <v>4499.37</v>
+        <v>7495.13</v>
       </c>
       <c r="J3" t="n">
-        <v>4423.86</v>
+        <v>7402.8</v>
       </c>
       <c r="K3" t="n">
-        <v>4343.91</v>
+        <v>7193.26</v>
       </c>
       <c r="L3" t="n">
-        <v>6.93</v>
+        <v>11.03</v>
       </c>
       <c r="M3" t="n">
-        <v>63.62</v>
+        <v>168.54</v>
       </c>
       <c r="N3" t="n">
-        <v>57.93</v>
+        <v>127.27</v>
       </c>
       <c r="O3" t="n">
-        <v>5.69</v>
+        <v>41.27</v>
       </c>
       <c r="P3" t="n">
-        <v>80.48</v>
+        <v>158.94</v>
       </c>
       <c r="Q3" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R3" t="n">
-        <v>48.2</v>
+        <v>48.8</v>
       </c>
       <c r="S3" t="n">
-        <v>0.32</v>
+        <v>0.28</v>
       </c>
       <c r="T3" t="n">
-        <v>-0.98</v>
+        <v>-1.13</v>
       </c>
       <c r="U3" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="V3" t="n">
-        <v>2.5</v>
+        <v>2.02</v>
       </c>
       <c r="W3" t="n">
         <v>-0.77</v>
       </c>
       <c r="X3" t="n">
-        <v>4774.35</v>
+        <v>7935</v>
       </c>
       <c r="Y3" t="n">
-        <v>4897.96</v>
+        <v>8081.8</v>
       </c>
       <c r="Z3" t="n">
-        <v>4889.26</v>
+        <v>7824.85</v>
       </c>
       <c r="AA3" t="n">
-        <v>4744.38</v>
+        <v>7696.58</v>
       </c>
       <c r="AB3" t="n">
-        <v>4807.8</v>
+        <v>7958.5</v>
       </c>
       <c r="AC3" t="n">
-        <v>4930.2</v>
+        <v>8020.5</v>
       </c>
       <c r="AD3" t="n">
-        <v>4995.3</v>
+        <v>8106</v>
       </c>
       <c r="AE3" t="n">
-        <v>72.59999999999999</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="AF3" t="n">
-        <v>0.29</v>
+        <v>0.26</v>
       </c>
       <c r="AG3" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH3" t="n">
         <v>0.15</v>
       </c>
       <c r="AI3" t="n">
-        <v>35.6</v>
+        <v>37.8</v>
       </c>
       <c r="AJ3" t="n">
-        <v>1.8</v>
+        <v>31.5</v>
       </c>
       <c r="AK3" t="n">
-        <v>27.5</v>
+        <v>23.2</v>
       </c>
       <c r="AL3" t="n">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="AM3" t="n">
-        <v>4991.18</v>
+        <v>8160.83</v>
       </c>
       <c r="AN3" t="n">
-        <v>4740.05</v>
+        <v>7743.58</v>
       </c>
       <c r="AO3" t="inlineStr">
         <is>
-          <t>HAL operates in the Industrials sector. With an estimated Market Cap of ₹325,332.29 Cr., a P/E ratio of 35.62, and YoY Revenue Growth of +1.8%, the company demonstrates strong institutional backing, solid operating profit margins (27.55%), and healthy Return on Equity (23.98%).</t>
+          <t>EICHERMOT operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹217,832.96 Cr., a P/E ratio of 37.78, and YoY Revenue Growth of +31.5%, the company demonstrates strong institutional backing, solid operating profit margins (23.21%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP3" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 72.57 (Bullish Momentum Zone), while MACD Line (63.62) trades above Signal (57.93) with an expanding histogram (+5.69). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +6.93% above the 200-day DMA (₹4343.91). Daily volatility envelope is bounded by ATR(14) of ₹80.48.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 75.06 (Bullish Momentum Zone), while MACD Line (168.54) trades above Signal (127.27) with an expanding histogram (+41.27). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +11.03% above the 200-day DMA (₹7193.26). Daily volatility envelope is bounded by ATR(14) of ₹158.94.</t>
         </is>
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for HAL. Current Market Price (₹4,865.10) is positioned above the 30-day DMA (₹4,499.37), 50-day DMA (₹4,423.86), and 200-day DMA (₹4,343.91). The price distance from 200 DMA is +6.93%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for EICHERMOT. Current Market Price (₹7,935.00) is positioned above the 30-day DMA (₹7,495.13), 50-day DMA (₹7,402.80), and 200-day DMA (₹7,193.26). The price distance from 200 DMA is +11.03%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR3" t="inlineStr">
         <is>
-          <t>[4865.1, 4879.7, 4894.29, 4908.89, 4923.48, 4938.08]</t>
+          <t>[7935.0, 8001.03, 8067.06, 8133.09, 8199.11, 8265.14]</t>
         </is>
       </c>
       <c r="AS3" t="inlineStr">
         <is>
-          <t>[4865.1, 4911.89, 4939.82, 4964.64, 4987.86, 5010.06]</t>
+          <t>[7935.0, 8064.61, 8156.97, 8243.21, 8326.27, 8407.31]</t>
         </is>
       </c>
       <c r="AT3" t="inlineStr">
         <is>
-          <t>[4865.1, 4855.55, 4860.15, 4867.07, 4875.19, 4884.09]</t>
+          <t>[7935.0, 7953.34, 7999.62, 8050.5, 8103.75, 8158.52]</t>
         </is>
       </c>
       <c r="AU3" t="n">
-        <v>4889.26</v>
+        <v>7824.85</v>
       </c>
     </row>
     <row r="4">
@@ -995,163 +995,163 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>EICHERMOT</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Basic Materials</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>220495.82</v>
+        <v>355915.84</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>8032</v>
+        <v>12099</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>₹8000.64 - ₹8079.04</t>
+          <t>₹12057.13 - ₹12161.8</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>8157.45</v>
+        <v>12266.47</v>
       </c>
       <c r="I4" t="n">
-        <v>7478.7</v>
+        <v>11541.28</v>
       </c>
       <c r="J4" t="n">
-        <v>7389.91</v>
+        <v>11320.31</v>
       </c>
       <c r="K4" t="n">
-        <v>7187.9</v>
+        <v>11571.01</v>
       </c>
       <c r="L4" t="n">
-        <v>10.39</v>
+        <v>5.35</v>
       </c>
       <c r="M4" t="n">
-        <v>160.7</v>
+        <v>200.35</v>
       </c>
       <c r="N4" t="n">
-        <v>116.95</v>
+        <v>157.57</v>
       </c>
       <c r="O4" t="n">
-        <v>43.75</v>
+        <v>42.78</v>
       </c>
       <c r="P4" t="n">
-        <v>156.81</v>
+        <v>209.34</v>
       </c>
       <c r="Q4" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R4" t="n">
-        <v>54</v>
+        <v>44.6</v>
       </c>
       <c r="S4" t="n">
-        <v>0.27</v>
+        <v>0.31</v>
       </c>
       <c r="T4" t="n">
-        <v>-1.01</v>
+        <v>-1.17</v>
       </c>
       <c r="U4" t="n">
-        <v>51.7</v>
+        <v>48.3</v>
       </c>
       <c r="V4" t="n">
-        <v>2.02</v>
+        <v>2.9</v>
       </c>
       <c r="W4" t="n">
         <v>-0.77</v>
       </c>
       <c r="X4" t="n">
-        <v>7925.36</v>
+        <v>11999.72</v>
       </c>
       <c r="Y4" t="n">
-        <v>8161.16</v>
+        <v>12195.97</v>
       </c>
       <c r="Z4" t="n">
-        <v>8120.14</v>
+        <v>12088.83</v>
       </c>
       <c r="AA4" t="n">
-        <v>7796.78</v>
+        <v>11784.99</v>
       </c>
       <c r="AB4" t="n">
-        <v>8011.33</v>
+        <v>12107.67</v>
       </c>
       <c r="AC4" t="n">
-        <v>8064.66</v>
+        <v>12195.34</v>
       </c>
       <c r="AD4" t="n">
-        <v>8097.33</v>
+        <v>12291.67</v>
       </c>
       <c r="AE4" t="n">
-        <v>74.3</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="AF4" t="n">
-        <v>0.21</v>
+        <v>0.32</v>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH4" t="n">
         <v>0.15</v>
       </c>
       <c r="AI4" t="n">
-        <v>38.2</v>
+        <v>41.2</v>
       </c>
       <c r="AJ4" t="n">
-        <v>31.5</v>
+        <v>15.9</v>
       </c>
       <c r="AK4" t="n">
-        <v>23.2</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="AL4" t="n">
         <v>15</v>
       </c>
       <c r="AM4" t="n">
-        <v>8246.41</v>
+        <v>12381.43</v>
       </c>
       <c r="AN4" t="n">
-        <v>7837.97</v>
+        <v>11832.33</v>
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>EICHERMOT operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹220,495.82 Cr., a P/E ratio of 38.23, and YoY Revenue Growth of +31.5%, the company demonstrates strong institutional backing, solid operating profit margins (23.21%), and healthy Return on Equity (15.00%).</t>
+          <t>ULTRACEMCO operates in the Basic Materials sector. With an estimated Market Cap of ₹355,915.84 Cr., a P/E ratio of 41.18, and YoY Revenue Growth of +15.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.29%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP4" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 74.31 (Bullish Momentum Zone), while MACD Line (160.70) trades above Signal (116.95) with an expanding histogram (+43.75). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +10.39% above the 200-day DMA (₹7187.90). Daily volatility envelope is bounded by ATR(14) of ₹156.81.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 75.88 (Bullish Momentum Zone), while MACD Line (200.35) trades above Signal (157.57) with an expanding histogram (+42.78). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +5.35% above the 200-day DMA (₹11571.01). Daily volatility envelope is bounded by ATR(14) of ₹209.34.</t>
         </is>
       </c>
       <c r="AQ4" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for EICHERMOT. Current Market Price (₹8,032.00) is positioned above the 30-day DMA (₹7,478.70), 50-day DMA (₹7,389.91), and 200-day DMA (₹7,187.90). The price distance from 200 DMA is +10.39%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ULTRACEMCO. Current Market Price (₹12,099.00) is positioned above the 30-day DMA (₹11,541.28), 50-day DMA (₹11,320.31), and 200-day DMA (₹11,571.01). The price distance from 200 DMA is +5.35%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR4" t="inlineStr">
         <is>
-          <t>[8032.0, 8056.1, 8080.19, 8104.29, 8128.38, 8152.48]</t>
+          <t>[12099.0, 12135.3, 12171.59, 12207.89, 12244.19, 12280.48]</t>
         </is>
       </c>
       <c r="AS4" t="inlineStr">
         <is>
-          <t>[8032.0, 8118.82, 8168.9, 8212.93, 8253.83, 8292.74]</t>
+          <t>[12099.0, 12219.03, 12290.01, 12352.93, 12411.66, 12467.72]</t>
         </is>
       </c>
       <c r="AT4" t="inlineStr">
         <is>
-          <t>[8032.0, 8009.05, 8013.66, 8022.81, 8034.3, 8047.29]</t>
+          <t>[12099.0, 12072.5, 12082.78, 12099.11, 12118.58, 12140.06]</t>
         </is>
       </c>
       <c r="AU4" t="n">
-        <v>8120.14</v>
+        <v>12088.83</v>
       </c>
     </row>
     <row r="5">
@@ -1162,163 +1162,163 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ALKEM</t>
+          <t>ASIANPAINT</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Basic Materials</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>67775.42</v>
+        <v>264106.49</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>5668.5</v>
+        <v>2755</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>₹5645.6 - ₹5702.85</t>
+          <t>₹2743.08 - ₹2772.88</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>5760.1</v>
+        <v>2802.69</v>
       </c>
       <c r="I5" t="n">
-        <v>5605.35</v>
+        <v>2701.3</v>
       </c>
       <c r="J5" t="n">
-        <v>5501.71</v>
+        <v>2690.11</v>
       </c>
       <c r="K5" t="n">
-        <v>5524.85</v>
+        <v>2579.42</v>
       </c>
       <c r="L5" t="n">
-        <v>1.51</v>
+        <v>7</v>
       </c>
       <c r="M5" t="n">
-        <v>48.94</v>
+        <v>26.48</v>
       </c>
       <c r="N5" t="n">
-        <v>53.54</v>
+        <v>18.67</v>
       </c>
       <c r="O5" t="n">
-        <v>-4.6</v>
+        <v>7.81</v>
       </c>
       <c r="P5" t="n">
-        <v>114.5</v>
+        <v>59.61</v>
       </c>
       <c r="Q5" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R5" t="n">
-        <v>54.9</v>
+        <v>45.2</v>
       </c>
       <c r="S5" t="n">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="T5" t="n">
-        <v>-1.02</v>
+        <v>-1.42</v>
       </c>
       <c r="U5" t="n">
         <v>53.3</v>
       </c>
       <c r="V5" t="n">
-        <v>2.74</v>
+        <v>1.72</v>
       </c>
       <c r="W5" t="n">
         <v>-0.77</v>
       </c>
       <c r="X5" t="n">
-        <v>5537.85</v>
+        <v>2718.8</v>
       </c>
       <c r="Y5" t="n">
-        <v>5691.58</v>
+        <v>2763.74</v>
       </c>
       <c r="Z5" t="n">
-        <v>5657.68</v>
+        <v>2731.16</v>
       </c>
       <c r="AA5" t="n">
-        <v>5496.75</v>
+        <v>2665.58</v>
       </c>
       <c r="AB5" t="n">
-        <v>5676.17</v>
+        <v>2761.53</v>
       </c>
       <c r="AC5" t="n">
-        <v>5687.84</v>
+        <v>2781.46</v>
       </c>
       <c r="AD5" t="n">
-        <v>5707.17</v>
+        <v>2807.93</v>
       </c>
       <c r="AE5" t="n">
-        <v>47.1</v>
+        <v>63.3</v>
       </c>
       <c r="AF5" t="n">
-        <v>-0.04</v>
+        <v>0.05</v>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Strong RSI | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH5" t="n">
         <v>0.15</v>
       </c>
       <c r="AI5" t="n">
-        <v>29.5</v>
+        <v>55.8</v>
       </c>
       <c r="AJ5" t="n">
-        <v>14.6</v>
+        <v>17.9</v>
       </c>
       <c r="AK5" t="n">
-        <v>15.6</v>
+        <v>12.8</v>
       </c>
       <c r="AL5" t="n">
-        <v>17.6</v>
+        <v>15</v>
       </c>
       <c r="AM5" t="n">
-        <v>5789.43</v>
+        <v>2820.4</v>
       </c>
       <c r="AN5" t="n">
-        <v>5547.69</v>
+        <v>2690.52</v>
       </c>
       <c r="AO5" t="inlineStr">
         <is>
-          <t>ALKEM operates in the Healthcare sector. With an estimated Market Cap of ₹67,775.42 Cr., a P/E ratio of 29.47, and YoY Revenue Growth of +14.6%, the company demonstrates strong institutional backing, solid operating profit margins (15.65%), and healthy Return on Equity (17.56%).</t>
+          <t>ASIANPAINT operates in the Basic Materials sector. With an estimated Market Cap of ₹264,106.49 Cr., a P/E ratio of 55.77, and YoY Revenue Growth of +17.9%, the company demonstrates strong institutional backing, solid operating profit margins (12.81%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP5" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 47.14 (Consolidation Zone), while MACD Line (48.94) trades below Signal (53.54) with an expanding histogram (-4.60). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +1.51% above the 200-day DMA (₹5524.85). Daily volatility envelope is bounded by ATR(14) of ₹114.50.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 63.35 (Bullish Momentum Zone), while MACD Line (26.48) trades above Signal (18.67) with an expanding histogram (+7.81). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +7.00% above the 200-day DMA (₹2579.42). Daily volatility envelope is bounded by ATR(14) of ₹59.61.</t>
         </is>
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ALKEM. Current Market Price (₹5,668.50) is positioned above the 30-day DMA (₹5,605.35), 50-day DMA (₹5,501.71), and 200-day DMA (₹5,524.85). The price distance from 200 DMA is +1.51%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ASIANPAINT. Current Market Price (₹2,755.00) is positioned above the 30-day DMA (₹2,701.30), 50-day DMA (₹2,690.11), and 200-day DMA (₹2,579.42). The price distance from 200 DMA is +7.00%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>[5668.5, 5685.51, 5702.51, 5719.52, 5736.52, 5753.53]</t>
+          <t>[2755.0, 2763.26, 2771.53, 2779.79, 2788.06, 2796.32]</t>
         </is>
       </c>
       <c r="AS5" t="inlineStr">
         <is>
-          <t>[5668.5, 5731.31, 5767.28, 5798.84, 5828.12, 5855.94]</t>
+          <t>[2755.0, 2787.11, 2805.25, 2821.1, 2835.75, 2849.65]</t>
         </is>
       </c>
       <c r="AT5" t="inlineStr">
         <is>
-          <t>[5668.5, 5651.16, 5653.93, 5660.02, 5667.82, 5676.72]</t>
+          <t>[2755.0, 2745.38, 2746.24, 2748.82, 2752.29, 2756.33]</t>
         </is>
       </c>
       <c r="AU5" t="n">
-        <v>5657.68</v>
+        <v>2731.16</v>
       </c>
     </row>
     <row r="6">
@@ -1329,16 +1329,16 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ULTRACEMCO</t>
+          <t>INDHOTEL</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Basic Materials</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>357269.01</v>
+        <v>104465.69</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1346,146 +1346,146 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>12145</v>
+        <v>733.9</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>₹12103.13 - ₹12207.8</t>
+          <t>₹730.83 - ₹738.51</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>12312.47</v>
+        <v>746.1900000000001</v>
       </c>
       <c r="I6" t="n">
-        <v>11541.28</v>
+        <v>732.2</v>
       </c>
       <c r="J6" t="n">
-        <v>11320.31</v>
+        <v>710.78</v>
       </c>
       <c r="K6" t="n">
-        <v>11571.01</v>
+        <v>686.49</v>
       </c>
       <c r="L6" t="n">
-        <v>5.35</v>
+        <v>7.95</v>
       </c>
       <c r="M6" t="n">
-        <v>200.35</v>
+        <v>8.74</v>
       </c>
       <c r="N6" t="n">
-        <v>157.57</v>
+        <v>9.07</v>
       </c>
       <c r="O6" t="n">
-        <v>42.78</v>
+        <v>-0.33</v>
       </c>
       <c r="P6" t="n">
-        <v>209.34</v>
+        <v>15.36</v>
       </c>
       <c r="Q6" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R6" t="n">
-        <v>44.6</v>
+        <v>43.6</v>
       </c>
       <c r="S6" t="n">
-        <v>0.31</v>
+        <v>0.25</v>
       </c>
       <c r="T6" t="n">
-        <v>-1.16</v>
+        <v>-1.42</v>
       </c>
       <c r="U6" t="n">
-        <v>48.3</v>
+        <v>53.3</v>
       </c>
       <c r="V6" t="n">
-        <v>2.9</v>
+        <v>5.79</v>
       </c>
       <c r="W6" t="n">
         <v>-0.77</v>
       </c>
       <c r="X6" t="n">
-        <v>11952.02</v>
+        <v>722.0700000000001</v>
       </c>
       <c r="Y6" t="n">
-        <v>12308.76</v>
+        <v>732.9</v>
       </c>
       <c r="Z6" t="n">
-        <v>12207.03</v>
+        <v>732.24</v>
       </c>
       <c r="AA6" t="n">
-        <v>11830.99</v>
+        <v>710.86</v>
       </c>
       <c r="AB6" t="n">
-        <v>12152.67</v>
+        <v>736.5700000000001</v>
       </c>
       <c r="AC6" t="n">
-        <v>12195.34</v>
+        <v>741.14</v>
       </c>
       <c r="AD6" t="n">
-        <v>12245.67</v>
+        <v>748.37</v>
       </c>
       <c r="AE6" t="n">
-        <v>75.90000000000001</v>
+        <v>55.9</v>
       </c>
       <c r="AF6" t="n">
-        <v>0.32</v>
+        <v>0.02</v>
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH6" t="n">
         <v>0.15</v>
       </c>
       <c r="AI6" t="n">
-        <v>41.3</v>
+        <v>49.3</v>
       </c>
       <c r="AJ6" t="n">
-        <v>15.9</v>
+        <v>15.1</v>
       </c>
       <c r="AK6" t="n">
-        <v>9.300000000000001</v>
+        <v>20.9</v>
       </c>
       <c r="AL6" t="n">
         <v>15</v>
       </c>
       <c r="AM6" t="n">
-        <v>12430.78</v>
+        <v>752.3</v>
       </c>
       <c r="AN6" t="n">
-        <v>11889.71</v>
+        <v>714.1</v>
       </c>
       <c r="AO6" t="inlineStr">
         <is>
-          <t>ULTRACEMCO operates in the Basic Materials sector. With an estimated Market Cap of ₹357,269.01 Cr., a P/E ratio of 41.34, and YoY Revenue Growth of +15.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.29%), and healthy Return on Equity (15.00%).</t>
+          <t>INDHOTEL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹104,465.69 Cr., a P/E ratio of 49.26, and YoY Revenue Growth of +15.1%, the company demonstrates strong institutional backing, solid operating profit margins (20.87%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP6" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 75.88 (Bullish Momentum Zone), while MACD Line (200.35) trades above Signal (157.57) with an expanding histogram (+42.78). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +5.35% above the 200-day DMA (₹11571.01). Daily volatility envelope is bounded by ATR(14) of ₹209.34.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 55.94 (Bullish Momentum Zone), while MACD Line (8.74) trades below Signal (9.07) with an expanding histogram (-0.33). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +7.95% above the 200-day DMA (₹686.49). Daily volatility envelope is bounded by ATR(14) of ₹15.36.</t>
         </is>
       </c>
       <c r="AQ6" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ULTRACEMCO. Current Market Price (₹12,145.00) is positioned above the 30-day DMA (₹11,541.28), 50-day DMA (₹11,320.31), and 200-day DMA (₹11,571.01). The price distance from 200 DMA is +5.35%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for INDHOTEL. Current Market Price (₹733.90) is positioned above the 30-day DMA (₹732.20), 50-day DMA (₹710.78), and 200-day DMA (₹686.49). The price distance from 200 DMA is +7.95%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR6" t="inlineStr">
         <is>
-          <t>[12145.0, 12181.43, 12217.87, 12254.3, 12290.74, 12327.17]</t>
+          <t>[733.9, 736.1, 738.3, 740.51, 742.71, 744.91]</t>
         </is>
       </c>
       <c r="AS6" t="inlineStr">
         <is>
-          <t>[12145.0, 12265.17, 12336.29, 12399.34, 12458.21, 12514.41]</t>
+          <t>[733.9, 742.24, 746.99, 751.14, 754.99, 758.64]</t>
         </is>
       </c>
       <c r="AT6" t="inlineStr">
         <is>
-          <t>[12145.0, 12118.63, 12129.05, 12145.53, 12165.14, 12186.75]</t>
+          <t>[733.9, 731.49, 731.79, 732.53, 733.49, 734.61]</t>
         </is>
       </c>
       <c r="AU6" t="n">
-        <v>12207.03</v>
+        <v>732.24</v>
       </c>
     </row>
     <row r="7">
@@ -1496,163 +1496,163 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>INDHOTEL</t>
+          <t>CIPLA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Healthcare</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>105497.68</v>
+        <v>119077.56</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>741.15</v>
+        <v>1474</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>₹738.08 - ₹745.76</t>
+          <t>₹1467.14 - ₹1484.29</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>753.4400000000001</v>
+        <v>1501.43</v>
       </c>
       <c r="I7" t="n">
-        <v>732.2</v>
+        <v>1443.74</v>
       </c>
       <c r="J7" t="n">
-        <v>710.78</v>
+        <v>1420.24</v>
       </c>
       <c r="K7" t="n">
-        <v>686.49</v>
+        <v>1394.5</v>
       </c>
       <c r="L7" t="n">
-        <v>7.95</v>
+        <v>4.61</v>
       </c>
       <c r="M7" t="n">
-        <v>8.74</v>
+        <v>11.95</v>
       </c>
       <c r="N7" t="n">
-        <v>9.07</v>
+        <v>9.52</v>
       </c>
       <c r="O7" t="n">
-        <v>-0.33</v>
+        <v>2.43</v>
       </c>
       <c r="P7" t="n">
-        <v>15.36</v>
+        <v>34.29</v>
       </c>
       <c r="Q7" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R7" t="n">
-        <v>52.2</v>
+        <v>48</v>
       </c>
       <c r="S7" t="n">
-        <v>0.26</v>
+        <v>0.23</v>
       </c>
       <c r="T7" t="n">
-        <v>-1.17</v>
+        <v>-1.54</v>
       </c>
       <c r="U7" t="n">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="V7" t="n">
-        <v>5.81</v>
+        <v>10.13</v>
       </c>
       <c r="W7" t="n">
         <v>-0.77</v>
       </c>
       <c r="X7" t="n">
-        <v>723.6</v>
+        <v>1446.53</v>
       </c>
       <c r="Y7" t="n">
-        <v>745.2</v>
+        <v>1486.61</v>
       </c>
       <c r="Z7" t="n">
-        <v>743.61</v>
+        <v>1486.61</v>
       </c>
       <c r="AA7" t="n">
-        <v>718.11</v>
+        <v>1422.56</v>
       </c>
       <c r="AB7" t="n">
-        <v>739.72</v>
+        <v>1474.37</v>
       </c>
       <c r="AC7" t="n">
-        <v>743.4400000000001</v>
+        <v>1487.74</v>
       </c>
       <c r="AD7" t="n">
-        <v>745.72</v>
+        <v>1501.47</v>
       </c>
       <c r="AE7" t="n">
-        <v>55.9</v>
+        <v>57.4</v>
       </c>
       <c r="AF7" t="n">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>TTM Squeeze | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH7" t="n">
         <v>0.15</v>
       </c>
       <c r="AI7" t="n">
-        <v>49.7</v>
+        <v>35.3</v>
       </c>
       <c r="AJ7" t="n">
-        <v>15.1</v>
+        <v>3.5</v>
       </c>
       <c r="AK7" t="n">
-        <v>20.9</v>
+        <v>12</v>
       </c>
       <c r="AL7" t="n">
         <v>15</v>
       </c>
       <c r="AM7" t="n">
-        <v>758.63</v>
+        <v>1504.26</v>
       </c>
       <c r="AN7" t="n">
-        <v>721.9299999999999</v>
+        <v>1443.79</v>
       </c>
       <c r="AO7" t="inlineStr">
         <is>
-          <t>INDHOTEL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹105,497.68 Cr., a P/E ratio of 49.74, and YoY Revenue Growth of +15.1%, the company demonstrates strong institutional backing, solid operating profit margins (20.87%), and healthy Return on Equity (15.00%).</t>
+          <t>CIPLA operates in the Healthcare sector. With an estimated Market Cap of ₹119,077.56 Cr., a P/E ratio of 35.33, and YoY Revenue Growth of +3.5%, the company demonstrates strong institutional backing, solid operating profit margins (12.01%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP7" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 55.94 (Bullish Momentum Zone), while MACD Line (8.74) trades below Signal (9.07) with an expanding histogram (-0.33). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +7.95% above the 200-day DMA (₹686.49). Daily volatility envelope is bounded by ATR(14) of ₹15.36.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 57.42 (Bullish Momentum Zone), while MACD Line (11.95) trades above Signal (9.52) with an expanding histogram (+2.43). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +4.61% above the 200-day DMA (₹1394.50). Daily volatility envelope is bounded by ATR(14) of ₹34.29.</t>
         </is>
       </c>
       <c r="AQ7" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for INDHOTEL. Current Market Price (₹741.15) is positioned above the 30-day DMA (₹732.20), 50-day DMA (₹710.78), and 200-day DMA (₹686.49). The price distance from 200 DMA is +7.95%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for CIPLA. Current Market Price (₹1,474.00) is positioned above the 30-day DMA (₹1,443.74), 50-day DMA (₹1,420.24), and 200-day DMA (₹1,394.50). The price distance from 200 DMA is +4.61%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR7" t="inlineStr">
         <is>
-          <t>[741.15, 743.37, 745.6, 747.82, 750.04, 752.27]</t>
+          <t>[1474.0, 1478.42, 1482.84, 1487.27, 1491.69, 1496.11]</t>
         </is>
       </c>
       <c r="AS7" t="inlineStr">
         <is>
-          <t>[741.15, 749.52, 754.28, 758.46, 762.33, 766.0]</t>
+          <t>[1474.0, 1492.14, 1502.24, 1511.02, 1519.12, 1526.78]</t>
         </is>
       </c>
       <c r="AT7" t="inlineStr">
         <is>
-          <t>[741.15, 738.77, 739.08, 739.84, 740.83, 741.97]</t>
+          <t>[1474.0, 1468.13, 1468.29, 1469.45, 1471.11, 1473.11]</t>
         </is>
       </c>
       <c r="AU7" t="n">
-        <v>743.61</v>
+        <v>1486.61</v>
       </c>
     </row>
     <row r="8">
@@ -1663,163 +1663,163 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ASIANPAINT</t>
+          <t>RECLTD</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Basic Materials</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>265132.26</v>
+        <v>95665.02</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>2765.7</v>
+        <v>363.3</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>₹2753.78 - ₹2783.58</t>
+          <t>₹361.73 - ₹365.65</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>2813.39</v>
+        <v>369.58</v>
       </c>
       <c r="I8" t="n">
-        <v>2701.3</v>
+        <v>358.57</v>
       </c>
       <c r="J8" t="n">
-        <v>2690.11</v>
+        <v>352.45</v>
       </c>
       <c r="K8" t="n">
-        <v>2579.42</v>
+        <v>347.8</v>
       </c>
       <c r="L8" t="n">
-        <v>7</v>
+        <v>5.23</v>
       </c>
       <c r="M8" t="n">
-        <v>26.48</v>
+        <v>4.61</v>
       </c>
       <c r="N8" t="n">
-        <v>18.67</v>
+        <v>3.76</v>
       </c>
       <c r="O8" t="n">
-        <v>7.81</v>
+        <v>0.85</v>
       </c>
       <c r="P8" t="n">
-        <v>59.61</v>
+        <v>7.85</v>
       </c>
       <c r="Q8" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R8" t="n">
-        <v>52.3</v>
+        <v>41.1</v>
       </c>
       <c r="S8" t="n">
         <v>0.25</v>
       </c>
       <c r="T8" t="n">
-        <v>-1.22</v>
+        <v>-1.68</v>
       </c>
       <c r="U8" t="n">
-        <v>55</v>
+        <v>46.7</v>
       </c>
       <c r="V8" t="n">
-        <v>1.72</v>
+        <v>3.32</v>
       </c>
       <c r="W8" t="n">
         <v>-0.77</v>
       </c>
       <c r="X8" t="n">
-        <v>2708.82</v>
+        <v>357.14</v>
       </c>
       <c r="Y8" t="n">
-        <v>2790.13</v>
+        <v>363.46</v>
       </c>
       <c r="Z8" t="n">
-        <v>2786.83</v>
+        <v>363.46</v>
       </c>
       <c r="AA8" t="n">
-        <v>2676.28</v>
+        <v>351.53</v>
       </c>
       <c r="AB8" t="n">
-        <v>2772.57</v>
+        <v>363.97</v>
       </c>
       <c r="AC8" t="n">
-        <v>2781.14</v>
+        <v>366.34</v>
       </c>
       <c r="AD8" t="n">
-        <v>2796.57</v>
+        <v>369.37</v>
       </c>
       <c r="AE8" t="n">
-        <v>63.3</v>
+        <v>73</v>
       </c>
       <c r="AF8" t="n">
-        <v>0.05</v>
+        <v>0.19</v>
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>Strong RSI | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH8" t="n">
         <v>0.15</v>
       </c>
       <c r="AI8" t="n">
-        <v>56</v>
+        <v>6</v>
       </c>
       <c r="AJ8" t="n">
-        <v>17.9</v>
+        <v>25.2</v>
       </c>
       <c r="AK8" t="n">
-        <v>12.8</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="AL8" t="n">
         <v>15</v>
       </c>
       <c r="AM8" t="n">
-        <v>2834.02</v>
+        <v>373.08</v>
       </c>
       <c r="AN8" t="n">
-        <v>2700.29</v>
+        <v>353.8</v>
       </c>
       <c r="AO8" t="inlineStr">
         <is>
-          <t>ASIANPAINT operates in the Basic Materials sector. With an estimated Market Cap of ₹265,132.26 Cr., a P/E ratio of 55.99, and YoY Revenue Growth of +17.9%, the company demonstrates strong institutional backing, solid operating profit margins (12.81%), and healthy Return on Equity (15.00%).</t>
+          <t>RECLTD operates in the Financial Services sector. With an estimated Market Cap of ₹95,665.02 Cr., a P/E ratio of 6.01, and YoY Revenue Growth of +25.2%, the company demonstrates strong institutional backing, solid operating profit margins (68.89%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP8" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 63.35 (Bullish Momentum Zone), while MACD Line (26.48) trades above Signal (18.67) with an expanding histogram (+7.81). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +7.00% above the 200-day DMA (₹2579.42). Daily volatility envelope is bounded by ATR(14) of ₹59.61.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 73.01 (Bullish Momentum Zone), while MACD Line (4.61) trades above Signal (3.76) with an expanding histogram (+0.85). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +5.23% above the 200-day DMA (₹347.80). Daily volatility envelope is bounded by ATR(14) of ₹7.85.</t>
         </is>
       </c>
       <c r="AQ8" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ASIANPAINT. Current Market Price (₹2,765.70) is positioned above the 30-day DMA (₹2,701.30), 50-day DMA (₹2,690.11), and 200-day DMA (₹2,579.42). The price distance from 200 DMA is +7.00%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for RECLTD. Current Market Price (₹363.30) is positioned above the 30-day DMA (₹358.57), 50-day DMA (₹352.45), and 200-day DMA (₹347.80). The price distance from 200 DMA is +5.23%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR8" t="inlineStr">
         <is>
-          <t>[2765.7, 2774.0, 2782.29, 2790.59, 2798.89, 2807.19]</t>
+          <t>[363.3, 364.39, 365.48, 366.57, 367.66, 368.75]</t>
         </is>
       </c>
       <c r="AS8" t="inlineStr">
         <is>
-          <t>[2765.7, 2797.84, 2816.02, 2831.89, 2846.58, 2860.51]</t>
+          <t>[363.3, 367.53, 369.92, 372.01, 373.94, 375.77]</t>
         </is>
       </c>
       <c r="AT8" t="inlineStr">
         <is>
-          <t>[2765.7, 2756.11, 2757.0, 2759.61, 2763.12, 2767.19]</t>
+          <t>[363.3, 362.04, 362.15, 362.49, 362.95, 363.48]</t>
         </is>
       </c>
       <c r="AU8" t="n">
-        <v>2786.83</v>
+        <v>363.46</v>
       </c>
     </row>
     <row r="9">
@@ -1839,7 +1839,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>334115.08</v>
+        <v>333571</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1847,15 +1847,15 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2087.9</v>
+        <v>2084.5</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>₹2078.51 - ₹2101.98</t>
+          <t>₹2075.11 - ₹2098.58</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>2125.45</v>
+        <v>2122.05</v>
       </c>
       <c r="I9" t="n">
         <v>1891.66</v>
@@ -1882,19 +1882,19 @@
         <v>46.94</v>
       </c>
       <c r="Q9" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R9" t="n">
-        <v>46.6</v>
+        <v>42.8</v>
       </c>
       <c r="S9" t="n">
         <v>0.24</v>
       </c>
       <c r="T9" t="n">
-        <v>-1.43</v>
+        <v>-1.69</v>
       </c>
       <c r="U9" t="n">
-        <v>48.3</v>
+        <v>46.7</v>
       </c>
       <c r="V9" t="n">
         <v>5.23</v>
@@ -1903,25 +1903,25 @@
         <v>-0.77</v>
       </c>
       <c r="X9" t="n">
-        <v>2050.2</v>
+        <v>2062.42</v>
       </c>
       <c r="Y9" t="n">
-        <v>2111.55</v>
+        <v>2111.77</v>
       </c>
       <c r="Z9" t="n">
-        <v>2081.03</v>
+        <v>2111.77</v>
       </c>
       <c r="AA9" t="n">
-        <v>2017.5</v>
+        <v>2014.1</v>
       </c>
       <c r="AB9" t="n">
-        <v>2082.6</v>
+        <v>2085.37</v>
       </c>
       <c r="AC9" t="n">
-        <v>2096.6</v>
+        <v>2102.14</v>
       </c>
       <c r="AD9" t="n">
-        <v>2105.3</v>
+        <v>2119.77</v>
       </c>
       <c r="AE9" t="n">
         <v>81.2</v>
@@ -1931,14 +1931,14 @@
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH9" t="n">
         <v>0.15</v>
       </c>
       <c r="AI9" t="n">
-        <v>33.1</v>
+        <v>33.3</v>
       </c>
       <c r="AJ9" t="n">
         <v>19.3</v>
@@ -1950,14 +1950,14 @@
         <v>15</v>
       </c>
       <c r="AM9" t="n">
-        <v>2140.84</v>
+        <v>2135.58</v>
       </c>
       <c r="AN9" t="n">
-        <v>2040.86</v>
+        <v>2031.52</v>
       </c>
       <c r="AO9" t="inlineStr">
         <is>
-          <t>BAJAJFINSV operates in the Financial Services sector. With an estimated Market Cap of ₹334,115.08 Cr., a P/E ratio of 33.09, and YoY Revenue Growth of +19.3%, the company demonstrates strong institutional backing, solid operating profit margins (6.47%), and healthy Return on Equity (15.00%).</t>
+          <t>BAJAJFINSV operates in the Financial Services sector. With an estimated Market Cap of ₹333,571.00 Cr., a P/E ratio of 33.31, and YoY Revenue Growth of +19.3%, the company demonstrates strong institutional backing, solid operating profit margins (6.47%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP9" t="inlineStr">
@@ -1967,26 +1967,26 @@
       </c>
       <c r="AQ9" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for BAJAJFINSV. Current Market Price (₹2,087.90) is positioned above the 30-day DMA (₹1,891.66), 50-day DMA (₹1,829.95), and 200-day DMA (₹1,912.06). The price distance from 200 DMA is +9.10%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for BAJAJFINSV. Current Market Price (₹2,084.50) is positioned above the 30-day DMA (₹1,891.66), 50-day DMA (₹1,829.95), and 200-day DMA (₹1,912.06). The price distance from 200 DMA is +9.10%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR9" t="inlineStr">
         <is>
-          <t>[2087.9, 2094.16, 2100.43, 2106.69, 2112.95, 2119.22]</t>
+          <t>[2084.5, 2090.75, 2097.01, 2103.26, 2109.51, 2115.77]</t>
         </is>
       </c>
       <c r="AS9" t="inlineStr">
         <is>
-          <t>[2087.9, 2112.94, 2126.98, 2139.21, 2150.5, 2161.2]</t>
+          <t>[2084.5, 2109.53, 2123.56, 2135.78, 2147.06, 2157.75]</t>
         </is>
       </c>
       <c r="AT9" t="inlineStr">
         <is>
-          <t>[2087.9, 2080.08, 2080.51, 2082.3, 2084.79, 2087.73]</t>
+          <t>[2084.5, 2076.67, 2077.09, 2078.87, 2081.35, 2084.28]</t>
         </is>
       </c>
       <c r="AU9" t="n">
-        <v>2081.03</v>
+        <v>2111.77</v>
       </c>
     </row>
     <row r="10">
@@ -1997,163 +1997,163 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>TECHM</t>
+          <t>M&amp;M</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>146758.62</v>
+        <v>409940.24</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>1656.7</v>
+        <v>3414</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>₹1648.28 - ₹1669.32</t>
+          <t>₹3396.85 - ₹3439.73</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>1690.36</v>
+        <v>3482.62</v>
       </c>
       <c r="I10" t="n">
-        <v>1512.55</v>
+        <v>3192.86</v>
       </c>
       <c r="J10" t="n">
-        <v>1479.9</v>
+        <v>3121.8</v>
       </c>
       <c r="K10" t="n">
-        <v>1463.61</v>
+        <v>3329.31</v>
       </c>
       <c r="L10" t="n">
-        <v>12.74</v>
+        <v>3.79</v>
       </c>
       <c r="M10" t="n">
-        <v>56.87</v>
+        <v>82.2</v>
       </c>
       <c r="N10" t="n">
-        <v>51.52</v>
+        <v>55.88</v>
       </c>
       <c r="O10" t="n">
-        <v>5.35</v>
+        <v>26.32</v>
       </c>
       <c r="P10" t="n">
-        <v>42.08</v>
+        <v>85.77</v>
       </c>
       <c r="Q10" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R10" t="n">
-        <v>52.3</v>
+        <v>47.3</v>
       </c>
       <c r="S10" t="n">
-        <v>0.23</v>
+        <v>0.21</v>
       </c>
       <c r="T10" t="n">
-        <v>-1.48</v>
+        <v>-1.72</v>
       </c>
       <c r="U10" t="n">
-        <v>51.7</v>
+        <v>53.3</v>
       </c>
       <c r="V10" t="n">
-        <v>7.51</v>
+        <v>3.48</v>
       </c>
       <c r="W10" t="n">
         <v>-0.77</v>
       </c>
       <c r="X10" t="n">
-        <v>1648.16</v>
+        <v>3348.98</v>
       </c>
       <c r="Y10" t="n">
-        <v>1696.73</v>
+        <v>3436.39</v>
       </c>
       <c r="Z10" t="n">
-        <v>1681.95</v>
+        <v>3436.39</v>
       </c>
       <c r="AA10" t="n">
-        <v>1593.58</v>
+        <v>3285.34</v>
       </c>
       <c r="AB10" t="n">
-        <v>1659.3</v>
+        <v>3424.33</v>
       </c>
       <c r="AC10" t="n">
-        <v>1667.4</v>
+        <v>3438.66</v>
       </c>
       <c r="AD10" t="n">
-        <v>1678.1</v>
+        <v>3463.33</v>
       </c>
       <c r="AE10" t="n">
-        <v>81.5</v>
+        <v>75.8</v>
       </c>
       <c r="AF10" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.12</v>
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH10" t="n">
         <v>0.15</v>
       </c>
       <c r="AI10" t="n">
-        <v>28.6</v>
+        <v>20.6</v>
       </c>
       <c r="AJ10" t="n">
-        <v>17.7</v>
+        <v>27.5</v>
       </c>
       <c r="AK10" t="n">
-        <v>8.699999999999999</v>
+        <v>8.6</v>
       </c>
       <c r="AL10" t="n">
         <v>15</v>
       </c>
       <c r="AM10" t="n">
-        <v>1700.95</v>
+        <v>3511.31</v>
       </c>
       <c r="AN10" t="n">
-        <v>1614.18</v>
+        <v>3317.13</v>
       </c>
       <c r="AO10" t="inlineStr">
         <is>
-          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹146,758.62 Cr., a P/E ratio of 28.60, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
+          <t>M&amp;M operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹409,940.24 Cr., a P/E ratio of 20.63, and YoY Revenue Growth of +27.5%, the company demonstrates strong institutional backing, solid operating profit margins (8.61%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP10" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 81.48 (Bullish Momentum Zone), while MACD Line (56.87) trades above Signal (51.52) with an expanding histogram (+5.35). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +12.74% above the 200-day DMA (₹1463.61). Daily volatility envelope is bounded by ATR(14) of ₹42.08.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 75.84 (Bullish Momentum Zone), while MACD Line (82.20) trades above Signal (55.88) with an expanding histogram (+26.32). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +3.79% above the 200-day DMA (₹3329.31). Daily volatility envelope is bounded by ATR(14) of ₹85.77.</t>
         </is>
       </c>
       <c r="AQ10" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,656.70) is positioned above the 30-day DMA (₹1,512.55), 50-day DMA (₹1,479.90), and 200-day DMA (₹1,463.61). The price distance from 200 DMA is +12.74%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for M&amp;M. Current Market Price (₹3,414.00) is positioned above the 30-day DMA (₹3,192.86), 50-day DMA (₹3,121.80), and 200-day DMA (₹3,329.31). The price distance from 200 DMA is +3.79%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR10" t="inlineStr">
         <is>
-          <t>[1656.7, 1671.0, 1685.31, 1699.61, 1713.91, 1728.22]</t>
+          <t>[3414.0, 3424.24, 3434.48, 3444.73, 3454.97, 3465.21]</t>
         </is>
       </c>
       <c r="AS10" t="inlineStr">
         <is>
-          <t>[1656.7, 1687.83, 1709.11, 1728.76, 1747.58, 1765.85]</t>
+          <t>[3414.0, 3458.55, 3483.0, 3504.15, 3523.59, 3541.93]</t>
         </is>
       </c>
       <c r="AT10" t="inlineStr">
         <is>
-          <t>[1656.7, 1658.38, 1667.45, 1677.74, 1688.67, 1699.99]</t>
+          <t>[3414.0, 3398.51, 3398.09, 3400.16, 3403.51, 3407.67]</t>
         </is>
       </c>
       <c r="AU10" t="n">
-        <v>1681.95</v>
+        <v>3436.39</v>
       </c>
     </row>
     <row r="11">
@@ -2164,16 +2164,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CIPLA</t>
+          <t>TECHM</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Healthcare</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>119392.62</v>
+        <v>144836.34</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2181,146 +2181,146 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1477.9</v>
+        <v>1635</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>₹1471.04 - ₹1488.19</t>
+          <t>₹1626.58 - ₹1647.62</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>1505.33</v>
+        <v>1668.66</v>
       </c>
       <c r="I11" t="n">
-        <v>1443.74</v>
+        <v>1512.55</v>
       </c>
       <c r="J11" t="n">
-        <v>1420.24</v>
+        <v>1479.9</v>
       </c>
       <c r="K11" t="n">
-        <v>1394.5</v>
+        <v>1463.61</v>
       </c>
       <c r="L11" t="n">
-        <v>4.61</v>
+        <v>12.74</v>
       </c>
       <c r="M11" t="n">
-        <v>11.95</v>
+        <v>56.87</v>
       </c>
       <c r="N11" t="n">
-        <v>9.52</v>
+        <v>51.52</v>
       </c>
       <c r="O11" t="n">
-        <v>2.43</v>
+        <v>5.35</v>
       </c>
       <c r="P11" t="n">
-        <v>34.29</v>
+        <v>42.08</v>
       </c>
       <c r="Q11" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R11" t="n">
-        <v>48</v>
+        <v>45.2</v>
       </c>
       <c r="S11" t="n">
-        <v>0.23</v>
+        <v>0.21</v>
       </c>
       <c r="T11" t="n">
-        <v>-1.53</v>
+        <v>-1.75</v>
       </c>
       <c r="U11" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="V11" t="n">
-        <v>10.14</v>
+        <v>7.51</v>
       </c>
       <c r="W11" t="n">
         <v>-0.77</v>
       </c>
       <c r="X11" t="n">
-        <v>1439.03</v>
+        <v>1635</v>
       </c>
       <c r="Y11" t="n">
-        <v>1485.03</v>
+        <v>1662.3</v>
       </c>
       <c r="Z11" t="n">
-        <v>1485.03</v>
+        <v>1606.52</v>
       </c>
       <c r="AA11" t="n">
-        <v>1426.46</v>
+        <v>1571.88</v>
       </c>
       <c r="AB11" t="n">
-        <v>1473.27</v>
+        <v>1645.33</v>
       </c>
       <c r="AC11" t="n">
-        <v>1485.54</v>
+        <v>1659.66</v>
       </c>
       <c r="AD11" t="n">
-        <v>1493.17</v>
+        <v>1684.33</v>
       </c>
       <c r="AE11" t="n">
-        <v>57.4</v>
+        <v>81.5</v>
       </c>
       <c r="AF11" t="n">
-        <v>0.04</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>TTM Squeeze | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH11" t="n">
         <v>0.15</v>
       </c>
       <c r="AI11" t="n">
-        <v>35.4</v>
+        <v>28.2</v>
       </c>
       <c r="AJ11" t="n">
-        <v>3.5</v>
+        <v>17.7</v>
       </c>
       <c r="AK11" t="n">
-        <v>12</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="AL11" t="n">
         <v>15</v>
       </c>
       <c r="AM11" t="n">
-        <v>1508.5</v>
+        <v>1679.93</v>
       </c>
       <c r="AN11" t="n">
-        <v>1446.8</v>
+        <v>1591.42</v>
       </c>
       <c r="AO11" t="inlineStr">
         <is>
-          <t>CIPLA operates in the Healthcare sector. With an estimated Market Cap of ₹119,392.62 Cr., a P/E ratio of 35.42, and YoY Revenue Growth of +3.5%, the company demonstrates strong institutional backing, solid operating profit margins (12.01%), and healthy Return on Equity (15.00%).</t>
+          <t>TECHM operates in the Technology sector. With an estimated Market Cap of ₹144,836.34 Cr., a P/E ratio of 28.23, and YoY Revenue Growth of +17.7%, the company demonstrates strong institutional backing, solid operating profit margins (8.68%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP11" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 57.42 (Bullish Momentum Zone), while MACD Line (11.95) trades above Signal (9.52) with an expanding histogram (+2.43). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +4.61% above the 200-day DMA (₹1394.50). Daily volatility envelope is bounded by ATR(14) of ₹34.29.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 81.48 (Bullish Momentum Zone), while MACD Line (56.87) trades above Signal (51.52) with an expanding histogram (+5.35). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +12.74% above the 200-day DMA (₹1463.61). Daily volatility envelope is bounded by ATR(14) of ₹42.08.</t>
         </is>
       </c>
       <c r="AQ11" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for CIPLA. Current Market Price (₹1,477.90) is positioned above the 30-day DMA (₹1,443.74), 50-day DMA (₹1,420.24), and 200-day DMA (₹1,394.50). The price distance from 200 DMA is +4.61%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for TECHM. Current Market Price (₹1,635.00) is positioned above the 30-day DMA (₹1,512.55), 50-day DMA (₹1,479.90), and 200-day DMA (₹1,463.61). The price distance from 200 DMA is +12.74%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR11" t="inlineStr">
         <is>
-          <t>[1477.9, 1482.33, 1486.77, 1491.2, 1495.63, 1500.07]</t>
+          <t>[1635.0, 1645.63, 1656.26, 1666.89, 1677.52, 1688.14]</t>
         </is>
       </c>
       <c r="AS11" t="inlineStr">
         <is>
-          <t>[1477.9, 1496.05, 1506.17, 1514.96, 1523.07, 1530.74]</t>
+          <t>[1635.0, 1662.46, 1680.06, 1696.04, 1711.18, 1725.78]</t>
         </is>
       </c>
       <c r="AT11" t="inlineStr">
         <is>
-          <t>[1477.9, 1472.05, 1472.22, 1473.38, 1475.06, 1477.06]</t>
+          <t>[1635.0, 1633.01, 1638.41, 1645.02, 1652.27, 1659.92]</t>
         </is>
       </c>
       <c r="AU11" t="n">
-        <v>1485.03</v>
+        <v>1606.52</v>
       </c>
     </row>
     <row r="12">
@@ -2331,163 +2331,163 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PERSISTENT</t>
+          <t>INDIGO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Industrials</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>86255.14999999999</v>
+        <v>206093.29</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>5521</v>
+        <v>5330</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>₹5485.82 - ₹5573.78</t>
+          <t>₹5301.71 - ₹5372.43</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>5661.74</v>
+        <v>5443.14</v>
       </c>
       <c r="I12" t="n">
-        <v>5032.34</v>
+        <v>5278.02</v>
       </c>
       <c r="J12" t="n">
-        <v>5021.77</v>
+        <v>5043.87</v>
       </c>
       <c r="K12" t="n">
-        <v>5453.52</v>
+        <v>4940.92</v>
       </c>
       <c r="L12" t="n">
-        <v>1.22</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="M12" t="n">
-        <v>172.8</v>
+        <v>66.64</v>
       </c>
       <c r="N12" t="n">
-        <v>139.73</v>
+        <v>59.95</v>
       </c>
       <c r="O12" t="n">
-        <v>33.07</v>
+        <v>6.69</v>
       </c>
       <c r="P12" t="n">
-        <v>175.92</v>
+        <v>141.43</v>
       </c>
       <c r="Q12" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R12" t="n">
-        <v>57.1</v>
+        <v>46.7</v>
       </c>
       <c r="S12" t="n">
-        <v>0.17</v>
+        <v>0.2</v>
       </c>
       <c r="T12" t="n">
-        <v>-1.59</v>
+        <v>-1.87</v>
       </c>
       <c r="U12" t="n">
-        <v>61.7</v>
+        <v>50</v>
       </c>
       <c r="V12" t="n">
-        <v>7.78</v>
+        <v>5.71</v>
       </c>
       <c r="W12" t="n">
         <v>-0.77</v>
       </c>
       <c r="X12" t="n">
-        <v>5347.92</v>
+        <v>5328.45</v>
       </c>
       <c r="Y12" t="n">
-        <v>5510.56</v>
+        <v>5414.12</v>
       </c>
       <c r="Z12" t="n">
-        <v>5502.84</v>
+        <v>5326.11</v>
       </c>
       <c r="AA12" t="n">
-        <v>5257.12</v>
+        <v>5117.86</v>
       </c>
       <c r="AB12" t="n">
-        <v>5526.67</v>
+        <v>5356.33</v>
       </c>
       <c r="AC12" t="n">
-        <v>5566.34</v>
+        <v>5397.66</v>
       </c>
       <c r="AD12" t="n">
-        <v>5611.67</v>
+        <v>5465.33</v>
       </c>
       <c r="AE12" t="n">
-        <v>72.5</v>
+        <v>55.9</v>
       </c>
       <c r="AF12" t="n">
-        <v>0.17</v>
+        <v>0.28</v>
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH12" t="n">
         <v>0.15</v>
       </c>
       <c r="AI12" t="n">
-        <v>46.3</v>
+        <v>23.4</v>
       </c>
       <c r="AJ12" t="n">
-        <v>29.1</v>
+        <v>6.2</v>
       </c>
       <c r="AK12" t="n">
-        <v>12.2</v>
+        <v>3.8</v>
       </c>
       <c r="AL12" t="n">
         <v>15</v>
       </c>
       <c r="AM12" t="n">
-        <v>5725.55</v>
+        <v>5514.27</v>
       </c>
       <c r="AN12" t="n">
-        <v>5323.6</v>
+        <v>5143.39</v>
       </c>
       <c r="AO12" t="inlineStr">
         <is>
-          <t>PERSISTENT operates in the Technology sector. With an estimated Market Cap of ₹86,255.15 Cr., a P/E ratio of 46.31, and YoY Revenue Growth of +29.1%, the company demonstrates strong institutional backing, solid operating profit margins (12.24%), and healthy Return on Equity (15.00%).</t>
+          <t>INDIGO operates in the Industrials sector. With an estimated Market Cap of ₹206,093.29 Cr., a P/E ratio of 23.39, and YoY Revenue Growth of +6.2%, the company demonstrates strong institutional backing, solid operating profit margins (3.79%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP12" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 72.50 (Bullish Momentum Zone), while MACD Line (172.80) trades above Signal (139.73) with an expanding histogram (+33.07). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +1.22% above the 200-day DMA (₹5453.52). Daily volatility envelope is bounded by ATR(14) of ₹175.92.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 55.89 (Bullish Momentum Zone), while MACD Line (66.64) trades above Signal (59.95) with an expanding histogram (+6.69). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +9.29% above the 200-day DMA (₹4940.92). Daily volatility envelope is bounded by ATR(14) of ₹141.43.</t>
         </is>
       </c>
       <c r="AQ12" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PERSISTENT. Current Market Price (₹5,521.00) is positioned above the 30-day DMA (₹5,032.34), 50-day DMA (₹5,021.77), and 200-day DMA (₹5,453.52). The price distance from 200 DMA is +1.22%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for INDIGO. Current Market Price (₹5,330.00) is positioned above the 30-day DMA (₹5,278.02), 50-day DMA (₹5,043.87), and 200-day DMA (₹4,940.92). The price distance from 200 DMA is +9.29%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR12" t="inlineStr">
         <is>
-          <t>[5521.0, 5537.56, 5554.13, 5570.69, 5587.25, 5603.81]</t>
+          <t>[5330.0, 5359.72, 5389.45, 5419.17, 5448.9, 5478.62]</t>
         </is>
       </c>
       <c r="AS12" t="inlineStr">
         <is>
-          <t>[5521.0, 5607.93, 5653.64, 5692.57, 5727.99, 5761.16]</t>
+          <t>[5330.0, 5416.3, 5469.45, 5517.16, 5562.04, 5605.12]</t>
         </is>
       </c>
       <c r="AT12" t="inlineStr">
         <is>
-          <t>[5521.0, 5484.79, 5479.49, 5479.28, 5481.7, 5485.81]</t>
+          <t>[5330.0, 5317.3, 5329.45, 5345.68, 5364.04, 5383.75]</t>
         </is>
       </c>
       <c r="AU12" t="n">
-        <v>5502.84</v>
+        <v>5326.11</v>
       </c>
     </row>
     <row r="13">
@@ -2507,7 +2507,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>39329.95</v>
+        <v>38956.76</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2515,15 +2515,15 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>516.4</v>
+        <v>511.5</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>₹513.74 - ₹520.4</t>
+          <t>₹508.84 - ₹515.5</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>527.05</v>
+        <v>522.15</v>
       </c>
       <c r="I13" t="n">
         <v>487.98</v>
@@ -2550,46 +2550,46 @@
         <v>13.32</v>
       </c>
       <c r="Q13" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R13" t="n">
-        <v>47</v>
+        <v>45.3</v>
       </c>
       <c r="S13" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="T13" t="n">
-        <v>-1.67</v>
+        <v>-1.89</v>
       </c>
       <c r="U13" t="n">
-        <v>48.3</v>
+        <v>46.7</v>
       </c>
       <c r="V13" t="n">
-        <v>6.69</v>
+        <v>6.67</v>
       </c>
       <c r="W13" t="n">
         <v>-0.77</v>
       </c>
       <c r="X13" t="n">
-        <v>501.03</v>
+        <v>500.09</v>
       </c>
       <c r="Y13" t="n">
-        <v>514.7</v>
+        <v>511.75</v>
       </c>
       <c r="Z13" t="n">
-        <v>514.7</v>
+        <v>511.75</v>
       </c>
       <c r="AA13" t="n">
-        <v>496.42</v>
+        <v>491.52</v>
       </c>
       <c r="AB13" t="n">
-        <v>517.0700000000001</v>
+        <v>514.5</v>
       </c>
       <c r="AC13" t="n">
-        <v>519.1900000000001</v>
+        <v>519</v>
       </c>
       <c r="AD13" t="n">
-        <v>521.97</v>
+        <v>526.5</v>
       </c>
       <c r="AE13" t="n">
         <v>64.3</v>
@@ -2599,14 +2599,14 @@
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH13" t="n">
         <v>0.15</v>
       </c>
       <c r="AI13" t="n">
-        <v>31.4</v>
+        <v>31.2</v>
       </c>
       <c r="AJ13" t="n">
         <v>0.3</v>
@@ -2618,14 +2618,14 @@
         <v>15</v>
       </c>
       <c r="AM13" t="n">
-        <v>529.9400000000001</v>
+        <v>523.74</v>
       </c>
       <c r="AN13" t="n">
-        <v>501.83</v>
+        <v>498.99</v>
       </c>
       <c r="AO13" t="inlineStr">
         <is>
-          <t>CONCOR operates in the Industrials sector. With an estimated Market Cap of ₹39,329.95 Cr., a P/E ratio of 31.45, and YoY Revenue Growth of +0.3%, the company demonstrates strong institutional backing, solid operating profit margins (13.67%), and healthy Return on Equity (15.00%).</t>
+          <t>CONCOR operates in the Industrials sector. With an estimated Market Cap of ₹38,956.76 Cr., a P/E ratio of 31.15, and YoY Revenue Growth of +0.3%, the company demonstrates strong institutional backing, solid operating profit margins (13.67%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP13" t="inlineStr">
@@ -2635,26 +2635,26 @@
       </c>
       <c r="AQ13" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for CONCOR. Current Market Price (₹516.40) is positioned above the 30-day DMA (₹487.98), 50-day DMA (₹476.36), and 200-day DMA (₹494.06). The price distance from 200 DMA is +4.51%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for CONCOR. Current Market Price (₹511.50) is positioned above the 30-day DMA (₹487.98), 50-day DMA (₹476.36), and 200-day DMA (₹494.06). The price distance from 200 DMA is +4.51%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR13" t="inlineStr">
         <is>
-          <t>[516.4, 517.95, 519.5, 521.05, 522.6, 524.15]</t>
+          <t>[511.5, 513.03, 514.57, 516.1, 517.64, 519.17]</t>
         </is>
       </c>
       <c r="AS13" t="inlineStr">
         <is>
-          <t>[516.4, 523.28, 527.03, 530.27, 533.25, 536.06]</t>
+          <t>[511.5, 518.36, 522.1, 525.33, 528.29, 531.08]</t>
         </is>
       </c>
       <c r="AT13" t="inlineStr">
         <is>
-          <t>[516.4, 513.95, 513.85, 514.13, 514.61, 515.21]</t>
+          <t>[511.5, 509.04, 508.92, 509.18, 509.65, 510.24]</t>
         </is>
       </c>
       <c r="AU13" t="n">
-        <v>514.7</v>
+        <v>511.75</v>
       </c>
     </row>
     <row r="14">
@@ -2665,163 +2665,163 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RECLTD</t>
+          <t>PERSISTENT</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>25000</v>
+        <v>85520.87</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>🔴 AVOID / HOLD</t>
+          <t>🟡 MODERATE BUY</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>364.65</v>
+        <v>5474</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>₹363.08 - ₹367.0</t>
+          <t>₹5438.82 - ₹5526.78</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>370.93</v>
+        <v>5614.74</v>
       </c>
       <c r="I14" t="n">
-        <v>358.57</v>
+        <v>5032.34</v>
       </c>
       <c r="J14" t="n">
-        <v>352.45</v>
+        <v>5021.77</v>
       </c>
       <c r="K14" t="n">
-        <v>347.8</v>
+        <v>5453.52</v>
       </c>
       <c r="L14" t="n">
-        <v>5.23</v>
+        <v>1.22</v>
       </c>
       <c r="M14" t="n">
-        <v>4.61</v>
+        <v>172.8</v>
       </c>
       <c r="N14" t="n">
-        <v>3.76</v>
+        <v>139.73</v>
       </c>
       <c r="O14" t="n">
-        <v>0.85</v>
+        <v>33.07</v>
       </c>
       <c r="P14" t="n">
-        <v>7.85</v>
+        <v>175.92</v>
       </c>
       <c r="Q14" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R14" t="n">
-        <v>40.9</v>
+        <v>53.8</v>
       </c>
       <c r="S14" t="n">
-        <v>0.25</v>
+        <v>0.17</v>
       </c>
       <c r="T14" t="n">
-        <v>-1.68</v>
+        <v>-1.94</v>
       </c>
       <c r="U14" t="n">
-        <v>46.7</v>
+        <v>60</v>
       </c>
       <c r="V14" t="n">
-        <v>3.33</v>
+        <v>7.78</v>
       </c>
       <c r="W14" t="n">
         <v>-0.77</v>
       </c>
       <c r="X14" t="n">
-        <v>355.66</v>
+        <v>5334.6</v>
       </c>
       <c r="Y14" t="n">
-        <v>365.75</v>
+        <v>5486.56</v>
       </c>
       <c r="Z14" t="n">
-        <v>365.75</v>
+        <v>5486.56</v>
       </c>
       <c r="AA14" t="n">
-        <v>352.88</v>
+        <v>5210.12</v>
       </c>
       <c r="AB14" t="n">
-        <v>365.08</v>
+        <v>5503.67</v>
       </c>
       <c r="AC14" t="n">
-        <v>366.56</v>
+        <v>5542.34</v>
       </c>
       <c r="AD14" t="n">
-        <v>368.48</v>
+        <v>5610.67</v>
       </c>
       <c r="AE14" t="n">
-        <v>73</v>
+        <v>72.5</v>
       </c>
       <c r="AF14" t="n">
-        <v>0.19</v>
+        <v>0.17</v>
       </c>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH14" t="n">
         <v>0.15</v>
       </c>
       <c r="AI14" t="n">
-        <v>6</v>
+        <v>46.1</v>
       </c>
       <c r="AJ14" t="n">
-        <v>25.2</v>
+        <v>29.1</v>
       </c>
       <c r="AK14" t="n">
-        <v>68.90000000000001</v>
+        <v>12.2</v>
       </c>
       <c r="AL14" t="n">
         <v>15</v>
       </c>
       <c r="AM14" t="n">
-        <v>374.1</v>
+        <v>5654.79</v>
       </c>
       <c r="AN14" t="n">
-        <v>354.24</v>
+        <v>5279.49</v>
       </c>
       <c r="AO14" t="inlineStr">
         <is>
-          <t>RECLTD operates in the Financial Services sector. With an estimated Market Cap of ₹25,000.00 Cr., a P/E ratio of 6.03, and YoY Revenue Growth of +25.2%, the company demonstrates strong institutional backing, solid operating profit margins (68.89%), and healthy Return on Equity (15.00%).</t>
+          <t>PERSISTENT operates in the Technology sector. With an estimated Market Cap of ₹85,520.87 Cr., a P/E ratio of 46.10, and YoY Revenue Growth of +29.1%, the company demonstrates strong institutional backing, solid operating profit margins (12.24%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP14" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 73.01 (Bullish Momentum Zone), while MACD Line (4.61) trades above Signal (3.76) with an expanding histogram (+0.85). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +5.23% above the 200-day DMA (₹347.80). Daily volatility envelope is bounded by ATR(14) of ₹7.85.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 72.50 (Bullish Momentum Zone), while MACD Line (172.80) trades above Signal (139.73) with an expanding histogram (+33.07). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +1.22% above the 200-day DMA (₹5453.52). Daily volatility envelope is bounded by ATR(14) of ₹175.92.</t>
         </is>
       </c>
       <c r="AQ14" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for RECLTD. Current Market Price (₹364.65) is positioned above the 30-day DMA (₹358.57), 50-day DMA (₹352.45), and 200-day DMA (₹347.80). The price distance from 200 DMA is +5.23%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PERSISTENT. Current Market Price (₹5,474.00) is positioned above the 30-day DMA (₹5,032.34), 50-day DMA (₹5,021.77), and 200-day DMA (₹5,453.52). The price distance from 200 DMA is +1.22%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR14" t="inlineStr">
         <is>
-          <t>[364.65, 365.74, 366.84, 367.93, 369.03, 370.12]</t>
+          <t>[5474.0, 5490.42, 5506.84, 5523.27, 5539.69, 5556.11]</t>
         </is>
       </c>
       <c r="AS14" t="inlineStr">
         <is>
-          <t>[364.65, 368.88, 371.28, 373.37, 375.31, 377.14]</t>
+          <t>[5474.0, 5560.79, 5606.36, 5645.15, 5680.42, 5713.46]</t>
         </is>
       </c>
       <c r="AT14" t="inlineStr">
         <is>
-          <t>[364.65, 363.39, 363.51, 363.85, 364.32, 364.85]</t>
+          <t>[5474.0, 5437.65, 5432.21, 5431.86, 5434.14, 5438.1]</t>
         </is>
       </c>
       <c r="AU14" t="n">
-        <v>365.75</v>
+        <v>5486.56</v>
       </c>
     </row>
     <row r="15">
@@ -2832,16 +2832,16 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>M&amp;M</t>
+          <t>CAMS</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>411417.18</v>
+        <v>19850.15</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2849,146 +2849,146 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>3426.3</v>
+        <v>799.45</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>₹3409.15 - ₹3452.03</t>
+          <t>₹795.09 - ₹806.0</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>3494.92</v>
+        <v>816.91</v>
       </c>
       <c r="I15" t="n">
-        <v>3192.86</v>
+        <v>781.22</v>
       </c>
       <c r="J15" t="n">
-        <v>3121.8</v>
+        <v>778.4299999999999</v>
       </c>
       <c r="K15" t="n">
-        <v>3329.31</v>
+        <v>742.8099999999999</v>
       </c>
       <c r="L15" t="n">
-        <v>3.79</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="M15" t="n">
-        <v>82.2</v>
+        <v>7.2</v>
       </c>
       <c r="N15" t="n">
-        <v>55.88</v>
+        <v>2.85</v>
       </c>
       <c r="O15" t="n">
-        <v>26.32</v>
+        <v>4.35</v>
       </c>
       <c r="P15" t="n">
-        <v>85.77</v>
+        <v>21.82</v>
       </c>
       <c r="Q15" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R15" t="n">
-        <v>44</v>
+        <v>46.6</v>
       </c>
       <c r="S15" t="n">
-        <v>0.21</v>
+        <v>0.2</v>
       </c>
       <c r="T15" t="n">
-        <v>-1.75</v>
+        <v>-1.94</v>
       </c>
       <c r="U15" t="n">
-        <v>53.3</v>
+        <v>50</v>
       </c>
       <c r="V15" t="n">
-        <v>3.48</v>
+        <v>6.74</v>
       </c>
       <c r="W15" t="n">
         <v>-0.77</v>
       </c>
       <c r="X15" t="n">
-        <v>3336.69</v>
+        <v>799.45</v>
       </c>
       <c r="Y15" t="n">
-        <v>3437.52</v>
+        <v>812.45</v>
       </c>
       <c r="Z15" t="n">
-        <v>3415.03</v>
+        <v>800.16</v>
       </c>
       <c r="AA15" t="n">
-        <v>3297.64</v>
+        <v>766.72</v>
       </c>
       <c r="AB15" t="n">
-        <v>3432.1</v>
+        <v>804.08</v>
       </c>
       <c r="AC15" t="n">
-        <v>3443.2</v>
+        <v>809.91</v>
       </c>
       <c r="AD15" t="n">
-        <v>3460.1</v>
+        <v>820.38</v>
       </c>
       <c r="AE15" t="n">
-        <v>75.8</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="AF15" t="n">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="AG15" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Strong RSI | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH15" t="n">
         <v>0.15</v>
       </c>
       <c r="AI15" t="n">
-        <v>20.7</v>
+        <v>40.2</v>
       </c>
       <c r="AJ15" t="n">
-        <v>27.5</v>
+        <v>11.5</v>
       </c>
       <c r="AK15" t="n">
-        <v>8.6</v>
+        <v>31.8</v>
       </c>
       <c r="AL15" t="n">
         <v>15</v>
       </c>
       <c r="AM15" t="n">
-        <v>3525.05</v>
+        <v>823.99</v>
       </c>
       <c r="AN15" t="n">
-        <v>3331.53</v>
+        <v>774.6</v>
       </c>
       <c r="AO15" t="inlineStr">
         <is>
-          <t>M&amp;M operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹411,417.18 Cr., a P/E ratio of 20.70, and YoY Revenue Growth of +27.5%, the company demonstrates strong institutional backing, solid operating profit margins (8.61%), and healthy Return on Equity (15.00%).</t>
+          <t>CAMS operates in the Technology sector. With an estimated Market Cap of ₹19,850.15 Cr., a P/E ratio of 40.19, and YoY Revenue Growth of +11.5%, the company demonstrates strong institutional backing, solid operating profit margins (31.79%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP15" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 75.84 (Bullish Momentum Zone), while MACD Line (82.20) trades above Signal (55.88) with an expanding histogram (+26.32). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +3.79% above the 200-day DMA (₹3329.31). Daily volatility envelope is bounded by ATR(14) of ₹85.77.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 74.63 (Bullish Momentum Zone), while MACD Line (7.20) trades above Signal (2.85) with an expanding histogram (+4.35). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +9.30% above the 200-day DMA (₹742.81). Daily volatility envelope is bounded by ATR(14) of ₹21.82.</t>
         </is>
       </c>
       <c r="AQ15" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for M&amp;M. Current Market Price (₹3,426.30) is positioned above the 30-day DMA (₹3,192.86), 50-day DMA (₹3,121.80), and 200-day DMA (₹3,329.31). The price distance from 200 DMA is +3.79%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for CAMS. Current Market Price (₹799.45) is positioned above the 30-day DMA (₹781.22), 50-day DMA (₹778.43), and 200-day DMA (₹742.81). The price distance from 200 DMA is +9.30%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR15" t="inlineStr">
         <is>
-          <t>[3426.3, 3436.58, 3446.86, 3457.14, 3467.42, 3477.69]</t>
+          <t>[799.45, 804.29, 809.12, 813.96, 818.8, 823.64]</t>
         </is>
       </c>
       <c r="AS15" t="inlineStr">
         <is>
-          <t>[3426.3, 3470.89, 3495.38, 3516.56, 3536.03, 3554.41]</t>
+          <t>[799.45, 813.02, 821.47, 829.08, 836.26, 843.15]</t>
         </is>
       </c>
       <c r="AT15" t="inlineStr">
         <is>
-          <t>[3426.3, 3410.85, 3410.47, 3412.57, 3415.95, 3420.16]</t>
+          <t>[799.45, 797.74, 799.87, 802.62, 805.71, 809.0]</t>
         </is>
       </c>
       <c r="AU15" t="n">
-        <v>3415.03</v>
+        <v>800.16</v>
       </c>
     </row>
     <row r="16">
@@ -2999,16 +2999,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>360ONE</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Financial Services</t>
+          <t>Consumer Cyclical</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>48574.43</v>
+        <v>291350.7</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3016,146 +3016,146 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>1193.8</v>
+        <v>316.5</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>₹1187.01 - ₹1203.98</t>
+          <t>₹314.56 - ₹319.42</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>1220.95</v>
+        <v>324.28</v>
       </c>
       <c r="I16" t="n">
-        <v>1113.86</v>
+        <v>288.12</v>
       </c>
       <c r="J16" t="n">
-        <v>1108.1</v>
+        <v>273.72</v>
       </c>
       <c r="K16" t="n">
-        <v>1101.31</v>
+        <v>273.2</v>
       </c>
       <c r="L16" t="n">
-        <v>8.23</v>
+        <v>13.6</v>
       </c>
       <c r="M16" t="n">
-        <v>15.9</v>
+        <v>10.42</v>
       </c>
       <c r="N16" t="n">
-        <v>9.369999999999999</v>
+        <v>9.5</v>
       </c>
       <c r="O16" t="n">
-        <v>6.53</v>
+        <v>0.93</v>
       </c>
       <c r="P16" t="n">
-        <v>33.94</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="Q16" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R16" t="n">
-        <v>51.1</v>
+        <v>50.8</v>
       </c>
       <c r="S16" t="n">
-        <v>0.19</v>
+        <v>0.17</v>
       </c>
       <c r="T16" t="n">
-        <v>-1.8</v>
+        <v>-2</v>
       </c>
       <c r="U16" t="n">
-        <v>51.7</v>
+        <v>53.3</v>
       </c>
       <c r="V16" t="n">
-        <v>2.18</v>
+        <v>2.34</v>
       </c>
       <c r="W16" t="n">
         <v>-0.77</v>
       </c>
       <c r="X16" t="n">
-        <v>1160.83</v>
+        <v>316.14</v>
       </c>
       <c r="Y16" t="n">
-        <v>1201.98</v>
+        <v>321.23</v>
       </c>
       <c r="Z16" t="n">
-        <v>1201.98</v>
+        <v>317.34</v>
       </c>
       <c r="AA16" t="n">
-        <v>1142.89</v>
+        <v>301.92</v>
       </c>
       <c r="AB16" t="n">
-        <v>1189.97</v>
+        <v>315.4</v>
       </c>
       <c r="AC16" t="n">
-        <v>1198.74</v>
+        <v>320.8</v>
       </c>
       <c r="AD16" t="n">
-        <v>1203.67</v>
+        <v>325.1</v>
       </c>
       <c r="AE16" t="n">
-        <v>71.40000000000001</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="AF16" t="n">
-        <v>0.2</v>
+        <v>0.14</v>
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH16" t="n">
         <v>0.15</v>
       </c>
       <c r="AI16" t="n">
-        <v>38.5</v>
+        <v>673.4</v>
       </c>
       <c r="AJ16" t="n">
-        <v>29.9</v>
+        <v>182</v>
       </c>
       <c r="AK16" t="n">
-        <v>26.5</v>
+        <v>0.6</v>
       </c>
       <c r="AL16" t="n">
         <v>15</v>
       </c>
       <c r="AM16" t="n">
-        <v>1230.89</v>
+        <v>328.4</v>
       </c>
       <c r="AN16" t="n">
-        <v>1156.9</v>
+        <v>305.07</v>
       </c>
       <c r="AO16" t="inlineStr">
         <is>
-          <t>360ONE operates in the Financial Services sector. With an estimated Market Cap of ₹48,574.43 Cr., a P/E ratio of 38.52, and YoY Revenue Growth of +29.9%, the company demonstrates strong institutional backing, solid operating profit margins (26.46%), and healthy Return on Equity (15.00%).</t>
+          <t>ETERNAL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹291,350.70 Cr., a P/E ratio of 673.40, and YoY Revenue Growth of +182.0%, the company demonstrates strong institutional backing, solid operating profit margins (0.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP16" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 71.45 (Bullish Momentum Zone), while MACD Line (15.90) trades above Signal (9.37) with an expanding histogram (+6.53). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +8.23% above the 200-day DMA (₹1101.31). Daily volatility envelope is bounded by ATR(14) of ₹33.94.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 68.11 (Bullish Momentum Zone), while MACD Line (10.42) trades above Signal (9.50) with an expanding histogram (+0.93). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +13.60% above the 200-day DMA (₹273.20). Daily volatility envelope is bounded by ATR(14) of ₹9.72.</t>
         </is>
       </c>
       <c r="AQ16" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for 360ONE. Current Market Price (₹1,193.80) is positioned above the 30-day DMA (₹1,113.86), 50-day DMA (₹1,108.10), and 200-day DMA (₹1,101.31). The price distance from 200 DMA is +8.23%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ETERNAL. Current Market Price (₹316.50) is positioned above the 30-day DMA (₹288.12), 50-day DMA (₹273.72), and 200-day DMA (₹273.20). The price distance from 200 DMA is +13.60%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR16" t="inlineStr">
         <is>
-          <t>[1193.8, 1197.38, 1200.96, 1204.54, 1208.13, 1211.71]</t>
+          <t>[316.5, 318.0, 319.49, 320.99, 322.48, 323.98]</t>
         </is>
       </c>
       <c r="AS16" t="inlineStr">
         <is>
-          <t>[1193.8, 1210.96, 1220.16, 1228.06, 1235.28, 1242.07]</t>
+          <t>[316.5, 321.88, 324.99, 327.72, 330.26, 332.67]</t>
         </is>
       </c>
       <c r="AT16" t="inlineStr">
         <is>
-          <t>[1193.8, 1187.2, 1186.56, 1186.91, 1187.76, 1188.94]</t>
+          <t>[316.5, 315.08, 315.37, 315.93, 316.65, 317.46]</t>
         </is>
       </c>
       <c r="AU16" t="n">
-        <v>1201.98</v>
+        <v>317.34</v>
       </c>
     </row>
     <row r="17">
@@ -3175,7 +3175,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>78976.03999999999</v>
+        <v>78710.42999999999</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -3183,98 +3183,98 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1784</v>
+        <v>1778</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>₹1772.36 - ₹1801.46</t>
+          <t>₹1766.18 - ₹1795.74</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>1830.55</v>
+        <v>1825.29</v>
       </c>
       <c r="I17" t="n">
-        <v>1530.06</v>
+        <v>1539.59</v>
       </c>
       <c r="J17" t="n">
-        <v>1489.66</v>
+        <v>1497.56</v>
       </c>
       <c r="K17" t="n">
-        <v>1504.99</v>
+        <v>1505.14</v>
       </c>
       <c r="L17" t="n">
-        <v>16.27</v>
+        <v>18.06</v>
       </c>
       <c r="M17" t="n">
-        <v>74.70999999999999</v>
+        <v>79.86</v>
       </c>
       <c r="N17" t="n">
-        <v>49.28</v>
+        <v>55.39</v>
       </c>
       <c r="O17" t="n">
-        <v>25.43</v>
+        <v>24.47</v>
       </c>
       <c r="P17" t="n">
-        <v>58.19</v>
+        <v>59.12</v>
       </c>
       <c r="Q17" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R17" t="n">
-        <v>51.9</v>
+        <v>50.7</v>
       </c>
       <c r="S17" t="n">
-        <v>0.26</v>
+        <v>0.16</v>
       </c>
       <c r="T17" t="n">
-        <v>-1.84</v>
+        <v>-2.05</v>
       </c>
       <c r="U17" t="n">
-        <v>50</v>
+        <v>51.7</v>
       </c>
       <c r="V17" t="n">
-        <v>7.73</v>
+        <v>7.06</v>
       </c>
       <c r="W17" t="n">
         <v>-0.77</v>
       </c>
       <c r="X17" t="n">
-        <v>1782.35</v>
+        <v>1772.85</v>
       </c>
       <c r="Y17" t="n">
-        <v>1834.6</v>
+        <v>1801.51</v>
       </c>
       <c r="Z17" t="n">
-        <v>1812.18</v>
+        <v>1750.26</v>
       </c>
       <c r="AA17" t="n">
-        <v>1696.71</v>
+        <v>1689.32</v>
       </c>
       <c r="AB17" t="n">
-        <v>1785.27</v>
+        <v>1783.27</v>
       </c>
       <c r="AC17" t="n">
-        <v>1812.64</v>
+        <v>1808.64</v>
       </c>
       <c r="AD17" t="n">
-        <v>1841.27</v>
+        <v>1839.27</v>
       </c>
       <c r="AE17" t="n">
-        <v>72.90000000000001</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="AF17" t="n">
-        <v>0.19</v>
+        <v>0.24</v>
       </c>
       <c r="AG17" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH17" t="n">
         <v>0.15</v>
       </c>
       <c r="AI17" t="n">
-        <v>36.5</v>
+        <v>36.4</v>
       </c>
       <c r="AJ17" t="n">
         <v>49.9</v>
@@ -3286,43 +3286,43 @@
         <v>15</v>
       </c>
       <c r="AM17" t="n">
-        <v>1858.65</v>
+        <v>1847.01</v>
       </c>
       <c r="AN17" t="n">
-        <v>1718.68</v>
+        <v>1709.64</v>
       </c>
       <c r="AO17" t="inlineStr">
         <is>
-          <t>COFORGE operates in the Technology sector. With an estimated Market Cap of ₹78,976.04 Cr., a P/E ratio of 36.54, and YoY Revenue Growth of +49.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.64%), and healthy Return on Equity (15.00%).</t>
+          <t>COFORGE operates in the Technology sector. With an estimated Market Cap of ₹78,710.43 Cr., a P/E ratio of 36.43, and YoY Revenue Growth of +49.9%, the company demonstrates strong institutional backing, solid operating profit margins (9.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP17" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 72.86 (Bullish Momentum Zone), while MACD Line (74.71) trades above Signal (49.28) with an expanding histogram (+25.43). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +16.27% above the 200-day DMA (₹1504.99). Daily volatility envelope is bounded by ATR(14) of ₹58.19.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 74.64 (Bullish Momentum Zone), while MACD Line (79.86) trades above Signal (55.39) with an expanding histogram (+24.47). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +18.06% above the 200-day DMA (₹1505.14). Daily volatility envelope is bounded by ATR(14) of ₹59.12.</t>
         </is>
       </c>
       <c r="AQ17" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for COFORGE. Current Market Price (₹1,784.00) is positioned above the 30-day DMA (₹1,530.06), 50-day DMA (₹1,489.66), and 200-day DMA (₹1,504.99). The price distance from 200 DMA is +16.27%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for COFORGE. Current Market Price (₹1,778.00) is positioned above the 30-day DMA (₹1,539.59), 50-day DMA (₹1,497.56), and 200-day DMA (₹1,505.14). The price distance from 200 DMA is +18.06%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR17" t="inlineStr">
         <is>
-          <t>[1784.0, 1806.94, 1829.88, 1852.82, 1875.76, 1898.7]</t>
+          <t>[1778.0, 1783.33, 1788.67, 1794.0, 1799.34, 1804.67]</t>
         </is>
       </c>
       <c r="AS17" t="inlineStr">
         <is>
-          <t>[1784.0, 1830.22, 1862.8, 1893.14, 1922.32, 1950.75]</t>
+          <t>[1778.0, 1806.98, 1822.11, 1834.96, 1846.63, 1857.55]</t>
         </is>
       </c>
       <c r="AT17" t="inlineStr">
         <is>
-          <t>[1784.0, 1789.48, 1805.19, 1822.58, 1840.84, 1859.66]</t>
+          <t>[1778.0, 1765.6, 1763.59, 1763.28, 1763.87, 1765.01]</t>
         </is>
       </c>
       <c r="AU17" t="n">
-        <v>1812.18</v>
+        <v>1750.26</v>
       </c>
     </row>
     <row r="18">
@@ -3333,16 +3333,16 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>INDIGO</t>
+          <t>360ONE</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Industrials</t>
+          <t>Financial Services</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>208645.3</v>
+        <v>48257.06</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3350,146 +3350,146 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>5396</v>
+        <v>1186</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>₹5367.71 - ₹5438.43</t>
+          <t>₹1179.21 - ₹1196.18</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>5509.14</v>
+        <v>1213.15</v>
       </c>
       <c r="I18" t="n">
-        <v>5278.02</v>
+        <v>1113.86</v>
       </c>
       <c r="J18" t="n">
-        <v>5043.87</v>
+        <v>1108.1</v>
       </c>
       <c r="K18" t="n">
-        <v>4940.92</v>
+        <v>1101.31</v>
       </c>
       <c r="L18" t="n">
-        <v>9.289999999999999</v>
+        <v>8.23</v>
       </c>
       <c r="M18" t="n">
-        <v>66.64</v>
+        <v>15.9</v>
       </c>
       <c r="N18" t="n">
-        <v>59.95</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="O18" t="n">
-        <v>6.69</v>
+        <v>6.53</v>
       </c>
       <c r="P18" t="n">
-        <v>141.43</v>
+        <v>33.94</v>
       </c>
       <c r="Q18" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R18" t="n">
-        <v>44.2</v>
+        <v>43.8</v>
       </c>
       <c r="S18" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="T18" t="n">
-        <v>-1.84</v>
+        <v>-2.19</v>
       </c>
       <c r="U18" t="n">
         <v>50</v>
       </c>
       <c r="V18" t="n">
-        <v>5.71</v>
+        <v>2.17</v>
       </c>
       <c r="W18" t="n">
         <v>-0.77</v>
       </c>
       <c r="X18" t="n">
-        <v>5357.01</v>
+        <v>1160.63</v>
       </c>
       <c r="Y18" t="n">
-        <v>5515.24</v>
+        <v>1187.15</v>
       </c>
       <c r="Z18" t="n">
-        <v>5378.25</v>
+        <v>1187.15</v>
       </c>
       <c r="AA18" t="n">
-        <v>5183.86</v>
+        <v>1135.09</v>
       </c>
       <c r="AB18" t="n">
-        <v>5401.83</v>
+        <v>1187.97</v>
       </c>
       <c r="AC18" t="n">
-        <v>5418.16</v>
+        <v>1195.04</v>
       </c>
       <c r="AD18" t="n">
-        <v>5440.33</v>
+        <v>1204.07</v>
       </c>
       <c r="AE18" t="n">
-        <v>55.9</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="AF18" t="n">
-        <v>0.28</v>
+        <v>0.2</v>
       </c>
       <c r="AG18" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH18" t="n">
         <v>0.15</v>
       </c>
       <c r="AI18" t="n">
-        <v>23.7</v>
+        <v>39.5</v>
       </c>
       <c r="AJ18" t="n">
-        <v>6.2</v>
+        <v>29.9</v>
       </c>
       <c r="AK18" t="n">
-        <v>3.8</v>
+        <v>26.5</v>
       </c>
       <c r="AL18" t="n">
         <v>15</v>
       </c>
       <c r="AM18" t="n">
-        <v>5586.43</v>
+        <v>1225.23</v>
       </c>
       <c r="AN18" t="n">
-        <v>5219.86</v>
+        <v>1150.2</v>
       </c>
       <c r="AO18" t="inlineStr">
         <is>
-          <t>INDIGO operates in the Industrials sector. With an estimated Market Cap of ₹208,645.30 Cr., a P/E ratio of 23.68, and YoY Revenue Growth of +6.2%, the company demonstrates strong institutional backing, solid operating profit margins (3.79%), and healthy Return on Equity (15.00%).</t>
+          <t>360ONE operates in the Financial Services sector. With an estimated Market Cap of ₹48,257.06 Cr., a P/E ratio of 39.48, and YoY Revenue Growth of +29.9%, the company demonstrates strong institutional backing, solid operating profit margins (26.46%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP18" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 55.89 (Bullish Momentum Zone), while MACD Line (66.64) trades above Signal (59.95) with an expanding histogram (+6.69). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +9.29% above the 200-day DMA (₹4940.92). Daily volatility envelope is bounded by ATR(14) of ₹141.43.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 71.45 (Bullish Momentum Zone), while MACD Line (15.90) trades above Signal (9.37) with an expanding histogram (+6.53). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +8.23% above the 200-day DMA (₹1101.31). Daily volatility envelope is bounded by ATR(14) of ₹33.94.</t>
         </is>
       </c>
       <c r="AQ18" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for INDIGO. Current Market Price (₹5,396.00) is positioned above the 30-day DMA (₹5,278.02), 50-day DMA (₹5,043.87), and 200-day DMA (₹4,940.92). The price distance from 200 DMA is +9.29%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for 360ONE. Current Market Price (₹1,186.00) is positioned above the 30-day DMA (₹1,113.86), 50-day DMA (₹1,108.10), and 200-day DMA (₹1,101.31). The price distance from 200 DMA is +8.23%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR18" t="inlineStr">
         <is>
-          <t>[5396.0, 5431.42, 5466.83, 5502.25, 5537.67, 5573.08]</t>
+          <t>[1186.0, 1189.56, 1193.12, 1196.67, 1200.23, 1203.79]</t>
         </is>
       </c>
       <c r="AS18" t="inlineStr">
         <is>
-          <t>[5396.0, 5487.99, 5546.84, 5600.24, 5650.81, 5699.58]</t>
+          <t>[1186.0, 1203.14, 1212.32, 1220.19, 1227.39, 1234.15]</t>
         </is>
       </c>
       <c r="AT18" t="inlineStr">
         <is>
-          <t>[5396.0, 5388.99, 5406.83, 5428.76, 5452.81, 5478.21]</t>
+          <t>[1186.0, 1179.38, 1178.72, 1179.04, 1179.87, 1181.02]</t>
         </is>
       </c>
       <c r="AU18" t="n">
-        <v>5378.25</v>
+        <v>1187.15</v>
       </c>
     </row>
     <row r="19">
@@ -3509,23 +3509,23 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>87025.75</v>
+        <v>86338.69</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>14313</v>
+        <v>14200</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>₹14228.06 - ₹14440.41</t>
+          <t>₹14115.06 - ₹14327.41</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>14652.77</v>
+        <v>14539.77</v>
       </c>
       <c r="I19" t="n">
         <v>13436.17</v>
@@ -3552,46 +3552,46 @@
         <v>424.71</v>
       </c>
       <c r="Q19" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R19" t="n">
-        <v>51.4</v>
+        <v>43</v>
       </c>
       <c r="S19" t="n">
         <v>0.18</v>
       </c>
       <c r="T19" t="n">
-        <v>-1.88</v>
+        <v>-2.21</v>
       </c>
       <c r="U19" t="n">
-        <v>50</v>
+        <v>48.3</v>
       </c>
       <c r="V19" t="n">
-        <v>5.33</v>
+        <v>5.32</v>
       </c>
       <c r="W19" t="n">
         <v>-0.77</v>
       </c>
       <c r="X19" t="n">
-        <v>14114.08</v>
+        <v>14090.25</v>
       </c>
       <c r="Y19" t="n">
-        <v>14534.33</v>
+        <v>14320.44</v>
       </c>
       <c r="Z19" t="n">
-        <v>14465.73</v>
+        <v>13967.07</v>
       </c>
       <c r="AA19" t="n">
-        <v>13675.93</v>
+        <v>13562.93</v>
       </c>
       <c r="AB19" t="n">
-        <v>14354.33</v>
+        <v>14260.67</v>
       </c>
       <c r="AC19" t="n">
-        <v>14403.66</v>
+        <v>14384.34</v>
       </c>
       <c r="AD19" t="n">
-        <v>14494.33</v>
+        <v>14568.67</v>
       </c>
       <c r="AE19" t="n">
         <v>46.3</v>
@@ -3601,14 +3601,14 @@
       </c>
       <c r="AG19" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH19" t="n">
         <v>0.15</v>
       </c>
       <c r="AI19" t="n">
-        <v>42.1</v>
+        <v>40.7</v>
       </c>
       <c r="AJ19" t="n">
         <v>21.1</v>
@@ -3620,14 +3620,14 @@
         <v>15</v>
       </c>
       <c r="AM19" t="n">
-        <v>14844.31</v>
+        <v>14722.25</v>
       </c>
       <c r="AN19" t="n">
-        <v>13773.23</v>
+        <v>13672.7</v>
       </c>
       <c r="AO19" t="inlineStr">
         <is>
-          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹87,025.75 Cr., a P/E ratio of 42.05, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
+          <t>DIXON operates in the Technology sector. With an estimated Market Cap of ₹86,338.69 Cr., a P/E ratio of 40.67, and YoY Revenue Growth of +21.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.64%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP19" t="inlineStr">
@@ -3637,26 +3637,26 @@
       </c>
       <c r="AQ19" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,313.00) is positioned above the 30-day DMA (₹13,436.17), 50-day DMA (₹12,790.96), and 200-day DMA (₹12,277.90). The price distance from 200 DMA is +16.55%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for DIXON. Current Market Price (₹14,200.00) is positioned above the 30-day DMA (₹13,436.17), 50-day DMA (₹12,790.96), and 200-day DMA (₹12,277.90). The price distance from 200 DMA is +16.55%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR19" t="inlineStr">
         <is>
-          <t>[14313.0, 14355.94, 14398.88, 14441.82, 14484.76, 14527.69]</t>
+          <t>[14200.0, 14242.6, 14285.2, 14327.8, 14370.4, 14413.0]</t>
         </is>
       </c>
       <c r="AS19" t="inlineStr">
         <is>
-          <t>[14313.0, 14525.82, 14639.13, 14736.07, 14824.53, 14907.57]</t>
+          <t>[14200.0, 14412.49, 14525.45, 14622.05, 14710.17, 14792.88]</t>
         </is>
       </c>
       <c r="AT19" t="inlineStr">
         <is>
-          <t>[14313.0, 14228.52, 14218.69, 14221.13, 14229.93, 14242.79]</t>
+          <t>[14200.0, 14115.19, 14105.01, 14107.11, 14115.57, 14128.09]</t>
         </is>
       </c>
       <c r="AU19" t="n">
-        <v>14465.73</v>
+        <v>13967.07</v>
       </c>
     </row>
     <row r="20">
@@ -3667,16 +3667,16 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CAMS</t>
+          <t>NAUKRI</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Communication Services</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>20052.51</v>
+        <v>79807.75</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3684,146 +3684,146 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>807.6</v>
+        <v>1232.1</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>₹803.24 - ₹814.15</t>
+          <t>₹1224.91 - ₹1242.89</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>825.0599999999999</v>
+        <v>1260.86</v>
       </c>
       <c r="I20" t="n">
-        <v>781.22</v>
+        <v>1149.22</v>
       </c>
       <c r="J20" t="n">
-        <v>778.4299999999999</v>
+        <v>1086.45</v>
       </c>
       <c r="K20" t="n">
-        <v>742.8099999999999</v>
+        <v>1148.99</v>
       </c>
       <c r="L20" t="n">
-        <v>9.300000000000001</v>
+        <v>8.09</v>
       </c>
       <c r="M20" t="n">
-        <v>7.2</v>
+        <v>47.94</v>
       </c>
       <c r="N20" t="n">
-        <v>2.85</v>
+        <v>48.71</v>
       </c>
       <c r="O20" t="n">
-        <v>4.35</v>
+        <v>-0.77</v>
       </c>
       <c r="P20" t="n">
-        <v>21.82</v>
+        <v>35.95</v>
       </c>
       <c r="Q20" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R20" t="n">
-        <v>43.8</v>
+        <v>41.2</v>
       </c>
       <c r="S20" t="n">
-        <v>0.2</v>
+        <v>0.18</v>
       </c>
       <c r="T20" t="n">
-        <v>-1.93</v>
+        <v>-2.24</v>
       </c>
       <c r="U20" t="n">
         <v>50</v>
       </c>
       <c r="V20" t="n">
-        <v>6.73</v>
+        <v>12.42</v>
       </c>
       <c r="W20" t="n">
         <v>-0.77</v>
       </c>
       <c r="X20" t="n">
-        <v>802.11</v>
+        <v>1199.92</v>
       </c>
       <c r="Y20" t="n">
-        <v>825.79</v>
+        <v>1216.32</v>
       </c>
       <c r="Z20" t="n">
-        <v>804.9400000000001</v>
+        <v>1216.11</v>
       </c>
       <c r="AA20" t="n">
-        <v>774.87</v>
+        <v>1178.17</v>
       </c>
       <c r="AB20" t="n">
-        <v>808.88</v>
+        <v>1239.53</v>
       </c>
       <c r="AC20" t="n">
-        <v>813.26</v>
+        <v>1249.56</v>
       </c>
       <c r="AD20" t="n">
-        <v>818.9299999999999</v>
+        <v>1267.03</v>
       </c>
       <c r="AE20" t="n">
-        <v>74.59999999999999</v>
+        <v>57.7</v>
       </c>
       <c r="AF20" t="n">
-        <v>0</v>
+        <v>-0.01</v>
       </c>
       <c r="AG20" t="inlineStr">
         <is>
-          <t>Strong RSI | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH20" t="n">
         <v>0.15</v>
       </c>
       <c r="AI20" t="n">
-        <v>42.2</v>
+        <v>55.2</v>
       </c>
       <c r="AJ20" t="n">
-        <v>11.5</v>
+        <v>15.9</v>
       </c>
       <c r="AK20" t="n">
-        <v>31.8</v>
+        <v>44.1</v>
       </c>
       <c r="AL20" t="n">
-        <v>15</v>
+        <v>4.6</v>
       </c>
       <c r="AM20" t="n">
-        <v>830.67</v>
+        <v>1270.33</v>
       </c>
       <c r="AN20" t="n">
-        <v>781.72</v>
+        <v>1192.23</v>
       </c>
       <c r="AO20" t="inlineStr">
         <is>
-          <t>CAMS operates in the Technology sector. With an estimated Market Cap of ₹20,052.51 Cr., a P/E ratio of 42.19, and YoY Revenue Growth of +11.5%, the company demonstrates strong institutional backing, solid operating profit margins (31.79%), and healthy Return on Equity (15.00%).</t>
+          <t>NAUKRI operates in the Communication Services sector. With an estimated Market Cap of ₹79,807.75 Cr., a P/E ratio of 55.18, and YoY Revenue Growth of +15.9%, the company demonstrates strong institutional backing, solid operating profit margins (44.14%), and healthy Return on Equity (4.57%).</t>
         </is>
       </c>
       <c r="AP20" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 74.63 (Bullish Momentum Zone), while MACD Line (7.20) trades above Signal (2.85) with an expanding histogram (+4.35). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +9.30% above the 200-day DMA (₹742.81). Daily volatility envelope is bounded by ATR(14) of ₹21.82.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 57.69 (Bullish Momentum Zone), while MACD Line (47.94) trades below Signal (48.71) with an expanding histogram (-0.77). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +8.09% above the 200-day DMA (₹1148.99). Daily volatility envelope is bounded by ATR(14) of ₹35.95.</t>
         </is>
       </c>
       <c r="AQ20" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for CAMS. Current Market Price (₹807.60) is positioned above the 30-day DMA (₹781.22), 50-day DMA (₹778.43), and 200-day DMA (₹742.81). The price distance from 200 DMA is +9.30%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for NAUKRI. Current Market Price (₹1,232.10) is positioned above the 30-day DMA (₹1,149.22), 50-day DMA (₹1,086.45), and 200-day DMA (₹1,148.99). The price distance from 200 DMA is +8.09%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR20" t="inlineStr">
         <is>
-          <t>[807.6, 813.25, 818.9, 824.55, 830.19, 835.84]</t>
+          <t>[1232.1, 1235.8, 1239.49, 1243.19, 1246.89, 1250.58]</t>
         </is>
       </c>
       <c r="AS20" t="inlineStr">
         <is>
-          <t>[807.6, 821.98, 831.24, 839.66, 847.65, 855.36]</t>
+          <t>[1232.1, 1250.18, 1259.83, 1268.1, 1275.65, 1282.74]</t>
         </is>
       </c>
       <c r="AT20" t="inlineStr">
         <is>
-          <t>[807.6, 806.7, 809.64, 813.21, 817.1, 821.21]</t>
+          <t>[1232.1, 1225.01, 1224.24, 1224.51, 1225.31, 1226.46]</t>
         </is>
       </c>
       <c r="AU20" t="n">
-        <v>804.9400000000001</v>
+        <v>1216.11</v>
       </c>
     </row>
     <row r="21">
@@ -3834,16 +3834,16 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ETERNAL</t>
+          <t>PGEL</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Consumer Cyclical</t>
+          <t>Technology</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>292041.1</v>
+        <v>17447.65</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3851,146 +3851,146 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>317.25</v>
+        <v>609</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>₹315.31 - ₹320.17</t>
+          <t>₹604.73 - ₹615.41</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>325.03</v>
+        <v>626.09</v>
       </c>
       <c r="I21" t="n">
-        <v>288.12</v>
+        <v>584.75</v>
       </c>
       <c r="J21" t="n">
-        <v>273.72</v>
+        <v>552.6900000000001</v>
       </c>
       <c r="K21" t="n">
-        <v>273.2</v>
+        <v>554.3099999999999</v>
       </c>
       <c r="L21" t="n">
-        <v>13.6</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="M21" t="n">
-        <v>10.42</v>
+        <v>14.33</v>
       </c>
       <c r="N21" t="n">
-        <v>9.5</v>
+        <v>15.59</v>
       </c>
       <c r="O21" t="n">
-        <v>0.93</v>
+        <v>-1.26</v>
       </c>
       <c r="P21" t="n">
-        <v>9.720000000000001</v>
+        <v>21.36</v>
       </c>
       <c r="Q21" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R21" t="n">
-        <v>51.2</v>
+        <v>49</v>
       </c>
       <c r="S21" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="T21" t="n">
-        <v>-1.97</v>
+        <v>-2.29</v>
       </c>
       <c r="U21" t="n">
-        <v>53.3</v>
+        <v>55</v>
       </c>
       <c r="V21" t="n">
-        <v>2.34</v>
+        <v>4.8</v>
       </c>
       <c r="W21" t="n">
         <v>-0.77</v>
       </c>
       <c r="X21" t="n">
-        <v>314.5</v>
+        <v>593.99</v>
       </c>
       <c r="Y21" t="n">
-        <v>323.81</v>
+        <v>605.35</v>
       </c>
       <c r="Z21" t="n">
-        <v>320.82</v>
+        <v>605.35</v>
       </c>
       <c r="AA21" t="n">
-        <v>302.67</v>
+        <v>576.95</v>
       </c>
       <c r="AB21" t="n">
-        <v>314.87</v>
+        <v>607.4</v>
       </c>
       <c r="AC21" t="n">
-        <v>319.74</v>
+        <v>617.8</v>
       </c>
       <c r="AD21" t="n">
-        <v>322.22</v>
+        <v>626.6</v>
       </c>
       <c r="AE21" t="n">
-        <v>68.09999999999999</v>
+        <v>42.4</v>
       </c>
       <c r="AF21" t="n">
-        <v>0.14</v>
+        <v>0.01</v>
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Strong RSI | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH21" t="n">
         <v>0.15</v>
       </c>
       <c r="AI21" t="n">
-        <v>675</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="AJ21" t="n">
-        <v>182</v>
+        <v>-10.1</v>
       </c>
       <c r="AK21" t="n">
-        <v>0.6</v>
+        <v>3.7</v>
       </c>
       <c r="AL21" t="n">
-        <v>15</v>
+        <v>6.7</v>
       </c>
       <c r="AM21" t="n">
-        <v>328.81</v>
+        <v>639.54</v>
       </c>
       <c r="AN21" t="n">
-        <v>306.71</v>
+        <v>578.51</v>
       </c>
       <c r="AO21" t="inlineStr">
         <is>
-          <t>ETERNAL operates in the Consumer Cyclical sector. With an estimated Market Cap of ₹292,041.10 Cr., a P/E ratio of 675.00, and YoY Revenue Growth of +182.0%, the company demonstrates strong institutional backing, solid operating profit margins (0.64%), and healthy Return on Equity (15.00%).</t>
+          <t>PGEL operates in the Technology sector. With an estimated Market Cap of ₹17,447.65 Cr., a P/E ratio of 87.88, and YoY Revenue Growth of -10.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.72%), and healthy Return on Equity (6.69%).</t>
         </is>
       </c>
       <c r="AP21" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 68.11 (Bullish Momentum Zone), while MACD Line (10.42) trades above Signal (9.50) with an expanding histogram (+0.93). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +13.60% above the 200-day DMA (₹273.20). Daily volatility envelope is bounded by ATR(14) of ₹9.72.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 42.40 (Consolidation Zone), while MACD Line (14.33) trades below Signal (15.59) with an expanding histogram (-1.26). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +8.78% above the 200-day DMA (₹554.31). Daily volatility envelope is bounded by ATR(14) of ₹21.36.</t>
         </is>
       </c>
       <c r="AQ21" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for ETERNAL. Current Market Price (₹317.25) is positioned above the 30-day DMA (₹288.12), 50-day DMA (₹273.72), and 200-day DMA (₹273.20). The price distance from 200 DMA is +13.60%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PGEL. Current Market Price (₹609.00) is positioned above the 30-day DMA (₹584.75), 50-day DMA (₹552.69), and 200-day DMA (₹554.31). The price distance from 200 DMA is +8.78%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR21" t="inlineStr">
         <is>
-          <t>[317.25, 318.87, 320.5, 322.12, 323.75, 325.37]</t>
+          <t>[609.0, 610.83, 612.65, 614.48, 616.31, 618.13]</t>
         </is>
       </c>
       <c r="AS21" t="inlineStr">
         <is>
-          <t>[317.25, 322.76, 326.0, 328.86, 331.52, 334.07]</t>
+          <t>[609.0, 619.37, 624.74, 629.28, 633.4, 637.24]</t>
         </is>
       </c>
       <c r="AT21" t="inlineStr">
         <is>
-          <t>[317.25, 315.96, 316.37, 317.07, 317.91, 318.85]</t>
+          <t>[609.0, 604.42, 603.59, 603.38, 603.49, 603.8]</t>
         </is>
       </c>
       <c r="AU21" t="n">
-        <v>320.82</v>
+        <v>605.35</v>
       </c>
     </row>
     <row r="22">
@@ -4010,7 +4010,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>11504.88</v>
+        <v>11383.04</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -4018,15 +4018,15 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>129.37</v>
+        <v>128</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>₹128.57 - ₹130.56</t>
+          <t>₹127.2 - ₹129.19</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>132.55</v>
+        <v>131.18</v>
       </c>
       <c r="I22" t="n">
         <v>124.58</v>
@@ -4053,46 +4053,46 @@
         <v>3.98</v>
       </c>
       <c r="Q22" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R22" t="n">
-        <v>45.9</v>
+        <v>43.5</v>
       </c>
       <c r="S22" t="n">
         <v>0.17</v>
       </c>
       <c r="T22" t="n">
-        <v>-2.27</v>
+        <v>-2.29</v>
       </c>
       <c r="U22" t="n">
         <v>46.7</v>
       </c>
       <c r="V22" t="n">
-        <v>3.63</v>
+        <v>3.62</v>
       </c>
       <c r="W22" t="n">
         <v>-0.77</v>
       </c>
       <c r="X22" t="n">
-        <v>124.74</v>
+        <v>124.36</v>
       </c>
       <c r="Y22" t="n">
-        <v>130.58</v>
+        <v>126.34</v>
       </c>
       <c r="Z22" t="n">
-        <v>130.58</v>
+        <v>126.34</v>
       </c>
       <c r="AA22" t="n">
-        <v>123.4</v>
+        <v>122.03</v>
       </c>
       <c r="AB22" t="n">
-        <v>129.55</v>
+        <v>128.69</v>
       </c>
       <c r="AC22" t="n">
-        <v>129.99</v>
+        <v>129.64</v>
       </c>
       <c r="AD22" t="n">
-        <v>130.62</v>
+        <v>131.27</v>
       </c>
       <c r="AE22" t="n">
         <v>58</v>
@@ -4102,14 +4102,14 @@
       </c>
       <c r="AG22" t="inlineStr">
         <is>
-          <t>Inst. Buying (CMF+) | Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Inst. Buying (CMF+) | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH22" t="n">
         <v>0.15</v>
       </c>
       <c r="AI22" t="n">
-        <v>22.7</v>
+        <v>22.4</v>
       </c>
       <c r="AJ22" t="n">
         <v>10.1</v>
@@ -4121,14 +4121,14 @@
         <v>15</v>
       </c>
       <c r="AM22" t="n">
-        <v>135.03</v>
+        <v>133.36</v>
       </c>
       <c r="AN22" t="n">
-        <v>123.59</v>
+        <v>122.2</v>
       </c>
       <c r="AO22" t="inlineStr">
         <is>
-          <t>IEX operates in the Financial Services sector. With an estimated Market Cap of ₹11,504.88 Cr., a P/E ratio of 22.66, and YoY Revenue Growth of +10.1%, the company demonstrates strong institutional backing, solid operating profit margins (66.22%), and healthy Return on Equity (15.00%).</t>
+          <t>IEX operates in the Financial Services sector. With an estimated Market Cap of ₹11,383.04 Cr., a P/E ratio of 22.42, and YoY Revenue Growth of +10.1%, the company demonstrates strong institutional backing, solid operating profit margins (66.22%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP22" t="inlineStr">
@@ -4138,26 +4138,26 @@
       </c>
       <c r="AQ22" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for IEX. Current Market Price (₹129.37) is positioned above the 30-day DMA (₹124.58), 50-day DMA (₹124.02), and 200-day DMA (₹127.98). The price distance from 200 DMA is +1.26%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for IEX. Current Market Price (₹128.00) is positioned above the 30-day DMA (₹124.58), 50-day DMA (₹124.02), and 200-day DMA (₹127.98). The price distance from 200 DMA is +1.26%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR22" t="inlineStr">
         <is>
-          <t>[129.37, 129.76, 130.15, 130.53, 130.92, 131.31]</t>
+          <t>[128.0, 128.38, 128.77, 129.15, 129.54, 129.92]</t>
         </is>
       </c>
       <c r="AS22" t="inlineStr">
         <is>
-          <t>[129.37, 131.35, 132.4, 133.29, 134.11, 134.87]</t>
+          <t>[128.0, 129.98, 131.02, 131.91, 132.72, 133.48]</t>
         </is>
       </c>
       <c r="AT22" t="inlineStr">
         <is>
-          <t>[129.37, 128.56, 128.46, 128.47, 128.53, 128.64]</t>
+          <t>[128.0, 127.19, 127.08, 127.08, 127.15, 127.25]</t>
         </is>
       </c>
       <c r="AU22" t="n">
-        <v>130.58</v>
+        <v>126.34</v>
       </c>
     </row>
     <row r="23">
@@ -4168,330 +4168,163 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PGEL</t>
+          <t>GODREJPROP</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Real Estate</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>17519.27</v>
+        <v>63106.84</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>🟡 MODERATE BUY</t>
+          <t>🔴 AVOID / HOLD</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>611.5</v>
+        <v>2095</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>₹607.23 - ₹617.91</t>
+          <t>₹2080.38 - ₹2116.92</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>628.59</v>
+        <v>2153.46</v>
       </c>
       <c r="I23" t="n">
-        <v>584.75</v>
+        <v>2038.04</v>
       </c>
       <c r="J23" t="n">
-        <v>552.6900000000001</v>
+        <v>1914.43</v>
       </c>
       <c r="K23" t="n">
-        <v>554.3099999999999</v>
+        <v>1879.78</v>
       </c>
       <c r="L23" t="n">
-        <v>8.779999999999999</v>
+        <v>11.66</v>
       </c>
       <c r="M23" t="n">
-        <v>14.33</v>
+        <v>44.12</v>
       </c>
       <c r="N23" t="n">
-        <v>15.59</v>
+        <v>57.51</v>
       </c>
       <c r="O23" t="n">
-        <v>-1.26</v>
+        <v>-13.39</v>
       </c>
       <c r="P23" t="n">
-        <v>21.36</v>
+        <v>73.08</v>
       </c>
       <c r="Q23" t="n">
-        <v>12.11</v>
+        <v>12.17</v>
       </c>
       <c r="R23" t="n">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="S23" t="n">
         <v>0.15</v>
       </c>
       <c r="T23" t="n">
-        <v>-2.28</v>
+        <v>-2.7</v>
       </c>
       <c r="U23" t="n">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="V23" t="n">
-        <v>4.81</v>
+        <v>6.47</v>
       </c>
       <c r="W23" t="n">
         <v>-0.77</v>
       </c>
       <c r="X23" t="n">
-        <v>592.17</v>
+        <v>2025.82</v>
       </c>
       <c r="Y23" t="n">
-        <v>625.75</v>
+        <v>2059.92</v>
       </c>
       <c r="Z23" t="n">
-        <v>625.75</v>
+        <v>2059.92</v>
       </c>
       <c r="AA23" t="n">
-        <v>579.45</v>
+        <v>1985.39</v>
       </c>
       <c r="AB23" t="n">
-        <v>606.8</v>
+        <v>2092.07</v>
       </c>
       <c r="AC23" t="n">
-        <v>616.6</v>
+        <v>2111.94</v>
       </c>
       <c r="AD23" t="n">
-        <v>621.7</v>
+        <v>2128.87</v>
       </c>
       <c r="AE23" t="n">
-        <v>42.4</v>
+        <v>51.8</v>
       </c>
       <c r="AF23" t="n">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="AG23" t="inlineStr">
         <is>
-          <t>Low VIX (12.11) | LSTM Deep Net</t>
+          <t>Vol Spike 2.3x | TTM Squeeze | Low VIX (12.17) | LSTM Deep Net</t>
         </is>
       </c>
       <c r="AH23" t="n">
         <v>0.15</v>
       </c>
       <c r="AI23" t="n">
-        <v>89.8</v>
+        <v>33</v>
       </c>
       <c r="AJ23" t="n">
-        <v>-10.1</v>
+        <v>16.5</v>
       </c>
       <c r="AK23" t="n">
-        <v>3.7</v>
+        <v>30.8</v>
       </c>
       <c r="AL23" t="n">
-        <v>6.7</v>
+        <v>15</v>
       </c>
       <c r="AM23" t="n">
-        <v>641.75</v>
+        <v>2168.04</v>
       </c>
       <c r="AN23" t="n">
-        <v>580.98</v>
+        <v>2023.34</v>
       </c>
       <c r="AO23" t="inlineStr">
         <is>
-          <t>PGEL operates in the Technology sector. With an estimated Market Cap of ₹17,519.27 Cr., a P/E ratio of 89.79, and YoY Revenue Growth of -10.1%, the company demonstrates strong institutional backing, solid operating profit margins (3.72%), and healthy Return on Equity (6.69%).</t>
+          <t>GODREJPROP operates in the Real Estate sector. With an estimated Market Cap of ₹63,106.84 Cr., a P/E ratio of 33.05, and YoY Revenue Growth of +16.5%, the company demonstrates strong institutional backing, solid operating profit margins (30.75%), and healthy Return on Equity (15.00%).</t>
         </is>
       </c>
       <c r="AP23" t="inlineStr">
         <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 42.40 (Consolidation Zone), while MACD Line (14.33) trades below Signal (15.59) with an expanding histogram (-1.26). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +8.78% above the 200-day DMA (₹554.31). Daily volatility envelope is bounded by ATR(14) of ₹21.36.</t>
+          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 51.76 (Consolidation Zone), while MACD Line (44.12) trades below Signal (57.51) with an expanding histogram (-13.39). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +11.66% above the 200-day DMA (₹1879.78). Daily volatility envelope is bounded by ATR(14) of ₹73.08.</t>
         </is>
       </c>
       <c r="AQ23" t="inlineStr">
         <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for PGEL. Current Market Price (₹611.50) is positioned above the 30-day DMA (₹584.75), 50-day DMA (₹552.69), and 200-day DMA (₹554.31). The price distance from 200 DMA is +8.78%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
+          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for GODREJPROP. Current Market Price (₹2,095.00) is positioned above the 30-day DMA (₹2,038.04), 50-day DMA (₹1,914.43), and 200-day DMA (₹1,879.78). The price distance from 200 DMA is +11.66%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
         </is>
       </c>
       <c r="AR23" t="inlineStr">
         <is>
-          <t>[611.5, 613.33, 615.17, 617.0, 618.84, 620.67]</t>
+          <t>[2095.0, 2101.28, 2107.57, 2113.85, 2120.14, 2126.42]</t>
         </is>
       </c>
       <c r="AS23" t="inlineStr">
         <is>
-          <t>[611.5, 621.88, 627.25, 631.81, 635.93, 639.78]</t>
+          <t>[2095.0, 2130.52, 2148.91, 2164.48, 2178.6, 2191.79]</t>
         </is>
       </c>
       <c r="AT23" t="inlineStr">
         <is>
-          <t>[611.5, 606.93, 606.1, 605.9, 606.02, 606.34]</t>
+          <t>[2095.0, 2079.36, 2076.57, 2075.88, 2076.29, 2077.4]</t>
         </is>
       </c>
       <c r="AU23" t="n">
-        <v>625.75</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>GODREJPROP</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Real Estate</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>62748.38</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>🔴 AVOID / HOLD</t>
-        </is>
-      </c>
-      <c r="F24" t="n">
-        <v>2083.1</v>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>₹2068.48 - ₹2105.02</t>
-        </is>
-      </c>
-      <c r="H24" t="n">
-        <v>2141.56</v>
-      </c>
-      <c r="I24" t="n">
-        <v>2038.04</v>
-      </c>
-      <c r="J24" t="n">
-        <v>1914.43</v>
-      </c>
-      <c r="K24" t="n">
-        <v>1879.78</v>
-      </c>
-      <c r="L24" t="n">
-        <v>11.66</v>
-      </c>
-      <c r="M24" t="n">
-        <v>44.12</v>
-      </c>
-      <c r="N24" t="n">
-        <v>57.51</v>
-      </c>
-      <c r="O24" t="n">
-        <v>-13.39</v>
-      </c>
-      <c r="P24" t="n">
-        <v>73.08</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>12.11</v>
-      </c>
-      <c r="R24" t="n">
-        <v>41.5</v>
-      </c>
-      <c r="S24" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="T24" t="n">
-        <v>-2.75</v>
-      </c>
-      <c r="U24" t="n">
-        <v>50</v>
-      </c>
-      <c r="V24" t="n">
-        <v>6.44</v>
-      </c>
-      <c r="W24" t="n">
-        <v>-0.77</v>
-      </c>
-      <c r="X24" t="n">
-        <v>1997.84</v>
-      </c>
-      <c r="Y24" t="n">
-        <v>2122.16</v>
-      </c>
-      <c r="Z24" t="n">
-        <v>2122.16</v>
-      </c>
-      <c r="AA24" t="n">
-        <v>1973.49</v>
-      </c>
-      <c r="AB24" t="n">
-        <v>2086.23</v>
-      </c>
-      <c r="AC24" t="n">
-        <v>2100.26</v>
-      </c>
-      <c r="AD24" t="n">
-        <v>2117.43</v>
-      </c>
-      <c r="AE24" t="n">
-        <v>51.8</v>
-      </c>
-      <c r="AF24" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="AG24" t="inlineStr">
-        <is>
-          <t>Vol Spike 2.3x | TTM Squeeze | Low VIX (12.11) | LSTM Deep Net</t>
-        </is>
-      </c>
-      <c r="AH24" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="AI24" t="n">
-        <v>32.9</v>
-      </c>
-      <c r="AJ24" t="n">
-        <v>16.5</v>
-      </c>
-      <c r="AK24" t="n">
-        <v>30.8</v>
-      </c>
-      <c r="AL24" t="n">
-        <v>15</v>
-      </c>
-      <c r="AM24" t="n">
-        <v>2160.12</v>
-      </c>
-      <c r="AN24" t="n">
-        <v>2010.81</v>
-      </c>
-      <c r="AO24" t="inlineStr">
-        <is>
-          <t>GODREJPROP operates in the Real Estate sector. With an estimated Market Cap of ₹62,748.38 Cr., a P/E ratio of 32.86, and YoY Revenue Growth of +16.5%, the company demonstrates strong institutional backing, solid operating profit margins (30.75%), and healthy Return on Equity (15.00%).</t>
-        </is>
-      </c>
-      <c r="AP24" t="inlineStr">
-        <is>
-          <t>Technical indicators confirm a Positive CAR Super Breakout. RSI(14) is currently at 51.76 (Consolidation Zone), while MACD Line (44.12) trades below Signal (57.51) with an expanding histogram (-13.39). Moving Averages are aligned in perfect Golden Stack (CMP &gt; 30 DMA &gt; 50 DMA &gt; 200 DMA) with price trading +11.66% above the 200-day DMA (₹1879.78). Daily volatility envelope is bounded by ATR(14) of ₹73.08.</t>
-        </is>
-      </c>
-      <c r="AQ24" t="inlineStr">
-        <is>
-          <t>Initialization.py scanner logic confirms a CAR (Cumulative Average Return) Super Breakout for GODREJPROP. Current Market Price (₹2,083.10) is positioned above the 30-day DMA (₹2,038.04), 50-day DMA (₹1,914.43), and 200-day DMA (₹1,879.78). The price distance from 200 DMA is +11.66%, indicating a high-conviction institutional momentum stack across short, medium, and long-term trend horizons.</t>
-        </is>
-      </c>
-      <c r="AR24" t="inlineStr">
-        <is>
-          <t>[2083.1, 2089.35, 2095.6, 2101.85, 2108.1, 2114.35]</t>
-        </is>
-      </c>
-      <c r="AS24" t="inlineStr">
-        <is>
-          <t>[2083.1, 2118.58, 2136.94, 2152.48, 2166.56, 2179.71]</t>
-        </is>
-      </c>
-      <c r="AT24" t="inlineStr">
-        <is>
-          <t>[2083.1, 2067.43, 2064.6, 2063.88, 2064.25, 2065.33]</t>
-        </is>
-      </c>
-      <c r="AU24" t="n">
-        <v>2122.16</v>
+        <v>2059.92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>